<commit_message>
Fix totalen en voeg omschrijving/waarvoor-kolommen toe
Totalen als vaste bedragen zodat subtotaal niet meer 0 toont.
Nieuwe kolommen: productomschrijving en waarvoor nodig.

Co-authored-by: bmverhagen <bmverhagen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Materiaalbenodigdheden_Vloerverwarming.xlsx
+++ b/Materiaalbenodigdheden_Vloerverwarming.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Bestelchecklist" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Boodschappenlijst'!$A$5:$L$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Boodschappenlijst'!$A$5:$N$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -144,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -178,7 +178,11 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -545,10 +549,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
@@ -568,7 +572,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>MAGNUM SlimFit 12 (lage opbouw ~14 mm) + PE-RT 12×1,5 mm</t>
+          <t>MAGNUM SlimFit 12 (~14 mm) + PE-RT 12×1,5 mm</t>
         </is>
       </c>
     </row>
@@ -592,7 +596,7 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>4 groepen (kamer 2× ±60–65 m, studeerkamer 1× ±80 m, +1)</t>
+          <t>4 groepen (kamer 2×, studeerkamer 1×, +1 reserve)</t>
         </is>
       </c>
     </row>
@@ -604,7 +608,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Kreisel Gruntolit-W 301 + Kreisel 418 (vezel)</t>
+          <t>Kreisel Gruntolit-W 301 + Kreisel 418</t>
         </is>
       </c>
     </row>
@@ -616,26 +620,25 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>H64-CC + master + 2 slave thermostaten + 4 actuators</t>
+          <t>H64-CC + master + 2 slaves + 4 actuators</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Kosten (uit Boodschappenlijst)</t>
+          <t>Kosten</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Totaal incl. BTW (actuele webshopprijzen)</t>
-        </is>
-      </c>
-      <c r="B10" s="5">
-        <f>Boodschappenlijst!H22</f>
-        <v/>
+          <t>Totaal incl. BTW</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>2487.32</v>
       </c>
     </row>
     <row r="11">
@@ -653,35 +656,28 @@
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Hoe te gebruiken</t>
+          <t>Kolommen in Boodschappenlijst</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>1. Open tabblad Boodschappenlijst</t>
+          <t>Omschrijving product = wat het is</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2. Pas gele cellen aan (hoeveelheid/prijs) indien nodig</t>
+          <t>Waarvoor nodig = waarom jij dit artikel nodig hebt</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>3. Klik op Product-URL om te bestellen</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>4. Controleer levertijd opnieuw op de webshop vóór bestelling</t>
+          <t>Totaal = hoeveelheid × prijs (vast bedrag, geen lege formule meer)</t>
         </is>
       </c>
     </row>
@@ -700,21 +696,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="28" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -727,7 +725,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Gebaseerd op jouw 4-groepen plan (±30 m²). Prijzen incl. BTW, gecontroleerd augustus 2026. Levertijden kunnen wijzigen.</t>
+          <t>Prijzen incl. BTW (augustus 2026). Totalen staan als bedragen (werken ook buiten Excel). Pas je een hoeveelheid/prijs aan, herbereken dan de totaalkolom (hoeveelheid × prijs).</t>
         </is>
       </c>
     </row>
@@ -743,7 +741,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="34" customHeight="1">
       <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Nr</t>
@@ -766,46 +764,56 @@
       </c>
       <c r="E5" s="10" t="inlineStr">
         <is>
+          <t>Omschrijving product</t>
+        </is>
+      </c>
+      <c r="F5" s="10" t="inlineStr">
+        <is>
+          <t>Waarvoor nodig</t>
+        </is>
+      </c>
+      <c r="G5" s="10" t="inlineStr">
+        <is>
           <t>Hoeveelheid</t>
         </is>
       </c>
-      <c r="F5" s="10" t="inlineStr">
+      <c r="H5" s="10" t="inlineStr">
         <is>
           <t>Eenheid</t>
         </is>
       </c>
-      <c r="G5" s="10" t="inlineStr">
+      <c r="I5" s="10" t="inlineStr">
         <is>
           <t>Prijs/eenheid incl. BTW</t>
         </is>
       </c>
-      <c r="H5" s="10" t="inlineStr">
+      <c r="J5" s="10" t="inlineStr">
         <is>
           <t>Totaal incl. BTW</t>
         </is>
       </c>
-      <c r="I5" s="10" t="inlineStr">
+      <c r="K5" s="10" t="inlineStr">
         <is>
           <t>Levertijd</t>
         </is>
       </c>
-      <c r="J5" s="10" t="inlineStr">
+      <c r="L5" s="10" t="inlineStr">
         <is>
           <t>Webshop</t>
         </is>
       </c>
-      <c r="K5" s="10" t="inlineStr">
+      <c r="M5" s="10" t="inlineStr">
         <is>
           <t>Product-URL</t>
         </is>
       </c>
-      <c r="L5" s="10" t="inlineStr">
+      <c r="N5" s="10" t="inlineStr">
         <is>
           <t>Opmerking</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1">
+    <row r="6" ht="72" customHeight="1">
       <c r="A6" s="11" t="n">
         <v>1</v>
       </c>
@@ -824,43 +832,52 @@
           <t>W61012</t>
         </is>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="11" t="inlineStr">
+        <is>
+          <t>Kunststof klikmatten (5 platen van 75×100 cm per pak = 3,75 m²) met lage opbouw (~14 mm). De 12 mm verwarmingsbuis klikt in de mat.</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="inlineStr">
+        <is>
+          <t>Vormt de basislaag waarin je de buizen vastlegt over het hele vloeroppervlak (±30 m²).</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="H6" s="11" t="inlineStr">
         <is>
           <t>pak</t>
         </is>
       </c>
-      <c r="G6" s="13" t="n">
+      <c r="I6" s="13" t="n">
         <v>86.94</v>
       </c>
-      <c r="H6" s="14">
-        <f>E6*G6</f>
-        <v/>
-      </c>
-      <c r="I6" s="11" t="inlineStr">
+      <c r="J6" s="14" t="n">
+        <v>695.52</v>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>1 werkdag</t>
         </is>
       </c>
-      <c r="J6" s="11" t="inlineStr">
+      <c r="L6" s="11" t="inlineStr">
         <is>
           <t>Elektramat</t>
         </is>
       </c>
-      <c r="K6" s="15" t="inlineStr">
+      <c r="M6" s="15" t="inlineStr">
         <is>
           <t>https://www.elektramat.nl/magnum-slimfit-12-bevestigingsmat-vloerverwarming-3-75-m2-5-stuks-van-75x100cm-w61012/</t>
         </is>
       </c>
-      <c r="L6" s="11" t="inlineStr">
+      <c r="N6" s="11" t="inlineStr">
         <is>
           <t>8 × 3,75 m² = 30 m² dekking</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1">
+    <row r="7" ht="72" customHeight="1">
       <c r="A7" s="16" t="n">
         <v>2</v>
       </c>
@@ -879,43 +896,52 @@
           <t>W12300</t>
         </is>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="16" t="inlineStr">
+        <is>
+          <t>Zuurstofdichte 5-laags PE-RT vloerverwarmingsbuis ø12 mm. Flexibel, KOMO-gekeurd, max. ±100 m per groep.</t>
+        </is>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>Voert het warme water door de vloer; hiermee leg je de 4 verwarmingscircuits.</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="H7" s="16" t="inlineStr">
         <is>
           <t>rol</t>
         </is>
       </c>
-      <c r="G7" s="13" t="n">
+      <c r="I7" s="13" t="n">
         <v>181.86</v>
       </c>
-      <c r="H7" s="14">
-        <f>E7*G7</f>
-        <v/>
-      </c>
-      <c r="I7" s="16" t="inlineStr">
+      <c r="J7" s="14" t="n">
+        <v>181.86</v>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
         <is>
           <t>1 werkdag</t>
         </is>
       </c>
-      <c r="J7" s="16" t="inlineStr">
+      <c r="L7" s="16" t="inlineStr">
         <is>
           <t>Elektramat</t>
         </is>
       </c>
-      <c r="K7" s="15" t="inlineStr">
+      <c r="M7" s="15" t="inlineStr">
         <is>
           <t>https://www.elektramat.nl/magnum-universele-vloerverwarmingsbuis-5-laags-pe-rt-12x1-5-mm-komo-rol-van-300-meter-w12300/</t>
         </is>
       </c>
-      <c r="L7" s="16" t="inlineStr">
-        <is>
-          <t>Voldoende voor 4 groepen (max. ±100 m/groep)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="36" customHeight="1">
+      <c r="N7" s="16" t="inlineStr">
+        <is>
+          <t>Voldoende voor 4 groepen</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1">
       <c r="A8" s="11" t="n">
         <v>3</v>
       </c>
@@ -934,43 +960,52 @@
           <t>W90012</t>
         </is>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Stalen knelkoppeling: verbindt 12 mm buis aan de ¾″ Euroconus-aansluiting van de verdeler. Set = 2 stuks.</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>Nodig om elke groep (aanvoer + retour) waterdicht op de verdeler aan te sluiten.</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="F8" s="11" t="inlineStr">
+      <c r="H8" s="11" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="G8" s="13" t="n">
+      <c r="I8" s="13" t="n">
         <v>4.69</v>
       </c>
-      <c r="H8" s="14">
-        <f>E8*G8</f>
-        <v/>
-      </c>
-      <c r="I8" s="11" t="inlineStr">
+      <c r="J8" s="14" t="n">
+        <v>18.76</v>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>1 werkdag</t>
         </is>
       </c>
-      <c r="J8" s="11" t="inlineStr">
+      <c r="L8" s="11" t="inlineStr">
         <is>
           <t>Elektramat</t>
         </is>
       </c>
-      <c r="K8" s="15" t="inlineStr">
+      <c r="M8" s="15" t="inlineStr">
         <is>
           <t>https://www.elektramat.nl/magnum-adaptor-euroconus-aansluitkoppeling-12x1-5mm-x-3-4-2-stuks-w90012/</t>
         </is>
       </c>
-      <c r="L8" s="11" t="inlineStr">
-        <is>
-          <t>1 set per groep (aanvoer + retour)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="36" customHeight="1">
+      <c r="N8" s="11" t="inlineStr">
+        <is>
+          <t>1 set per groep</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
       <c r="A9" s="16" t="n">
         <v>4</v>
       </c>
@@ -989,43 +1024,52 @@
           <t>W90125</t>
         </is>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="16" t="inlineStr">
+        <is>
+          <t>Kunststof geleider die de buis in een vaste 90°-hoek houdt zonder knikken.</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Beschermt de buis waar die vanaf de verdeler de vloer in gaat; voorkomt beschadiging en doorstromingsproblemen.</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="F9" s="16" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="G9" s="13" t="n">
+      <c r="I9" s="13" t="n">
         <v>1.18</v>
       </c>
-      <c r="H9" s="14">
-        <f>E9*G9</f>
-        <v/>
-      </c>
-      <c r="I9" s="16" t="inlineStr">
+      <c r="J9" s="14" t="n">
+        <v>4.72</v>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
         <is>
           <t>1–2 werkdagen</t>
         </is>
       </c>
-      <c r="J9" s="16" t="inlineStr">
+      <c r="L9" s="16" t="inlineStr">
         <is>
           <t>123InstallatieMaterialen</t>
         </is>
       </c>
-      <c r="K9" s="15" t="inlineStr">
+      <c r="M9" s="15" t="inlineStr">
         <is>
           <t>https://123installatiematerialen.nl/90-bochtondersteuning-buismaat-o-10-12mm-2-stuks/</t>
         </is>
       </c>
-      <c r="L9" s="16" t="inlineStr">
-        <is>
-          <t>8 stuks totaal; bij opgang naar verdeler</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="36" customHeight="1">
+      <c r="N9" s="16" t="inlineStr">
+        <is>
+          <t>8 stuks totaal</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
       <c r="A10" s="11" t="n">
         <v>5</v>
       </c>
@@ -1044,43 +1088,52 @@
           <t>W61027</t>
         </is>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <t>Spuitlijm (500 ml) om SlimFit-matten te verlijmen op een droge, stofvrije ondervloer. ±1 bus per 5 m².</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>Houdt de matten vast op de bestaande vloer zodat ze niet verschuiven tijdens het leggen en egaliseren.</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="F10" s="11" t="inlineStr">
+      <c r="H10" s="11" t="inlineStr">
         <is>
           <t>bus</t>
         </is>
       </c>
-      <c r="G10" s="13" t="n">
+      <c r="I10" s="13" t="n">
         <v>9.050000000000001</v>
       </c>
-      <c r="H10" s="14">
-        <f>E10*G10</f>
-        <v/>
-      </c>
-      <c r="I10" s="11" t="inlineStr">
+      <c r="J10" s="14" t="n">
+        <v>54.3</v>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>1 werkdag</t>
         </is>
       </c>
-      <c r="J10" s="11" t="inlineStr">
+      <c r="L10" s="11" t="inlineStr">
         <is>
           <t>Elektramat</t>
         </is>
       </c>
-      <c r="K10" s="15" t="inlineStr">
+      <c r="M10" s="15" t="inlineStr">
         <is>
           <t>https://www.elektramat.nl/magnum-contactlijm-voor-verlijmen-magnum-verlegsystemen-w61027/</t>
         </is>
       </c>
-      <c r="L10" s="11" t="inlineStr">
-        <is>
-          <t>±1 bus per 5 m² → 6 bussen voor 30 m²</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="36" customHeight="1">
+      <c r="N10" s="11" t="inlineStr">
+        <is>
+          <t>6 bussen voor 30 m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1">
       <c r="A11" s="16" t="n">
         <v>6</v>
       </c>
@@ -1099,43 +1152,52 @@
           <t>M-90111</t>
         </is>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="16" t="inlineStr">
+        <is>
+          <t>PE-schuimstrook 8 mm dik / 150 mm hoog met kleefrand en flap, rol van 25 m.</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>Plak je rondom tegen de muren: voorkomt koudebruggen en vangt uitzetting van de egaline/dekvloer op.</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="H11" s="16" t="inlineStr">
         <is>
           <t>rol</t>
         </is>
       </c>
-      <c r="G11" s="13" t="n">
+      <c r="I11" s="13" t="n">
         <v>16.9</v>
       </c>
-      <c r="H11" s="14">
-        <f>E11*G11</f>
-        <v/>
-      </c>
-      <c r="I11" s="16" t="inlineStr">
+      <c r="J11" s="14" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
         <is>
           <t>Volgende werkdag</t>
         </is>
       </c>
-      <c r="J11" s="16" t="inlineStr">
+      <c r="L11" s="16" t="inlineStr">
         <is>
           <t>Vloerverwarmingshop</t>
         </is>
       </c>
-      <c r="K11" s="15" t="inlineStr">
+      <c r="M11" s="15" t="inlineStr">
         <is>
           <t>https://vloerverwarmingshop.nl/shop/product/randisolatie-8mm-x-150mm-met-flap-rol-25-meter</t>
         </is>
       </c>
-      <c r="L11" s="16" t="inlineStr">
-        <is>
-          <t>3 × 25 m = 75 m omtrek</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="36" customHeight="1">
+      <c r="N11" s="16" t="inlineStr">
+        <is>
+          <t>3 × 25 m = 75 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="72" customHeight="1">
       <c r="A12" s="11" t="n">
         <v>7</v>
       </c>
@@ -1154,43 +1216,52 @@
           <t>Gruntolit-W 301</t>
         </is>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>Watergedragen hechtprimer (voorstrijk) voor cementgebonden ondergronden, bus 5 liter.</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="inlineStr">
+        <is>
+          <t>Zorgt dat de egaline goed hecht op de ondervloer (en SlimFit-opbouw); zonder primer kan egaline loslaten.</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="H12" s="11" t="inlineStr">
         <is>
           <t>bus 5L</t>
         </is>
       </c>
-      <c r="G12" s="13" t="n">
+      <c r="I12" s="13" t="n">
         <v>9.289999999999999</v>
       </c>
-      <c r="H12" s="14">
-        <f>E12*G12</f>
-        <v/>
-      </c>
-      <c r="I12" s="11" t="inlineStr">
+      <c r="J12" s="14" t="n">
+        <v>18.58</v>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>2–5 werkdagen</t>
         </is>
       </c>
-      <c r="J12" s="11" t="inlineStr">
+      <c r="L12" s="11" t="inlineStr">
         <is>
           <t>EgalineXXL</t>
         </is>
       </c>
-      <c r="K12" s="15" t="inlineStr">
+      <c r="M12" s="15" t="inlineStr">
         <is>
           <t>https://egalinexxl.nl/products/kreisel-gruntolit-w-301-voorstrijk-5l</t>
         </is>
       </c>
-      <c r="L12" s="11" t="inlineStr">
-        <is>
-          <t>2 × 5 L = 10 liter totaal</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="36" customHeight="1">
+      <c r="N12" s="11" t="inlineStr">
+        <is>
+          <t>2 × 5 L = 10 liter</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="72" customHeight="1">
       <c r="A13" s="16" t="n">
         <v>8</v>
       </c>
@@ -1209,43 +1280,52 @@
           <t>418</t>
         </is>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="16" t="inlineStr">
+        <is>
+          <t>Zelfnivellerende, vezelversterkte egaline 1–50 mm. Geschikt over vloerverwarming. Verbruik ±1,5 kg/m² per mm.</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>Gietlaag die buizen en matten inbedt tot een vlakke, sterke vloer klaar voor tegels/PVC/lijmparket.</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="n">
         <v>33</v>
       </c>
-      <c r="F13" s="16" t="inlineStr">
+      <c r="H13" s="16" t="inlineStr">
         <is>
           <t>zak</t>
         </is>
       </c>
-      <c r="G13" s="13" t="n">
+      <c r="I13" s="13" t="n">
         <v>14.87</v>
       </c>
-      <c r="H13" s="14">
-        <f>E13*G13</f>
-        <v/>
-      </c>
-      <c r="I13" s="16" t="inlineStr">
+      <c r="J13" s="14" t="n">
+        <v>490.71</v>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
         <is>
           <t>2–5 werkdagen</t>
         </is>
       </c>
-      <c r="J13" s="16" t="inlineStr">
+      <c r="L13" s="16" t="inlineStr">
         <is>
           <t>EgalineXXL</t>
         </is>
       </c>
-      <c r="K13" s="15" t="inlineStr">
+      <c r="M13" s="15" t="inlineStr">
         <is>
           <t>https://egalinexxl.nl/products/kreisel-418-vezelversterkte-egalisatie-25kg-1-50mm</t>
         </is>
       </c>
-      <c r="L13" s="16" t="inlineStr">
-        <is>
-          <t>Midden van 30–36 zakken; check laagdikte (verbruik ±1,5 kg/m²/mm)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="36" customHeight="1">
+      <c r="N13" s="16" t="inlineStr">
+        <is>
+          <t>Midden van 30–36 zakken; check laagdikte</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="72" customHeight="1">
       <c r="A14" s="11" t="n">
         <v>9</v>
       </c>
@@ -1264,43 +1344,52 @@
           <t>W40004</t>
         </is>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Stalen mengverdeler voor 4 groepen met thermostatische menging, A-label pomp, thermometer en ontluchter.</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>Hart van het systeem: mengt CV-water naar vloertemperatuur en verdeelt het over de 4 groepen.</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="11" t="inlineStr">
+      <c r="H14" s="11" t="inlineStr">
         <is>
           <t>st</t>
         </is>
       </c>
-      <c r="G14" s="13" t="n">
+      <c r="I14" s="13" t="n">
         <v>406.52</v>
       </c>
-      <c r="H14" s="14">
-        <f>E14*G14</f>
-        <v/>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
+      <c r="J14" s="14" t="n">
+        <v>406.52</v>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>1 werkdag</t>
         </is>
       </c>
-      <c r="J14" s="11" t="inlineStr">
+      <c r="L14" s="11" t="inlineStr">
         <is>
           <t>Elektramat</t>
         </is>
       </c>
-      <c r="K14" s="15" t="inlineStr">
+      <c r="M14" s="15" t="inlineStr">
         <is>
           <t>https://www.elektramat.nl/magnum-basic-staal-vloerverwarming-verdeler-4-groeps-incl-a-label-pomp-w40004/</t>
         </is>
       </c>
-      <c r="L14" s="11" t="inlineStr">
-        <is>
-          <t>Inclusief mengregeling + pomp; primaire aansluiting ½″</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="36" customHeight="1">
+      <c r="N14" s="11" t="inlineStr">
+        <is>
+          <t>Primaire aansluiting ½″</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="72" customHeight="1">
       <c r="A15" s="16" t="n">
         <v>10</v>
       </c>
@@ -1319,43 +1408,52 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="16" t="inlineStr">
+        <is>
+          <t>Leidingwerk tussen cv-ketel/warmtepomp en de verdeler (aanvoer warm + retour koel).</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Brengt warm water van de warmtebron naar de verdeler en weer terug; lengte hangt af van de afstand.</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="F15" s="16" t="inlineStr">
+      <c r="H15" s="16" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="G15" s="13" t="n">
+      <c r="I15" s="13" t="n">
         <v>8.5</v>
       </c>
-      <c r="H15" s="14">
-        <f>E15*G15</f>
-        <v/>
-      </c>
-      <c r="I15" s="16" t="inlineStr">
+      <c r="J15" s="14" t="n">
+        <v>85</v>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
         <is>
           <t>1–3 werkdagen</t>
         </is>
       </c>
-      <c r="J15" s="16" t="inlineStr">
+      <c r="L15" s="16" t="inlineStr">
         <is>
           <t>Bouwmarkt / installatiezaak</t>
         </is>
       </c>
-      <c r="K15" s="15" t="inlineStr">
+      <c r="M15" s="15" t="inlineStr">
         <is>
           <t>https://www.elektramat.nl/bonfix-meerlagenbuis-alu-pers-systeembuis-16mm-x-2-0mm-op-rol-25-meter-2002715/</t>
         </is>
       </c>
-      <c r="L15" s="16" t="inlineStr">
-        <is>
-          <t>Lengte afhankelijk van afstand cv→verdeler; pas meters aan</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="36" customHeight="1">
+      <c r="N15" s="16" t="inlineStr">
+        <is>
+          <t>Pas meters aan op jouw situatie</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="72" customHeight="1">
       <c r="A16" s="11" t="n">
         <v>11</v>
       </c>
@@ -1374,43 +1472,52 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Afsluitkranen en hulpstukken om de verdeler te kunnen afsluiten en aan te koppelen op het CV-net.</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Maakt service mogelijk (verdeler demontabel/afsluitbaar) zonder het hele CV-systeem leeg te laten.</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="11" t="inlineStr">
+      <c r="H16" s="11" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="G16" s="13" t="n">
+      <c r="I16" s="13" t="n">
         <v>34.95</v>
       </c>
-      <c r="H16" s="14">
-        <f>E16*G16</f>
-        <v/>
-      </c>
-      <c r="I16" s="11" t="inlineStr">
+      <c r="J16" s="14" t="n">
+        <v>34.95</v>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>1–3 werkdagen</t>
         </is>
       </c>
-      <c r="J16" s="11" t="inlineStr">
+      <c r="L16" s="11" t="inlineStr">
         <is>
           <t>Online-vloerverwarming</t>
         </is>
       </c>
-      <c r="K16" s="15" t="inlineStr">
+      <c r="M16" s="15" t="inlineStr">
         <is>
           <t>https://online-vloerverwarming.nl/kogelkraan-set-1-rvs-verdeler/</t>
         </is>
       </c>
-      <c r="L16" s="11" t="inlineStr">
-        <is>
-          <t>Controleer of jouw verdeler al primaire afsluiters heeft (Basic Staal vaak wel)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="36" customHeight="1">
+      <c r="N16" s="11" t="inlineStr">
+        <is>
+          <t>Check of Basic Staal al primaire afsluiters heeft</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="72" customHeight="1">
       <c r="A17" s="16" t="n">
         <v>12</v>
       </c>
@@ -1429,43 +1536,52 @@
           <t>W81004</t>
         </is>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="E17" s="16" t="inlineStr">
+        <is>
+          <t>Bedrade zonecontroller (max. 8 zones) inclusief master WiFi-thermostaat met app-bediening.</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="inlineStr">
+        <is>
+          <t>Stuurt de actuators aan op basis van ruimtetemperatuur; masterthermostaat = hoofdbediening + WiFi.</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="16" t="inlineStr">
+      <c r="H17" s="16" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="G17" s="13" t="n">
+      <c r="I17" s="13" t="n">
         <v>225</v>
       </c>
-      <c r="H17" s="14">
-        <f>E17*G17</f>
-        <v/>
-      </c>
-      <c r="I17" s="16" t="inlineStr">
-        <is>
-          <t>1–2 werkdagen (vaak dinsdag)</t>
-        </is>
-      </c>
-      <c r="J17" s="16" t="inlineStr">
+      <c r="J17" s="14" t="n">
+        <v>225</v>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>1–2 werkdagen</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
         <is>
           <t>Vloerverwarmingstore</t>
         </is>
       </c>
-      <c r="K17" s="15" t="inlineStr">
+      <c r="M17" s="15" t="inlineStr">
         <is>
           <t>https://www.vloerverwarmingstore.nl/p/h64-cc-regelunit-cc-regelunit-en-h64-mt-thermostaat-ral-9011-zwart</t>
         </is>
       </c>
-      <c r="L17" s="16" t="inlineStr">
-        <is>
-          <t>Masterthermostaat zit in deze set – niet apart bestellen</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="36" customHeight="1">
+      <c r="N17" s="16" t="inlineStr">
+        <is>
+          <t>Master zit in deze set – niet apart bestellen</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="72" customHeight="1">
       <c r="A18" s="11" t="n">
         <v>13</v>
       </c>
@@ -1484,43 +1600,52 @@
           <t>W81003</t>
         </is>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Extra bedrade programmeerbare ruimtethermostaat (slave) voor het H64-systeem.</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="inlineStr">
+        <is>
+          <t>Nodig voor aparte temperatuurregeling in de 2e en 3e ruimte (naast de master).</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="11" t="inlineStr">
+      <c r="H18" s="11" t="inlineStr">
         <is>
           <t>st</t>
         </is>
       </c>
-      <c r="G18" s="13" t="n">
+      <c r="I18" s="13" t="n">
         <v>57.95</v>
       </c>
-      <c r="H18" s="14">
-        <f>E18*G18</f>
-        <v/>
-      </c>
-      <c r="I18" s="11" t="inlineStr">
+      <c r="J18" s="14" t="n">
+        <v>115.9</v>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>1–2 werkdagen</t>
         </is>
       </c>
-      <c r="J18" s="11" t="inlineStr">
+      <c r="L18" s="11" t="inlineStr">
         <is>
           <t>Vloerverwarmingstore</t>
         </is>
       </c>
-      <c r="K18" s="15" t="inlineStr">
+      <c r="M18" s="15" t="inlineStr">
         <is>
           <t>https://www.vloerverwarmingstore.nl/p/h64-st-klokthermostaat-bedrade-ruimtethermostaat</t>
         </is>
       </c>
-      <c r="L18" s="11" t="inlineStr">
-        <is>
-          <t>Extra zones (bijv. 2e en 3e ruimte)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="36" customHeight="1">
+      <c r="N18" s="11" t="inlineStr">
+        <is>
+          <t>2 extra zones</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="72" customHeight="1">
       <c r="A19" s="16" t="n">
         <v>14</v>
       </c>
@@ -1539,43 +1664,52 @@
           <t>W80003</t>
         </is>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="16" t="inlineStr">
+        <is>
+          <t>Elektrische thermomotor (normaal gesloten) die op de groepsafsluiter van de verdeler past.</t>
+        </is>
+      </c>
+      <c r="F19" s="16" t="inlineStr">
+        <is>
+          <t>Opent/sluit per groep de watertoevoer wanneer die ruimte warmte vraagt of voldoende warm is.</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="F19" s="16" t="inlineStr">
+      <c r="H19" s="16" t="inlineStr">
         <is>
           <t>st</t>
         </is>
       </c>
-      <c r="G19" s="13" t="n">
+      <c r="I19" s="13" t="n">
         <v>19.95</v>
       </c>
-      <c r="H19" s="14">
-        <f>E19*G19</f>
-        <v/>
-      </c>
-      <c r="I19" s="16" t="inlineStr">
+      <c r="J19" s="14" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
         <is>
           <t>1–2 werkdagen</t>
         </is>
       </c>
-      <c r="J19" s="16" t="inlineStr">
+      <c r="L19" s="16" t="inlineStr">
         <is>
           <t>Vloerverwarmingstore</t>
         </is>
       </c>
-      <c r="K19" s="15" t="inlineStr">
+      <c r="M19" s="15" t="inlineStr">
         <is>
           <t>https://www.vloerverwarmingstore.nl/p/mw-a-actuator-nc-magnum-actuator-normaal-gesloten</t>
         </is>
       </c>
-      <c r="L19" s="16" t="inlineStr">
-        <is>
-          <t>1 actuator per groep</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="36" customHeight="1">
+      <c r="N19" s="16" t="inlineStr">
+        <is>
+          <t>1 per groep = 4 stuks</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="72" customHeight="1">
       <c r="A20" s="11" t="n">
         <v>15</v>
       </c>
@@ -1594,65 +1728,73 @@
           <t>—</t>
         </is>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E20" s="11" t="inlineStr">
+        <is>
+          <t>230V voedingskabel en eventueel signaaldraad tussen thermostaten, regelunit en pomp.</t>
+        </is>
+      </c>
+      <c r="F20" s="11" t="inlineStr">
+        <is>
+          <t>Levert stroom aan pomp + H64-regelunit en verbindt de thermostaten met de controller.</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="11" t="inlineStr">
+      <c r="H20" s="11" t="inlineStr">
         <is>
           <t>kleinmateriaal</t>
         </is>
       </c>
-      <c r="G20" s="13" t="n">
+      <c r="I20" s="13" t="n">
         <v>25</v>
       </c>
-      <c r="H20" s="14">
-        <f>E20*G20</f>
-        <v/>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
+      <c r="J20" s="14" t="n">
+        <v>25</v>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>Direct / bouwmarkt</t>
         </is>
       </c>
-      <c r="J20" s="11" t="inlineStr">
+      <c r="L20" s="11" t="inlineStr">
         <is>
           <t>Bouwmarkt</t>
         </is>
       </c>
-      <c r="K20" s="15" t="inlineStr">
+      <c r="M20" s="15" t="inlineStr">
         <is>
           <t>https://www.gamma.nl/assortiment/elektra/elektradraad-en-kabel</t>
         </is>
       </c>
-      <c r="L20" s="11" t="inlineStr">
+      <c r="N20" s="11" t="inlineStr">
         <is>
           <t>Laat aansluiting bij voorkeur door elektricien doen</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="F22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>Subtotaal materiaal</t>
         </is>
       </c>
-      <c r="H22" s="17">
-        <f>SUM(H6:H20)</f>
-        <v/>
+      <c r="J22" s="17" t="n">
+        <v>2487.32</v>
       </c>
     </row>
     <row r="23">
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Raming bandbreedte (zoals in chat)</t>
-        </is>
-      </c>
-      <c r="G23" s="18" t="inlineStr">
+      <c r="H23" s="8" t="inlineStr">
+        <is>
+          <t>Chat-raming destijds</t>
+        </is>
+      </c>
+      <c r="I23" s="18" t="inlineStr">
         <is>
           <t>€ 2.800 – € 3.100</t>
         </is>
       </c>
-      <c r="H23" s="8" t="inlineStr">
+      <c r="J23" s="19" t="inlineStr">
         <is>
           <t>(bij hogere webshopprijzen / meer egaline)</t>
         </is>
@@ -1668,50 +1810,42 @@
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>Geel = aanpasbare hoeveelheid/prijs. Groen = berekend totaal. Klik op Product-URL om de webshop te openen.</t>
+          <t>Geel = hoeveelheid/prijs aanpasbaar. Groen = totaal (al ingevuld als bedrag). Wijzig je hoeveelheid of prijs: zet in kolom Totaal de formule =G×I (bijv. =G6*I6) of reken zelf na.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>Niet meegenomen: arbeidsloon, eindafwerking (tegel/PVC/hout), elektra-aansluiting door professional, afvoer oud materiaal.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
-        <is>
-          <t>H64 masterthermostaat staat niet apart: die zit in regelunit-set W81004.</t>
+          <t>H64 masterthermostaat staat niet apart: die zit in regelunit-set W81004. Arbeid en eindafwerking zijn niet meegenomen.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:L20"/>
-  <mergeCells count="6">
-    <mergeCell ref="A26:L26"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="A28:L28"/>
-    <mergeCell ref="A27:L27"/>
+  <autoFilter ref="A5:N20"/>
+  <mergeCells count="5">
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="A27:N27"/>
+    <mergeCell ref="A26:N26"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M7" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M8" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M9" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M10" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M11" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M12" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M13" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M14" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M15" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M16" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M17" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M18" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M19" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M20" r:id="rId15"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1723,14 +1857,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="70" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1748,256 +1883,336 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
+          <t>Waarvoor nodig</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
           <t>Besteld?</t>
         </is>
       </c>
-      <c r="C3" s="10" t="inlineStr">
-        <is>
-          <t>Webshop ordernr</t>
-        </is>
-      </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>Verwachte leverdatum</t>
+          <t>Ordernr</t>
         </is>
       </c>
       <c r="E3" s="10" t="inlineStr">
         <is>
+          <t>Leverdatum</t>
+        </is>
+      </c>
+      <c r="F3" s="10" t="inlineStr">
+        <is>
           <t>Ontvangen?</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+    <row r="4" ht="40" customHeight="1">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>MAGNUM SlimFit 12 bevestigingsmat 3,75 m² (5 platen 75×100 cm)</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Vormt de basislaag waarin je de buizen vastlegt over het hele vloeroppervlak (±30 m²).</t>
+        </is>
+      </c>
+      <c r="C4" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C4" s="20" t="n"/>
-      <c r="D4" s="20" t="n"/>
-      <c r="E4" s="20" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="D4" s="22" t="n"/>
+      <c r="E4" s="22" t="n"/>
+      <c r="F4" s="22" t="n"/>
+    </row>
+    <row r="5" ht="40" customHeight="1">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>MAGNUM PE-RT buis 12×1,5 mm KOMO – rol 300 m</t>
         </is>
       </c>
-      <c r="B5" s="20" t="inlineStr">
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Voert het warme water door de vloer; hiermee leg je de 4 verwarmingscircuits.</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C5" s="20" t="n"/>
-      <c r="D5" s="20" t="n"/>
-      <c r="E5" s="20" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="22" t="n"/>
+      <c r="F5" s="22" t="n"/>
+    </row>
+    <row r="6" ht="40" customHeight="1">
+      <c r="A6" s="20" t="inlineStr">
         <is>
           <t>MAGNUM Euroconus / adaptor 12×1,5 mm × ¾″ (set van 2)</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Nodig om elke groep (aanvoer + retour) waterdicht op de verdeler aan te sluiten.</t>
+        </is>
+      </c>
+      <c r="C6" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C6" s="20" t="n"/>
-      <c r="D6" s="20" t="n"/>
-      <c r="E6" s="20" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="22" t="n"/>
+      <c r="F6" s="22" t="n"/>
+    </row>
+    <row r="7" ht="40" customHeight="1">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>MAGNUM 90° bochtondersteuning ø10–12 mm (set van 2)</t>
         </is>
       </c>
-      <c r="B7" s="20" t="inlineStr">
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Beschermt de buis waar die vanaf de verdeler de vloer in gaat; voorkomt beschadiging en doorstromingsproblemen.</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n"/>
-      <c r="D7" s="20" t="n"/>
-      <c r="E7" s="20" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="19" t="inlineStr">
+      <c r="D7" s="22" t="n"/>
+      <c r="E7" s="22" t="n"/>
+      <c r="F7" s="22" t="n"/>
+    </row>
+    <row r="8" ht="40" customHeight="1">
+      <c r="A8" s="20" t="inlineStr">
         <is>
           <t>MAGNUM Contactlijm SlimFit / verlegsystemen 500 ml</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Houdt de matten vast op de bestaande vloer zodat ze niet verschuiven tijdens het leggen en egaliseren.</t>
+        </is>
+      </c>
+      <c r="C8" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n"/>
-      <c r="D8" s="20" t="n"/>
-      <c r="E8" s="20" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="D8" s="22" t="n"/>
+      <c r="E8" s="22" t="n"/>
+      <c r="F8" s="22" t="n"/>
+    </row>
+    <row r="9" ht="40" customHeight="1">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Randisolatie 8×150 mm met flap – rol 25 m</t>
         </is>
       </c>
-      <c r="B9" s="20" t="inlineStr">
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Plak je rondom tegen de muren: voorkomt koudebruggen en vangt uitzetting van de egaline/dekvloer op.</t>
+        </is>
+      </c>
+      <c r="C9" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n"/>
-      <c r="D9" s="20" t="n"/>
-      <c r="E9" s="20" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="19" t="inlineStr">
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
+      <c r="F9" s="22" t="n"/>
+    </row>
+    <row r="10" ht="40" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Kreisel Gruntolit-W 301 voorstrijk / primer 5 L</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Zorgt dat de egaline goed hecht op de ondervloer (en SlimFit-opbouw); zonder primer kan egaline loslaten.</t>
+        </is>
+      </c>
+      <c r="C10" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n"/>
-      <c r="D10" s="20" t="n"/>
-      <c r="E10" s="20" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="D10" s="22" t="n"/>
+      <c r="E10" s="22" t="n"/>
+      <c r="F10" s="22" t="n"/>
+    </row>
+    <row r="11" ht="40" customHeight="1">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Kreisel 418 vezelversterkte egaline 25 kg (1–50 mm)</t>
         </is>
       </c>
-      <c r="B11" s="20" t="inlineStr">
+      <c r="B11" s="21" t="inlineStr">
+        <is>
+          <t>Gietlaag die buizen en matten inbedt tot een vlakke, sterke vloer klaar voor tegels/PVC/lijmparket.</t>
+        </is>
+      </c>
+      <c r="C11" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n"/>
-      <c r="D11" s="20" t="n"/>
-      <c r="E11" s="20" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="D11" s="22" t="n"/>
+      <c r="E11" s="22" t="n"/>
+      <c r="F11" s="22" t="n"/>
+    </row>
+    <row r="12" ht="40" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>MAGNUM Basic Staal 4-groeps mengverdeler + A-label pomp</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t>Hart van het systeem: mengt CV-water naar vloertemperatuur en verdeelt het over de 4 groepen.</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n"/>
-      <c r="D12" s="20" t="n"/>
-      <c r="E12" s="20" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="D12" s="22" t="n"/>
+      <c r="E12" s="22" t="n"/>
+      <c r="F12" s="22" t="n"/>
+    </row>
+    <row r="13" ht="40" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Aanvoer + retourleiding vanaf cv (meerlagenbuis 16×2 of koper 15 mm)</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B13" s="21" t="inlineStr">
+        <is>
+          <t>Brengt warm water van de warmtebron naar de verdeler en weer terug; lengte hangt af van de afstand.</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C13" s="20" t="n"/>
-      <c r="D13" s="20" t="n"/>
-      <c r="E13" s="20" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="19" t="inlineStr">
+      <c r="D13" s="22" t="n"/>
+      <c r="E13" s="22" t="n"/>
+      <c r="F13" s="22" t="n"/>
+    </row>
+    <row r="14" ht="40" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>Kogelkranen / koppelingen / verloopstukken (set)</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
+        <is>
+          <t>Maakt service mogelijk (verdeler demontabel/afsluitbaar) zonder het hele CV-systeem leeg te laten.</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C14" s="20" t="n"/>
-      <c r="D14" s="20" t="n"/>
-      <c r="E14" s="20" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="D14" s="22" t="n"/>
+      <c r="E14" s="22" t="n"/>
+      <c r="F14" s="22" t="n"/>
+    </row>
+    <row r="15" ht="40" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>MAGNUM H64-CC regelunit + H64-MT master WiFi-thermostaat</t>
         </is>
       </c>
-      <c r="B15" s="20" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>Stuurt de actuators aan op basis van ruimtetemperatuur; masterthermostaat = hoofdbediening + WiFi.</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C15" s="20" t="n"/>
-      <c r="D15" s="20" t="n"/>
-      <c r="E15" s="20" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="D15" s="22" t="n"/>
+      <c r="E15" s="22" t="n"/>
+      <c r="F15" s="22" t="n"/>
+    </row>
+    <row r="16" ht="40" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>MAGNUM H64-ST slave / klokthermostaat</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
+        <is>
+          <t>Nodig voor aparte temperatuurregeling in de 2e en 3e ruimte (naast de master).</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C16" s="20" t="n"/>
-      <c r="D16" s="20" t="n"/>
-      <c r="E16" s="20" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="19" t="inlineStr">
+      <c r="D16" s="22" t="n"/>
+      <c r="E16" s="22" t="n"/>
+      <c r="F16" s="22" t="n"/>
+    </row>
+    <row r="17" ht="40" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>MAGNUM MW-A thermische actuator 230V NC M30×1,5</t>
         </is>
       </c>
-      <c r="B17" s="20" t="inlineStr">
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t>Opent/sluit per groep de watertoevoer wanneer die ruimte warmte vraagt of voldoende warm is.</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C17" s="20" t="n"/>
-      <c r="D17" s="20" t="n"/>
-      <c r="E17" s="20" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="19" t="inlineStr">
+      <c r="D17" s="22" t="n"/>
+      <c r="E17" s="22" t="n"/>
+      <c r="F17" s="22" t="n"/>
+    </row>
+    <row r="18" ht="40" customHeight="1">
+      <c r="A18" s="20" t="inlineStr">
         <is>
           <t>Elektrakabel 230V naar regelunit + pomp (VD-draad / YMvK)</t>
         </is>
       </c>
-      <c r="B18" s="20" t="inlineStr">
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>Levert stroom aan pomp + H64-regelunit en verbindt de thermostaten met de controller.</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="C18" s="20" t="n"/>
-      <c r="D18" s="20" t="n"/>
-      <c r="E18" s="20" t="n"/>
+      <c r="D18" s="22" t="n"/>
+      <c r="E18" s="22" t="n"/>
+      <c r="F18" s="22" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B4:B18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="C4:C18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Nee,Ja,Deels"</formula1>
     </dataValidation>
-    <dataValidation sqref="E4:E18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F4:F18" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Nee,Ja"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Group all materials under Kopje Vloerverwarming
Adds a Kopje column and section banners so future categories
can be added alongside Vloerverwarming.

Co-authored-by: bmverhagen <bmverhagen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Materiaalbenodigdheden_Vloerverwarming.xlsx
+++ b/Materiaalbenodigdheden_Vloerverwarming.xlsx
@@ -7,14 +7,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Projectkort" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Overzicht" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Regeling-keuze" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Boodschappenlijst" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Tado-aansluiting" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Bestelchecklist" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Boodschappenlijst'!$A$5:$O$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Boodschappenlijst'!$A$6:$P$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Bestelchecklist'!$A$4:$G$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -25,7 +26,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="€ #,##0.00"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -48,7 +49,22 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="002874A6"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -61,23 +77,14 @@
       <sz val="11"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="002874A6"/>
-      <sz val="12"/>
+      <color rgb="001B4F72"/>
     </font>
     <font>
       <name val="Calibri"/>
       <color rgb="000563C1"/>
       <sz val="10"/>
       <u val="single"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="7">
@@ -89,12 +96,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCF3CF"/>
+        <fgColor rgb="001B4F72"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001B4F72"/>
+        <fgColor rgb="00D5F5E3"/>
       </patternFill>
     </fill>
     <fill>
@@ -104,7 +111,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D5F5E3"/>
+        <fgColor rgb="00FCF3CF"/>
       </patternFill>
     </fill>
     <fill>
@@ -183,56 +190,62 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="9" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -598,123 +611,149 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>SlimFit-project + Tado/H64 regeling</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+          <t>Materiaallijst project</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Alles staat onder kopjes. Nu: alleen Vloerverwarming. Later kun je andere kopjes toevoegen (bijv. Badkamer, Elektra, Afwerking).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>KOPJE: Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Oppervlak / groepen</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>±30 m² · 4 groepen · 3 ruimten apart</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Systeem</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>MAGNUM SlimFit 12 + PE-RT 12×1,5 + Kreisel egaline</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Gekozen regeling</t>
         </is>
       </c>
-      <c r="B4" s="4">
+      <c r="B7" s="7">
         <f>'Regeling-keuze'!B4</f>
         <v/>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>Kostenvergelijking (incl. BTW)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>Basis materiaal (vloer + verdeler + actuators)</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n">
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Kosten Vloerverwarming (incl. BTW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>Basis (zonder thermostaat-keuze)</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
         <v>2156.42</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>Met Tado draadloos (aanbevolen draadloos)</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="n">
+    <row r="11">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>Met Tado draadloos (3 ruimten)</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="n">
         <v>2543.42</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>Met Tado bedraad (vaak goedkoopst)</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="n">
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>Met Tado bedraad (3 ruimten)</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="n">
         <v>2486.41</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Met Magnum H64</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B13" s="11" t="n">
         <v>2497.32</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>Tado-materialen kort</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Draadloos: 3× Starterskit (Ontvanger + Sensor) ≈ €387 + bestaande 4 actuators</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Bedraad: 1× Starter (thermostaat+Bridge) + 2× Thermostaat X ≈ €330 + bestaande 4 actuators</t>
-        </is>
-      </c>
-    </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Zie tabblad Regeling-keuze voor uitleg per kamer</t>
-        </is>
-      </c>
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>Andere kopjes (later)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Nog leeg – voeg hier later kopjes toe, bijv. Badkamer / Keuken / Elektra / Afwerking</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>(Placeholder)</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="6">
+    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A16:C16"/>
+    <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -726,300 +765,222 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>3 ruimten apart regelen: Magnum H64 of tado°?</t>
-        </is>
-      </c>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>KOPJE: Vloerverwarming — regeling kiezen</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="n"/>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="n"/>
+      <c r="E1" s="4" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>Jouw zones: Kamer 15 m² (2 groepen) · Studeerkamer 10 m² (1 groep) · 3e ruimte (1 groep). Actuators op de verdeler blijven in alle opties nodig.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>3 ruimten apart: Magnum H64 of tado°?</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Zones: Kamer 15 m² (2 groepen) · Studeerkamer 10 m² (1 groep) · 3e ruimte (1 groep). Actuators blijven in alle opties nodig.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Kies hier je regeling →</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Tado draadloos (3 ruimten)</t>
         </is>
       </c>
-      <c r="C4" s="10" t="inlineStr">
-        <is>
-          <t>← wijzig dit veld; totalen op Boodschappenlijst volgen de keuze via kolom Keuze</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+    </row>
+    <row r="7">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Onderdeel</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t>Tado draadloos</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C7" s="15" t="inlineStr">
         <is>
           <t>Tado bedraad</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="D7" s="15" t="inlineStr">
         <is>
           <t>Magnum H64</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E7" s="15" t="inlineStr">
         <is>
           <t>Toelichting</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Ruimten apart</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>Ja – 3 zones</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>Ja – 3 zones</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>Ja – master + 2 slaves</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>Alle drie kunnen 3 kamers apart</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="28" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>App / slim</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>tado° app + Matter</t>
-        </is>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
-        <is>
-          <t>tado° app + Matter</t>
-        </is>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>MAGNUM HeatLink app</t>
-        </is>
-      </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>Tado: HomeKit/Alexa/Google/Matter</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Hardware</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>3× Starterskit draadloos</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>1× Starter + 2× bedrade thermostaat</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>1× H64-CC + 2× H64-ST</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr"/>
-    </row>
-    <row r="10" ht="28" customHeight="1">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Bij verdeler</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>3× Ontvanger X → actuators</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
-        <is>
-          <t>Bedrading thermostaat → actuators</t>
-        </is>
-      </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Bedrading → actuators</t>
+        </is>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>H64-unit → actuators</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
-        <is>
-          <t>Kamer met 2 groepen: 2 actuators parallel</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="28" customHeight="1">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
+        <is>
+          <t>2 groepen in 1 kamer = actuators parallel</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Actuators 4×</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>Ja, houden</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>Ja, houden</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>Ja, houden</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>MW-A 230V NC op verdeler</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="28" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Indicatie regeling only</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Indicatie regeling</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>± € 387</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>± € 330</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="D12" s="16" t="inlineStr">
         <is>
           <t>± € 341</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
-          <t>Excl. basisvloerverwarming</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="28" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>Levertijd</t>
-        </is>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>2–4 werkdagen</t>
-        </is>
-      </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>2–4 werkdagen</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>1–2 werkdagen</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Hoe Tado de 3 ruimten aanstuurt</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>Per ruimte meet een tado°-thermostaat/sensor de temperatuur. Bij warmtevraag schakelt de bijbehorende Ontvanger X (draadloos) of het relais van de bedrade thermostaat de 230V-actuators van die zone op de verdeler. Kamer 15 m² heeft 2 groepen → koppel beide actuators van die kamer aan dezelfde Tado-zone. Studeerkamer en 3e ruimte elk 1 actuator/zone. De mengverdeler + pomp blijven gewoon hun werk doen; Tado regelt alleen open/dicht per kamer. H64-regelunit + H64-thermostaten koop je dan NIET.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>Bron: tado° Help – meerdere vloerverwarmingszones = 1 smart thermostat / starterkit per zone.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="15" t="inlineStr">
-        <is>
-          <t>https://help.tado.com/en/articles/8953202-how-does-tado-x-control-underfloor-heating-systems</t>
+      <c r="E12" s="16" t="inlineStr">
+        <is>
+          <t>Excl. basis</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Koop niet zowel H64 als Tado. Filter in Boodschappenlijst op kolom Kopje = Vloerverwarming en Keuze.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A14:E14"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A16:E18"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Tado draadloos (3 ruimten),Tado bedraad (3 ruimten),Magnum H64"</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1030,1531 +991,1690 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O33"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="48" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
-    <col width="40" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
     <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="42" customWidth="1" min="14" max="14"/>
-    <col width="28" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Boodschappenlijst – SlimFit + regeling (H64 of Tado)</t>
+          <t>Boodschappenlijst per kopje</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
-        <is>
-          <t>Totalen zijn vaste bedragen. Filter kolom Keuze op jouw regeling. Geel = aanpasbaar.</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Kolom Kopje groepeert alles. Nu alles = Vloerverwarming. Later: nieuwe rijen met ander kopje toevoegen. Totalen = vaste bedragen.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Actieve regeling (zelfde als Regeling-keuze!B4)</t>
-        </is>
-      </c>
-      <c r="B3" s="4">
-        <f>IFERROR('Regeling-keuze'!B4,"Tado draadloos (3 ruimten)")</f>
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Actieve regeling</t>
+        </is>
+      </c>
+      <c r="B3" s="7">
+        <f>IFERROR('Regeling-keuze'!B5,"Tado draadloos (3 ruimten)")</f>
         <v/>
       </c>
-      <c r="C3" s="16" t="n"/>
-      <c r="D3" s="17" t="n"/>
-    </row>
-    <row r="5" ht="34" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="C3" s="17" t="n"/>
+      <c r="D3" s="18" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>KOPJE: Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n"/>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+      <c r="I5" s="4" t="n"/>
+      <c r="J5" s="4" t="n"/>
+      <c r="K5" s="4" t="n"/>
+      <c r="L5" s="4" t="n"/>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="n"/>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Kopje</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>Nr</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>Keuze</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="D6" s="15" t="inlineStr">
         <is>
           <t>Categorie</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="E6" s="15" t="inlineStr">
         <is>
           <t>Benodigd artikel</t>
         </is>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="F6" s="15" t="inlineStr">
         <is>
           <t>Artikelnr</t>
         </is>
       </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="G6" s="15" t="inlineStr">
         <is>
           <t>Omschrijving product</t>
         </is>
       </c>
-      <c r="G5" s="12" t="inlineStr">
+      <c r="H6" s="15" t="inlineStr">
         <is>
           <t>Waarvoor nodig</t>
         </is>
       </c>
-      <c r="H5" s="12" t="inlineStr">
+      <c r="I6" s="15" t="inlineStr">
         <is>
           <t>Hoeveelheid</t>
         </is>
       </c>
-      <c r="I5" s="12" t="inlineStr">
+      <c r="J6" s="15" t="inlineStr">
         <is>
           <t>Eenheid</t>
         </is>
       </c>
-      <c r="J5" s="12" t="inlineStr">
+      <c r="K6" s="15" t="inlineStr">
         <is>
           <t>Prijs/eenheid incl. BTW</t>
         </is>
       </c>
-      <c r="K5" s="12" t="inlineStr">
+      <c r="L6" s="15" t="inlineStr">
         <is>
           <t>Totaal incl. BTW</t>
         </is>
       </c>
-      <c r="L5" s="12" t="inlineStr">
+      <c r="M6" s="15" t="inlineStr">
         <is>
           <t>Levertijd</t>
         </is>
       </c>
-      <c r="M5" s="12" t="inlineStr">
+      <c r="N6" s="15" t="inlineStr">
         <is>
           <t>Webshop</t>
         </is>
       </c>
-      <c r="N5" s="12" t="inlineStr">
+      <c r="O6" s="15" t="inlineStr">
         <is>
           <t>Product-URL</t>
         </is>
       </c>
-      <c r="O5" s="12" t="inlineStr">
+      <c r="P6" s="15" t="inlineStr">
         <is>
           <t>Opmerking</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="68" customHeight="1">
-      <c r="A6" s="13" t="n">
+    <row r="7" ht="64" customHeight="1">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>Bevestiging</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>MAGNUM SlimFit 12 bevestigingsmat 3,75 m² (5 platen 75×100 cm)</t>
         </is>
       </c>
-      <c r="E6" s="13" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>W61012</t>
         </is>
       </c>
-      <c r="F6" s="13" t="inlineStr">
+      <c r="G7" s="16" t="inlineStr">
         <is>
           <t>Kunststof klikmatten (5 platen van 75×100 cm per pak = 3,75 m²) met lage opbouw (~14 mm). De 12 mm verwarmingsbuis klikt in de mat.</t>
         </is>
       </c>
-      <c r="G6" s="13" t="inlineStr">
+      <c r="H7" s="16" t="inlineStr">
         <is>
           <t>Vormt de basislaag waarin je de buizen vastlegt over het hele vloeroppervlak (±30 m²).</t>
         </is>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="I7" s="20" t="n">
         <v>8</v>
       </c>
-      <c r="I6" s="13" t="inlineStr">
+      <c r="J7" s="16" t="inlineStr">
         <is>
           <t>pak</t>
         </is>
       </c>
-      <c r="J6" s="19" t="n">
+      <c r="K7" s="21" t="n">
         <v>86.94</v>
       </c>
-      <c r="K6" s="20" t="n">
+      <c r="L7" s="22" t="n">
         <v>695.52</v>
       </c>
-      <c r="L6" s="13" t="inlineStr">
+      <c r="M7" s="16" t="inlineStr">
         <is>
           <t>1 werkdag</t>
         </is>
       </c>
-      <c r="M6" s="13" t="inlineStr">
+      <c r="N7" s="16" t="inlineStr">
         <is>
           <t>Elektramat</t>
         </is>
       </c>
-      <c r="N6" s="21" t="inlineStr">
+      <c r="O7" s="23" t="inlineStr">
         <is>
           <t>https://www.elektramat.nl/magnum-slimfit-12-bevestigingsmat-vloerverwarming-3-75-m2-5-stuks-van-75x100cm-w61012/</t>
         </is>
       </c>
-      <c r="O6" s="13" t="inlineStr">
+      <c r="P7" s="16" t="inlineStr">
         <is>
           <t>8 × 3,75 m² = 30 m²</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="68" customHeight="1">
-      <c r="A7" s="13" t="n">
+    <row r="8" ht="64" customHeight="1">
+      <c r="A8" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="D8" s="16" t="inlineStr">
         <is>
           <t>Buis</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>MAGNUM PE-RT buis 12×1,5 mm KOMO – rol 300 m</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>W12300</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
+      <c r="G8" s="16" t="inlineStr">
         <is>
           <t>Zuurstofdichte 5-laags PE-RT vloerverwarmingsbuis ø12 mm. Flexibel, KOMO-gekeurd, max. ±100 m per groep.</t>
         </is>
       </c>
-      <c r="G7" s="13" t="inlineStr">
+      <c r="H8" s="16" t="inlineStr">
         <is>
           <t>Voert het warme water door de vloer; hiermee leg je de 4 verwarmingscircuits.</t>
         </is>
       </c>
-      <c r="H7" s="18" t="n">
+      <c r="I8" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I7" s="13" t="inlineStr">
+      <c r="J8" s="16" t="inlineStr">
         <is>
           <t>rol</t>
         </is>
       </c>
-      <c r="J7" s="19" t="n">
+      <c r="K8" s="21" t="n">
         <v>181.86</v>
       </c>
-      <c r="K7" s="20" t="n">
+      <c r="L8" s="22" t="n">
         <v>181.86</v>
       </c>
-      <c r="L7" s="13" t="inlineStr">
+      <c r="M8" s="16" t="inlineStr">
         <is>
           <t>1 werkdag</t>
         </is>
       </c>
-      <c r="M7" s="13" t="inlineStr">
+      <c r="N8" s="16" t="inlineStr">
         <is>
           <t>Elektramat</t>
         </is>
       </c>
-      <c r="N7" s="21" t="inlineStr">
+      <c r="O8" s="23" t="inlineStr">
         <is>
           <t>https://www.elektramat.nl/magnum-universele-vloerverwarmingsbuis-5-laags-pe-rt-12x1-5-mm-komo-rol-van-300-meter-w12300/</t>
         </is>
       </c>
-      <c r="O7" s="13" t="inlineStr">
+      <c r="P8" s="16" t="inlineStr">
         <is>
           <t>Voldoende voor 4 groepen</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="68" customHeight="1">
-      <c r="A8" s="13" t="n">
+    <row r="9" ht="64" customHeight="1">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C8" s="13" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>Aansluiting</t>
         </is>
       </c>
-      <c r="D8" s="13" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>MAGNUM Euroconus / adaptor 12×1,5 mm × ¾″ (set van 2)</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>W90012</t>
         </is>
       </c>
-      <c r="F8" s="13" t="inlineStr">
+      <c r="G9" s="16" t="inlineStr">
         <is>
           <t>Stalen knelkoppeling: verbindt 12 mm buis aan de ¾″ Euroconus van de verdeler. Set = 2 stuks.</t>
         </is>
       </c>
-      <c r="G8" s="13" t="inlineStr">
+      <c r="H9" s="16" t="inlineStr">
         <is>
           <t>Nodig om elke groep (aanvoer + retour) waterdicht op de verdeler aan te sluiten.</t>
         </is>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="I9" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="I8" s="13" t="inlineStr">
+      <c r="J9" s="16" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="J8" s="19" t="n">
+      <c r="K9" s="21" t="n">
         <v>4.69</v>
       </c>
-      <c r="K8" s="20" t="n">
+      <c r="L9" s="22" t="n">
         <v>18.76</v>
       </c>
-      <c r="L8" s="13" t="inlineStr">
+      <c r="M9" s="16" t="inlineStr">
         <is>
           <t>1 werkdag</t>
         </is>
       </c>
-      <c r="M8" s="13" t="inlineStr">
+      <c r="N9" s="16" t="inlineStr">
         <is>
           <t>Elektramat</t>
         </is>
       </c>
-      <c r="N8" s="21" t="inlineStr">
+      <c r="O9" s="23" t="inlineStr">
         <is>
           <t>https://www.elektramat.nl/magnum-adaptor-euroconus-aansluitkoppeling-12x1-5mm-x-3-4-2-stuks-w90012/</t>
         </is>
       </c>
-      <c r="O8" s="13" t="inlineStr">
+      <c r="P9" s="16" t="inlineStr">
         <is>
           <t>1 set per groep</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="68" customHeight="1">
-      <c r="A9" s="13" t="n">
+    <row r="10" ht="64" customHeight="1">
+      <c r="A10" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="13" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="D10" s="16" t="inlineStr">
         <is>
           <t>Aansluiting</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>MAGNUM 90° bochtondersteuning ø10–12 mm (set van 2)</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>W90125</t>
         </is>
       </c>
-      <c r="F9" s="13" t="inlineStr">
+      <c r="G10" s="16" t="inlineStr">
         <is>
           <t>Kunststof geleider die de buis in een vaste 90°-hoek houdt zonder knikken.</t>
         </is>
       </c>
-      <c r="G9" s="13" t="inlineStr">
+      <c r="H10" s="16" t="inlineStr">
         <is>
           <t>Beschermt de buis waar die vanaf de verdeler de vloer in gaat.</t>
         </is>
       </c>
-      <c r="H9" s="18" t="n">
+      <c r="I10" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="I9" s="13" t="inlineStr">
+      <c r="J10" s="16" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="J9" s="19" t="n">
+      <c r="K10" s="21" t="n">
         <v>1.18</v>
       </c>
-      <c r="K9" s="20" t="n">
+      <c r="L10" s="22" t="n">
         <v>4.72</v>
       </c>
-      <c r="L9" s="13" t="inlineStr">
+      <c r="M10" s="16" t="inlineStr">
         <is>
           <t>1–2 werkdagen</t>
         </is>
       </c>
-      <c r="M9" s="13" t="inlineStr">
+      <c r="N10" s="16" t="inlineStr">
         <is>
           <t>123InstallatieMaterialen</t>
         </is>
       </c>
-      <c r="N9" s="21" t="inlineStr">
+      <c r="O10" s="23" t="inlineStr">
         <is>
           <t>https://123installatiematerialen.nl/90-bochtondersteuning-buismaat-o-10-12mm-2-stuks/</t>
         </is>
       </c>
-      <c r="O9" s="13" t="inlineStr">
+      <c r="P10" s="16" t="inlineStr">
         <is>
           <t>8 stuks totaal</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="68" customHeight="1">
-      <c r="A10" s="13" t="n">
+    <row r="11" ht="64" customHeight="1">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C10" s="13" t="inlineStr">
+      <c r="D11" s="16" t="inlineStr">
         <is>
           <t>Bevestiging</t>
         </is>
       </c>
-      <c r="D10" s="13" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>MAGNUM Contactlijm SlimFit / verlegsystemen 500 ml</t>
         </is>
       </c>
-      <c r="E10" s="13" t="inlineStr">
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>W61027</t>
         </is>
       </c>
-      <c r="F10" s="13" t="inlineStr">
+      <c r="G11" s="16" t="inlineStr">
         <is>
           <t>Spuitlijm (500 ml) om SlimFit-matten te verlijmen. ±1 bus per 5 m².</t>
         </is>
       </c>
-      <c r="G10" s="13" t="inlineStr">
+      <c r="H11" s="16" t="inlineStr">
         <is>
           <t>Houdt de matten vast op de ondervloer tijdens leggen en egaliseren.</t>
         </is>
       </c>
-      <c r="H10" s="18" t="n">
+      <c r="I11" s="20" t="n">
         <v>6</v>
       </c>
-      <c r="I10" s="13" t="inlineStr">
+      <c r="J11" s="16" t="inlineStr">
         <is>
           <t>bus</t>
         </is>
       </c>
-      <c r="J10" s="19" t="n">
+      <c r="K11" s="21" t="n">
         <v>9.050000000000001</v>
       </c>
-      <c r="K10" s="20" t="n">
+      <c r="L11" s="22" t="n">
         <v>54.3</v>
       </c>
-      <c r="L10" s="13" t="inlineStr">
+      <c r="M11" s="16" t="inlineStr">
         <is>
           <t>1 werkdag</t>
         </is>
       </c>
-      <c r="M10" s="13" t="inlineStr">
+      <c r="N11" s="16" t="inlineStr">
         <is>
           <t>Elektramat</t>
         </is>
       </c>
-      <c r="N10" s="21" t="inlineStr">
+      <c r="O11" s="23" t="inlineStr">
         <is>
           <t>https://www.elektramat.nl/magnum-contactlijm-voor-verlijmen-magnum-verlegsystemen-w61027/</t>
         </is>
       </c>
-      <c r="O10" s="13" t="inlineStr">
+      <c r="P11" s="16" t="inlineStr">
         <is>
           <t>6 bussen voor 30 m²</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="68" customHeight="1">
-      <c r="A11" s="13" t="n">
+    <row r="12" ht="64" customHeight="1">
+      <c r="A12" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="D12" s="16" t="inlineStr">
         <is>
           <t>Isolatie</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>Randisolatie 8×150 mm met flap – rol 25 m</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="F12" s="16" t="inlineStr">
         <is>
           <t>M-90111</t>
         </is>
       </c>
-      <c r="F11" s="13" t="inlineStr">
+      <c r="G12" s="16" t="inlineStr">
         <is>
           <t>PE-schuimstrook 8 mm dik / 150 mm hoog met kleefrand en flap, rol 25 m.</t>
         </is>
       </c>
-      <c r="G11" s="13" t="inlineStr">
+      <c r="H12" s="16" t="inlineStr">
         <is>
           <t>Rondom tegen muren: voorkomt koudebruggen en vangt uitzetting op.</t>
         </is>
       </c>
-      <c r="H11" s="18" t="n">
+      <c r="I12" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="I11" s="13" t="inlineStr">
+      <c r="J12" s="16" t="inlineStr">
         <is>
           <t>rol</t>
         </is>
       </c>
-      <c r="J11" s="19" t="n">
+      <c r="K12" s="21" t="n">
         <v>16.9</v>
       </c>
-      <c r="K11" s="20" t="n">
+      <c r="L12" s="22" t="n">
         <v>50.7</v>
       </c>
-      <c r="L11" s="13" t="inlineStr">
+      <c r="M12" s="16" t="inlineStr">
         <is>
           <t>Volgende werkdag</t>
         </is>
       </c>
-      <c r="M11" s="13" t="inlineStr">
+      <c r="N12" s="16" t="inlineStr">
         <is>
           <t>Vloerverwarmingshop</t>
         </is>
       </c>
-      <c r="N11" s="21" t="inlineStr">
+      <c r="O12" s="23" t="inlineStr">
         <is>
           <t>https://vloerverwarmingshop.nl/shop/product/randisolatie-8mm-x-150mm-met-flap-rol-25-meter</t>
         </is>
       </c>
-      <c r="O11" s="13" t="inlineStr">
+      <c r="P12" s="16" t="inlineStr">
         <is>
           <t>3 × 25 m = 75 m</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="68" customHeight="1">
-      <c r="A12" s="13" t="n">
+    <row r="13" ht="64" customHeight="1">
+      <c r="A13" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C12" s="13" t="inlineStr">
+      <c r="D13" s="16" t="inlineStr">
         <is>
           <t>Egalisatie</t>
         </is>
       </c>
-      <c r="D12" s="13" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>Kreisel Gruntolit-W 301 voorstrijk / primer 5 L</t>
         </is>
       </c>
-      <c r="E12" s="13" t="inlineStr">
+      <c r="F13" s="16" t="inlineStr">
         <is>
           <t>Gruntolit-W 301</t>
         </is>
       </c>
-      <c r="F12" s="13" t="inlineStr">
+      <c r="G13" s="16" t="inlineStr">
         <is>
           <t>Watergedragen hechtprimer voor cementgebonden ondergronden, 5 liter.</t>
         </is>
       </c>
-      <c r="G12" s="13" t="inlineStr">
+      <c r="H13" s="16" t="inlineStr">
         <is>
           <t>Zorgt dat egaline goed hecht; zonder primer kan egaline loslaten.</t>
         </is>
       </c>
-      <c r="H12" s="18" t="n">
+      <c r="I13" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="I12" s="13" t="inlineStr">
+      <c r="J13" s="16" t="inlineStr">
         <is>
           <t>bus 5L</t>
         </is>
       </c>
-      <c r="J12" s="19" t="n">
+      <c r="K13" s="21" t="n">
         <v>9.289999999999999</v>
       </c>
-      <c r="K12" s="20" t="n">
+      <c r="L13" s="22" t="n">
         <v>18.58</v>
       </c>
-      <c r="L12" s="13" t="inlineStr">
+      <c r="M13" s="16" t="inlineStr">
         <is>
           <t>2–5 werkdagen</t>
         </is>
       </c>
-      <c r="M12" s="13" t="inlineStr">
+      <c r="N13" s="16" t="inlineStr">
         <is>
           <t>EgalineXXL</t>
         </is>
       </c>
-      <c r="N12" s="21" t="inlineStr">
+      <c r="O13" s="23" t="inlineStr">
         <is>
           <t>https://egalinexxl.nl/products/kreisel-gruntolit-w-301-voorstrijk-5l</t>
         </is>
       </c>
-      <c r="O12" s="13" t="inlineStr">
+      <c r="P13" s="16" t="inlineStr">
         <is>
           <t>2 × 5 L = 10 liter</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="68" customHeight="1">
-      <c r="A13" s="13" t="n">
+    <row r="14" ht="64" customHeight="1">
+      <c r="A14" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="B13" s="13" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>Egalisatie</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>Kreisel 418 vezelversterkte egaline 25 kg (1–50 mm)</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="F14" s="16" t="inlineStr">
         <is>
           <t>418</t>
         </is>
       </c>
-      <c r="F13" s="13" t="inlineStr">
+      <c r="G14" s="16" t="inlineStr">
         <is>
           <t>Zelfnivellerende vezelversterkte egaline 1–50 mm, geschikt over vloerverwarming.</t>
         </is>
       </c>
-      <c r="G13" s="13" t="inlineStr">
+      <c r="H14" s="16" t="inlineStr">
         <is>
           <t>Gietlaag die buizen/matten inbedt tot vlakke vloer klaar voor afwerking.</t>
         </is>
       </c>
-      <c r="H13" s="18" t="n">
+      <c r="I14" s="20" t="n">
         <v>33</v>
       </c>
-      <c r="I13" s="13" t="inlineStr">
+      <c r="J14" s="16" t="inlineStr">
         <is>
           <t>zak</t>
         </is>
       </c>
-      <c r="J13" s="19" t="n">
+      <c r="K14" s="21" t="n">
         <v>14.87</v>
       </c>
-      <c r="K13" s="20" t="n">
+      <c r="L14" s="22" t="n">
         <v>490.71</v>
       </c>
-      <c r="L13" s="13" t="inlineStr">
+      <c r="M14" s="16" t="inlineStr">
         <is>
           <t>2–5 werkdagen</t>
         </is>
       </c>
-      <c r="M13" s="13" t="inlineStr">
+      <c r="N14" s="16" t="inlineStr">
         <is>
           <t>EgalineXXL</t>
         </is>
       </c>
-      <c r="N13" s="21" t="inlineStr">
+      <c r="O14" s="23" t="inlineStr">
         <is>
           <t>https://egalinexxl.nl/products/kreisel-418-vezelversterkte-egalisatie-25kg-1-50mm</t>
         </is>
       </c>
-      <c r="O13" s="13" t="inlineStr">
+      <c r="P14" s="16" t="inlineStr">
         <is>
           <t>Check laagdikte (verbruik ±1,5 kg/m²/mm)</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="68" customHeight="1">
-      <c r="A14" s="13" t="n">
+    <row r="15" ht="64" customHeight="1">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B15" s="16" t="n">
         <v>9</v>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C14" s="13" t="inlineStr">
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>Verdeler</t>
         </is>
       </c>
-      <c r="D14" s="13" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>MAGNUM Basic Staal 4-groeps mengverdeler + A-label pomp</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
+      <c r="F15" s="16" t="inlineStr">
         <is>
           <t>W40004</t>
         </is>
       </c>
-      <c r="F14" s="13" t="inlineStr">
+      <c r="G15" s="16" t="inlineStr">
         <is>
           <t>Stalen mengverdeler 4 groepen met thermostatische menging, A-label pomp, thermometer, ontluchter.</t>
         </is>
       </c>
-      <c r="G14" s="13" t="inlineStr">
+      <c r="H15" s="16" t="inlineStr">
         <is>
           <t>Hart van het systeem: mengt CV-water en verdeelt over de 4 groepen.</t>
         </is>
       </c>
-      <c r="H14" s="18" t="n">
+      <c r="I15" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I14" s="13" t="inlineStr">
+      <c r="J15" s="16" t="inlineStr">
         <is>
           <t>st</t>
         </is>
       </c>
-      <c r="J14" s="19" t="n">
+      <c r="K15" s="21" t="n">
         <v>406.52</v>
       </c>
-      <c r="K14" s="20" t="n">
+      <c r="L15" s="22" t="n">
         <v>406.52</v>
       </c>
-      <c r="L14" s="13" t="inlineStr">
+      <c r="M15" s="16" t="inlineStr">
         <is>
           <t>1 werkdag</t>
         </is>
       </c>
-      <c r="M14" s="13" t="inlineStr">
+      <c r="N15" s="16" t="inlineStr">
         <is>
           <t>Elektramat</t>
         </is>
       </c>
-      <c r="N14" s="21" t="inlineStr">
+      <c r="O15" s="23" t="inlineStr">
         <is>
           <t>https://www.elektramat.nl/magnum-basic-staal-vloerverwarming-verdeler-4-groeps-incl-a-label-pomp-w40004/</t>
         </is>
       </c>
-      <c r="O14" s="13" t="inlineStr">
+      <c r="P15" s="16" t="inlineStr">
         <is>
           <t>Primaire aansluiting ½″</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="68" customHeight="1">
-      <c r="A15" s="13" t="n">
+    <row r="16" ht="64" customHeight="1">
+      <c r="A16" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="n">
         <v>10</v>
       </c>
-      <c r="B15" s="13" t="inlineStr">
+      <c r="C16" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="D16" s="16" t="inlineStr">
         <is>
           <t>CV-aansluiting</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>Aanvoer + retourleiding vanaf cv (meerlagenbuis 16×2 of koper 15 mm)</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="F16" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F15" s="13" t="inlineStr">
+      <c r="G16" s="16" t="inlineStr">
         <is>
           <t>Leidingwerk tussen warmtebron en verdeler (aanvoer + retour).</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr">
+      <c r="H16" s="16" t="inlineStr">
         <is>
           <t>Brengt warm water van cv/wp naar de verdeler; lengte hangt af van afstand.</t>
         </is>
       </c>
-      <c r="H15" s="18" t="n">
+      <c r="I16" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="I15" s="13" t="inlineStr">
+      <c r="J16" s="16" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="J15" s="19" t="n">
+      <c r="K16" s="21" t="n">
         <v>8.5</v>
       </c>
-      <c r="K15" s="20" t="n">
+      <c r="L16" s="22" t="n">
         <v>85</v>
       </c>
-      <c r="L15" s="13" t="inlineStr">
+      <c r="M16" s="16" t="inlineStr">
         <is>
           <t>1–3 werkdagen</t>
         </is>
       </c>
-      <c r="M15" s="13" t="inlineStr">
+      <c r="N16" s="16" t="inlineStr">
         <is>
           <t>Bouwmarkt / installatiezaak</t>
         </is>
       </c>
-      <c r="N15" s="21" t="inlineStr">
+      <c r="O16" s="23" t="inlineStr">
         <is>
           <t>https://www.elektramat.nl/bonfix-meerlagenbuis-alu-pers-systeembuis-16mm-x-2-0mm-op-rol-25-meter-2002715/</t>
         </is>
       </c>
-      <c r="O15" s="13" t="inlineStr">
+      <c r="P16" s="16" t="inlineStr">
         <is>
           <t>Pas meters aan</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="68" customHeight="1">
-      <c r="A16" s="13" t="n">
+    <row r="17" ht="64" customHeight="1">
+      <c r="A17" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="n">
         <v>11</v>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="C17" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C16" s="13" t="inlineStr">
+      <c r="D17" s="16" t="inlineStr">
         <is>
           <t>CV-aansluiting</t>
         </is>
       </c>
-      <c r="D16" s="13" t="inlineStr">
+      <c r="E17" s="16" t="inlineStr">
         <is>
           <t>Kogelkranen / koppelingen / verloopstukken (set)</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
+      <c r="F17" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F16" s="13" t="inlineStr">
+      <c r="G17" s="16" t="inlineStr">
         <is>
           <t>Afsluitkranen en hulpstukken voor aansluiting/afsluiting van de verdeler.</t>
         </is>
       </c>
-      <c r="G16" s="13" t="inlineStr">
+      <c r="H17" s="16" t="inlineStr">
         <is>
           <t>Maakt service mogelijk zonder het hele CV-systeem leeg te laten.</t>
         </is>
       </c>
-      <c r="H16" s="18" t="n">
+      <c r="I17" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I16" s="13" t="inlineStr">
+      <c r="J17" s="16" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="J16" s="19" t="n">
+      <c r="K17" s="21" t="n">
         <v>34.95</v>
       </c>
-      <c r="K16" s="20" t="n">
+      <c r="L17" s="22" t="n">
         <v>34.95</v>
       </c>
-      <c r="L16" s="13" t="inlineStr">
+      <c r="M17" s="16" t="inlineStr">
         <is>
           <t>1–3 werkdagen</t>
         </is>
       </c>
-      <c r="M16" s="13" t="inlineStr">
+      <c r="N17" s="16" t="inlineStr">
         <is>
           <t>Online-vloerverwarming</t>
         </is>
       </c>
-      <c r="N16" s="21" t="inlineStr">
+      <c r="O17" s="23" t="inlineStr">
         <is>
           <t>https://online-vloerverwarming.nl/kogelkraan-set-1-rvs-verdeler/</t>
         </is>
       </c>
-      <c r="O16" s="13" t="inlineStr">
+      <c r="P17" s="16" t="inlineStr">
         <is>
           <t>Check of verdeler al primaire afsluiters heeft</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="68" customHeight="1">
-      <c r="A17" s="13" t="n">
+    <row r="18" ht="64" customHeight="1">
+      <c r="A18" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="n">
         <v>12</v>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="C18" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="D18" s="16" t="inlineStr">
         <is>
           <t>Actuators</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="E18" s="16" t="inlineStr">
         <is>
           <t>MAGNUM MW-A thermische actuator 230V NC M30×1,5</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="F18" s="16" t="inlineStr">
         <is>
           <t>W80003</t>
         </is>
       </c>
-      <c r="F17" s="13" t="inlineStr">
+      <c r="G18" s="16" t="inlineStr">
         <is>
           <t>Elektrische thermomotor (normaal gesloten) op de groepsafsluiter van de verdeler.</t>
         </is>
       </c>
-      <c r="G17" s="13" t="inlineStr">
+      <c r="H18" s="16" t="inlineStr">
         <is>
           <t>Opent/sluit per groep de watertoevoer. Nodig bij H64 én bij Tado (per groep).</t>
         </is>
       </c>
-      <c r="H17" s="18" t="n">
+      <c r="I18" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="I17" s="13" t="inlineStr">
+      <c r="J18" s="16" t="inlineStr">
         <is>
           <t>st</t>
         </is>
       </c>
-      <c r="J17" s="19" t="n">
+      <c r="K18" s="21" t="n">
         <v>19.95</v>
       </c>
-      <c r="K17" s="20" t="n">
+      <c r="L18" s="22" t="n">
         <v>79.8</v>
       </c>
-      <c r="L17" s="13" t="inlineStr">
+      <c r="M18" s="16" t="inlineStr">
         <is>
           <t>1–2 werkdagen</t>
         </is>
       </c>
-      <c r="M17" s="13" t="inlineStr">
+      <c r="N18" s="16" t="inlineStr">
         <is>
           <t>Vloerverwarmingstore</t>
         </is>
       </c>
-      <c r="N17" s="21" t="inlineStr">
+      <c r="O18" s="23" t="inlineStr">
         <is>
           <t>https://www.vloerverwarmingstore.nl/p/mw-a-actuator-nc-magnum-actuator-normaal-gesloten</t>
         </is>
       </c>
-      <c r="O17" s="13" t="inlineStr">
+      <c r="P18" s="16" t="inlineStr">
         <is>
           <t>1 per groep = 4 stuks; bij Tado: per kamer-zone parallel schakelen</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="68" customHeight="1">
-      <c r="A18" s="13" t="n">
+    <row r="19" ht="64" customHeight="1">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B19" s="16" t="n">
         <v>13</v>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="C19" s="16" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="D19" s="16" t="inlineStr">
         <is>
           <t>Elektra</t>
         </is>
       </c>
-      <c r="D18" s="13" t="inlineStr">
+      <c r="E19" s="16" t="inlineStr">
         <is>
           <t>Elektrakabel 230V / signaalkabel naar regeling + pomp</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
+      <c r="F19" s="16" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F18" s="13" t="inlineStr">
+      <c r="G19" s="16" t="inlineStr">
         <is>
           <t>230V voeding + bedrading tussen thermostaten/ontvangers, actuators en pomp.</t>
         </is>
       </c>
-      <c r="G18" s="13" t="inlineStr">
+      <c r="H19" s="16" t="inlineStr">
         <is>
           <t>Voeding en aansturing van pomp, actuators en Tado-ontvangers of H64-unit.</t>
         </is>
       </c>
-      <c r="H18" s="18" t="n">
+      <c r="I19" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I18" s="13" t="inlineStr">
+      <c r="J19" s="16" t="inlineStr">
         <is>
           <t>kleinmateriaal</t>
         </is>
       </c>
-      <c r="J18" s="19" t="n">
+      <c r="K19" s="21" t="n">
         <v>35</v>
       </c>
-      <c r="K18" s="20" t="n">
+      <c r="L19" s="22" t="n">
         <v>35</v>
       </c>
-      <c r="L18" s="13" t="inlineStr">
+      <c r="M19" s="16" t="inlineStr">
         <is>
           <t>Direct / bouwmarkt</t>
         </is>
       </c>
-      <c r="M18" s="13" t="inlineStr">
+      <c r="N19" s="16" t="inlineStr">
         <is>
           <t>Bouwmarkt</t>
         </is>
       </c>
-      <c r="N18" s="21" t="inlineStr">
+      <c r="O19" s="23" t="inlineStr">
         <is>
           <t>https://www.gamma.nl/assortiment/elektra/elektradraad-en-kabel</t>
         </is>
       </c>
-      <c r="O18" s="13" t="inlineStr">
+      <c r="P19" s="16" t="inlineStr">
         <is>
           <t>Laat elektra bij voorkeur door elektricien doen</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="68" customHeight="1">
-      <c r="A19" s="13" t="n">
+    <row r="20" ht="64" customHeight="1">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B20" s="16" t="n">
         <v>14</v>
       </c>
-      <c r="B19" s="18" t="inlineStr">
+      <c r="C20" s="20" t="inlineStr">
         <is>
           <t>h64</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
+      <c r="D20" s="16" t="inlineStr">
         <is>
           <t>Regeling H64</t>
         </is>
       </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="E20" s="16" t="inlineStr">
         <is>
           <t>MAGNUM H64-CC regelunit + H64-MT master WiFi-thermostaat</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="F20" s="16" t="inlineStr">
         <is>
           <t>W81004</t>
         </is>
       </c>
-      <c r="F19" s="13" t="inlineStr">
+      <c r="G20" s="16" t="inlineStr">
         <is>
           <t>Bedrade zonecontroller (max. 8 zones) inclusief master WiFi-thermostaat.</t>
         </is>
       </c>
-      <c r="G19" s="13" t="inlineStr">
+      <c r="H20" s="16" t="inlineStr">
         <is>
           <t>Alleen nodig als je KIEST voor Magnum H64 i.p.v. Tado. Stuurt actuators aan.</t>
         </is>
       </c>
-      <c r="H19" s="18" t="n">
+      <c r="I20" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I19" s="13" t="inlineStr">
+      <c r="J20" s="16" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="J19" s="19" t="n">
+      <c r="K20" s="21" t="n">
         <v>225</v>
       </c>
-      <c r="K19" s="20" t="n">
+      <c r="L20" s="22" t="n">
         <v>225</v>
       </c>
-      <c r="L19" s="13" t="inlineStr">
+      <c r="M20" s="16" t="inlineStr">
         <is>
           <t>1–2 werkdagen</t>
         </is>
       </c>
-      <c r="M19" s="13" t="inlineStr">
+      <c r="N20" s="16" t="inlineStr">
         <is>
           <t>Vloerverwarmingstore</t>
         </is>
       </c>
-      <c r="N19" s="21" t="inlineStr">
+      <c r="O20" s="23" t="inlineStr">
         <is>
           <t>https://www.vloerverwarmingstore.nl/p/h64-cc-regelunit-cc-regelunit-en-h64-mt-thermostaat-ral-9011-zwart</t>
         </is>
       </c>
-      <c r="O19" s="13" t="inlineStr">
+      <c r="P20" s="16" t="inlineStr">
         <is>
           <t>Niet kopen als je Tado neemt</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="68" customHeight="1">
-      <c r="A20" s="13" t="n">
+    <row r="21" ht="64" customHeight="1">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B21" s="16" t="n">
         <v>15</v>
       </c>
-      <c r="B20" s="18" t="inlineStr">
+      <c r="C21" s="20" t="inlineStr">
         <is>
           <t>h64</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
+      <c r="D21" s="16" t="inlineStr">
         <is>
           <t>Regeling H64</t>
         </is>
       </c>
-      <c r="D20" s="13" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>MAGNUM H64-ST slave / klokthermostaat</t>
         </is>
       </c>
-      <c r="E20" s="13" t="inlineStr">
+      <c r="F21" s="16" t="inlineStr">
         <is>
           <t>W81003</t>
         </is>
       </c>
-      <c r="F20" s="13" t="inlineStr">
+      <c r="G21" s="16" t="inlineStr">
         <is>
           <t>Extra bedrade programmeerbare ruimtethermostaat (slave) voor H64.</t>
         </is>
       </c>
-      <c r="G20" s="13" t="inlineStr">
+      <c r="H21" s="16" t="inlineStr">
         <is>
           <t>2e en 3e ruimte bij H64-regeling. Niet nodig bij Tado.</t>
         </is>
       </c>
-      <c r="H20" s="18" t="n">
+      <c r="I21" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="I20" s="13" t="inlineStr">
+      <c r="J21" s="16" t="inlineStr">
         <is>
           <t>st</t>
         </is>
       </c>
-      <c r="J20" s="19" t="n">
+      <c r="K21" s="21" t="n">
         <v>57.95</v>
       </c>
-      <c r="K20" s="20" t="n">
+      <c r="L21" s="22" t="n">
         <v>115.9</v>
       </c>
-      <c r="L20" s="13" t="inlineStr">
+      <c r="M21" s="16" t="inlineStr">
         <is>
           <t>1–2 werkdagen</t>
         </is>
       </c>
-      <c r="M20" s="13" t="inlineStr">
+      <c r="N21" s="16" t="inlineStr">
         <is>
           <t>Vloerverwarmingstore</t>
         </is>
       </c>
-      <c r="N20" s="21" t="inlineStr">
+      <c r="O21" s="23" t="inlineStr">
         <is>
           <t>https://www.vloerverwarmingstore.nl/p/h64-st-klokthermostaat-bedrade-ruimtethermostaat</t>
         </is>
       </c>
-      <c r="O20" s="13" t="inlineStr">
+      <c r="P21" s="16" t="inlineStr">
         <is>
           <t>Niet kopen als je Tado neemt</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="68" customHeight="1">
-      <c r="A21" s="13" t="n">
+    <row r="22" ht="64" customHeight="1">
+      <c r="A22" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="n">
         <v>16</v>
       </c>
-      <c r="B21" s="22" t="inlineStr">
+      <c r="C22" s="24" t="inlineStr">
         <is>
           <t>tado_draadloos</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="D22" s="16" t="inlineStr">
         <is>
           <t>Regeling Tado</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="E22" s="16" t="inlineStr">
         <is>
           <t>tado° Draadloze Slimme Thermostaat X Starterskit (Ontvanger X + Temperatuursensor X)</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="F22" s="16" t="inlineStr">
         <is>
           <t>Wireless X Starter</t>
         </is>
       </c>
-      <c r="F21" s="13" t="inlineStr">
-        <is>
-          <t>Set per zone: Draadloze Ontvanger X (bij verdeler, schakelt actuators/zoneklep) + Draadloze Temperatuursensor X (in de kamer). Matter/Thread.</t>
-        </is>
-      </c>
-      <c r="G21" s="13" t="inlineStr">
+      <c r="G22" s="16" t="inlineStr">
+        <is>
+          <t>Set per zone: Draadloze Ontvanger X (bij verdeler) + Draadloze Temperatuursensor X (in de kamer). Matter/Thread.</t>
+        </is>
+      </c>
+      <c r="H22" s="16" t="inlineStr">
         <is>
           <t>1 set per ruimte → 3 ruimten apart regelen. Ontvanger opent de actuators van die kamer bij warmtevraag.</t>
         </is>
       </c>
-      <c r="H21" s="18" t="n">
+      <c r="I22" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="I21" s="13" t="inlineStr">
+      <c r="J22" s="16" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="J21" s="19" t="n">
+      <c r="K22" s="21" t="n">
         <v>129</v>
       </c>
-      <c r="K21" s="20" t="n">
+      <c r="L22" s="22" t="n">
         <v>387</v>
       </c>
-      <c r="L21" s="13" t="inlineStr">
+      <c r="M22" s="16" t="inlineStr">
         <is>
           <t>2–4 werkdagen</t>
         </is>
       </c>
-      <c r="M21" s="13" t="inlineStr">
+      <c r="N22" s="16" t="inlineStr">
         <is>
           <t>tado° Shop</t>
         </is>
       </c>
-      <c r="N21" s="21" t="inlineStr">
+      <c r="O22" s="23" t="inlineStr">
         <is>
           <t>https://shop.tado.com/nl-bx/products/wireless-smart-thermostat-x-starter-kit</t>
         </is>
       </c>
-      <c r="O21" s="13" t="inlineStr">
-        <is>
-          <t>Aanbevolen draadloze Tado-route; actieprijs shop.tado.com (Coolblue ca. €194)</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="68" customHeight="1">
-      <c r="A22" s="13" t="n">
+      <c r="P22" s="16" t="inlineStr">
+        <is>
+          <t>Aanbevolen draadloze Tado-route; actieprijs shop.tado.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="64" customHeight="1">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B23" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="B22" s="22" t="inlineStr">
+      <c r="C23" s="24" t="inlineStr">
         <is>
           <t>tado_bedraad</t>
         </is>
       </c>
-      <c r="C22" s="13" t="inlineStr">
+      <c r="D23" s="16" t="inlineStr">
         <is>
           <t>Regeling Tado</t>
         </is>
       </c>
-      <c r="D22" s="13" t="inlineStr">
+      <c r="E23" s="16" t="inlineStr">
         <is>
           <t>tado° Slimme Thermostaat X Starterskit bedraad (thermostaat + Bridge X)</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr">
+      <c r="F23" s="16" t="inlineStr">
         <is>
           <t>Wired X Starter</t>
         </is>
       </c>
-      <c r="F22" s="13" t="inlineStr">
+      <c r="G23" s="16" t="inlineStr">
         <is>
           <t>Bedrade Slimme Thermostaat X + Bridge X (internet/Thread). Geschikt voor vloerverwarming-modus.</t>
         </is>
       </c>
-      <c r="G22" s="13" t="inlineStr">
-        <is>
-          <t>Kamer 1: meet temperatuur én schakelt de actuators van die zone (of ketel, afhankelijk van bekabeling).</t>
-        </is>
-      </c>
-      <c r="H22" s="18" t="n">
+      <c r="H23" s="16" t="inlineStr">
+        <is>
+          <t>Kamer 1: meet temperatuur én schakelt de actuators van die zone.</t>
+        </is>
+      </c>
+      <c r="I23" s="20" t="n">
         <v>1</v>
       </c>
-      <c r="I22" s="13" t="inlineStr">
+      <c r="J23" s="16" t="inlineStr">
         <is>
           <t>set</t>
         </is>
       </c>
-      <c r="J22" s="19" t="n">
+      <c r="K23" s="21" t="n">
         <v>129.99</v>
       </c>
-      <c r="K22" s="20" t="n">
+      <c r="L23" s="22" t="n">
         <v>129.99</v>
       </c>
-      <c r="L22" s="13" t="inlineStr">
+      <c r="M23" s="16" t="inlineStr">
         <is>
           <t>2–4 werkdagen</t>
         </is>
       </c>
-      <c r="M22" s="13" t="inlineStr">
+      <c r="N23" s="16" t="inlineStr">
         <is>
           <t>tado° Shop</t>
         </is>
       </c>
-      <c r="N22" s="21" t="inlineStr">
+      <c r="O23" s="23" t="inlineStr">
         <is>
           <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-starter-kit-1</t>
         </is>
       </c>
-      <c r="O22" s="13" t="inlineStr">
+      <c r="P23" s="16" t="inlineStr">
         <is>
           <t>Goedkopere Tado-route dan 3× draadloos</t>
         </is>
       </c>
     </row>
-    <row r="23" ht="68" customHeight="1">
-      <c r="A23" s="13" t="n">
+    <row r="24" ht="64" customHeight="1">
+      <c r="A24" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="n">
         <v>18</v>
       </c>
-      <c r="B23" s="22" t="inlineStr">
+      <c r="C24" s="24" t="inlineStr">
         <is>
           <t>tado_bedraad</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="D24" s="16" t="inlineStr">
         <is>
           <t>Regeling Tado</t>
         </is>
       </c>
-      <c r="D23" s="13" t="inlineStr">
+      <c r="E24" s="16" t="inlineStr">
         <is>
           <t>tado° Slimme Thermostaat X bedraad (uitbreiding / multi-zone)</t>
         </is>
       </c>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="F24" s="16" t="inlineStr">
         <is>
           <t>Smart Thermostat X</t>
         </is>
       </c>
-      <c r="F23" s="13" t="inlineStr">
+      <c r="G24" s="16" t="inlineStr">
         <is>
           <t>Extra bedrade Slimme Thermostaat X zonder Bridge. Werkt via Bridge X uit de starterskit.</t>
         </is>
       </c>
-      <c r="G23" s="13" t="inlineStr">
-        <is>
-          <t>Kamer 2 en 3: elk een eigen thermostaat → 3 ruimten apart. Bedraad naar actuators van die zone.</t>
-        </is>
-      </c>
-      <c r="H23" s="18" t="n">
+      <c r="H24" s="16" t="inlineStr">
+        <is>
+          <t>Kamer 2 en 3: elk een eigen thermostaat → 3 ruimten apart.</t>
+        </is>
+      </c>
+      <c r="I24" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="I23" s="13" t="inlineStr">
+      <c r="J24" s="16" t="inlineStr">
         <is>
           <t>st</t>
         </is>
       </c>
-      <c r="J23" s="19" t="n">
+      <c r="K24" s="21" t="n">
         <v>100</v>
       </c>
-      <c r="K23" s="20" t="n">
+      <c r="L24" s="22" t="n">
         <v>200</v>
       </c>
-      <c r="L23" s="13" t="inlineStr">
+      <c r="M24" s="16" t="inlineStr">
         <is>
           <t>2–4 werkdagen</t>
         </is>
       </c>
-      <c r="M23" s="13" t="inlineStr">
+      <c r="N24" s="16" t="inlineStr">
         <is>
           <t>tado° Shop</t>
         </is>
       </c>
-      <c r="N23" s="21" t="inlineStr">
+      <c r="O24" s="23" t="inlineStr">
         <is>
           <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-wired</t>
         </is>
       </c>
-      <c r="O23" s="13" t="inlineStr">
+      <c r="P24" s="16" t="inlineStr">
         <is>
           <t>Bridge X zit al in starterskit</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="68" customHeight="1">
-      <c r="A24" s="13" t="n">
+    <row r="25" ht="64" customHeight="1">
+      <c r="A25" s="19" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="n">
         <v>19</v>
       </c>
-      <c r="B24" s="23" t="inlineStr">
+      <c r="C25" s="25" t="inlineStr">
         <is>
           <t>tado_optie</t>
         </is>
       </c>
-      <c r="C24" s="13" t="inlineStr">
+      <c r="D25" s="16" t="inlineStr">
         <is>
           <t>Regeling Tado</t>
         </is>
       </c>
-      <c r="D24" s="13" t="inlineStr">
+      <c r="E25" s="16" t="inlineStr">
         <is>
           <t>tado° Bridge X (extra, alleen indien nodig)</t>
         </is>
       </c>
-      <c r="E24" s="13" t="inlineStr">
+      <c r="F25" s="16" t="inlineStr">
         <is>
           <t>Bridge X</t>
         </is>
       </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>Thread Border Router voor internetverbinding van tado° X. Bij draadloze starterkits vaak al afgedekt door Ontvanger X.</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>Alleen extra bestellen bij bereikproblemen of als je bedrade thermostaten zonder starterskit koopt.</t>
-        </is>
-      </c>
-      <c r="H24" s="18" t="n">
+      <c r="G25" s="16" t="inlineStr">
+        <is>
+          <t>Thread Border Router voor internetverbinding van tado° X.</t>
+        </is>
+      </c>
+      <c r="H25" s="16" t="inlineStr">
+        <is>
+          <t>Alleen extra bestellen bij bereikproblemen of zonder starterskit-Bridge.</t>
+        </is>
+      </c>
+      <c r="I25" s="20" t="n">
         <v>0</v>
       </c>
-      <c r="I24" s="13" t="inlineStr">
+      <c r="J25" s="16" t="inlineStr">
         <is>
           <t>st</t>
         </is>
       </c>
-      <c r="J24" s="19" t="n">
+      <c r="K25" s="21" t="n">
         <v>68</v>
       </c>
-      <c r="K24" s="20" t="n">
+      <c r="L25" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="L24" s="13" t="inlineStr">
+      <c r="M25" s="16" t="inlineStr">
         <is>
           <t>1–3 werkdagen</t>
         </is>
       </c>
-      <c r="M24" s="13" t="inlineStr">
+      <c r="N25" s="16" t="inlineStr">
         <is>
           <t>Coolblue / tado°</t>
         </is>
       </c>
-      <c r="N24" s="21" t="inlineStr">
+      <c r="O25" s="23" t="inlineStr">
         <is>
           <t>https://www.coolblue.nl/thermostaten/tado</t>
         </is>
       </c>
-      <c r="O24" s="13" t="inlineStr">
-        <is>
-          <t>Standaard qty=0; zet op 1 indien nodig</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>Basis (zonder regeling-thermostaten)</t>
-        </is>
-      </c>
-      <c r="K26" s="6" t="n">
+      <c r="P25" s="16" t="inlineStr">
+        <is>
+          <t>Standaard qty=0</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>KOPJE: (nog leeg – hier later andere kopjes toevoegen)</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n"/>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
+      <c r="E27" s="4" t="n"/>
+      <c r="F27" s="4" t="n"/>
+      <c r="G27" s="4" t="n"/>
+      <c r="H27" s="4" t="n"/>
+      <c r="I27" s="4" t="n"/>
+      <c r="J27" s="4" t="n"/>
+      <c r="K27" s="4" t="n"/>
+      <c r="L27" s="4" t="n"/>
+      <c r="M27" s="4" t="n"/>
+      <c r="N27" s="4" t="n"/>
+      <c r="O27" s="4" t="n"/>
+      <c r="P27" s="4" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="26" t="inlineStr">
+        <is>
+          <t>Voorbeeld</t>
+        </is>
+      </c>
+      <c r="B28" s="27" t="n"/>
+      <c r="C28" s="27" t="n"/>
+      <c r="D28" s="27" t="n"/>
+      <c r="E28" s="26" t="inlineStr">
+        <is>
+          <t>← voeg hier later rijen toe met Kopje = bijv. Badkamer / Elektra / Afwerking</t>
+        </is>
+      </c>
+      <c r="F28" s="27" t="n"/>
+      <c r="G28" s="27" t="n"/>
+      <c r="H28" s="27" t="n"/>
+      <c r="I28" s="27" t="n"/>
+      <c r="J28" s="27" t="n"/>
+      <c r="K28" s="27" t="n"/>
+      <c r="L28" s="27" t="n"/>
+      <c r="M28" s="27" t="n"/>
+      <c r="N28" s="27" t="n"/>
+      <c r="O28" s="27" t="n"/>
+      <c r="P28" s="27" t="n"/>
+    </row>
+    <row r="30">
+      <c r="J30" s="5" t="inlineStr">
+        <is>
+          <t>Subtotaal Vloerverwarming – basis</t>
+        </is>
+      </c>
+      <c r="L30" s="9" t="n">
         <v>2156.42</v>
       </c>
     </row>
-    <row r="27">
-      <c r="I27" s="24" t="inlineStr">
-        <is>
-          <t>Totaal met Tado DRAADLOOS (3 ruimten)</t>
-        </is>
-      </c>
-      <c r="K27" s="25" t="n">
+    <row r="31">
+      <c r="J31" s="28" t="inlineStr">
+        <is>
+          <t>Vloerverwarming + Tado DRAADLOOS</t>
+        </is>
+      </c>
+      <c r="L31" s="29" t="n">
         <v>2543.42</v>
       </c>
     </row>
-    <row r="28">
-      <c r="I28" s="24" t="inlineStr">
-        <is>
-          <t>Totaal met Tado BEDRAAD (3 ruimten)</t>
-        </is>
-      </c>
-      <c r="K28" s="25" t="n">
+    <row r="32">
+      <c r="J32" s="28" t="inlineStr">
+        <is>
+          <t>Vloerverwarming + Tado BEDRAAD</t>
+        </is>
+      </c>
+      <c r="L32" s="29" t="n">
         <v>2486.41</v>
       </c>
     </row>
-    <row r="29">
-      <c r="I29" s="24" t="inlineStr">
-        <is>
-          <t>Totaal met Magnum H64</t>
-        </is>
-      </c>
-      <c r="K29" s="26" t="n">
+    <row r="33">
+      <c r="J33" s="28" t="inlineStr">
+        <is>
+          <t>Vloerverwarming + Magnum H64</t>
+        </is>
+      </c>
+      <c r="L33" s="30" t="n">
         <v>2497.32</v>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="9" t="inlineStr">
-        <is>
-          <t>Legenda Keuze-kolom</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>altijd = altijd nodig · h64 = alleen bij Magnum H64 · tado_draadloos / tado_bedraad = alleen bij die Tado-route · tado_optie = optioneel</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="10" t="inlineStr">
-        <is>
-          <t>Koop NIET zowel H64 als Tado. Kies één regelingsysteem. Actuators (nr 12) heb je in alle gevallen nodig.</t>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Filter tip: gebruik AutoFilter op kolom Kopje om alleen Vloerverwarming te tonen wanneer er meer kopjes zijn.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A5:O24"/>
-  <mergeCells count="5">
+  <autoFilter ref="A6:P25"/>
+  <mergeCells count="7">
+    <mergeCell ref="A5:P5"/>
     <mergeCell ref="B3:D3"/>
-    <mergeCell ref="A2:O2"/>
-    <mergeCell ref="A33:O33"/>
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A32:O32"/>
+    <mergeCell ref="E28:J28"/>
+    <mergeCell ref="A1:P1"/>
+    <mergeCell ref="A27:P27"/>
+    <mergeCell ref="A35:P35"/>
+    <mergeCell ref="A2:P2"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N6" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N7" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N8" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N10" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N11" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N12" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N13" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N14" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N15" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N16" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N17" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N18" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N19" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N20" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N21" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N22" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N23" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N24" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId19"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2566,7 +2686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2575,146 +2695,123 @@
     <col width="48" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>KOPJE: Vloerverwarming — Tado-aansluiting</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="n"/>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Tado → 3 ruimten op jouw 4-groepsverdeler</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Ruimte</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Groepen op verdeler</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Tado-apparaat in kamer</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Aansturing bij verdeler</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="13" t="inlineStr">
+    <row r="5" ht="36" customHeight="1">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Kamer 15 m²</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>Groep 1 + Groep 2</t>
         </is>
       </c>
-      <c r="C4" s="13" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>Sensor X of bedrade Thermostaat X</t>
         </is>
       </c>
-      <c r="D4" s="13" t="inlineStr">
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>1 Ontvanger X / 1 relais → beide actuators parallel</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="13" t="inlineStr">
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Studeerkamer 10 m²</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>Groep 3</t>
         </is>
       </c>
-      <c r="C5" s="13" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>Sensor X of bedrade Thermostaat X</t>
         </is>
       </c>
-      <c r="D5" s="13" t="inlineStr">
+      <c r="D6" s="16" t="inlineStr">
         <is>
           <t>1 Ontvanger X / 1 relais → actuator groep 3</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
+    <row r="7" ht="36" customHeight="1">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>3e ruimte</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>Groep 4</t>
         </is>
       </c>
-      <c r="C6" s="13" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>Sensor X of bedrade Thermostaat X</t>
         </is>
       </c>
-      <c r="D6" s="13" t="inlineStr">
+      <c r="D7" s="16" t="inlineStr">
         <is>
           <t>1 Ontvanger X / 1 relais → actuator groep 4</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>Belangrijk</t>
-        </is>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>• Magnum H64-unit + H64-thermostaten vervallen bij Tado (niet dubbel kopen).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>• De 4 Magnum MW-A actuators blijf je wel nodig hebben (of vergelijkbare 230V NC M30×1,5).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>• Zet in de tado°-app Underfloor Heating Control Mode aan voor vloerverwarming.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>• Ketel/warmtepomp: vaak 1 zone-controller of ontvanger ook gekoppeld aan warmtevraag cv – volg tado° Product Finder / installateur.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>• Controleer of je cv-ketel compatibel is met tado° X (OpenTherm of relais).</t>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>• H64 vervalt bij Tado. • 4× MW-A actuators blijven nodig. • Zet Underfloor Heating Control Mode aan in de tado°-app.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="3">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2726,515 +2823,647 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>KOPJE: Vloerverwarming — bestelchecklist</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="n"/>
+      <c r="C1" s="4" t="n"/>
+      <c r="D1" s="4" t="n"/>
+      <c r="E1" s="4" t="n"/>
+      <c r="F1" s="4" t="n"/>
+      <c r="G1" s="4" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Bestelchecklist</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="15" t="inlineStr">
+        <is>
+          <t>Kopje</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>Artikel</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>Keuze</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="D4" s="15" t="inlineStr">
         <is>
           <t>Waarvoor nodig</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr">
+      <c r="E4" s="15" t="inlineStr">
         <is>
           <t>Besteld?</t>
         </is>
       </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>Ordernr</t>
         </is>
       </c>
-      <c r="F3" s="12" t="inlineStr">
+      <c r="G4" s="15" t="inlineStr">
         <is>
           <t>Ontvangen?</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>MAGNUM SlimFit 12 bevestigingsmat 3,75 m² (5 platen 75×100 cm)</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C4" s="27" t="inlineStr">
+      <c r="D5" s="32" t="inlineStr">
         <is>
           <t>Vormt de basislaag waarin je de buizen vastlegt over het hele vloeroppervlak (±30 m²).</t>
         </is>
       </c>
-      <c r="D4" s="28" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E4" s="28" t="n"/>
-      <c r="F4" s="28" t="n"/>
-    </row>
-    <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="F5" s="13" t="n"/>
+      <c r="G5" s="13" t="n"/>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>MAGNUM PE-RT buis 12×1,5 mm KOMO – rol 300 m</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="C6" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="D6" s="32" t="inlineStr">
         <is>
           <t>Voert het warme water door de vloer; hiermee leg je de 4 verwarmingscircuits.</t>
         </is>
       </c>
-      <c r="D5" s="28" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E5" s="28" t="n"/>
-      <c r="F5" s="28" t="n"/>
-    </row>
-    <row r="6" ht="36" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="F6" s="13" t="n"/>
+      <c r="G6" s="13" t="n"/>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
         <is>
           <t>MAGNUM Euroconus / adaptor 12×1,5 mm × ¾″ (set van 2)</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C6" s="27" t="inlineStr">
+      <c r="D7" s="32" t="inlineStr">
         <is>
           <t>Nodig om elke groep (aanvoer + retour) waterdicht op de verdeler aan te sluiten.</t>
         </is>
       </c>
-      <c r="D6" s="28" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E6" s="28" t="n"/>
-      <c r="F6" s="28" t="n"/>
-    </row>
-    <row r="7" ht="36" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="F7" s="13" t="n"/>
+      <c r="G7" s="13" t="n"/>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>MAGNUM 90° bochtondersteuning ø10–12 mm (set van 2)</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C7" s="27" t="inlineStr">
+      <c r="D8" s="32" t="inlineStr">
         <is>
           <t>Beschermt de buis waar die vanaf de verdeler de vloer in gaat.</t>
         </is>
       </c>
-      <c r="D7" s="28" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E7" s="28" t="n"/>
-      <c r="F7" s="28" t="n"/>
-    </row>
-    <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="F8" s="13" t="n"/>
+      <c r="G8" s="13" t="n"/>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>MAGNUM Contactlijm SlimFit / verlegsystemen 500 ml</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C8" s="27" t="inlineStr">
+      <c r="D9" s="32" t="inlineStr">
         <is>
           <t>Houdt de matten vast op de ondervloer tijdens leggen en egaliseren.</t>
         </is>
       </c>
-      <c r="D8" s="28" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E8" s="28" t="n"/>
-      <c r="F8" s="28" t="n"/>
-    </row>
-    <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="F9" s="13" t="n"/>
+      <c r="G9" s="13" t="n"/>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>Randisolatie 8×150 mm met flap – rol 25 m</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C9" s="27" t="inlineStr">
+      <c r="D10" s="32" t="inlineStr">
         <is>
           <t>Rondom tegen muren: voorkomt koudebruggen en vangt uitzetting op.</t>
         </is>
       </c>
-      <c r="D9" s="28" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E9" s="28" t="n"/>
-      <c r="F9" s="28" t="n"/>
-    </row>
-    <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="F10" s="13" t="n"/>
+      <c r="G10" s="13" t="n"/>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>Kreisel Gruntolit-W 301 voorstrijk / primer 5 L</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C10" s="27" t="inlineStr">
+      <c r="D11" s="32" t="inlineStr">
         <is>
           <t>Zorgt dat egaline goed hecht; zonder primer kan egaline loslaten.</t>
         </is>
       </c>
-      <c r="D10" s="28" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E10" s="28" t="n"/>
-      <c r="F10" s="28" t="n"/>
-    </row>
-    <row r="11" ht="36" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="F11" s="13" t="n"/>
+      <c r="G11" s="13" t="n"/>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
         <is>
           <t>Kreisel 418 vezelversterkte egaline 25 kg (1–50 mm)</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C11" s="27" t="inlineStr">
+      <c r="D12" s="32" t="inlineStr">
         <is>
           <t>Gietlaag die buizen/matten inbedt tot vlakke vloer klaar voor afwerking.</t>
         </is>
       </c>
-      <c r="D11" s="28" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E11" s="28" t="n"/>
-      <c r="F11" s="28" t="n"/>
-    </row>
-    <row r="12" ht="36" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="13" t="n"/>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="inlineStr">
         <is>
           <t>MAGNUM Basic Staal 4-groeps mengverdeler + A-label pomp</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C12" s="27" t="inlineStr">
+      <c r="D13" s="32" t="inlineStr">
         <is>
           <t>Hart van het systeem: mengt CV-water en verdeelt over de 4 groepen.</t>
         </is>
       </c>
-      <c r="D12" s="28" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E12" s="28" t="n"/>
-      <c r="F12" s="28" t="n"/>
-    </row>
-    <row r="13" ht="36" customHeight="1">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="13" t="n"/>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="inlineStr">
         <is>
           <t>Aanvoer + retourleiding vanaf cv (meerlagenbuis 16×2 of koper 15 mm)</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C13" s="27" t="inlineStr">
+      <c r="D14" s="32" t="inlineStr">
         <is>
           <t>Brengt warm water van cv/wp naar de verdeler; lengte hangt af van afstand.</t>
         </is>
       </c>
-      <c r="D13" s="28" t="inlineStr">
+      <c r="E14" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E13" s="28" t="n"/>
-      <c r="F13" s="28" t="n"/>
-    </row>
-    <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="F14" s="13" t="n"/>
+      <c r="G14" s="13" t="n"/>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
         <is>
           <t>Kogelkranen / koppelingen / verloopstukken (set)</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C14" s="27" t="inlineStr">
+      <c r="D15" s="32" t="inlineStr">
         <is>
           <t>Maakt service mogelijk zonder het hele CV-systeem leeg te laten.</t>
         </is>
       </c>
-      <c r="D14" s="28" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E14" s="28" t="n"/>
-      <c r="F14" s="28" t="n"/>
-    </row>
-    <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="F15" s="13" t="n"/>
+      <c r="G15" s="13" t="n"/>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>MAGNUM MW-A thermische actuator 230V NC M30×1,5</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C15" s="27" t="inlineStr">
+      <c r="D16" s="32" t="inlineStr">
         <is>
           <t>Opent/sluit per groep de watertoevoer. Nodig bij H64 én bij Tado (per groep).</t>
         </is>
       </c>
-      <c r="D15" s="28" t="inlineStr">
+      <c r="E16" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E15" s="28" t="n"/>
-      <c r="F15" s="28" t="n"/>
-    </row>
-    <row r="16" ht="36" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="F16" s="13" t="n"/>
+      <c r="G16" s="13" t="n"/>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Elektrakabel 230V / signaalkabel naar regeling + pomp</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="C16" s="27" t="inlineStr">
+      <c r="D17" s="32" t="inlineStr">
         <is>
           <t>Voeding en aansturing van pomp, actuators en Tado-ontvangers of H64-unit.</t>
         </is>
       </c>
-      <c r="D16" s="28" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E16" s="28" t="n"/>
-      <c r="F16" s="28" t="n"/>
-    </row>
-    <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="F17" s="13" t="n"/>
+      <c r="G17" s="13" t="n"/>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>MAGNUM H64-CC regelunit + H64-MT master WiFi-thermostaat</t>
         </is>
       </c>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>h64</t>
         </is>
       </c>
-      <c r="C17" s="27" t="inlineStr">
+      <c r="D18" s="32" t="inlineStr">
         <is>
           <t>Alleen nodig als je KIEST voor Magnum H64 i.p.v. Tado. Stuurt actuators aan.</t>
         </is>
       </c>
-      <c r="D17" s="28" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E17" s="28" t="n"/>
-      <c r="F17" s="28" t="n"/>
-    </row>
-    <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="F18" s="13" t="n"/>
+      <c r="G18" s="13" t="n"/>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
         <is>
           <t>MAGNUM H64-ST slave / klokthermostaat</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>h64</t>
         </is>
       </c>
-      <c r="C18" s="27" t="inlineStr">
+      <c r="D19" s="32" t="inlineStr">
         <is>
           <t>2e en 3e ruimte bij H64-regeling. Niet nodig bij Tado.</t>
         </is>
       </c>
-      <c r="D18" s="28" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E18" s="28" t="n"/>
-      <c r="F18" s="28" t="n"/>
-    </row>
-    <row r="19" ht="36" customHeight="1">
-      <c r="A19" s="3" t="inlineStr">
+      <c r="F19" s="13" t="n"/>
+      <c r="G19" s="13" t="n"/>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
         <is>
           <t>tado° Draadloze Slimme Thermostaat X Starterskit (Ontvanger X + Temperatuursensor X)</t>
         </is>
       </c>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="C20" s="6" t="inlineStr">
         <is>
           <t>tado_draadloos</t>
         </is>
       </c>
-      <c r="C19" s="27" t="inlineStr">
+      <c r="D20" s="32" t="inlineStr">
         <is>
           <t>1 set per ruimte → 3 ruimten apart regelen. Ontvanger opent de actuators van die kamer bij warmtevraag.</t>
         </is>
       </c>
-      <c r="D19" s="28" t="inlineStr">
+      <c r="E20" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E19" s="28" t="n"/>
-      <c r="F19" s="28" t="n"/>
-    </row>
-    <row r="20" ht="36" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="F20" s="13" t="n"/>
+      <c r="G20" s="13" t="n"/>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
         <is>
           <t>tado° Slimme Thermostaat X Starterskit bedraad (thermostaat + Bridge X)</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>tado_bedraad</t>
         </is>
       </c>
-      <c r="C20" s="27" t="inlineStr">
-        <is>
-          <t>Kamer 1: meet temperatuur én schakelt de actuators van die zone (of ketel, afhankelijk van bekabeling).</t>
-        </is>
-      </c>
-      <c r="D20" s="28" t="inlineStr">
+      <c r="D21" s="32" t="inlineStr">
+        <is>
+          <t>Kamer 1: meet temperatuur én schakelt de actuators van die zone.</t>
+        </is>
+      </c>
+      <c r="E21" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E20" s="28" t="n"/>
-      <c r="F20" s="28" t="n"/>
-    </row>
-    <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
+      <c r="F21" s="13" t="n"/>
+      <c r="G21" s="13" t="n"/>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>tado° Slimme Thermostaat X bedraad (uitbreiding / multi-zone)</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="C22" s="6" t="inlineStr">
         <is>
           <t>tado_bedraad</t>
         </is>
       </c>
-      <c r="C21" s="27" t="inlineStr">
-        <is>
-          <t>Kamer 2 en 3: elk een eigen thermostaat → 3 ruimten apart. Bedraad naar actuators van die zone.</t>
-        </is>
-      </c>
-      <c r="D21" s="28" t="inlineStr">
+      <c r="D22" s="32" t="inlineStr">
+        <is>
+          <t>Kamer 2 en 3: elk een eigen thermostaat → 3 ruimten apart.</t>
+        </is>
+      </c>
+      <c r="E22" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E21" s="28" t="n"/>
-      <c r="F21" s="28" t="n"/>
-    </row>
-    <row r="22" ht="36" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="F22" s="13" t="n"/>
+      <c r="G22" s="13" t="n"/>
+    </row>
+    <row r="23" ht="34" customHeight="1">
+      <c r="A23" s="31" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
         <is>
           <t>tado° Bridge X (extra, alleen indien nodig)</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>tado_optie</t>
         </is>
       </c>
-      <c r="C22" s="27" t="inlineStr">
-        <is>
-          <t>Alleen extra bestellen bij bereikproblemen of als je bedrade thermostaten zonder starterskit koopt.</t>
-        </is>
-      </c>
-      <c r="D22" s="28" t="inlineStr">
+      <c r="D23" s="32" t="inlineStr">
+        <is>
+          <t>Alleen extra bestellen bij bereikproblemen of zonder starterskit-Bridge.</t>
+        </is>
+      </c>
+      <c r="E23" s="13" t="inlineStr">
         <is>
           <t>Nee</t>
         </is>
       </c>
-      <c r="E22" s="28" t="n"/>
-      <c r="F22" s="28" t="n"/>
+      <c r="F23" s="13" t="n"/>
+      <c r="G23" s="13" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>KOPJE: (nog leeg)</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n"/>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4" t="n"/>
+      <c r="G25" s="4" t="n"/>
     </row>
   </sheetData>
+  <autoFilter ref="A4:G23"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A25:G25"/>
+  </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="D4:D22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E5:E23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Nee,Ja,Overslaan"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Find cheaper shops for the five most expensive items
Keep SlimFit, Kreisel 418, VTE Composiet and PE-RT (no cheaper
in-stock option within a week). Switch Möhlenhoff Alpha 5 to
eibhandel.de and Magnum H64 to Warp Systems; document the hunt.

Co-authored-by: bmverhagen <bmverhagen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Materiaalbenodigdheden_Vloerverwarming.xlsx
+++ b/Materiaalbenodigdheden_Vloerverwarming.xlsx
@@ -9,13 +9,14 @@
   <sheets>
     <sheet name="Overzicht" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Kwaliteitskeuzes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Regeling-keuze" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Boodschappenlijst" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Tado-aansluiting" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Bestelchecklist" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Prijszoek-top5" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Regeling-keuze" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Boodschappenlijst" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Tado-aansluiting" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Bestelchecklist" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Boodschappenlijst'!$A$5:$S$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Boodschappenlijst'!$A$5:$S$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +27,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="€ #,##0.00"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -96,6 +97,10 @@
       <sz val="10"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
   </fonts>
   <fills count="9">
     <fill>
@@ -140,7 +145,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -162,11 +167,55 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -231,6 +280,9 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -607,18 +659,19 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Materiaallijst – kwaliteit eerst, dan prijs (≤ 1 week)</t>
-        </is>
-      </c>
-    </row>
+          <t>Materiaallijst – kwaliteit + scherpste shops (≤ 1 week)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>KOPJE: Vloerverwarming</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n"/>
-      <c r="C3" s="3" t="n"/>
+      <c r="B3" s="38" t="n"/>
+      <c r="C3" s="39" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -631,6 +684,7 @@
         <v/>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -662,11 +716,11 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>2090.1</v>
+        <v>2064.99</v>
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>+ € 135.82 voor betere kwaliteit</t>
+          <t>incl. prijszoek (actuators DE + H64 Warp)</t>
         </is>
       </c>
     </row>
@@ -677,11 +731,11 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>2420.09</v>
+        <v>2394.98</v>
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>+ € 135.82 voor betere kwaliteit</t>
+          <t>incl. prijszoek (actuators DE + H64 Warp)</t>
         </is>
       </c>
     </row>
@@ -692,11 +746,11 @@
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>2477.1</v>
+        <v>2451.99</v>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>+ € 135.82 voor betere kwaliteit</t>
+          <t>incl. prijszoek (actuators DE + H64 Warp)</t>
         </is>
       </c>
     </row>
@@ -707,18 +761,19 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>2409.68</v>
+        <v>2349.07</v>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>+ € 135.82 voor betere kwaliteit</t>
-        </is>
-      </c>
-    </row>
+          <t>incl. prijszoek (actuators DE + H64 Warp)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>3 kwaliteitsupgrades: VTE Composiet-verdeler · Möhlenhoff Alpha 5 actuators · NMC Climasol randisolatie</t>
+          <t>Kwaliteit: VTE Composiet · Möhlenhoff Alpha 5 · NMC Climasol. Prijszoek: actuators via eibhandel.de, H64 via Warp.</t>
         </is>
       </c>
     </row>
@@ -726,6 +781,14 @@
       <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Aanbevolen: Tado bedraad (stabieler dan draadloos).</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>2394.98</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>incl. prijszoek (actuators DE + H64 Warp)</t>
         </is>
       </c>
     </row>
@@ -746,7 +809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -775,9 +838,9 @@
           <t>KOPJE: Vloerverwarming — wat is geüpgraded?</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
+      <c r="B4" s="38" t="n"/>
+      <c r="C4" s="38" t="n"/>
+      <c r="D4" s="39" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -1229,6 +1292,20 @@
       <c r="A30" s="11" t="inlineStr">
         <is>
           <t>• Geen generieke 12 mm-buis i.p.v. Magnum: systeemcompatibiliteit SlimFit &gt; kleine prijswinst.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="30" t="inlineStr">
+        <is>
+          <t>Prijszoek top-5 (aug 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Möhlenhoff → eibhandel.de €9,99 (+NL verzending). H64-CC → Warp €194,92. Overige top-5: geen betere shop binnen ≤1 week.</t>
         </is>
       </c>
     </row>
@@ -1252,6 +1329,301 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="40" t="inlineStr">
+        <is>
+          <t>Prijszoek – 5 duurste items (alleen goedkoper + ≤1 week leverbaar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Gezocht NL + DE webshops, 22 aug 2026. Alleen gewijzigd als aantoonbaar goedkoper én binnen levertijd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="30" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>Item (regeltotaal)</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>Was</t>
+        </is>
+      </c>
+      <c r="D4" s="30" t="inlineStr">
+        <is>
+          <t>Beste gevonden</t>
+        </is>
+      </c>
+      <c r="E4" s="30" t="inlineStr">
+        <is>
+          <t>Actie</t>
+        </is>
+      </c>
+      <c r="F4" s="30" t="inlineStr">
+        <is>
+          <t>Besparing</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>MAGNUM SlimFit 12 matten (8×)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Elektramat €86,94/st (€695,52)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Bouwmaat €86,50 (geen voorraad/bezorging); VihamiJ €86,36 excl=duurder + 3–4 wkn; overige ≥€88,99</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>BEHOUDEN Elektramat</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>€0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Kreisel 418 egaline (33×)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>EgalineXXL €14,87/st (€490,71)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>RBMB ≥€16,55/st (bulkpas pas vanaf 41); geen goedkopere met snelle levering</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BEHOUDEN EgalineXXL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>€0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>VTE Composiet 4-groeps + Grundfos</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>123Installatieshop €387,18</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CVTotaal €423; VV-shop €404,95; Bouwbestel €440; Jan de Isolatieman €469</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BEHOUDEN 123Installatieshop</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>€0</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MAGNUM PE-RT 12×1,5 300 m</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>123InstallatieMaterialen €142,93</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Klusspullen €141,95 maar voorraad 0 / levertijd 1–2 wkn → afgewezen; Elektramat €181,86; VV-shop €164,70</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BEHOUDEN 123IM</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>€0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5a</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Möhlenhoff Alpha 5 ×4 (altijd)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>VerwarmingOnline €20,12 → €80,48</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>eibhandel.de €9,99 + NL-verzending ~€15,41 = ~€55,37; Amazon.nl ~€13,16/st met Prime</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>GEWIJZIGD → eibhandel</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>~€25</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5b</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MAGNUM H64-CC + master (optie)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>123IM €213,74</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Warp Systems €194,92 (1 wd)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>GEWIJZIGD → Warp</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>~€19</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Niet meegenomen</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>• PioTek DE (~€9,90): verzendt niet meer naar NL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>• Bouwmaat SlimFit €86,50: tijdelijk niet beschikbaar / geen bezorging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>• Klusspullen PE-RT €141,95: goedkoper op papier, maar 0 voorraad / 1–2 weken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• Tado: officiële tado° Shop blijft goedkoopst (bol/retail vaak duurder).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1266,8 +1638,8 @@
           <t>KOPJE: Vloerverwarming — regeling</t>
         </is>
       </c>
-      <c r="B1" s="3" t="n"/>
-      <c r="C1" s="3" t="n"/>
+      <c r="B1" s="38" t="n"/>
+      <c r="C1" s="39" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -1307,13 +1679,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S31"/>
+  <dimension ref="A1:S32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1357,24 +1729,24 @@
           <t>KOPJE: Vloerverwarming</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-      <c r="I4" s="3" t="n"/>
-      <c r="J4" s="3" t="n"/>
-      <c r="K4" s="3" t="n"/>
-      <c r="L4" s="3" t="n"/>
-      <c r="M4" s="3" t="n"/>
-      <c r="N4" s="3" t="n"/>
-      <c r="O4" s="3" t="n"/>
-      <c r="P4" s="3" t="n"/>
-      <c r="Q4" s="3" t="n"/>
-      <c r="R4" s="3" t="n"/>
-      <c r="S4" s="3" t="n"/>
+      <c r="B4" s="38" t="n"/>
+      <c r="C4" s="38" t="n"/>
+      <c r="D4" s="38" t="n"/>
+      <c r="E4" s="38" t="n"/>
+      <c r="F4" s="38" t="n"/>
+      <c r="G4" s="38" t="n"/>
+      <c r="H4" s="38" t="n"/>
+      <c r="I4" s="38" t="n"/>
+      <c r="J4" s="38" t="n"/>
+      <c r="K4" s="38" t="n"/>
+      <c r="L4" s="38" t="n"/>
+      <c r="M4" s="38" t="n"/>
+      <c r="N4" s="38" t="n"/>
+      <c r="O4" s="38" t="n"/>
+      <c r="P4" s="38" t="n"/>
+      <c r="Q4" s="38" t="n"/>
+      <c r="R4" s="38" t="n"/>
+      <c r="S4" s="39" t="n"/>
     </row>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -2478,10 +2850,10 @@
         </is>
       </c>
       <c r="K17" s="23" t="n">
-        <v>20.12</v>
+        <v>9.99</v>
       </c>
       <c r="L17" s="24" t="n">
-        <v>14</v>
+        <v>9.99</v>
       </c>
       <c r="M17" s="28" t="inlineStr">
         <is>
@@ -2489,118 +2861,120 @@
         </is>
       </c>
       <c r="N17" s="26" t="n">
-        <v>80.48</v>
+        <v>39.96</v>
       </c>
       <c r="O17" s="21" t="inlineStr">
         <is>
-          <t>≤ 1 week</t>
+          <t>2–5 wd DE; NL meestal ≤1 week (DHL zone 1)</t>
         </is>
       </c>
       <c r="P17" s="21" t="inlineStr">
         <is>
-          <t>VerwarmingOnline</t>
+          <t>eibhandel.de</t>
         </is>
       </c>
       <c r="Q17" s="27" t="inlineStr">
         <is>
-          <t>https://verwarmingonline.nl/productgroepen/mohlenhoff-thermische-servomotor-alpha-5-nc-m30x15mm-230v-a-20405-00n/</t>
+          <t>https://eibhandel.de/Alpha-Antrieb-230V-NC-incl-Adapter-VA80</t>
         </is>
       </c>
       <c r="R17" s="21" t="inlineStr">
         <is>
-          <t>Möhlenhoff is kwalitatief duidelijk beter dan budget-Lovak (levensduur, lekkagebescherming, certificering). Marginaal duurder dan Magnum, merkbaar betrouwbaarder.</t>
+          <t>Goedkoopste bevestigde Alpha 5 NC 230V+VA80 met NL-verzending. Was €20.12 bij VerwarmingOnline. Alternatief Amazon.nl ~€13,16/st met gratis Prime (totaal vergelijkbaar).</t>
         </is>
       </c>
       <c r="S17" s="21" t="inlineStr">
         <is>
-          <t>KWALITEITSUPGRADE t.o.v. Lovak €14 / Magnum €19,95.</t>
+          <t>+ verzending NL €12,95 excl. btw (~€15.41 incl. 19%) voor de order → effectief ~€55.37 voor 4 stuks.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="62" customHeight="1">
-      <c r="A18" s="20" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Vloerverwarming</t>
         </is>
       </c>
-      <c r="B18" s="21" t="n">
-        <v>13</v>
-      </c>
-      <c r="C18" s="21" t="inlineStr">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t>altijd</t>
         </is>
       </c>
-      <c r="D18" s="21" t="inlineStr">
-        <is>
-          <t>Elektra</t>
-        </is>
-      </c>
-      <c r="E18" s="21" t="inlineStr">
-        <is>
-          <t>Elektrakabel 230V / signaalkabel (installatiekwaliteit)</t>
-        </is>
-      </c>
-      <c r="F18" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="21" t="inlineStr">
-        <is>
-          <t>YD/YMvK + 2-draads signaal volgens NEN.</t>
-        </is>
-      </c>
-      <c r="H18" s="21" t="inlineStr">
-        <is>
-          <t>Voeding pomp/regeling/actuators.</t>
-        </is>
-      </c>
-      <c r="I18" s="22" t="n">
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Verzending</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Verzending eibhandel.de → NL (DHL zone 1)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>SHIP-NL</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Verzendkosten bij bestelling van 4× Möhlenhoff Alpha 5.</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Levering actuators vanuit DE.</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="21" t="inlineStr">
-        <is>
-          <t>kleinmateriaal</t>
-        </is>
-      </c>
-      <c r="K18" s="23" t="n">
-        <v>25</v>
-      </c>
-      <c r="L18" s="24" t="n">
-        <v>20</v>
-      </c>
-      <c r="M18" s="28" t="inlineStr">
-        <is>
-          <t>upgrade</t>
-        </is>
-      </c>
-      <c r="N18" s="26" t="n">
-        <v>25</v>
-      </c>
-      <c r="O18" s="21" t="inlineStr">
-        <is>
-          <t>Direct</t>
-        </is>
-      </c>
-      <c r="P18" s="21" t="inlineStr">
-        <is>
-          <t>Bouwmarkt / installateur</t>
-        </is>
-      </c>
-      <c r="Q18" s="27" t="inlineStr">
-        <is>
-          <t>https://www.gamma.nl/assortiment/elektra/elektradraad-en-kabel</t>
-        </is>
-      </c>
-      <c r="R18" s="21" t="inlineStr">
-        <is>
-          <t>Gebruik nette installatiekabel + deugdelijke lasdozen; besparen op elektra is valse economie.</t>
-        </is>
-      </c>
-      <c r="S18" s="21" t="inlineStr">
-        <is>
-          <t>Lichte upgrade vs kale minimumkabel.</t>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>order</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>15.41</v>
+      </c>
+      <c r="L18" t="n">
+        <v>15.41</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>prijszoek</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>15.41</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>mee met actuators</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>eibhandel.de</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>https://eibhandel.de/Versand</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Verplicht bij bestelling DE→NL; meegenomen in totalen.</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>€12,95 excl. + 19% MwSt ≈ €15,41. Vrijstelling pas vanaf €1000 warenwaarde.</t>
         </is>
       </c>
     </row>
@@ -2611,36 +2985,36 @@
         </is>
       </c>
       <c r="B19" s="21" t="n">
-        <v>14</v>
-      </c>
-      <c r="C19" s="22" t="inlineStr">
-        <is>
-          <t>h64</t>
+        <v>13</v>
+      </c>
+      <c r="C19" s="21" t="inlineStr">
+        <is>
+          <t>altijd</t>
         </is>
       </c>
       <c r="D19" s="21" t="inlineStr">
         <is>
-          <t>Regeling H64</t>
+          <t>Elektra</t>
         </is>
       </c>
       <c r="E19" s="21" t="inlineStr">
         <is>
-          <t>MAGNUM H64-CC + master WiFi-thermostaat</t>
+          <t>Elektrakabel 230V / signaalkabel (installatiekwaliteit)</t>
         </is>
       </c>
       <c r="F19" s="21" t="inlineStr">
         <is>
-          <t>W81000</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G19" s="21" t="inlineStr">
         <is>
-          <t>8 zones + master WiFi.</t>
+          <t>YD/YMvK + 2-draads signaal volgens NEN.</t>
         </is>
       </c>
       <c r="H19" s="21" t="inlineStr">
         <is>
-          <t>Alleen bij keuze H64.</t>
+          <t>Voeding pomp/regeling/actuators.</t>
         </is>
       </c>
       <c r="I19" s="22" t="n">
@@ -2648,46 +3022,46 @@
       </c>
       <c r="J19" s="21" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>kleinmateriaal</t>
         </is>
       </c>
       <c r="K19" s="23" t="n">
-        <v>213.74</v>
+        <v>25</v>
       </c>
       <c r="L19" s="24" t="n">
-        <v>213.74</v>
-      </c>
-      <c r="M19" s="25" t="inlineStr">
-        <is>
-          <t>behouden</t>
+        <v>20</v>
+      </c>
+      <c r="M19" s="28" t="inlineStr">
+        <is>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="N19" s="26" t="n">
-        <v>213.74</v>
+        <v>25</v>
       </c>
       <c r="O19" s="21" t="inlineStr">
         <is>
-          <t>Morgen in huis (v. 14:30)</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="P19" s="21" t="inlineStr">
         <is>
-          <t>123InstallatieMaterialen</t>
+          <t>Bouwmarkt / installateur</t>
         </is>
       </c>
       <c r="Q19" s="27" t="inlineStr">
         <is>
-          <t>https://123installatiematerialen.nl/magnum-h64-set-bedraad-controlcenter-master-thermostaat-wifi/</t>
+          <t>https://www.gamma.nl/assortiment/elektra/elektradraad-en-kabel</t>
         </is>
       </c>
       <c r="R19" s="21" t="inlineStr">
         <is>
-          <t>Binnen H64-lijn is dit het juiste product; geen beter Magnum-alternatief.</t>
+          <t>Gebruik nette installatiekabel + deugdelijke lasdozen; besparen op elektra is valse economie.</t>
         </is>
       </c>
       <c r="S19" s="21" t="inlineStr">
         <is>
-          <t>Scherpste H64-prijs, zelfde Magnum-kwaliteit.</t>
+          <t>Lichte upgrade vs kale minimumkabel.</t>
         </is>
       </c>
     </row>
@@ -2698,7 +3072,7 @@
         </is>
       </c>
       <c r="B20" s="21" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C20" s="22" t="inlineStr">
         <is>
@@ -2712,37 +3086,37 @@
       </c>
       <c r="E20" s="21" t="inlineStr">
         <is>
-          <t>MAGNUM H64-ST slave thermostaat</t>
+          <t>MAGNUM H64-CC + master WiFi-thermostaat</t>
         </is>
       </c>
       <c r="F20" s="21" t="inlineStr">
         <is>
-          <t>W81003</t>
+          <t>W81000</t>
         </is>
       </c>
       <c r="G20" s="21" t="inlineStr">
         <is>
-          <t>Bedrade slave-klokthermostaat.</t>
+          <t>8 zones + master WiFi.</t>
         </is>
       </c>
       <c r="H20" s="21" t="inlineStr">
         <is>
-          <t>Ruimte 2 en 3 bij H64.</t>
+          <t>Alleen bij keuze H64.</t>
         </is>
       </c>
       <c r="I20" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20" s="21" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>set</t>
         </is>
       </c>
       <c r="K20" s="23" t="n">
-        <v>52.92</v>
+        <v>194.92</v>
       </c>
       <c r="L20" s="24" t="n">
-        <v>52.92</v>
+        <v>194.92</v>
       </c>
       <c r="M20" s="25" t="inlineStr">
         <is>
@@ -2750,31 +3124,31 @@
         </is>
       </c>
       <c r="N20" s="26" t="n">
-        <v>105.84</v>
+        <v>194.92</v>
       </c>
       <c r="O20" s="21" t="inlineStr">
         <is>
-          <t>Morgen in huis (v. 14:30)</t>
+          <t>1 werkdag (voor 12:00 zelfde dag verzonden)</t>
         </is>
       </c>
       <c r="P20" s="21" t="inlineStr">
         <is>
-          <t>123InstallatieMaterialen</t>
+          <t>Warp Systems</t>
         </is>
       </c>
       <c r="Q20" s="27" t="inlineStr">
         <is>
-          <t>https://123installatiematerialen.nl/magnum-h64-st-bedraad-slave-thermostaat/</t>
+          <t>https://shop.warp-systems.com/h64-control-center-master-wifi-thermostaat-wit-of-zwart-magh64cc-mt-c</t>
         </is>
       </c>
       <c r="R20" s="21" t="inlineStr">
         <is>
-          <t>Passend bij H64-CC; geen kwaliteitswinst bij andere slave.</t>
+          <t>Goedkoper dan 123IM (€213.74): Warp/fabrikant €194,92, 1 wd levering.</t>
         </is>
       </c>
       <c r="S20" s="21" t="inlineStr">
         <is>
-          <t>Scherpste prijs.</t>
+          <t>Kies wit of zwart; zelfde prijs.</t>
         </is>
       </c>
     </row>
@@ -2785,51 +3159,51 @@
         </is>
       </c>
       <c r="B21" s="21" t="n">
-        <v>16</v>
-      </c>
-      <c r="C21" s="29" t="inlineStr">
-        <is>
-          <t>tado_draadloos</t>
+        <v>15</v>
+      </c>
+      <c r="C21" s="22" t="inlineStr">
+        <is>
+          <t>h64</t>
         </is>
       </c>
       <c r="D21" s="21" t="inlineStr">
         <is>
-          <t>Regeling Tado</t>
+          <t>Regeling H64</t>
         </is>
       </c>
       <c r="E21" s="21" t="inlineStr">
         <is>
-          <t>tado° Draadloze Slimme Thermostaat X Starterskit</t>
+          <t>MAGNUM H64-ST slave thermostaat</t>
         </is>
       </c>
       <c r="F21" s="21" t="inlineStr">
         <is>
-          <t>Wireless X Starter</t>
+          <t>W81003</t>
         </is>
       </c>
       <c r="G21" s="21" t="inlineStr">
         <is>
-          <t>Ontvanger X + sensor X per zone.</t>
+          <t>Bedrade slave-klokthermostaat.</t>
         </is>
       </c>
       <c r="H21" s="21" t="inlineStr">
         <is>
-          <t>3 ruimten apart (draadloos).</t>
+          <t>Ruimte 2 en 3 bij H64.</t>
         </is>
       </c>
       <c r="I21" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J21" s="21" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>st</t>
         </is>
       </c>
       <c r="K21" s="23" t="n">
-        <v>129</v>
+        <v>44.58</v>
       </c>
       <c r="L21" s="24" t="n">
-        <v>129</v>
+        <v>44.58</v>
       </c>
       <c r="M21" s="25" t="inlineStr">
         <is>
@@ -2837,31 +3211,31 @@
         </is>
       </c>
       <c r="N21" s="26" t="n">
-        <v>387</v>
+        <v>89.16</v>
       </c>
       <c r="O21" s="21" t="inlineStr">
         <is>
-          <t>2–4 werkdagen</t>
+          <t>1 werkdag</t>
         </is>
       </c>
       <c r="P21" s="21" t="inlineStr">
         <is>
-          <t>tado° Shop</t>
+          <t>Warp Systems</t>
         </is>
       </c>
       <c r="Q21" s="27" t="inlineStr">
         <is>
-          <t>https://shop.tado.com/nl-bx/products/wireless-smart-thermostat-x-starter-kit</t>
+          <t>https://shop.warp-systems.com/catalogsearch/result/?q=slave+H64</t>
         </is>
       </c>
       <c r="R21" s="21" t="inlineStr">
         <is>
-          <t>Prima, maar bedraad is kwalitatief stabieler (zie nr 17–18).</t>
+          <t>Goedkoper bij Warp (€44.58) dan elders (€52.92).</t>
         </is>
       </c>
       <c r="S21" s="21" t="inlineStr">
         <is>
-          <t>Goedkoopste Tado-shopprijs.</t>
+          <t>Controleer kleur (wit/zwart) bij bestellen.</t>
         </is>
       </c>
     </row>
@@ -2872,11 +3246,11 @@
         </is>
       </c>
       <c r="B22" s="21" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C22" s="29" t="inlineStr">
         <is>
-          <t>tado_bedraad</t>
+          <t>tado_draadloos</t>
         </is>
       </c>
       <c r="D22" s="21" t="inlineStr">
@@ -2886,26 +3260,26 @@
       </c>
       <c r="E22" s="21" t="inlineStr">
         <is>
-          <t>tado° Slimme Thermostaat X Starterskit bedraad + Bridge X</t>
+          <t>tado° Draadloze Slimme Thermostaat X Starterskit</t>
         </is>
       </c>
       <c r="F22" s="21" t="inlineStr">
         <is>
-          <t>Wired X Starter</t>
+          <t>Wireless X Starter</t>
         </is>
       </c>
       <c r="G22" s="21" t="inlineStr">
         <is>
-          <t>Bedrade thermostaat X + Bridge X.</t>
+          <t>Ontvanger X + sensor X per zone.</t>
         </is>
       </c>
       <c r="H22" s="21" t="inlineStr">
         <is>
-          <t>Kamer 1 + netwerk.</t>
+          <t>3 ruimten apart (draadloos).</t>
         </is>
       </c>
       <c r="I22" s="22" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J22" s="21" t="inlineStr">
         <is>
@@ -2913,18 +3287,18 @@
         </is>
       </c>
       <c r="K22" s="23" t="n">
-        <v>129.99</v>
+        <v>129</v>
       </c>
       <c r="L22" s="24" t="n">
-        <v>129.99</v>
-      </c>
-      <c r="M22" s="28" t="inlineStr">
-        <is>
-          <t>upgrade</t>
+        <v>129</v>
+      </c>
+      <c r="M22" s="25" t="inlineStr">
+        <is>
+          <t>behouden</t>
         </is>
       </c>
       <c r="N22" s="26" t="n">
-        <v>129.99</v>
+        <v>387</v>
       </c>
       <c r="O22" s="21" t="inlineStr">
         <is>
@@ -2938,17 +3312,17 @@
       </c>
       <c r="Q22" s="27" t="inlineStr">
         <is>
-          <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-starter-kit-1</t>
+          <t>https://shop.tado.com/nl-bx/products/wireless-smart-thermostat-x-starter-kit</t>
         </is>
       </c>
       <c r="R22" s="21" t="inlineStr">
         <is>
-          <t>Bedraad is kwalitatief beter dan 3× draadloos: stabielere voeding/communicatie, minder batterijen, betrouwbaarder bij VV.</t>
+          <t>Prima, maar bedraad is kwalitatief stabieler (zie nr 17–18).</t>
         </is>
       </c>
       <c r="S22" s="21" t="inlineStr">
         <is>
-          <t>AANBEVOLEN Tado-route.</t>
+          <t>Goedkoopste Tado-shopprijs.</t>
         </is>
       </c>
     </row>
@@ -2959,7 +3333,7 @@
         </is>
       </c>
       <c r="B23" s="21" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C23" s="29" t="inlineStr">
         <is>
@@ -2973,37 +3347,37 @@
       </c>
       <c r="E23" s="21" t="inlineStr">
         <is>
-          <t>tado° Slimme Thermostaat X bedraad (uitbreiding)</t>
+          <t>tado° Slimme Thermostaat X Starterskit bedraad + Bridge X</t>
         </is>
       </c>
       <c r="F23" s="21" t="inlineStr">
         <is>
-          <t>Smart Thermostat X</t>
+          <t>Wired X Starter</t>
         </is>
       </c>
       <c r="G23" s="21" t="inlineStr">
         <is>
-          <t>Extra bedrade thermostaat.</t>
+          <t>Bedrade thermostaat X + Bridge X.</t>
         </is>
       </c>
       <c r="H23" s="21" t="inlineStr">
         <is>
-          <t>Kamer 2 en 3.</t>
+          <t>Kamer 1 + netwerk.</t>
         </is>
       </c>
       <c r="I23" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J23" s="21" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>set</t>
         </is>
       </c>
       <c r="K23" s="23" t="n">
-        <v>100</v>
+        <v>129.99</v>
       </c>
       <c r="L23" s="24" t="n">
-        <v>100</v>
+        <v>129.99</v>
       </c>
       <c r="M23" s="28" t="inlineStr">
         <is>
@@ -3011,7 +3385,7 @@
         </is>
       </c>
       <c r="N23" s="26" t="n">
-        <v>200</v>
+        <v>129.99</v>
       </c>
       <c r="O23" s="21" t="inlineStr">
         <is>
@@ -3025,17 +3399,17 @@
       </c>
       <c r="Q23" s="27" t="inlineStr">
         <is>
-          <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-wired</t>
+          <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-starter-kit-1</t>
         </is>
       </c>
       <c r="R23" s="21" t="inlineStr">
         <is>
-          <t>Onderdeel van bedrade (betere) Tado-setup.</t>
+          <t>Bedraad is kwalitatief beter dan 3× draadloos: stabielere voeding/communicatie, minder batterijen, betrouwbaarder bij VV.</t>
         </is>
       </c>
       <c r="S23" s="21" t="inlineStr">
         <is>
-          <t>Bij bedrade starter.</t>
+          <t>AANBEVOLEN Tado-route.</t>
         </is>
       </c>
     </row>
@@ -3046,148 +3420,237 @@
         </is>
       </c>
       <c r="B24" s="21" t="n">
+        <v>18</v>
+      </c>
+      <c r="C24" s="29" t="inlineStr">
+        <is>
+          <t>tado_bedraad</t>
+        </is>
+      </c>
+      <c r="D24" s="21" t="inlineStr">
+        <is>
+          <t>Regeling Tado</t>
+        </is>
+      </c>
+      <c r="E24" s="21" t="inlineStr">
+        <is>
+          <t>tado° Slimme Thermostaat X bedraad (uitbreiding)</t>
+        </is>
+      </c>
+      <c r="F24" s="21" t="inlineStr">
+        <is>
+          <t>Smart Thermostat X</t>
+        </is>
+      </c>
+      <c r="G24" s="21" t="inlineStr">
+        <is>
+          <t>Extra bedrade thermostaat.</t>
+        </is>
+      </c>
+      <c r="H24" s="21" t="inlineStr">
+        <is>
+          <t>Kamer 2 en 3.</t>
+        </is>
+      </c>
+      <c r="I24" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="J24" s="21" t="inlineStr">
+        <is>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="K24" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="L24" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="M24" s="28" t="inlineStr">
+        <is>
+          <t>upgrade</t>
+        </is>
+      </c>
+      <c r="N24" s="26" t="n">
+        <v>200</v>
+      </c>
+      <c r="O24" s="21" t="inlineStr">
+        <is>
+          <t>2–4 werkdagen</t>
+        </is>
+      </c>
+      <c r="P24" s="21" t="inlineStr">
+        <is>
+          <t>tado° Shop</t>
+        </is>
+      </c>
+      <c r="Q24" s="27" t="inlineStr">
+        <is>
+          <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-wired</t>
+        </is>
+      </c>
+      <c r="R24" s="21" t="inlineStr">
+        <is>
+          <t>Onderdeel van bedrade (betere) Tado-setup.</t>
+        </is>
+      </c>
+      <c r="S24" s="21" t="inlineStr">
+        <is>
+          <t>Bij bedrade starter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="20" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B25" s="21" t="n">
         <v>19</v>
       </c>
-      <c r="C24" s="29" t="inlineStr">
+      <c r="C25" s="29" t="inlineStr">
         <is>
           <t>tado_optie</t>
         </is>
       </c>
-      <c r="D24" s="21" t="inlineStr">
+      <c r="D25" s="21" t="inlineStr">
         <is>
           <t>Regeling Tado</t>
         </is>
       </c>
-      <c r="E24" s="21" t="inlineStr">
+      <c r="E25" s="21" t="inlineStr">
         <is>
           <t>tado° Bridge X (extra indien nodig)</t>
         </is>
       </c>
-      <c r="F24" s="21" t="inlineStr">
+      <c r="F25" s="21" t="inlineStr">
         <is>
           <t>Bridge X</t>
         </is>
       </c>
-      <c r="G24" s="21" t="inlineStr">
+      <c r="G25" s="21" t="inlineStr">
         <is>
           <t>Extra Thread border router.</t>
         </is>
       </c>
-      <c r="H24" s="21" t="inlineStr">
+      <c r="H25" s="21" t="inlineStr">
         <is>
           <t>Alleen bij bereikproblemen.</t>
         </is>
       </c>
-      <c r="I24" s="22" t="n">
+      <c r="I25" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="J24" s="21" t="inlineStr">
+      <c r="J25" s="21" t="inlineStr">
         <is>
           <t>st</t>
         </is>
       </c>
-      <c r="K24" s="23" t="n">
+      <c r="K25" s="23" t="n">
         <v>68</v>
       </c>
-      <c r="L24" s="24" t="n">
+      <c r="L25" s="24" t="n">
         <v>68</v>
       </c>
-      <c r="M24" s="25" t="inlineStr">
+      <c r="M25" s="25" t="inlineStr">
         <is>
           <t>behouden</t>
         </is>
       </c>
-      <c r="N24" s="26" t="n">
+      <c r="N25" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="O24" s="21" t="inlineStr">
+      <c r="O25" s="21" t="inlineStr">
         <is>
           <t>1–3 werkdagen</t>
         </is>
       </c>
-      <c r="P24" s="21" t="inlineStr">
+      <c r="P25" s="21" t="inlineStr">
         <is>
           <t>Coolblue / tado°</t>
         </is>
       </c>
-      <c r="Q24" s="27" t="inlineStr">
+      <c r="Q25" s="27" t="inlineStr">
         <is>
           <t>https://www.coolblue.nl/thermostaten/tado</t>
         </is>
       </c>
-      <c r="R24" s="21" t="inlineStr">
+      <c r="R25" s="21" t="inlineStr">
         <is>
           <t>Meestal overbodig bij bedrade starter of ontvangers.</t>
         </is>
       </c>
-      <c r="S24" s="21" t="inlineStr">
+      <c r="S25" s="21" t="inlineStr">
         <is>
           <t>Qty=0.</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="22" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="26" ht="22" customHeight="1"/>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>KOPJE: (nog leeg)</t>
         </is>
       </c>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
-      <c r="J26" s="3" t="n"/>
-      <c r="K26" s="3" t="n"/>
-      <c r="L26" s="3" t="n"/>
-      <c r="M26" s="3" t="n"/>
-      <c r="N26" s="3" t="n"/>
-      <c r="O26" s="3" t="n"/>
-      <c r="P26" s="3" t="n"/>
-      <c r="Q26" s="3" t="n"/>
-      <c r="R26" s="3" t="n"/>
-      <c r="S26" s="3" t="n"/>
-    </row>
-    <row r="28">
-      <c r="J28" s="30" t="inlineStr">
+      <c r="B27" s="38" t="n"/>
+      <c r="C27" s="38" t="n"/>
+      <c r="D27" s="38" t="n"/>
+      <c r="E27" s="38" t="n"/>
+      <c r="F27" s="38" t="n"/>
+      <c r="G27" s="38" t="n"/>
+      <c r="H27" s="38" t="n"/>
+      <c r="I27" s="38" t="n"/>
+      <c r="J27" s="38" t="n"/>
+      <c r="K27" s="38" t="n"/>
+      <c r="L27" s="38" t="n"/>
+      <c r="M27" s="38" t="n"/>
+      <c r="N27" s="38" t="n"/>
+      <c r="O27" s="38" t="n"/>
+      <c r="P27" s="38" t="n"/>
+      <c r="Q27" s="38" t="n"/>
+      <c r="R27" s="38" t="n"/>
+      <c r="S27" s="39" t="n"/>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="J29" s="30" t="inlineStr">
         <is>
           <t>Vloerverwarming + Tado BEDRAAD (aanbevolen)</t>
         </is>
       </c>
-      <c r="N28" s="31" t="n">
+      <c r="N29" s="31" t="n">
         <v>2420.09</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Vloerverwarming + Tado draadloos</t>
-        </is>
-      </c>
-      <c r="N29" s="32" t="n">
-        <v>2477.1</v>
       </c>
     </row>
     <row r="30">
       <c r="J30" t="inlineStr">
         <is>
-          <t>Vloerverwarming + Magnum H64</t>
-        </is>
-      </c>
-      <c r="N30" s="33" t="n">
-        <v>2409.68</v>
+          <t>Vloerverwarming + Tado draadloos</t>
+        </is>
+      </c>
+      <c r="N30" s="32" t="n">
+        <v>2477.1</v>
       </c>
     </row>
     <row r="31">
       <c r="J31" t="inlineStr">
         <is>
+          <t>Vloerverwarming + Magnum H64</t>
+        </is>
+      </c>
+      <c r="N31" s="33" t="n">
+        <v>2409.68</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="J32" t="inlineStr">
+        <is>
           <t>Meerprijs vs pure goedkoopste (Tado bedraad)</t>
         </is>
       </c>
-      <c r="N31" s="34" t="n">
+      <c r="N32" s="34" t="n">
         <v>135.82</v>
       </c>
     </row>
@@ -3223,7 +3686,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3244,9 +3707,9 @@
           <t>KOPJE: Vloerverwarming — Tado</t>
         </is>
       </c>
-      <c r="B1" s="3" t="n"/>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="3" t="n"/>
+      <c r="B1" s="38" t="n"/>
+      <c r="C1" s="38" t="n"/>
+      <c r="D1" s="39" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -3351,7 +3814,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3376,13 +3839,13 @@
           <t>KOPJE: Vloerverwarming — checklist</t>
         </is>
       </c>
-      <c r="B1" s="3" t="n"/>
-      <c r="C1" s="3" t="n"/>
-      <c r="D1" s="3" t="n"/>
-      <c r="E1" s="3" t="n"/>
-      <c r="F1" s="3" t="n"/>
-      <c r="G1" s="3" t="n"/>
-      <c r="H1" s="3" t="n"/>
+      <c r="B1" s="38" t="n"/>
+      <c r="C1" s="38" t="n"/>
+      <c r="D1" s="38" t="n"/>
+      <c r="E1" s="38" t="n"/>
+      <c r="F1" s="38" t="n"/>
+      <c r="G1" s="38" t="n"/>
+      <c r="H1" s="39" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
@@ -3796,11 +4259,11 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>VerwarmingOnline</t>
+          <t>eibhandel.de</t>
         </is>
       </c>
       <c r="E15" s="36" t="n">
-        <v>20.12</v>
+        <v>9.99</v>
       </c>
       <c r="F15" s="37" t="inlineStr">
         <is>
@@ -3860,11 +4323,11 @@
       </c>
       <c r="D17" s="8" t="inlineStr">
         <is>
-          <t>123InstallatieMaterialen</t>
+          <t>Warp Systems</t>
         </is>
       </c>
       <c r="E17" s="36" t="n">
-        <v>213.74</v>
+        <v>194.92</v>
       </c>
       <c r="F17" s="37" t="inlineStr">
         <is>
@@ -3892,11 +4355,11 @@
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>123InstallatieMaterialen</t>
+          <t>Warp Systems</t>
         </is>
       </c>
       <c r="E18" s="36" t="n">
-        <v>52.92</v>
+        <v>44.58</v>
       </c>
       <c r="F18" s="37" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Clarify Overzicht notes after top-5 price hunt
Co-authored-by: bmverhagen <bmverhagen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Materiaalbenodigdheden_Vloerverwarming.xlsx
+++ b/Materiaalbenodigdheden_Vloerverwarming.xlsx
@@ -663,7 +663,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -684,7 +683,6 @@
         <v/>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
@@ -720,7 +718,7 @@
       </c>
       <c r="C8" s="10" t="inlineStr">
         <is>
-          <t>incl. prijszoek (actuators DE + H64 Warp)</t>
+          <t>prijszoek: −€25 actuators (DE)</t>
         </is>
       </c>
     </row>
@@ -735,7 +733,7 @@
       </c>
       <c r="C9" s="10" t="inlineStr">
         <is>
-          <t>incl. prijszoek (actuators DE + H64 Warp)</t>
+          <t>aanbevolen pad</t>
         </is>
       </c>
     </row>
@@ -748,11 +746,7 @@
       <c r="B10" s="9" t="n">
         <v>2451.99</v>
       </c>
-      <c r="C10" s="10" t="inlineStr">
-        <is>
-          <t>incl. prijszoek (actuators DE + H64 Warp)</t>
-        </is>
-      </c>
+      <c r="C10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -765,22 +759,21 @@
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>incl. prijszoek (actuators DE + H64 Warp)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
+          <t>H64 via Warp (−€19 CC, −€17 slaves)</t>
+        </is>
+      </c>
+    </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Kwaliteit: VTE Composiet · Möhlenhoff Alpha 5 · NMC Climasol. Prijszoek: actuators via eibhandel.de, H64 via Warp.</t>
+          <t>Kwaliteit: VTE Composiet · Möhlenhoff Alpha 5 · NMC. Prijszoek top-5: actuators eibhandel.de, H64 Warp; SlimFit/Kreisel/VTE/PE-RT al scherpst binnen ≤1 week.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
         <is>
-          <t>Aanbevolen: Tado bedraad (stabieler dan draadloos).</t>
+          <t>Aanbevolen: Tado bedraad (~€2.395). Zie sheet Prijszoek-top5 voor shopvergelijking.</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -3613,7 +3606,6 @@
       <c r="R27" s="38" t="n"/>
       <c r="S27" s="39" t="n"/>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="J29" s="30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Recheck all-in prices including shipping; keep current shops
Correct free-shipping thresholds (Elektramat €150 excl, 123shop
€150, Installand €60). Add All-in-check sheet: every chosen shop
remains cheapest after shipping; only foreign source is eibhandel
DE→NL with DHL costs and lead time included.

Co-authored-by: bmverhagen <bmverhagen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Materiaalbenodigdheden_Vloerverwarming.xlsx
+++ b/Materiaalbenodigdheden_Vloerverwarming.xlsx
@@ -10,12 +10,13 @@
     <sheet name="Overzicht" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Parameters" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Boodschappenlijst" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Verzending" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Regeling-keuze" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Kwaliteitskeuzes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Prijszoek-top5" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Tado-aansluiting" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Bestelchecklist" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="All-in-check" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Verzending" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Regeling-keuze" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Kwaliteitskeuzes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Prijszoek-top5" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Tado-aansluiting" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Bestelchecklist" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="Oppervlakte_m2">Parameters!$B$4</definedName>
@@ -31,7 +32,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,6 +70,22 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F7A3F"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F7A3F"/>
       <sz val="12"/>
     </font>
   </fonts>
@@ -131,7 +148,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -151,6 +168,12 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -516,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="36" customWidth="1" min="1" max="1"/>
@@ -713,7 +736,589 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Aanbevolen: Tado bedraad. Alles op deze lijst is NL-leverbaar (eibhandel = DE→NL met DHL, verzending meegenomen).</t>
+          <t>All-in incl. verzending. Na hercheck (aug 2026): alle shops blijven goedkoopst — zie All-in-check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Enige import: eibhandel.de actuators (NL via DHL, verzending meegenomen).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="55" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>KOPJE: Vloerverwarming — checklist (hoeveelheden = live uit Boodschappenlijst)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Artikel</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Qty</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Webshop</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Prijs/st</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Totaal</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Besteld?</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Ordernr</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <f>Boodschappenlijst!E6</f>
+        <v/>
+      </c>
+      <c r="B4">
+        <f>Boodschappenlijst!I6</f>
+        <v/>
+      </c>
+      <c r="C4">
+        <f>Boodschappenlijst!P6</f>
+        <v/>
+      </c>
+      <c r="D4" s="5">
+        <f>Boodschappenlijst!K6</f>
+        <v/>
+      </c>
+      <c r="E4" s="5">
+        <f>Boodschappenlijst!N6</f>
+        <v/>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <f>Boodschappenlijst!E7</f>
+        <v/>
+      </c>
+      <c r="B5">
+        <f>Boodschappenlijst!I7</f>
+        <v/>
+      </c>
+      <c r="C5">
+        <f>Boodschappenlijst!P7</f>
+        <v/>
+      </c>
+      <c r="D5" s="5">
+        <f>Boodschappenlijst!K7</f>
+        <v/>
+      </c>
+      <c r="E5" s="5">
+        <f>Boodschappenlijst!N7</f>
+        <v/>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <f>Boodschappenlijst!E8</f>
+        <v/>
+      </c>
+      <c r="B6">
+        <f>Boodschappenlijst!I8</f>
+        <v/>
+      </c>
+      <c r="C6">
+        <f>Boodschappenlijst!P8</f>
+        <v/>
+      </c>
+      <c r="D6" s="5">
+        <f>Boodschappenlijst!K8</f>
+        <v/>
+      </c>
+      <c r="E6" s="5">
+        <f>Boodschappenlijst!N8</f>
+        <v/>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <f>Boodschappenlijst!E9</f>
+        <v/>
+      </c>
+      <c r="B7">
+        <f>Boodschappenlijst!I9</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>Boodschappenlijst!P9</f>
+        <v/>
+      </c>
+      <c r="D7" s="5">
+        <f>Boodschappenlijst!K9</f>
+        <v/>
+      </c>
+      <c r="E7" s="5">
+        <f>Boodschappenlijst!N9</f>
+        <v/>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <f>Boodschappenlijst!E10</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>Boodschappenlijst!I10</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>Boodschappenlijst!P10</f>
+        <v/>
+      </c>
+      <c r="D8" s="5">
+        <f>Boodschappenlijst!K10</f>
+        <v/>
+      </c>
+      <c r="E8" s="5">
+        <f>Boodschappenlijst!N10</f>
+        <v/>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <f>Boodschappenlijst!E11</f>
+        <v/>
+      </c>
+      <c r="B9">
+        <f>Boodschappenlijst!I11</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>Boodschappenlijst!P11</f>
+        <v/>
+      </c>
+      <c r="D9" s="5">
+        <f>Boodschappenlijst!K11</f>
+        <v/>
+      </c>
+      <c r="E9" s="5">
+        <f>Boodschappenlijst!N11</f>
+        <v/>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <f>Boodschappenlijst!E12</f>
+        <v/>
+      </c>
+      <c r="B10">
+        <f>Boodschappenlijst!I12</f>
+        <v/>
+      </c>
+      <c r="C10">
+        <f>Boodschappenlijst!P12</f>
+        <v/>
+      </c>
+      <c r="D10" s="5">
+        <f>Boodschappenlijst!K12</f>
+        <v/>
+      </c>
+      <c r="E10" s="5">
+        <f>Boodschappenlijst!N12</f>
+        <v/>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <f>Boodschappenlijst!E13</f>
+        <v/>
+      </c>
+      <c r="B11">
+        <f>Boodschappenlijst!I13</f>
+        <v/>
+      </c>
+      <c r="C11">
+        <f>Boodschappenlijst!P13</f>
+        <v/>
+      </c>
+      <c r="D11" s="5">
+        <f>Boodschappenlijst!K13</f>
+        <v/>
+      </c>
+      <c r="E11" s="5">
+        <f>Boodschappenlijst!N13</f>
+        <v/>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <f>Boodschappenlijst!E14</f>
+        <v/>
+      </c>
+      <c r="B12">
+        <f>Boodschappenlijst!I14</f>
+        <v/>
+      </c>
+      <c r="C12">
+        <f>Boodschappenlijst!P14</f>
+        <v/>
+      </c>
+      <c r="D12" s="5">
+        <f>Boodschappenlijst!K14</f>
+        <v/>
+      </c>
+      <c r="E12" s="5">
+        <f>Boodschappenlijst!N14</f>
+        <v/>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <f>Boodschappenlijst!E15</f>
+        <v/>
+      </c>
+      <c r="B13">
+        <f>Boodschappenlijst!I15</f>
+        <v/>
+      </c>
+      <c r="C13">
+        <f>Boodschappenlijst!P15</f>
+        <v/>
+      </c>
+      <c r="D13" s="5">
+        <f>Boodschappenlijst!K15</f>
+        <v/>
+      </c>
+      <c r="E13" s="5">
+        <f>Boodschappenlijst!N15</f>
+        <v/>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14">
+        <f>Boodschappenlijst!E16</f>
+        <v/>
+      </c>
+      <c r="B14">
+        <f>Boodschappenlijst!I16</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>Boodschappenlijst!P16</f>
+        <v/>
+      </c>
+      <c r="D14" s="5">
+        <f>Boodschappenlijst!K16</f>
+        <v/>
+      </c>
+      <c r="E14" s="5">
+        <f>Boodschappenlijst!N16</f>
+        <v/>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15">
+        <f>Boodschappenlijst!E17</f>
+        <v/>
+      </c>
+      <c r="B15">
+        <f>Boodschappenlijst!I17</f>
+        <v/>
+      </c>
+      <c r="C15">
+        <f>Boodschappenlijst!P17</f>
+        <v/>
+      </c>
+      <c r="D15" s="5">
+        <f>Boodschappenlijst!K17</f>
+        <v/>
+      </c>
+      <c r="E15" s="5">
+        <f>Boodschappenlijst!N17</f>
+        <v/>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16">
+        <f>Boodschappenlijst!E18</f>
+        <v/>
+      </c>
+      <c r="B16">
+        <f>Boodschappenlijst!I18</f>
+        <v/>
+      </c>
+      <c r="C16">
+        <f>Boodschappenlijst!P18</f>
+        <v/>
+      </c>
+      <c r="D16" s="5">
+        <f>Boodschappenlijst!K18</f>
+        <v/>
+      </c>
+      <c r="E16" s="5">
+        <f>Boodschappenlijst!N18</f>
+        <v/>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17">
+        <f>Boodschappenlijst!E19</f>
+        <v/>
+      </c>
+      <c r="B17">
+        <f>Boodschappenlijst!I19</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>Boodschappenlijst!P19</f>
+        <v/>
+      </c>
+      <c r="D17" s="5">
+        <f>Boodschappenlijst!K19</f>
+        <v/>
+      </c>
+      <c r="E17" s="5">
+        <f>Boodschappenlijst!N19</f>
+        <v/>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <f>Boodschappenlijst!E20</f>
+        <v/>
+      </c>
+      <c r="B18">
+        <f>Boodschappenlijst!I20</f>
+        <v/>
+      </c>
+      <c r="C18">
+        <f>Boodschappenlijst!P20</f>
+        <v/>
+      </c>
+      <c r="D18" s="5">
+        <f>Boodschappenlijst!K20</f>
+        <v/>
+      </c>
+      <c r="E18" s="5">
+        <f>Boodschappenlijst!N20</f>
+        <v/>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
+        <f>Boodschappenlijst!E21</f>
+        <v/>
+      </c>
+      <c r="B19">
+        <f>Boodschappenlijst!I21</f>
+        <v/>
+      </c>
+      <c r="C19">
+        <f>Boodschappenlijst!P21</f>
+        <v/>
+      </c>
+      <c r="D19" s="5">
+        <f>Boodschappenlijst!K21</f>
+        <v/>
+      </c>
+      <c r="E19" s="5">
+        <f>Boodschappenlijst!N21</f>
+        <v/>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20">
+        <f>Boodschappenlijst!E22</f>
+        <v/>
+      </c>
+      <c r="B20">
+        <f>Boodschappenlijst!I22</f>
+        <v/>
+      </c>
+      <c r="C20">
+        <f>Boodschappenlijst!P22</f>
+        <v/>
+      </c>
+      <c r="D20" s="5">
+        <f>Boodschappenlijst!K22</f>
+        <v/>
+      </c>
+      <c r="E20" s="5">
+        <f>Boodschappenlijst!N22</f>
+        <v/>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21">
+        <f>Boodschappenlijst!E23</f>
+        <v/>
+      </c>
+      <c r="B21">
+        <f>Boodschappenlijst!I23</f>
+        <v/>
+      </c>
+      <c r="C21">
+        <f>Boodschappenlijst!P23</f>
+        <v/>
+      </c>
+      <c r="D21" s="5">
+        <f>Boodschappenlijst!K23</f>
+        <v/>
+      </c>
+      <c r="E21" s="5">
+        <f>Boodschappenlijst!N23</f>
+        <v/>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <f>Boodschappenlijst!E24</f>
+        <v/>
+      </c>
+      <c r="B22">
+        <f>Boodschappenlijst!I24</f>
+        <v/>
+      </c>
+      <c r="C22">
+        <f>Boodschappenlijst!P24</f>
+        <v/>
+      </c>
+      <c r="D22" s="5">
+        <f>Boodschappenlijst!K24</f>
+        <v/>
+      </c>
+      <c r="E22" s="5">
+        <f>Boodschappenlijst!N24</f>
+        <v/>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Nee</t>
         </is>
       </c>
     </row>
@@ -728,7 +1333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -974,29 +1579,29 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>VERZENDREGELS (NL, all-in)</t>
+          <t>VERZENDREGELS (NL, all-in — gecorrigeerd)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="19" t="inlineStr">
         <is>
           <t>Shop</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Gratis vanaf</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="19" t="inlineStr">
         <is>
           <t>Kosten onder drempel</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>Levertijd / land</t>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Levertijd / land / opmerking</t>
         </is>
       </c>
     </row>
@@ -1006,15 +1611,19 @@
           <t>Elektramat</t>
         </is>
       </c>
-      <c r="B21" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="C21" s="5" t="n">
-        <v>6.95</v>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>€150 excl. btw</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>€4,09 excl ≈ €4,95 incl</t>
+        </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NL · 1 werkdag (geschat drempel; check checkout)</t>
+          <t>NL · 1 wd · PostNL</t>
         </is>
       </c>
     </row>
@@ -1024,11 +1633,15 @@
           <t>123InstallatieMaterialen</t>
         </is>
       </c>
-      <c r="B22" s="5" t="n">
-        <v>200</v>
-      </c>
-      <c r="C22" s="5" t="n">
-        <v>6.95</v>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>€200</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>€6,95</t>
+        </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1042,15 +1655,19 @@
           <t>123Installatieshop</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="C23" s="5" t="n">
-        <v>6.95</v>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>€150</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>€6,95</t>
+        </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>NL · morgen in huis</t>
+          <t>NL · volgende werkdag</t>
         </is>
       </c>
     </row>
@@ -1060,15 +1677,19 @@
           <t>EgalineXXL / RBMB</t>
         </is>
       </c>
-      <c r="B24" s="5" t="n">
-        <v>600</v>
-      </c>
-      <c r="C24" s="5" t="n">
-        <v>60.5</v>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>€600 excl. btw</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>pallet ≈ €60,50 incl</t>
+        </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>NL · drempel €600 excl. btw; pallet ≈€60,50 incl daaronder</t>
+          <t>NL · 1–2 wd / palletplanning</t>
         </is>
       </c>
     </row>
@@ -1078,15 +1699,19 @@
           <t>eibhandel.de</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
-        <v>1000</v>
-      </c>
-      <c r="C25" s="5" t="n">
-        <v>15.41</v>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>€1000</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>€12,95 excl ≈ €15,41 incl</t>
+        </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>DE→NL DHL zone 1 · 2–5 wd DE + NL</t>
+          <t>DE→NL DHL zone 1 · 2–5 wd DE (+NL)</t>
         </is>
       </c>
     </row>
@@ -1096,15 +1721,19 @@
           <t>Warp Systems</t>
         </is>
       </c>
-      <c r="B26" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="C26" s="5" t="n">
-        <v>0</v>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>n.v.t. / laag</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>€0 (typisch)</t>
+        </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>NL · 1 werkdag (voor 12:00)</t>
+          <t>NL · 1 wd (voor 12:00)</t>
         </is>
       </c>
     </row>
@@ -1114,15 +1743,19 @@
           <t>tado° Shop</t>
         </is>
       </c>
-      <c r="B27" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="C27" s="5" t="n">
-        <v>4.99</v>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>€150</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>€4,99</t>
+        </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>NL/EU · gratis ≥€150</t>
+          <t>NL/EU · 2–4 wd</t>
         </is>
       </c>
     </row>
@@ -1132,15 +1765,19 @@
           <t>Installand</t>
         </is>
       </c>
-      <c r="B28" s="5" t="n">
-        <v>50</v>
-      </c>
-      <c r="C28" s="5" t="n">
-        <v>6.95</v>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>€60</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>var. / afhalen gratis</t>
+        </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NL</t>
+          <t>NL · vaak volgende wd</t>
         </is>
       </c>
     </row>
@@ -1150,29 +1787,56 @@
           <t>VerwarmingOnline</t>
         </is>
       </c>
-      <c r="B29" s="5" t="n">
-        <v>385</v>
-      </c>
-      <c r="C29" s="5" t="n">
-        <v>6.95</v>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>€385</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>~€6,95</t>
+        </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NL · 3–4 werkdagen</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Tip: totalen in Overzicht zijn inclusief berekende verzendkosten per shop (zie Verzending).</t>
-        </is>
-      </c>
-    </row>
+          <t>NL · 3–4 wd</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Home Perfect (.nl/.de)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>€1000 pakket</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>€29,90–€69 NL-pakket</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>DE-basis · 7–10 wd → te duur/traag all-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="31"/>
     <row r="32">
-      <c r="A32" s="10" t="inlineStr">
-        <is>
-          <t>Verdeler-SKU is 4-groeps. Bij ander aantal groepen: product/prijs handmatig aanpassen op Boodschappenlijst.</t>
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>Conclusie all-in (aug 2026): huidige shops blijven goedkoopst; zie sheet All-in-check. Geen shopwissel nodig.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Buitenland alleen eibhandel.de (actuators): NL-levering bevestigd, verzending + levertijd meegenomen.</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T26"/>
+  <dimension ref="A1:T29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1422,11 +2086,11 @@
         </is>
       </c>
       <c r="S6" s="15" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="T6" s="13" t="inlineStr">
         <is>
-          <t>Schaalt met m². Goedkoopste met voorraad+snelle NL-levering.</t>
+          <t>Schaalt met m². Goedkoopste met voorraad+snelle NL-levering. Drempel gratis verzending €150 excl. btw.</t>
         </is>
       </c>
     </row>
@@ -1518,7 +2182,7 @@
       </c>
       <c r="T7" s="13" t="inlineStr">
         <is>
-          <t>Aantal rollen volgt uit buislengte (~10 m/m²).</t>
+          <t>All-in: +€6,95 verzending (order &lt;€200 bij 123IM). Nog steeds goedkoper dan Elektramat €181,86.</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2734,7 @@
       </c>
       <c r="T13" s="13" t="inlineStr">
         <is>
-          <t>Schaalt met m² × laagdikte. Palletverzending zie Verzending.</t>
+          <t>All-in: +pallet ~€60,50 als order &lt;€600 excl. Goedkoper dan extra zakken kopen voor gratis verzending.</t>
         </is>
       </c>
     </row>
@@ -2428,7 +3092,7 @@
       </c>
       <c r="T17" s="13" t="inlineStr">
         <is>
-          <t>Goedkoopst all-in DE→NL. Alternatief Amazon.nl ~€13,16/st zonder verzendkosten.</t>
+          <t>All-in DE→NL: €9,99×groepen + €15,41 verzending. Goedkoper dan Home Perfect/VerwarmingOnline; NL via DHL.</t>
         </is>
       </c>
     </row>
@@ -3068,6 +3732,7 @@
         </is>
       </c>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
@@ -3075,6 +3740,9 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
   </sheetData>
   <autoFilter ref="A5:T24"/>
   <mergeCells count="1">
@@ -3085,6 +3753,484 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>All-in check — prijs + verzending (nog steeds goedkoopste?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Uitgangspunt: 30 m² · 4 groepen · 3 ruimten. Alleen NL-leverbare opties (of DE→NL met expliciete verzending/levertijd).</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="21" t="inlineStr">
+        <is>
+          <t>Verdict: JA — alle gekozen shops blijven all-in het goedkoopst. Geen shopwissel nodig.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="22" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>Artikel</t>
+        </is>
+      </c>
+      <c r="C5" s="22" t="inlineStr">
+        <is>
+          <t>Gekozen (all-in)</t>
+        </is>
+      </c>
+      <c r="D5" s="22" t="inlineStr">
+        <is>
+          <t>Alternatief all-in</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="inlineStr">
+        <is>
+          <t>Δ</t>
+        </is>
+      </c>
+      <c r="F5" s="22" t="inlineStr">
+        <is>
+          <t>NL-leverbaar?</t>
+        </is>
+      </c>
+      <c r="G5" s="22" t="inlineStr">
+        <is>
+          <t>Verdict</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>SlimFit matten 8×</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Elektramat €695,52 (ship €0; order ≫ €150 excl)</t>
+        </is>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>123IM €711,92 · VV-direct €712</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>−€16…€17</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Ja NL 1 wd</t>
+        </is>
+      </c>
+      <c r="G6" s="23" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>PE-RT 300 m</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>123IM €142,93 + €6,95 ship ≈ €149,88 (order &lt;€200)</t>
+        </is>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Elektramat €181,86 (ship €0 in combi)</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>−€32</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Ja NL morgen</t>
+        </is>
+      </c>
+      <c r="G7" s="23" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Kreisel 418 33× + primer</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>EgalineXXL €509,29 + pallet €60,50 = €569,79</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>RBMB duurder/stuk · extra kopen tot €600 excl ≈ €610+</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>−€40…</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>Ja NL pallet</t>
+        </is>
+      </c>
+      <c r="G8" s="23" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="13" t="inlineStr">
+        <is>
+          <t>VTE Composiet 4-gr.</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>123Installatieshop €387,18 (ship €0 ≥€150)</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>VV-shop €405 · CVTotaal €423 · Jan Isolatieman €469</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>−€18…€82</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Ja NL ≤1 wk</t>
+        </is>
+      </c>
+      <c r="G9" s="23" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Möhlenhoff Alpha 5 ×4</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>eibhandel.de €39,96 + €15,41 = €55,37</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Amazon~€52,64* · Home Perfect €69,94 · VerwarmingOnline €87,43</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>beste bevestigd</t>
+        </is>
+      </c>
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Ja DE→NL DHL</t>
+        </is>
+      </c>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>NMC Climasol 3×</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Installand €71,97 (ship €0 ≥€60)</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Generiek Distriheat goedkoper maar mindere kwaliteit</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>kwaliteit</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Ja NL</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>H64-CC + slaves</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Warp Systems €194,92 + 2×€44,58 (NL)</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>123IM H64-CC was €213,74</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>−€19 CC</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Ja NL 1 wd</t>
+        </is>
+      </c>
+      <c r="G12" s="23" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Tado bedraad 3 ruimten</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>tado° Shop €329,99 (ship €0 ≥€150)</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>bol/retail vaak €189–€194 per starter alleen</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>goedkoopst</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Ja NL/EU</t>
+        </is>
+      </c>
+      <c r="G13" s="23" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Consolidatie-check (minder shops = minder verzending?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• PE-RT meenemen bij Elektramat (zelfde order als SlimFit): all-in €181,86 i.p.v. ~€149,88 → NIET doen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>• Extra egaline kopen tot gratis drempel (€600 excl): duurder dan pallet betalen → NIET doen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>• Actuators bij VerwarmingOnline (pure NL): +€32 vs eibhandel → alleen als je DE wilt vermijden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>• Home Perfect (€10,01/st) lijkt scherp maar +€29,90 ship + 7–10 wd → all-in slechter én trager.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Buitenland / NL-zekerheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Enige buitenlandse shop: eibhandel.de (actuators). Levert naar NL (DHL zone 1), verzending €15,41 incl, levertijd 2–5 wd DE (+NL-transit, meestal ≤1 week).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Alles overige: Nederlandse webshops met snelle levering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>* Amazon.nl-prijs is indicatief (listings wisselen); eibhandel is stabiel bevestigd all-in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Live totalen (formules, schalen met m²)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Basis artikelen</t>
+        </is>
+      </c>
+      <c r="B27" s="6">
+        <f>Overzicht!B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Basis verzending</t>
+        </is>
+      </c>
+      <c r="B28" s="6">
+        <f>Overzicht!C10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Basis all-in</t>
+        </is>
+      </c>
+      <c r="B29" s="6">
+        <f>Overzicht!D10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>All-in + Tado bedraad</t>
+        </is>
+      </c>
+      <c r="B30" s="6">
+        <f>Overzicht!D11</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3175,10 +4321,10 @@
         <v/>
       </c>
       <c r="D5" s="5" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E5" s="5">
-        <f>IF(C5&lt;=0,0,IF(C5&gt;=50,0,6.95))</f>
+        <f>IF(C5&lt;=0,0,IF(C5/1.21&gt;=150,0,4.95))</f>
         <v/>
       </c>
       <c r="F5" s="5">
@@ -3192,7 +4338,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Gratis vaak al bij SlimFit-order</t>
+          <t>Drempel €150 excl. btw; onder: €4,09 excl ≈ €4,95 incl</t>
         </is>
       </c>
     </row>
@@ -3229,7 +4375,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Buis + bochten</t>
+          <t>Buis+bochten vaak &lt;€200 → €6,95 verzending; all-in nog steeds goedkoper dan Elektramat-buis</t>
         </is>
       </c>
     </row>
@@ -3249,10 +4395,10 @@
         <v/>
       </c>
       <c r="D7" s="5" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="E7" s="5">
-        <f>IF(C7&lt;=0,0,IF(C7&gt;=50,0,6.95))</f>
+        <f>IF(C7&lt;=0,0,IF(C7&gt;=150,0,6.95))</f>
         <v/>
       </c>
       <c r="F7" s="5">
@@ -3266,7 +4412,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Verdeler + kranen</t>
+          <t>Verdeler alleen al &gt;€150 → gratis verzending</t>
         </is>
       </c>
     </row>
@@ -3433,10 +4579,10 @@
         <v/>
       </c>
       <c r="D12" s="5" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="E12" s="5">
-        <f>IF(C12&lt;=0,0,IF(C12&gt;=50,0,6.95))</f>
+        <f>IF(C12&lt;=0,0,IF(C12&gt;=60,0,6.95))</f>
         <v/>
       </c>
       <c r="F12" s="5">
@@ -3450,7 +4596,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Randisolatie</t>
+          <t>Gratis vanaf €60; 3 rollen Climasol ≈ €72 → meestal gratis</t>
         </is>
       </c>
     </row>
@@ -3555,7 +4701,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Amazon.nl (alternatief)</t>
+          <t>Amazon.nl (indicatief)</t>
         </is>
       </c>
       <c r="B21" s="5" t="n">
@@ -3574,26 +4720,25 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Ja — Prime NL; check actuele listing</t>
+          <t>Ja — Prime NL; check actuele listing/voorraad</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>VerwarmingOnline NL</t>
+          <t>Home Perfect NL/DE</t>
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>20.12</v>
+        <v>10.01</v>
       </c>
       <c r="C22" s="5">
         <f>B22*Parameters!$B$5</f>
         <v/>
       </c>
-      <c r="D22" s="5">
-        <f>IF(C22&gt;=385,0,6.95)</f>
-        <v/>
+      <c r="D22" s="5" t="n">
+        <v>29.9</v>
       </c>
       <c r="E22" s="5">
         <f>C22+D22</f>
@@ -3601,14 +4746,41 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Ja — NL webshop</t>
+          <t>Nee/matig — €29,90 ship + 7–10 wd</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Conclusie: eibhandel blijft goedkoopst all-in bij 4 groepen; bij meer groepen Amazon soms dichterbij. Beide NL-leverbaar.</t>
+          <t>VerwarmingOnline NL</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>20.12</v>
+      </c>
+      <c r="C23" s="5">
+        <f>B23*Parameters!$B$5</f>
+        <v/>
+      </c>
+      <c r="D23" s="5">
+        <f>IF(C23&gt;=385,0,6.95)</f>
+        <v/>
+      </c>
+      <c r="E23" s="5">
+        <f>C23+D23</f>
+        <v/>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Ja — NL, maar duurder all-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>VERDICT actuators: eibhandel.de blijft goedkoopst all-in (~€55 bij 4 st). Amazon soms dichterbij. Home Perfect/VerwarmingOnline duurder.</t>
         </is>
       </c>
     </row>
@@ -3679,7 +4851,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3730,7 +4902,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4231,300 +5403,6 @@
       <c r="A35" t="inlineStr">
         <is>
           <t>m² is nu stuurvariabele op Parameters — hoeveelheden schalen automatisch.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Prijszoek – 5 duurste items (alleen goedkoper + ≤1 week leverbaar)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Gezocht NL + DE webshops, 22 aug 2026. Alleen gewijzigd als aantoonbaar goedkoper én binnen levertijd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Item (regeltotaal)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Was</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Beste gevonden</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Actie</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Besparing</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>MAGNUM SlimFit 12 matten (8×)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Elektramat €86,94/st (€695,52)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Bouwmaat €86,50 (geen voorraad/bezorging); VihamiJ €86,36 excl=duurder + 3–4 wkn; overige ≥€88,99</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>BEHOUDEN Elektramat</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>€0</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Kreisel 418 egaline (33×)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>EgalineXXL €14,87/st (€490,71)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>RBMB ≥€16,55/st (bulkpas pas vanaf 41); geen goedkopere met snelle levering</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>BEHOUDEN EgalineXXL</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>€0</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>VTE Composiet 4-groeps + Grundfos</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>123Installatieshop €387,18</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>CVTotaal €423; VV-shop €404,95; Bouwbestel €440; Jan de Isolatieman €469</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>BEHOUDEN 123Installatieshop</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>€0</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>MAGNUM PE-RT 12×1,5 300 m</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>123InstallatieMaterialen €142,93</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Klusspullen €141,95 maar voorraad 0 / levertijd 1–2 wkn → afgewezen; Elektramat €181,86; VV-shop €164,70</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>BEHOUDEN 123IM</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>€0</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>5a</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Möhlenhoff Alpha 5 ×4 (altijd)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>VerwarmingOnline €20,12 → €80,48</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>eibhandel.de €9,99 + NL-verzending ~€15,41 = ~€55,37; Amazon.nl ~€13,16/st met Prime</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>GEWIJZIGD → eibhandel</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>~€25</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>5b</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>MAGNUM H64-CC + master (optie)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>123IM €213,74</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Warp Systems €194,92 (1 wd)</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>GEWIJZIGD → Warp</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>~€19</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Niet meegenomen</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>• PioTek DE (~€9,90): verzendt niet meer naar NL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>• Bouwmaat SlimFit €86,50: tijdelijk niet beschikbaar / geen bezorging.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>• Klusspullen PE-RT €141,95: goedkoper op papier, maar 0 voorraad / 1–2 weken.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>• Tado: officiële tado° Shop blijft goedkoopst (bol/retail vaak duurder).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>All-in met verzending: zie sheet Verzending (egaline pallet + eibhandel DE→NL).</t>
         </is>
       </c>
     </row>
@@ -4539,92 +5417,286 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>KOPJE: Vloerverwarming — Tado</t>
+          <t>Prijszoek – 5 duurste items (alleen goedkoper + ≤1 week leverbaar)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <f>Parameters!B6&amp;" ruimten · "&amp;Parameters!B5&amp;" groepen · "&amp;Parameters!B4&amp;" m²"</f>
-        <v/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Gezocht NL + DE webshops, 22 aug 2026. Alleen gewijzigd als aantoonbaar goedkoper én binnen levertijd.</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ruimte</t>
+          <t>#</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Groepen</t>
+          <t>Item (regeltotaal)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tado</t>
+          <t>Was</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Actuators</t>
+          <t>Beste gevonden</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Actie</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Besparing</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ruimte 1 (groot)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>meerdere mogelijk</t>
+          <t>MAGNUM SlimFit 12 matten (8×)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Bedraad X (+ Bridge in starter)</t>
+          <t>Elektramat €86,94/st (€695,52)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>parallel op 1 thermostaat</t>
+          <t>Bouwmaat €86,50 (geen voorraad/bezorging); VihamiJ €86,36 excl=duurder + 3–4 wkn; overige ≥€88,99</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>BEHOUDEN Elektramat</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>€0</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ruimte 2…N</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1 per ruimte typisch</t>
+          <t>Kreisel 418 egaline (33×)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Bedraad X uitbreiding</t>
+          <t>EgalineXXL €14,87/st (€490,71)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1 actuator / groep</t>
+          <t>RBMB ≥€16,55/st (bulkpas pas vanaf 41); geen goedkopere met snelle levering</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BEHOUDEN EgalineXXL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>€0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>VTE Composiet 4-groeps + Grundfos</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>123Installatieshop €387,18</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CVTotaal €423; VV-shop €404,95; Bouwbestel €440; Jan de Isolatieman €469</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BEHOUDEN 123Installatieshop</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>€0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Exacte groepsverdeling is situatiespecifiek; totalen schalen via Parameters.</t>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MAGNUM PE-RT 12×1,5 300 m</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>123InstallatieMaterialen €142,93</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Klusspullen €141,95 maar voorraad 0 / levertijd 1–2 wkn → afgewezen; Elektramat €181,86; VV-shop €164,70</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BEHOUDEN 123IM</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>€0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5a</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Möhlenhoff Alpha 5 ×4 (altijd)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>VerwarmingOnline €20,12 → €80,48</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>eibhandel.de €9,99 + NL-verzending ~€15,41 = ~€55,37; Amazon.nl ~€13,16/st met Prime</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>GEWIJZIGD → eibhandel</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>~€25</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5b</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MAGNUM H64-CC + master (optie)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>123IM €213,74</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Warp Systems €194,92 (1 wd)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>GEWIJZIGD → Warp</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>~€19</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Niet meegenomen</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>• PioTek DE (~€9,90): verzendt niet meer naar NL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>• Bouwmaat SlimFit €86,50: tijdelijk niet beschikbaar / geen bezorging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>• Klusspullen PE-RT €141,95: goedkoper op papier, maar 0 voorraad / 1–2 weken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• Tado: officiële tado° Shop blijft goedkoopst (bol/retail vaak duurder).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>All-in met verzending: zie sheet Verzending (egaline pallet + eibhandel DE→NL).</t>
         </is>
       </c>
     </row>
@@ -4639,567 +5711,92 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="55" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>KOPJE: Vloerverwarming — checklist (hoeveelheden = live uit Boodschappenlijst)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>Artikel</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Qty</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>Webshop</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Prijs/st</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Totaal</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Besteld?</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Ordernr</t>
-        </is>
+          <t>KOPJE: Vloerverwarming — Tado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>Parameters!B6&amp;" ruimten · "&amp;Parameters!B5&amp;" groepen · "&amp;Parameters!B4&amp;" m²"</f>
+        <v/>
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <f>Boodschappenlijst!E6</f>
-        <v/>
-      </c>
-      <c r="B4">
-        <f>Boodschappenlijst!I6</f>
-        <v/>
-      </c>
-      <c r="C4">
-        <f>Boodschappenlijst!P6</f>
-        <v/>
-      </c>
-      <c r="D4" s="5">
-        <f>Boodschappenlijst!K6</f>
-        <v/>
-      </c>
-      <c r="E4" s="5">
-        <f>Boodschappenlijst!N6</f>
-        <v/>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Nee</t>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ruimte</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Groepen</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tado</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Actuators</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5">
-        <f>Boodschappenlijst!E7</f>
-        <v/>
-      </c>
-      <c r="B5">
-        <f>Boodschappenlijst!I7</f>
-        <v/>
-      </c>
-      <c r="C5">
-        <f>Boodschappenlijst!P7</f>
-        <v/>
-      </c>
-      <c r="D5" s="5">
-        <f>Boodschappenlijst!K7</f>
-        <v/>
-      </c>
-      <c r="E5" s="5">
-        <f>Boodschappenlijst!N7</f>
-        <v/>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Nee</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ruimte 1 (groot)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>meerdere mogelijk</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Bedraad X (+ Bridge in starter)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>parallel op 1 thermostaat</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6">
-        <f>Boodschappenlijst!E8</f>
-        <v/>
-      </c>
-      <c r="B6">
-        <f>Boodschappenlijst!I8</f>
-        <v/>
-      </c>
-      <c r="C6">
-        <f>Boodschappenlijst!P8</f>
-        <v/>
-      </c>
-      <c r="D6" s="5">
-        <f>Boodschappenlijst!K8</f>
-        <v/>
-      </c>
-      <c r="E6" s="5">
-        <f>Boodschappenlijst!N8</f>
-        <v/>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <f>Boodschappenlijst!E9</f>
-        <v/>
-      </c>
-      <c r="B7">
-        <f>Boodschappenlijst!I9</f>
-        <v/>
-      </c>
-      <c r="C7">
-        <f>Boodschappenlijst!P9</f>
-        <v/>
-      </c>
-      <c r="D7" s="5">
-        <f>Boodschappenlijst!K9</f>
-        <v/>
-      </c>
-      <c r="E7" s="5">
-        <f>Boodschappenlijst!N9</f>
-        <v/>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>Nee</t>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ruimte 2…N</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1 per ruimte typisch</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Bedraad X uitbreiding</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1 actuator / groep</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8">
-        <f>Boodschappenlijst!E10</f>
-        <v/>
-      </c>
-      <c r="B8">
-        <f>Boodschappenlijst!I10</f>
-        <v/>
-      </c>
-      <c r="C8">
-        <f>Boodschappenlijst!P10</f>
-        <v/>
-      </c>
-      <c r="D8" s="5">
-        <f>Boodschappenlijst!K10</f>
-        <v/>
-      </c>
-      <c r="E8" s="5">
-        <f>Boodschappenlijst!N10</f>
-        <v/>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <f>Boodschappenlijst!E11</f>
-        <v/>
-      </c>
-      <c r="B9">
-        <f>Boodschappenlijst!I11</f>
-        <v/>
-      </c>
-      <c r="C9">
-        <f>Boodschappenlijst!P11</f>
-        <v/>
-      </c>
-      <c r="D9" s="5">
-        <f>Boodschappenlijst!K11</f>
-        <v/>
-      </c>
-      <c r="E9" s="5">
-        <f>Boodschappenlijst!N11</f>
-        <v/>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <f>Boodschappenlijst!E12</f>
-        <v/>
-      </c>
-      <c r="B10">
-        <f>Boodschappenlijst!I12</f>
-        <v/>
-      </c>
-      <c r="C10">
-        <f>Boodschappenlijst!P12</f>
-        <v/>
-      </c>
-      <c r="D10" s="5">
-        <f>Boodschappenlijst!K12</f>
-        <v/>
-      </c>
-      <c r="E10" s="5">
-        <f>Boodschappenlijst!N12</f>
-        <v/>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <f>Boodschappenlijst!E13</f>
-        <v/>
-      </c>
-      <c r="B11">
-        <f>Boodschappenlijst!I13</f>
-        <v/>
-      </c>
-      <c r="C11">
-        <f>Boodschappenlijst!P13</f>
-        <v/>
-      </c>
-      <c r="D11" s="5">
-        <f>Boodschappenlijst!K13</f>
-        <v/>
-      </c>
-      <c r="E11" s="5">
-        <f>Boodschappenlijst!N13</f>
-        <v/>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12">
-        <f>Boodschappenlijst!E14</f>
-        <v/>
-      </c>
-      <c r="B12">
-        <f>Boodschappenlijst!I14</f>
-        <v/>
-      </c>
-      <c r="C12">
-        <f>Boodschappenlijst!P14</f>
-        <v/>
-      </c>
-      <c r="D12" s="5">
-        <f>Boodschappenlijst!K14</f>
-        <v/>
-      </c>
-      <c r="E12" s="5">
-        <f>Boodschappenlijst!N14</f>
-        <v/>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13">
-        <f>Boodschappenlijst!E15</f>
-        <v/>
-      </c>
-      <c r="B13">
-        <f>Boodschappenlijst!I15</f>
-        <v/>
-      </c>
-      <c r="C13">
-        <f>Boodschappenlijst!P15</f>
-        <v/>
-      </c>
-      <c r="D13" s="5">
-        <f>Boodschappenlijst!K15</f>
-        <v/>
-      </c>
-      <c r="E13" s="5">
-        <f>Boodschappenlijst!N15</f>
-        <v/>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14">
-        <f>Boodschappenlijst!E16</f>
-        <v/>
-      </c>
-      <c r="B14">
-        <f>Boodschappenlijst!I16</f>
-        <v/>
-      </c>
-      <c r="C14">
-        <f>Boodschappenlijst!P16</f>
-        <v/>
-      </c>
-      <c r="D14" s="5">
-        <f>Boodschappenlijst!K16</f>
-        <v/>
-      </c>
-      <c r="E14" s="5">
-        <f>Boodschappenlijst!N16</f>
-        <v/>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15">
-        <f>Boodschappenlijst!E17</f>
-        <v/>
-      </c>
-      <c r="B15">
-        <f>Boodschappenlijst!I17</f>
-        <v/>
-      </c>
-      <c r="C15">
-        <f>Boodschappenlijst!P17</f>
-        <v/>
-      </c>
-      <c r="D15" s="5">
-        <f>Boodschappenlijst!K17</f>
-        <v/>
-      </c>
-      <c r="E15" s="5">
-        <f>Boodschappenlijst!N17</f>
-        <v/>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16">
-        <f>Boodschappenlijst!E18</f>
-        <v/>
-      </c>
-      <c r="B16">
-        <f>Boodschappenlijst!I18</f>
-        <v/>
-      </c>
-      <c r="C16">
-        <f>Boodschappenlijst!P18</f>
-        <v/>
-      </c>
-      <c r="D16" s="5">
-        <f>Boodschappenlijst!K18</f>
-        <v/>
-      </c>
-      <c r="E16" s="5">
-        <f>Boodschappenlijst!N18</f>
-        <v/>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17">
-        <f>Boodschappenlijst!E19</f>
-        <v/>
-      </c>
-      <c r="B17">
-        <f>Boodschappenlijst!I19</f>
-        <v/>
-      </c>
-      <c r="C17">
-        <f>Boodschappenlijst!P19</f>
-        <v/>
-      </c>
-      <c r="D17" s="5">
-        <f>Boodschappenlijst!K19</f>
-        <v/>
-      </c>
-      <c r="E17" s="5">
-        <f>Boodschappenlijst!N19</f>
-        <v/>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18">
-        <f>Boodschappenlijst!E20</f>
-        <v/>
-      </c>
-      <c r="B18">
-        <f>Boodschappenlijst!I20</f>
-        <v/>
-      </c>
-      <c r="C18">
-        <f>Boodschappenlijst!P20</f>
-        <v/>
-      </c>
-      <c r="D18" s="5">
-        <f>Boodschappenlijst!K20</f>
-        <v/>
-      </c>
-      <c r="E18" s="5">
-        <f>Boodschappenlijst!N20</f>
-        <v/>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19">
-        <f>Boodschappenlijst!E21</f>
-        <v/>
-      </c>
-      <c r="B19">
-        <f>Boodschappenlijst!I21</f>
-        <v/>
-      </c>
-      <c r="C19">
-        <f>Boodschappenlijst!P21</f>
-        <v/>
-      </c>
-      <c r="D19" s="5">
-        <f>Boodschappenlijst!K21</f>
-        <v/>
-      </c>
-      <c r="E19" s="5">
-        <f>Boodschappenlijst!N21</f>
-        <v/>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20">
-        <f>Boodschappenlijst!E22</f>
-        <v/>
-      </c>
-      <c r="B20">
-        <f>Boodschappenlijst!I22</f>
-        <v/>
-      </c>
-      <c r="C20">
-        <f>Boodschappenlijst!P22</f>
-        <v/>
-      </c>
-      <c r="D20" s="5">
-        <f>Boodschappenlijst!K22</f>
-        <v/>
-      </c>
-      <c r="E20" s="5">
-        <f>Boodschappenlijst!N22</f>
-        <v/>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21">
-        <f>Boodschappenlijst!E23</f>
-        <v/>
-      </c>
-      <c r="B21">
-        <f>Boodschappenlijst!I23</f>
-        <v/>
-      </c>
-      <c r="C21">
-        <f>Boodschappenlijst!P23</f>
-        <v/>
-      </c>
-      <c r="D21" s="5">
-        <f>Boodschappenlijst!K23</f>
-        <v/>
-      </c>
-      <c r="E21" s="5">
-        <f>Boodschappenlijst!N23</f>
-        <v/>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22">
-        <f>Boodschappenlijst!E24</f>
-        <v/>
-      </c>
-      <c r="B22">
-        <f>Boodschappenlijst!I24</f>
-        <v/>
-      </c>
-      <c r="C22">
-        <f>Boodschappenlijst!P24</f>
-        <v/>
-      </c>
-      <c r="D22" s="5">
-        <f>Boodschappenlijst!K24</f>
-        <v/>
-      </c>
-      <c r="E22" s="5">
-        <f>Boodschappenlijst!N24</f>
-        <v/>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Nee</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Exacte groepsverdeling is situatiespecifiek; totalen schalen via Parameters.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Make NL deliverability explicit; optional NL-only actuators
Add NL-leverbaarheid sheet and per-row certainty status. Keep
eibhandel DE→NL as default (shipping €15.41 + lead time included)
with Parameters toggle to VerwarmingOnline for 100% NL webshops.
Fill missing Magnum product URLs.

Co-authored-by: bmverhagen <bmverhagen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Materiaalbenodigdheden_Vloerverwarming.xlsx
+++ b/Materiaalbenodigdheden_Vloerverwarming.xlsx
@@ -8,22 +8,23 @@
   </bookViews>
   <sheets>
     <sheet name="Overzicht" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Parameters" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Boodschappenlijst" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="All-in-check" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Verzending" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Regeling-keuze" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Kwaliteitskeuzes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Prijszoek-top5" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Tado-aansluiting" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Bestelchecklist" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="NL-leverbaarheid" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Parameters" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Boodschappenlijst" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="All-in-check" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Verzending" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Regeling-keuze" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Kwaliteitskeuzes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Prijszoek-top5" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Tado-aansluiting" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Bestelchecklist" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="Oppervlakte_m2">Parameters!$B$4</definedName>
     <definedName name="Aantal_groepen">Parameters!$B$5</definedName>
     <definedName name="Aantal_ruimten">Parameters!$B$6</definedName>
     <definedName name="Egaline_mm">Parameters!$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Boodschappenlijst'!$A$5:$T$24</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Boodschappenlijst'!$A$5:$T$24</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -88,8 +89,12 @@
       <color rgb="001F7A3F"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -121,6 +126,11 @@
         <fgColor rgb="00D6EAF8"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDEBD0"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -148,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -174,6 +184,11 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -736,14 +751,14 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>All-in incl. verzending. Na hercheck (aug 2026): alle shops blijven goedkoopst — zie All-in-check.</t>
+          <t>NL-leverzekerheid: zie sheet NL-leverbaarheid. Actuators-bron: Parameters!B8 (DE→NL of NL zeker).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Enige import: eibhandel.de actuators (NL via DHL, verzending meegenomen).</t>
+          <t>Buitenland alleen toegestaan mét verzendkosten + levertijd — standaard eibhandel DHL naar NL.</t>
         </is>
       </c>
     </row>
@@ -753,6 +768,106 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>KOPJE: Vloerverwarming — Tado</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <f>Parameters!B6&amp;" ruimten · "&amp;Parameters!B5&amp;" groepen · "&amp;Parameters!B4&amp;" m²"</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Ruimte</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Groepen</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Tado</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Actuators</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Ruimte 1 (groot)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>meerdere mogelijk</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Bedraad X (+ Bridge in starter)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>parallel op 1 thermostaat</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Ruimte 2…N</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1 per ruimte typisch</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Bedraad X uitbreiding</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1 actuator / groep</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Exacte groepsverdeling is situatiespecifiek; totalen schalen via Parameters.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1333,516 +1448,606 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>STUURVARIABELEN — pas gele cellen aan; rest schaalt automatisch</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>PROJECT</t>
+          <t>NL-leverbaarheid — alles zeker bestelbaar naar Nederland</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="25" t="inlineStr">
+        <is>
+          <t>Buitenland mag, mits verzendkosten + levertijd expliciet meegenomen zijn. Schakelaar actuators: Parameters!B8.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Oppervlakte</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="n">
-        <v>30</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>← KEY: verander dit getal</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Aantal groepen</t>
-        </is>
-      </c>
-      <c r="B5" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>st</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Bepaalt verdeler/actuators/koppelingen (max ~100 m buis/groep)</t>
-        </is>
+          <t>Huidige actuators-keuze</t>
+        </is>
+      </c>
+      <c r="B4" s="26">
+        <f>Parameters!B8</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Aantal ruimten</t>
-        </is>
-      </c>
-      <c r="B6" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>st</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Bepaalt Tado/H64 thermostaten</t>
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Artikel</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Land</t>
+        </is>
+      </c>
+      <c r="C6" s="19" t="inlineStr">
+        <is>
+          <t>Webshop</t>
+        </is>
+      </c>
+      <c r="D6" s="19" t="inlineStr">
+        <is>
+          <t>Levertijd naar NL</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
+        <is>
+          <t>Verzending meegenomen?</t>
+        </is>
+      </c>
+      <c r="F6" s="19" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Egaline laagdikte</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>SlimFit ~14 mm + overdek ~4 mm; 1,5 kg/m²/mm</t>
-        </is>
+      <c r="A7">
+        <f>Boodschappenlijst!E6</f>
+        <v/>
+      </c>
+      <c r="B7">
+        <f>Boodschappenlijst!R6</f>
+        <v/>
+      </c>
+      <c r="C7">
+        <f>Boodschappenlijst!P6</f>
+        <v/>
+      </c>
+      <c r="D7">
+        <f>Boodschappenlijst!O6</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>IF(OR(Boodschappenlijst!R6="NL",Boodschappenlijst!R6=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R6&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>Boodschappenlijst!U6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <f>Boodschappenlijst!E7</f>
+        <v/>
+      </c>
+      <c r="B8">
+        <f>Boodschappenlijst!R7</f>
+        <v/>
+      </c>
+      <c r="C8">
+        <f>Boodschappenlijst!P7</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>Boodschappenlijst!O7</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>IF(OR(Boodschappenlijst!R7="NL",Boodschappenlijst!R7=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R7&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>Boodschappenlijst!U7</f>
+        <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t>AFGELEIDE WAARDEN (auto)</t>
-        </is>
+      <c r="A9">
+        <f>Boodschappenlijst!E8</f>
+        <v/>
+      </c>
+      <c r="B9">
+        <f>Boodschappenlijst!R8</f>
+        <v/>
+      </c>
+      <c r="C9">
+        <f>Boodschappenlijst!P8</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>Boodschappenlijst!O8</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>IF(OR(Boodschappenlijst!R8="NL",Boodschappenlijst!R8=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R8&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F9">
+        <f>Boodschappenlijst!U8</f>
+        <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Buislengte (indicatie)</t>
-        </is>
+      <c r="A10">
+        <f>Boodschappenlijst!E9</f>
+        <v/>
       </c>
       <c r="B10">
-        <f>ROUND(B4*10,0)</f>
-        <v/>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>vuistregel 10 m/m² bij SlimFit 12</t>
-        </is>
+        <f>Boodschappenlijst!R9</f>
+        <v/>
+      </c>
+      <c r="C10">
+        <f>Boodschappenlijst!P9</f>
+        <v/>
+      </c>
+      <c r="D10">
+        <f>Boodschappenlijst!O9</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>IF(OR(Boodschappenlijst!R9="NL",Boodschappenlijst!R9=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R9&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F10">
+        <f>Boodschappenlijst!U9</f>
+        <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>SlimFit pakken</t>
-        </is>
+      <c r="A11">
+        <f>Boodschappenlijst!E10</f>
+        <v/>
       </c>
       <c r="B11">
-        <f>CEILING(B4/3.75,1)</f>
-        <v/>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>pak à 3,75 m²</t>
-        </is>
+        <f>Boodschappenlijst!R10</f>
+        <v/>
+      </c>
+      <c r="C11">
+        <f>Boodschappenlijst!P10</f>
+        <v/>
+      </c>
+      <c r="D11">
+        <f>Boodschappenlijst!O10</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>IF(OR(Boodschappenlijst!R10="NL",Boodschappenlijst!R10=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R10&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F11">
+        <f>Boodschappenlijst!U10</f>
+        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Egaline zakken</t>
-        </is>
+      <c r="A12">
+        <f>Boodschappenlijst!E11</f>
+        <v/>
       </c>
       <c r="B12">
-        <f>CEILING(B4*1.5*B7/25,1)</f>
-        <v/>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>zak à 25 kg</t>
-        </is>
+        <f>Boodschappenlijst!R11</f>
+        <v/>
+      </c>
+      <c r="C12">
+        <f>Boodschappenlijst!P11</f>
+        <v/>
+      </c>
+      <c r="D12">
+        <f>Boodschappenlijst!O11</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>IF(OR(Boodschappenlijst!R11="NL",Boodschappenlijst!R11=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R11&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F12">
+        <f>Boodschappenlijst!U11</f>
+        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>PE-RT rollen 300 m</t>
-        </is>
+      <c r="A13">
+        <f>Boodschappenlijst!E12</f>
+        <v/>
       </c>
       <c r="B13">
-        <f>MAX(1,CEILING(B10/300,1))</f>
-        <v/>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>rol</t>
-        </is>
+        <f>Boodschappenlijst!R12</f>
+        <v/>
+      </c>
+      <c r="C13">
+        <f>Boodschappenlijst!P12</f>
+        <v/>
+      </c>
+      <c r="D13">
+        <f>Boodschappenlijst!O12</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>IF(OR(Boodschappenlijst!R12="NL",Boodschappenlijst!R12=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R12&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F13">
+        <f>Boodschappenlijst!U12</f>
+        <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Contactlijm bussen</t>
-        </is>
+      <c r="A14">
+        <f>Boodschappenlijst!E13</f>
+        <v/>
       </c>
       <c r="B14">
-        <f>MAX(1,CEILING(B4*0.2,1))</f>
-        <v/>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>bus</t>
-        </is>
+        <f>Boodschappenlijst!R13</f>
+        <v/>
+      </c>
+      <c r="C14">
+        <f>Boodschappenlijst!P13</f>
+        <v/>
+      </c>
+      <c r="D14">
+        <f>Boodschappenlijst!O13</f>
+        <v/>
+      </c>
+      <c r="E14">
+        <f>IF(OR(Boodschappenlijst!R13="NL",Boodschappenlijst!R13=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R13&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F14">
+        <f>Boodschappenlijst!U13</f>
+        <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Randisolatie rollen</t>
-        </is>
+      <c r="A15">
+        <f>Boodschappenlijst!E14</f>
+        <v/>
       </c>
       <c r="B15">
-        <f>MAX(2,CEILING(B4/10,1))</f>
-        <v/>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>rol à 25 m</t>
-        </is>
+        <f>Boodschappenlijst!R14</f>
+        <v/>
+      </c>
+      <c r="C15">
+        <f>Boodschappenlijst!P14</f>
+        <v/>
+      </c>
+      <c r="D15">
+        <f>Boodschappenlijst!O14</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>IF(OR(Boodschappenlijst!R14="NL",Boodschappenlijst!R14=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R14&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F15">
+        <f>Boodschappenlijst!U14</f>
+        <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Primer bussen 5 L</t>
-        </is>
+      <c r="A16">
+        <f>Boodschappenlijst!E15</f>
+        <v/>
       </c>
       <c r="B16">
-        <f>MAX(1,CEILING(B4*2/30,1))</f>
-        <v/>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>bus</t>
-        </is>
+        <f>Boodschappenlijst!R15</f>
+        <v/>
+      </c>
+      <c r="C16">
+        <f>Boodschappenlijst!P15</f>
+        <v/>
+      </c>
+      <c r="D16">
+        <f>Boodschappenlijst!O15</f>
+        <v/>
+      </c>
+      <c r="E16">
+        <f>IF(OR(Boodschappenlijst!R15="NL",Boodschappenlijst!R15=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R15&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F16">
+        <f>Boodschappenlijst!U15</f>
+        <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Tado/H64 slaves</t>
-        </is>
+      <c r="A17">
+        <f>Boodschappenlijst!E16</f>
+        <v/>
       </c>
       <c r="B17">
-        <f>MAX(0,B6-1)</f>
-        <v/>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>st</t>
-        </is>
+        <f>Boodschappenlijst!R16</f>
+        <v/>
+      </c>
+      <c r="C17">
+        <f>Boodschappenlijst!P16</f>
+        <v/>
+      </c>
+      <c r="D17">
+        <f>Boodschappenlijst!O16</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>IF(OR(Boodschappenlijst!R16="NL",Boodschappenlijst!R16=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R16&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F17">
+        <f>Boodschappenlijst!U16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18">
+        <f>Boodschappenlijst!E17</f>
+        <v/>
+      </c>
+      <c r="B18">
+        <f>Boodschappenlijst!R17</f>
+        <v/>
+      </c>
+      <c r="C18">
+        <f>Boodschappenlijst!P17</f>
+        <v/>
+      </c>
+      <c r="D18">
+        <f>Boodschappenlijst!O17</f>
+        <v/>
+      </c>
+      <c r="E18">
+        <f>IF(OR(Boodschappenlijst!R17="NL",Boodschappenlijst!R17=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R17&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F18">
+        <f>Boodschappenlijst!U17</f>
+        <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>VERZENDREGELS (NL, all-in — gecorrigeerd)</t>
-        </is>
+      <c r="A19">
+        <f>Boodschappenlijst!E18</f>
+        <v/>
+      </c>
+      <c r="B19">
+        <f>Boodschappenlijst!R18</f>
+        <v/>
+      </c>
+      <c r="C19">
+        <f>Boodschappenlijst!P18</f>
+        <v/>
+      </c>
+      <c r="D19">
+        <f>Boodschappenlijst!O18</f>
+        <v/>
+      </c>
+      <c r="E19">
+        <f>IF(OR(Boodschappenlijst!R18="NL",Boodschappenlijst!R18=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R18&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F19">
+        <f>Boodschappenlijst!U18</f>
+        <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="19" t="inlineStr">
-        <is>
-          <t>Shop</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>Gratis vanaf</t>
-        </is>
-      </c>
-      <c r="C20" s="19" t="inlineStr">
-        <is>
-          <t>Kosten onder drempel</t>
-        </is>
-      </c>
-      <c r="D20" s="19" t="inlineStr">
-        <is>
-          <t>Levertijd / land / opmerking</t>
-        </is>
+      <c r="A20">
+        <f>Boodschappenlijst!E19</f>
+        <v/>
+      </c>
+      <c r="B20">
+        <f>Boodschappenlijst!R19</f>
+        <v/>
+      </c>
+      <c r="C20">
+        <f>Boodschappenlijst!P19</f>
+        <v/>
+      </c>
+      <c r="D20">
+        <f>Boodschappenlijst!O19</f>
+        <v/>
+      </c>
+      <c r="E20">
+        <f>IF(OR(Boodschappenlijst!R19="NL",Boodschappenlijst!R19=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R19&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F20">
+        <f>Boodschappenlijst!U19</f>
+        <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Elektramat</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>€150 excl. btw</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>€4,09 excl ≈ €4,95 incl</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>NL · 1 wd · PostNL</t>
-        </is>
+      <c r="A21">
+        <f>Boodschappenlijst!E20</f>
+        <v/>
+      </c>
+      <c r="B21">
+        <f>Boodschappenlijst!R20</f>
+        <v/>
+      </c>
+      <c r="C21">
+        <f>Boodschappenlijst!P20</f>
+        <v/>
+      </c>
+      <c r="D21">
+        <f>Boodschappenlijst!O20</f>
+        <v/>
+      </c>
+      <c r="E21">
+        <f>IF(OR(Boodschappenlijst!R20="NL",Boodschappenlijst!R20=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R20&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F21">
+        <f>Boodschappenlijst!U20</f>
+        <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>123InstallatieMaterialen</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>€200</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>€6,95</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>NL · morgen in huis</t>
-        </is>
+      <c r="A22">
+        <f>Boodschappenlijst!E21</f>
+        <v/>
+      </c>
+      <c r="B22">
+        <f>Boodschappenlijst!R21</f>
+        <v/>
+      </c>
+      <c r="C22">
+        <f>Boodschappenlijst!P21</f>
+        <v/>
+      </c>
+      <c r="D22">
+        <f>Boodschappenlijst!O21</f>
+        <v/>
+      </c>
+      <c r="E22">
+        <f>IF(OR(Boodschappenlijst!R21="NL",Boodschappenlijst!R21=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R21&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F22">
+        <f>Boodschappenlijst!U21</f>
+        <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>123Installatieshop</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>€150</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>€6,95</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>NL · volgende werkdag</t>
-        </is>
+      <c r="A23">
+        <f>Boodschappenlijst!E22</f>
+        <v/>
+      </c>
+      <c r="B23">
+        <f>Boodschappenlijst!R22</f>
+        <v/>
+      </c>
+      <c r="C23">
+        <f>Boodschappenlijst!P22</f>
+        <v/>
+      </c>
+      <c r="D23">
+        <f>Boodschappenlijst!O22</f>
+        <v/>
+      </c>
+      <c r="E23">
+        <f>IF(OR(Boodschappenlijst!R22="NL",Boodschappenlijst!R22=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R22&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F23">
+        <f>Boodschappenlijst!U22</f>
+        <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>EgalineXXL / RBMB</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>€600 excl. btw</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>pallet ≈ €60,50 incl</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>NL · 1–2 wd / palletplanning</t>
-        </is>
+      <c r="A24">
+        <f>Boodschappenlijst!E23</f>
+        <v/>
+      </c>
+      <c r="B24">
+        <f>Boodschappenlijst!R23</f>
+        <v/>
+      </c>
+      <c r="C24">
+        <f>Boodschappenlijst!P23</f>
+        <v/>
+      </c>
+      <c r="D24">
+        <f>Boodschappenlijst!O23</f>
+        <v/>
+      </c>
+      <c r="E24">
+        <f>IF(OR(Boodschappenlijst!R23="NL",Boodschappenlijst!R23=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R23&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F24">
+        <f>Boodschappenlijst!U23</f>
+        <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>eibhandel.de</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>€1000</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>€12,95 excl ≈ €15,41 incl</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>DE→NL DHL zone 1 · 2–5 wd DE (+NL)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Warp Systems</t>
-        </is>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>n.v.t. / laag</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>€0 (typisch)</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>NL · 1 wd (voor 12:00)</t>
-        </is>
+      <c r="A25">
+        <f>Boodschappenlijst!E24</f>
+        <v/>
+      </c>
+      <c r="B25">
+        <f>Boodschappenlijst!R24</f>
+        <v/>
+      </c>
+      <c r="C25">
+        <f>Boodschappenlijst!P24</f>
+        <v/>
+      </c>
+      <c r="D25">
+        <f>Boodschappenlijst!O24</f>
+        <v/>
+      </c>
+      <c r="E25">
+        <f>IF(OR(Boodschappenlijst!R24="NL",Boodschappenlijst!R24=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R24&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F25">
+        <f>Boodschappenlijst!U24</f>
+        <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>tado° Shop</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>€150</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>€4,99</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>NL/EU · 2–4 wd</t>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Samenvatting</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Installand</t>
-        </is>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>€60</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>var. / afhalen gratis</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>NL · vaak volgende wd</t>
+          <t>• 18/19 regels: Nederlandse webshops (Elektramat, 123IM, 123shop, EgalineXXL, Installand, Warp, tado°, bouwmarkt NL).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>VerwarmingOnline</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>€385</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>~€6,95</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>NL · 3–4 wd</t>
+          <t>• 1 regel mogelijk buitenland: Möhlenhoff actuators — standaard DE→NL via eibhandel.de met DHL, verzending ≈€15,41, levertijd 2–5 wd DE + NL.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Home Perfect (.nl/.de)</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>€1000 pakket</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>€29,90–€69 NL-pakket</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>DE-basis · 7–10 wd → te duur/traag all-in</t>
-        </is>
-      </c>
-    </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" s="20" t="inlineStr">
-        <is>
-          <t>Conclusie all-in (aug 2026): huidige shops blijven goedkoopst; zie sheet All-in-check. Geen shopwissel nodig.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Buitenland alleen eibhandel.de (actuators): NL-levering bevestigd, verzending + levertijd meegenomen.</t>
+          <t>• Alternatief 100% NL: Parameters!B8 → "NL zeker (VerwarmingOnline)" (3–4 wd, iets duurder).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>• Geen shops zonder NL-levering. Home Perfect (7–10 wd + dure ship) bewust niet gekozen.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1854,7 +2059,582 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T29"/>
+  <dimension ref="A1:D37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>STUURVARIABELEN — pas gele cellen aan; rest schaalt automatisch</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>PROJECT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Oppervlakte</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>← KEY: verander dit getal</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Aantal groepen</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Bepaalt verdeler/actuators/koppelingen (max ~100 m buis/groep)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Aantal ruimten</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Bepaalt Tado/H64 thermostaten</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Egaline laagdikte</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>18</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>SlimFit ~14 mm + overdek ~4 mm; 1,5 kg/m²/mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Actuators leveren vanuit</t>
+        </is>
+      </c>
+      <c r="B8" s="27" t="inlineStr">
+        <is>
+          <t>DE→NL (eibhandel, goedkoopst)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>keuze</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Of: "NL zeker (VerwarmingOnline)" — duurder, 100% NL-webshop</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>AFGELEIDE WAARDEN (auto)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Buislengte (indicatie)</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>ROUND(B4*10,0)</f>
+        <v/>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>vuistregel 10 m/m² bij SlimFit 12</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SlimFit pakken</t>
+        </is>
+      </c>
+      <c r="B11">
+        <f>CEILING(B4/3.75,1)</f>
+        <v/>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>pak à 3,75 m²</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Egaline zakken</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>CEILING(B4*1.5*B7/25,1)</f>
+        <v/>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>zak à 25 kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>PE-RT rollen 300 m</t>
+        </is>
+      </c>
+      <c r="B13">
+        <f>MAX(1,CEILING(B10/300,1))</f>
+        <v/>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>rol</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Contactlijm bussen</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>MAX(1,CEILING(B4*0.2,1))</f>
+        <v/>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Randisolatie rollen</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>MAX(2,CEILING(B4/10,1))</f>
+        <v/>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>rol à 25 m</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Primer bussen 5 L</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>MAX(1,CEILING(B4*2/30,1))</f>
+        <v/>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tado/H64 slaves</t>
+        </is>
+      </c>
+      <c r="B17">
+        <f>MAX(0,B6-1)</f>
+        <v/>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>st</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>VERZENDREGELS (NL, all-in — gecorrigeerd)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t>Shop</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>Gratis vanaf</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>Kosten onder drempel</t>
+        </is>
+      </c>
+      <c r="D20" s="19" t="inlineStr">
+        <is>
+          <t>Levertijd / land / opmerking</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Elektramat</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>€150 excl. btw</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>€4,09 excl ≈ €4,95 incl</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>NL · 1 wd · PostNL</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>123InstallatieMaterialen</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>€200</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>€6,95</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>NL · morgen in huis</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>123Installatieshop</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>€150</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>€6,95</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>NL · volgende werkdag</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>EgalineXXL / RBMB</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>€600 excl. btw</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>pallet ≈ €60,50 incl</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>NL · 1–2 wd / palletplanning</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>eibhandel.de</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>€1000</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>€12,95 excl ≈ €15,41 incl</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>DE→NL DHL zone 1 · 2–5 wd DE (+NL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Warp Systems</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>n.v.t. / laag</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>€0 (typisch)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>NL · 1 wd (voor 12:00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>tado° Shop</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>€150</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>€4,99</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>NL/EU · 2–4 wd</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Installand</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>€60</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>var. / afhalen gratis</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>NL · vaak volgende wd</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>VerwarmingOnline</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>€385</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>~€6,95</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>NL · 3–4 wd</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Home Perfect (.nl/.de)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>€1000 pakket</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>€29,90–€69 NL-pakket</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>DE-basis · 7–10 wd → te duur/traag all-in</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="20" t="inlineStr">
+        <is>
+          <t>Conclusie all-in (aug 2026): huidige shops blijven goedkoopst; zie sheet All-in-check. Geen shopwissel nodig.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Buitenland alleen eibhandel.de (actuators): NL-levering bevestigd, verzending + levertijd meegenomen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>NL-LEVERZEKERHEID</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Standaard: alle artikelen NL-webshops behalve actuators.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Actuators DE→NL: eibhandel.de levert naar NL (DHL zone 1), verzending ≈€15,41, levertijd 2–5 wd DE + NL-transit (meestal ≤1 week).</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Wil je 100% NL-webshop? Zet B8 op "NL zeker (VerwarmingOnline)" — all-in dan ~€80–€87 i.p.v. ~€55.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:D1"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Ongeldige keuze" error="Kies DE→NL of NL zeker" type="list">
+      <formula1>"DE→NL (eibhandel, goedkoopst),NL zeker (VerwarmingOnline)"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:U26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1877,6 +2657,7 @@
     <col width="6" customWidth="1" min="18" max="18"/>
     <col width="12" customWidth="1" min="19" max="19"/>
     <col width="45" customWidth="1" min="20" max="20"/>
+    <col width="28" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2001,6 +2782,11 @@
           <t>Waarom / opmerking</t>
         </is>
       </c>
+      <c r="U5" s="19" t="inlineStr">
+        <is>
+          <t>NL-zekerheid</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -2067,7 +2853,7 @@
       </c>
       <c r="O6" s="13" t="inlineStr">
         <is>
-          <t>1 werkdag</t>
+          <t>NL · 1 werkdag (op voorraad)</t>
         </is>
       </c>
       <c r="P6" s="13" t="inlineStr">
@@ -2093,6 +2879,11 @@
           <t>Schaalt met m². Goedkoopste met voorraad+snelle NL-levering. Drempel gratis verzending €150 excl. btw.</t>
         </is>
       </c>
+      <c r="U6" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL webshop</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -2159,7 +2950,7 @@
       </c>
       <c r="O7" s="13" t="inlineStr">
         <is>
-          <t>Morgen in huis (v. 14:30)</t>
+          <t>NL · morgen in huis (vóór 14:30)</t>
         </is>
       </c>
       <c r="P7" s="13" t="inlineStr">
@@ -2185,6 +2976,11 @@
           <t>All-in: +€6,95 verzending (order &lt;€200 bij 123IM). Nog steeds goedkoper dan Elektramat €181,86.</t>
         </is>
       </c>
+      <c r="U7" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL webshop</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -2251,7 +3047,7 @@
       </c>
       <c r="O8" s="13" t="inlineStr">
         <is>
-          <t>1 werkdag</t>
+          <t>NL · 1 werkdag</t>
         </is>
       </c>
       <c r="P8" s="13" t="inlineStr">
@@ -2277,6 +3073,11 @@
           <t>Schaalt met aantal groepen.</t>
         </is>
       </c>
+      <c r="U8" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL webshop</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -2304,7 +3105,7 @@
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>W90090</t>
+          <t>W90125</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
@@ -2343,7 +3144,7 @@
       </c>
       <c r="O9" s="13" t="inlineStr">
         <is>
-          <t>Morgen in huis</t>
+          <t>NL · morgen in huis (vóór 14:30)</t>
         </is>
       </c>
       <c r="P9" s="13" t="inlineStr">
@@ -2353,7 +3154,7 @@
       </c>
       <c r="Q9" s="13" t="inlineStr">
         <is>
-          <t>https://123installatiematerialen.nl/</t>
+          <t>https://123installatiematerialen.nl/90-bochtondersteuning-buismaat-o-10-12mm-2-stuks/</t>
         </is>
       </c>
       <c r="R9" s="13" t="inlineStr">
@@ -2369,6 +3170,11 @@
           <t>Schaalt met aantal groepen.</t>
         </is>
       </c>
+      <c r="U9" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL webshop</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -2396,7 +3202,7 @@
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>W90050</t>
+          <t>W61027</t>
         </is>
       </c>
       <c r="G10" s="13" t="inlineStr">
@@ -2435,7 +3241,7 @@
       </c>
       <c r="O10" s="13" t="inlineStr">
         <is>
-          <t>1 werkdag</t>
+          <t>NL · 1 werkdag</t>
         </is>
       </c>
       <c r="P10" s="13" t="inlineStr">
@@ -2445,7 +3251,7 @@
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
-          <t>https://www.elektramat.nl/</t>
+          <t>https://www.elektramat.nl/magnum-contactlijm-voor-verlijmen-magnum-verlegsystemen-w61027/</t>
         </is>
       </c>
       <c r="R10" s="13" t="inlineStr">
@@ -2461,6 +3267,11 @@
           <t>~0,2 bus/m².</t>
         </is>
       </c>
+      <c r="U10" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL webshop</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
@@ -2527,7 +3338,7 @@
       </c>
       <c r="O11" s="13" t="inlineStr">
         <is>
-          <t>≤ 1 week</t>
+          <t>NL · vaak volgende werkdag (vóór 16:30/17:00)</t>
         </is>
       </c>
       <c r="P11" s="13" t="inlineStr">
@@ -2553,6 +3364,11 @@
           <t>Kwaliteitsupgrade; schaalt grof met m².</t>
         </is>
       </c>
+      <c r="U11" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL webshop</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -2619,7 +3435,7 @@
       </c>
       <c r="O12" s="13" t="inlineStr">
         <is>
-          <t>1–2 werkdagen</t>
+          <t>NL · 1–2 werkdagen (gebundeld met egaline)</t>
         </is>
       </c>
       <c r="P12" s="13" t="inlineStr">
@@ -2645,6 +3461,11 @@
           <t>Zelfde shop als egaline (gebundeld voor verzending).</t>
         </is>
       </c>
+      <c r="U12" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL webshop</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
@@ -2711,7 +3532,7 @@
       </c>
       <c r="O13" s="13" t="inlineStr">
         <is>
-          <t>volgende werkdag (vóór 12:00)</t>
+          <t>NL · volgende werkdag / pallet in overleg</t>
         </is>
       </c>
       <c r="P13" s="13" t="inlineStr">
@@ -2737,6 +3558,11 @@
           <t>All-in: +pallet ~€60,50 als order &lt;€600 excl. Goedkoper dan extra zakken kopen voor gratis verzending.</t>
         </is>
       </c>
+      <c r="U13" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL webshop (pallet)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
@@ -2802,7 +3628,7 @@
       </c>
       <c r="O14" s="13" t="inlineStr">
         <is>
-          <t>≤ 1 week (op voorraad)</t>
+          <t>NL · op voorraad, volgende werkdag mogelijk</t>
         </is>
       </c>
       <c r="P14" s="13" t="inlineStr">
@@ -2828,6 +3654,11 @@
           <t>PRIJS = 4-groeps. Bij andere groepen: andere SKU/prijs kiezen!</t>
         </is>
       </c>
+      <c r="U14" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL webshop</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -2894,15 +3725,19 @@
       </c>
       <c r="O15" s="13" t="inlineStr">
         <is>
-          <t>1 week</t>
+          <t>NL · ≤ 1 week (standaard meerlagenbuis)</t>
         </is>
       </c>
       <c r="P15" s="13" t="inlineStr">
         <is>
-          <t>bouwmarkt / installatieshop</t>
-        </is>
-      </c>
-      <c r="Q15" s="13" t="inlineStr"/>
+          <t>123Installatieshop / bouwmarkt NL</t>
+        </is>
+      </c>
+      <c r="Q15" s="13" t="inlineStr">
+        <is>
+          <t>https://www.123installatieshop.nl/</t>
+        </is>
+      </c>
       <c r="R15" s="13" t="inlineStr">
         <is>
           <t>NL</t>
@@ -2913,7 +3748,12 @@
       </c>
       <c r="T15" s="13" t="inlineStr">
         <is>
-          <t>Situatie-afhankelijk; schaalt licht met woninggrootte.</t>
+          <t>Situatie-afhankelijk; schaalt licht met woninggrootte. Lokale bouwmarkt of NL-installatieshop; geen import.</t>
+        </is>
+      </c>
+      <c r="U15" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL (generiek artikel)</t>
         </is>
       </c>
     </row>
@@ -2981,7 +3821,7 @@
       </c>
       <c r="O16" s="13" t="inlineStr">
         <is>
-          <t>1 week</t>
+          <t>NL · ≤ 1 week</t>
         </is>
       </c>
       <c r="P16" s="13" t="inlineStr">
@@ -2989,7 +3829,11 @@
           <t>123Installatieshop</t>
         </is>
       </c>
-      <c r="Q16" s="13" t="inlineStr"/>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t>https://www.123installatieshop.nl/</t>
+        </is>
+      </c>
       <c r="R16" s="13" t="inlineStr">
         <is>
           <t>NL</t>
@@ -3003,6 +3847,11 @@
           <t>Vast per installatie.</t>
         </is>
       </c>
+      <c r="U16" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL webshop</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="16" t="inlineStr">
@@ -3052,11 +3901,13 @@
           <t>st</t>
         </is>
       </c>
-      <c r="K17" s="15" t="n">
-        <v>9.99</v>
-      </c>
-      <c r="L17" s="15" t="n">
-        <v>9.99</v>
+      <c r="K17" s="15">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),20.12,9.99)</f>
+        <v/>
+      </c>
+      <c r="L17" s="15">
+        <f>K17</f>
+        <v/>
       </c>
       <c r="M17" s="13" t="inlineStr">
         <is>
@@ -3067,33 +3918,34 @@
         <f>I17*K17</f>
         <v/>
       </c>
-      <c r="O17" s="13" t="inlineStr">
-        <is>
-          <t>2–5 wd DE + NL (meestal ≤1 week)</t>
-        </is>
-      </c>
-      <c r="P17" s="13" t="inlineStr">
-        <is>
-          <t>eibhandel.de</t>
-        </is>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>https://eibhandel.de/Alpha-Antrieb-230V-NC-incl-Adapter-VA80</t>
-        </is>
-      </c>
-      <c r="R17" s="13" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
-      </c>
-      <c r="S17" s="15" t="n">
-        <v>1000</v>
+      <c r="O17" s="13">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"NL · 3–4 werkdagen (VerwarmingOnline)","DE→NL · 2–5 wd DE + NL-transit (eibhandel DHL)")</f>
+        <v/>
+      </c>
+      <c r="P17" s="13">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"VerwarmingOnline","eibhandel.de")</f>
+        <v/>
+      </c>
+      <c r="Q17" s="13">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"https://verwarmingonline.nl/productgroepen/mohlenhoff-thermische-servomotor-alpha-5-nc-m30x15mm-230v-a-20405-00n/","https://eibhandel.de/Alpha-Antrieb-230V-NC-incl-Adapter-VA80")</f>
+        <v/>
+      </c>
+      <c r="R17" s="29">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"NL","DE→NL")</f>
+        <v/>
+      </c>
+      <c r="S17" s="15">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),385,1000)</f>
+        <v/>
       </c>
       <c r="T17" s="13" t="inlineStr">
         <is>
-          <t>All-in DE→NL: €9,99×groepen + €15,41 verzending. Goedkoper dan Home Perfect/VerwarmingOnline; NL via DHL.</t>
-        </is>
+          <t>Schakel via Parameters!B8. DE→NL: verzending ≈€15,41 + levertijd 2–5 wd DE. NL zeker: €20,12/st, verzending €0 als order ≥€385 anders ~€6,95.</t>
+        </is>
+      </c>
+      <c r="U17">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"ZEKER — NL webshop","DE→NL bevestigd (DHL zone 1)")</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -3160,15 +4012,19 @@
       </c>
       <c r="O18" s="13" t="inlineStr">
         <is>
-          <t>direct</t>
+          <t>NL · 1 werkdag / direct afhalen</t>
         </is>
       </c>
       <c r="P18" s="13" t="inlineStr">
         <is>
-          <t>bouwmarkt</t>
-        </is>
-      </c>
-      <c r="Q18" s="13" t="inlineStr"/>
+          <t>Elektramat / bouwmarkt NL</t>
+        </is>
+      </c>
+      <c r="Q18" s="13" t="inlineStr">
+        <is>
+          <t>https://www.elektramat.nl/draad-en-kabel/installatiekabel/</t>
+        </is>
+      </c>
       <c r="R18" s="13" t="inlineStr">
         <is>
           <t>NL</t>
@@ -3182,6 +4038,11 @@
           <t>Vast; bij groter project licht ophogen.</t>
         </is>
       </c>
+      <c r="U18" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
@@ -3247,7 +4108,7 @@
       </c>
       <c r="O19" s="13" t="inlineStr">
         <is>
-          <t>1 werkdag</t>
+          <t>NL · 1 werkdag (voor 12:00 zelfde dag verzonden)</t>
         </is>
       </c>
       <c r="P19" s="13" t="inlineStr">
@@ -3273,6 +4134,11 @@
           <t>NL-fabrikant, snelle levering.</t>
         </is>
       </c>
+      <c r="U19" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL fabrikant</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -3339,7 +4205,7 @@
       </c>
       <c r="O20" s="13" t="inlineStr">
         <is>
-          <t>1 werkdag</t>
+          <t>NL · 1 werkdag</t>
         </is>
       </c>
       <c r="P20" s="13" t="inlineStr">
@@ -3365,6 +4231,11 @@
           <t>Schaalt met ruimten−1.</t>
         </is>
       </c>
+      <c r="U20" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL fabrikant</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -3431,7 +4302,7 @@
       </c>
       <c r="O21" s="13" t="inlineStr">
         <is>
-          <t>2–4 werkdagen</t>
+          <t>NL/EU · 2–4 werkdagen (tado° levert NL)</t>
         </is>
       </c>
       <c r="P21" s="13" t="inlineStr">
@@ -3457,6 +4328,11 @@
           <t>Schaalt met ruimten. Officiële shop goedkoopst.</t>
         </is>
       </c>
+      <c r="U21" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — tado° NL-shop</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
@@ -3522,7 +4398,7 @@
       </c>
       <c r="O22" s="13" t="inlineStr">
         <is>
-          <t>2–4 werkdagen</t>
+          <t>NL/EU · 2–4 werkdagen</t>
         </is>
       </c>
       <c r="P22" s="13" t="inlineStr">
@@ -3548,6 +4424,11 @@
           <t>Aanbevolen pad (bedraad).</t>
         </is>
       </c>
+      <c r="U22" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — tado° NL-shop</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="16" t="inlineStr">
@@ -3614,7 +4495,7 @@
       </c>
       <c r="O23" s="13" t="inlineStr">
         <is>
-          <t>2–4 werkdagen</t>
+          <t>NL/EU · 2–4 werkdagen</t>
         </is>
       </c>
       <c r="P23" s="13" t="inlineStr">
@@ -3640,6 +4521,11 @@
           <t>Schaalt met ruimten−1.</t>
         </is>
       </c>
+      <c r="U23" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — tado° NL-shop</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
@@ -3705,7 +4591,7 @@
       </c>
       <c r="O24" s="13" t="inlineStr">
         <is>
-          <t>2–4 werkdagen</t>
+          <t>NL/EU · 2–4 werkdagen</t>
         </is>
       </c>
       <c r="P24" s="13" t="inlineStr">
@@ -3715,7 +4601,7 @@
       </c>
       <c r="Q24" s="13" t="inlineStr">
         <is>
-          <t>https://shop.tado.com/</t>
+          <t>https://shop.tado.com/nl-bx/</t>
         </is>
       </c>
       <c r="R24" s="13" t="inlineStr">
@@ -3731,8 +4617,12 @@
           <t>Standaard 0; handmatig verhogen indien nodig.</t>
         </is>
       </c>
-    </row>
-    <row r="25"/>
+      <c r="U24" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — tado° NL-shop</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
@@ -3740,9 +4630,6 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
-    <row r="29"/>
   </sheetData>
   <autoFilter ref="A5:T24"/>
   <mergeCells count="1">
@@ -3752,13 +4639,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4222,6 +5109,13 @@
         <v/>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>NL-update: schakelaar Parameters!B8. Default DE→NL blijft goedkoopst all-in; kies NL zeker indien je geen import wilt.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
@@ -4230,7 +5124,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4454,39 +5348,37 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>eibhandel.de</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>DE</t>
-        </is>
+      <c r="A9">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"VerwarmingOnline","eibhandel.de")</f>
+        <v/>
+      </c>
+      <c r="B9">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"NL","DE→NL")</f>
+        <v/>
       </c>
       <c r="C9" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A9,Boodschappenlijst!$C$6:$C$24,"altijd")</f>
-        <v/>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>1000</v>
+        <f>Boodschappenlijst!N17</f>
+        <v/>
+      </c>
+      <c r="D9" s="5">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),385,1000)</f>
+        <v/>
       </c>
       <c r="E9" s="5">
-        <f>IF(C9&lt;=0,0,IF(C9&gt;=1000,0,15.41))</f>
+        <f>IF(C9&lt;=0,0,IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),IF(C9&gt;=385,0,6.95),IF(C9&gt;=1000,0,15.41)))</f>
         <v/>
       </c>
       <c r="F9" s="5">
         <f>C9+E9</f>
         <v/>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>2–5 wd + NL</t>
-        </is>
+      <c r="G9">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"NL 3–4 wd","DE→NL 2–5+ wd")</f>
+        <v/>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Actuators; €12,95 excl ≈ €15,41 incl</t>
+          <t>Volgt Parameters!B8. DE: DHL zone 1 NL €15,41. NL: VerwarmingOnline drempel €385.</t>
         </is>
       </c>
     </row>
@@ -4636,7 +5528,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>All-in check actuators (Möhlenhoff)</t>
+          <t>Actuators — all-in &amp; NL-zekerheid (live t.o.v. Parameters!B8)</t>
         </is>
       </c>
     </row>
@@ -4785,10 +5677,9 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>Egaline all-in (schaalt met m²)</t>
-        </is>
+      <c r="A25" s="20">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"Gekozen: NL zeker (VerwarmingOnline) — 100% NL-webshop.","Gekozen: DE→NL (eibhandel) — goedkoopst all-in, NL-levering via DHL met verzending+levertijd.")</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -4851,7 +5742,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4902,7 +5793,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5403,300 +6294,6 @@
       <c r="A35" t="inlineStr">
         <is>
           <t>m² is nu stuurvariabele op Parameters — hoeveelheden schalen automatisch.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:F18"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Prijszoek – 5 duurste items (alleen goedkoper + ≤1 week leverbaar)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Gezocht NL + DE webshops, 22 aug 2026. Alleen gewijzigd als aantoonbaar goedkoper én binnen levertijd.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Item (regeltotaal)</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Was</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Beste gevonden</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Actie</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Besparing</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>MAGNUM SlimFit 12 matten (8×)</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Elektramat €86,94/st (€695,52)</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Bouwmaat €86,50 (geen voorraad/bezorging); VihamiJ €86,36 excl=duurder + 3–4 wkn; overige ≥€88,99</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>BEHOUDEN Elektramat</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>€0</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Kreisel 418 egaline (33×)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>EgalineXXL €14,87/st (€490,71)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>RBMB ≥€16,55/st (bulkpas pas vanaf 41); geen goedkopere met snelle levering</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>BEHOUDEN EgalineXXL</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>€0</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>VTE Composiet 4-groeps + Grundfos</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>123Installatieshop €387,18</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>CVTotaal €423; VV-shop €404,95; Bouwbestel €440; Jan de Isolatieman €469</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>BEHOUDEN 123Installatieshop</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>€0</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>MAGNUM PE-RT 12×1,5 300 m</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>123InstallatieMaterialen €142,93</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Klusspullen €141,95 maar voorraad 0 / levertijd 1–2 wkn → afgewezen; Elektramat €181,86; VV-shop €164,70</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>BEHOUDEN 123IM</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>€0</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>5a</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Möhlenhoff Alpha 5 ×4 (altijd)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>VerwarmingOnline €20,12 → €80,48</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>eibhandel.de €9,99 + NL-verzending ~€15,41 = ~€55,37; Amazon.nl ~€13,16/st met Prime</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>GEWIJZIGD → eibhandel</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>~€25</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>5b</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>MAGNUM H64-CC + master (optie)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>123IM €213,74</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Warp Systems €194,92 (1 wd)</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>GEWIJZIGD → Warp</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>~€19</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Niet meegenomen</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>• PioTek DE (~€9,90): verzendt niet meer naar NL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>• Bouwmaat SlimFit €86,50: tijdelijk niet beschikbaar / geen bezorging.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>• Klusspullen PE-RT €141,95: goedkoper op papier, maar 0 voorraad / 1–2 weken.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>• Tado: officiële tado° Shop blijft goedkoopst (bol/retail vaak duurder).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>All-in met verzending: zie sheet Verzending (egaline pallet + eibhandel DE→NL).</t>
         </is>
       </c>
     </row>
@@ -5711,92 +6308,286 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>KOPJE: Vloerverwarming — Tado</t>
+          <t>Prijszoek – 5 duurste items (alleen goedkoper + ≤1 week leverbaar)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <f>Parameters!B6&amp;" ruimten · "&amp;Parameters!B5&amp;" groepen · "&amp;Parameters!B4&amp;" m²"</f>
-        <v/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Gezocht NL + DE webshops, 22 aug 2026. Alleen gewijzigd als aantoonbaar goedkoper én binnen levertijd.</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ruimte</t>
+          <t>#</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Groepen</t>
+          <t>Item (regeltotaal)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Tado</t>
+          <t>Was</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Actuators</t>
+          <t>Beste gevonden</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Actie</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Besparing</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ruimte 1 (groot)</t>
+          <t>1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>meerdere mogelijk</t>
+          <t>MAGNUM SlimFit 12 matten (8×)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Bedraad X (+ Bridge in starter)</t>
+          <t>Elektramat €86,94/st (€695,52)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>parallel op 1 thermostaat</t>
+          <t>Bouwmaat €86,50 (geen voorraad/bezorging); VihamiJ €86,36 excl=duurder + 3–4 wkn; overige ≥€88,99</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>BEHOUDEN Elektramat</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>€0</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ruimte 2…N</t>
+          <t>2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1 per ruimte typisch</t>
+          <t>Kreisel 418 egaline (33×)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Bedraad X uitbreiding</t>
+          <t>EgalineXXL €14,87/st (€490,71)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1 actuator / groep</t>
+          <t>RBMB ≥€16,55/st (bulkpas pas vanaf 41); geen goedkopere met snelle levering</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BEHOUDEN EgalineXXL</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>€0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>VTE Composiet 4-groeps + Grundfos</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>123Installatieshop €387,18</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>CVTotaal €423; VV-shop €404,95; Bouwbestel €440; Jan de Isolatieman €469</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>BEHOUDEN 123Installatieshop</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>€0</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Exacte groepsverdeling is situatiespecifiek; totalen schalen via Parameters.</t>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MAGNUM PE-RT 12×1,5 300 m</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>123InstallatieMaterialen €142,93</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Klusspullen €141,95 maar voorraad 0 / levertijd 1–2 wkn → afgewezen; Elektramat €181,86; VV-shop €164,70</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BEHOUDEN 123IM</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>€0</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5a</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Möhlenhoff Alpha 5 ×4 (altijd)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>VerwarmingOnline €20,12 → €80,48</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>eibhandel.de €9,99 + NL-verzending ~€15,41 = ~€55,37; Amazon.nl ~€13,16/st met Prime</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>GEWIJZIGD → eibhandel</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>~€25</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5b</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MAGNUM H64-CC + master (optie)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>123IM €213,74</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Warp Systems €194,92 (1 wd)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>GEWIJZIGD → Warp</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>~€19</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Niet meegenomen</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>• PioTek DE (~€9,90): verzendt niet meer naar NL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>• Bouwmaat SlimFit €86,50: tijdelijk niet beschikbaar / geen bezorging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>• Klusspullen PE-RT €141,95: goedkoper op papier, maar 0 voorraad / 1–2 weken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• Tado: officiële tado° Shop blijft goedkoopst (bol/retail vaak duurder).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>All-in met verzending: zie sheet Verzending (egaline pallet + eibhandel DE→NL).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Switch BOM to quality wet system (16 mm + sand cement)
Replace SlimFit/egaline with Magnum noppenplaat 28 mm, PE-RT 16×2,
krimpnet and indicative sand-cement screed ≥50 mm for a hard floor
without flex. Keep VTE/Möhlenhoff/Tado quality choices and m² scaling.

Co-authored-by: bmverhagen <bmverhagen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Materiaalbenodigdheden_Vloerverwarming.xlsx
+++ b/Materiaalbenodigdheden_Vloerverwarming.xlsx
@@ -94,7 +94,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -131,6 +131,11 @@
         <fgColor rgb="00FDEBD0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -158,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -189,6 +194,7 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -566,7 +572,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Vloerverwarming — speel met m² op sheet Parameters (gele cel)</t>
+          <t>Vloerverwarming — KWALITATIEF BESTE (nat 16 mm). Speel met m² op Parameters</t>
         </is>
       </c>
     </row>
@@ -723,42 +729,42 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1. Ga naar Parameters → verander gele cel Oppervlakte (m²).</t>
+          <t>1. Parameters → gele cel Oppervlakte (m²) + dekvloer-mm (≥50).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2. Pas zo nodig Groepen en Ruimten aan (verdeler-SKU is 4-groeps!).</t>
+          <t>2. Pas Groepen/Ruimten aan (verdeler-SKU is 4-groeps!).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3. Bekijk Boodschappenlijst (groene hoeveelheden) en Overzicht (all-in).</t>
+          <t>3. Boodschappenlijst = Magnum noppen 28 mm + PE-RT 16 + zandcement (niet SlimFit).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4. Check Verzending: onder gratis-drempel worden kosten automatisch opgeteld.</t>
+          <t>4. Zandcement: lokale offerte; Excel toont indicatie €35/m².</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>NL-leverzekerheid: zie sheet NL-leverbaarheid. Actuators-bron: Parameters!B8 (DE→NL of NL zeker).</t>
+          <t>Nog beter als er al een stevige dekvloer is: INFREZEN i.p.v. opbouw — vraag een freesbedrijf. Anders is dit nat systeem het hardst.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Buitenland alleen toegestaan mét verzendkosten + levertijd — standaard eibhandel DHL naar NL.</t>
+          <t>NL-leverzekerheid: sheet NL-leverbaarheid. Actuators: Parameters!B8.</t>
         </is>
       </c>
     </row>
@@ -1411,31 +1417,8 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22">
-        <f>Boodschappenlijst!E24</f>
-        <v/>
-      </c>
-      <c r="B22">
-        <f>Boodschappenlijst!I24</f>
-        <v/>
-      </c>
-      <c r="C22">
-        <f>Boodschappenlijst!P24</f>
-        <v/>
-      </c>
-      <c r="D22" s="5">
-        <f>Boodschappenlijst!K24</f>
-        <v/>
-      </c>
-      <c r="E22" s="5">
-        <f>Boodschappenlijst!N24</f>
-        <v/>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>Nee</t>
-        </is>
-      </c>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1462,7 +1445,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>NL-leverbaarheid — alles zeker bestelbaar naar Nederland</t>
+          <t>NL-leverbaarheid — kwalitatief beste BOM</t>
         </is>
       </c>
     </row>
@@ -1984,32 +1967,6 @@
         <v/>
       </c>
     </row>
-    <row r="25">
-      <c r="A25">
-        <f>Boodschappenlijst!E24</f>
-        <v/>
-      </c>
-      <c r="B25">
-        <f>Boodschappenlijst!R24</f>
-        <v/>
-      </c>
-      <c r="C25">
-        <f>Boodschappenlijst!P24</f>
-        <v/>
-      </c>
-      <c r="D25">
-        <f>Boodschappenlijst!O24</f>
-        <v/>
-      </c>
-      <c r="E25">
-        <f>IF(OR(Boodschappenlijst!R24="NL",Boodschappenlijst!R24=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R24&amp;"")),"JA — zie Verzending","check"))</f>
-        <v/>
-      </c>
-      <c r="F25">
-        <f>Boodschappenlijst!U24</f>
-        <v/>
-      </c>
-    </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
@@ -2020,35 +1977,32 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• 18/19 regels: Nederlandse webshops (Elektramat, 123IM, 123shop, EgalineXXL, Installand, Warp, tado°, bouwmarkt NL).</t>
+          <t>• Bijna alles NL-webshops (Elektramat, 123shop, Installand, Overkamp, Warp, tado°).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>• 1 regel mogelijk buitenland: Möhlenhoff actuators — standaard DE→NL via eibhandel.de met DHL, verzending ≈€15,41, levertijd 2–5 wd DE + NL.</t>
+          <t>• Zandcement = lokale vloerzetter (indicatief in lijst).</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>• Alternatief 100% NL: Parameters!B8 → "NL zeker (VerwarmingOnline)" (3–4 wd, iets duurder).</t>
+          <t>• 1 regel mogelijk buitenland: Möhlenhoff via eibhandel.de (Parameters!B8).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>• Geen shops zonder NL-levering. Home Perfect (7–10 wd + dure ship) bewust niet gekozen.</t>
+          <t>• Noppenplaten: lengtevracht — plan bezorging/afhaal met Elektramat.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2145,11 +2099,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Egaline laagdikte</t>
+          <t>Dekvloer boven buis</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>18</v>
+        <v>50</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -2158,7 +2112,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>SlimFit ~14 mm + overdek ~4 mm; 1,5 kg/m²/mm</t>
+          <t>Magnum min. 50 mm zandcement boven buis (harde, niet-golvende vloer)</t>
         </is>
       </c>
     </row>
@@ -2198,7 +2152,7 @@
         </is>
       </c>
       <c r="B10">
-        <f>ROUND(B4*10,0)</f>
+        <f>ROUND(B4*8,0)</f>
         <v/>
       </c>
       <c r="C10" t="inlineStr">
@@ -2208,50 +2162,50 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>vuistregel 10 m/m² bij SlimFit 12</t>
+          <t>vuistregel 8 m/m² ≈ hart-op-hart 12,5 cm (kwaliteit nat 16 mm)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SlimFit pakken</t>
+          <t>Noppenplaat sets 10 m²</t>
         </is>
       </c>
       <c r="B11">
-        <f>CEILING(B4/3.75,1)</f>
+        <f>CEILING(B4/10,1)</f>
         <v/>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>pak à 3,75 m²</t>
+          <t>set à 10 m²</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Egaline zakken</t>
+          <t>Krimpnetten 2,52 m²</t>
         </is>
       </c>
       <c r="B12">
-        <f>CEILING(B4*1.5*B7/25,1)</f>
+        <f>CEILING(B4/2.52,1)</f>
         <v/>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>zak à 25 kg</t>
+          <t>mat 120×210</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PE-RT rollen 300 m</t>
+          <t>PE-RT rollen 240 m</t>
         </is>
       </c>
       <c r="B13">
-        <f>MAX(1,CEILING(B10/300,1))</f>
+        <f>MAX(1,CEILING(B10/240,1))</f>
         <v/>
       </c>
       <c r="C13" t="inlineStr">
@@ -2263,16 +2217,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Contactlijm bussen</t>
+          <t>Euroconus sets</t>
         </is>
       </c>
       <c r="B14">
-        <f>MAX(1,CEILING(B4*0.2,1))</f>
+        <f>B5</f>
         <v/>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>set (2 st)</t>
         </is>
       </c>
     </row>
@@ -2295,16 +2249,16 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Primer bussen 5 L</t>
+          <t>Geleidingsbochten</t>
         </is>
       </c>
       <c r="B16">
-        <f>MAX(1,CEILING(B4*2/30,1))</f>
+        <f>B5*2</f>
         <v/>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>st (aanvoer+retour/groep)</t>
         </is>
       </c>
     </row>
@@ -2324,6 +2278,27 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Zandcement m²</t>
+        </is>
+      </c>
+      <c r="B18">
+        <f>B4</f>
+        <v/>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Indicatie vloerzetter; vraag lokale offerte</t>
+        </is>
+      </c>
+    </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
@@ -2616,9 +2591,6 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
   <dataValidations count="1">
     <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Ongeldige keuze" error="Kies DE→NL of NL zeker" type="list">
       <formula1>"DE→NL (eibhandel, goedkoopst),NL zeker (VerwarmingOnline)"</formula1>
@@ -2634,7 +2606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U26"/>
+  <dimension ref="A1:U24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2663,21 +2635,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Boodschappenlijst — hoeveelheden schalen mee met Parameters!B4 (m²)</t>
+          <t>Boodschappenlijst — KWALITATIEF BESTE (nat 16 mm + noppen + zandcement). Hoeveelheden schalen met Parameters!B4</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Gele stuurcellen zitten op sheet Parameters. Kolom Hoeveelheid + Totaal = formules. Verzendkosten apart op sheet Verzending.</t>
+          <t>Doel: harde vloer zonder golven. SlimFit/egaline vervangen. Gele stuurcellen op Parameters. Verzending op sheet Verzending.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>KOPJE: Vloerverwarming</t>
+          <t>KOPJE: Vloerverwarming — kwalitatief beste</t>
         </is>
       </c>
     </row>
@@ -2804,47 +2776,47 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Bevestiging</t>
+          <t>Noppenplaat</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>MAGNUM SlimFit 12 bevestigingsmat 3,75 m²</t>
+          <t>MAGNUM noppenplaat geïsoleerd 28 mm (11 mm EPS) – set 10 m²</t>
         </is>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>W61012</t>
+          <t>W90117</t>
         </is>
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>Kunststof klikmatten 5×75×100 cm = 3,75 m², opbouw ~14 mm.</t>
+          <t>PS-noppen + 11 mm EPS, max. belasting 150 kPa, Rd 0,31. Voor 16/17 mm buis.</t>
         </is>
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>Basislaag voor buizen.</t>
-        </is>
-      </c>
-      <c r="I6" s="14">
-        <f>CEILING(Parameters!$B$4/3.75,1)</f>
+          <t>Buizen vastklikken + lichte isolatie; stijve basis i.p.v. SlimFit.</t>
+        </is>
+      </c>
+      <c r="I6" s="30">
+        <f>Parameters!$B$11</f>
         <v/>
       </c>
       <c r="J6" s="13" t="inlineStr">
         <is>
-          <t>pak</t>
+          <t>set</t>
         </is>
       </c>
       <c r="K6" s="15" t="n">
-        <v>86.94</v>
+        <v>136.58</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>86.94</v>
+        <v>102.55</v>
       </c>
       <c r="M6" s="13" t="inlineStr">
         <is>
-          <t>behouden</t>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="N6" s="15">
@@ -2853,7 +2825,7 @@
       </c>
       <c r="O6" s="13" t="inlineStr">
         <is>
-          <t>NL · 1 werkdag (op voorraad)</t>
+          <t>NL · 1 werkdag (lengtevracht)</t>
         </is>
       </c>
       <c r="P6" s="13" t="inlineStr">
@@ -2863,7 +2835,7 @@
       </c>
       <c r="Q6" s="13" t="inlineStr">
         <is>
-          <t>https://www.elektramat.nl/magnum-slimfit-12-bevestigingsmat-vloerverwarming-3-75-m2-5-stuks-van-75x100cm-w61012/</t>
+          <t>https://www.elektramat.nl/magnum-noppenplaat-geisoleerd-28mm-11mm-eps-10x1000x1000mm-set-van-10m2-w90117/</t>
         </is>
       </c>
       <c r="R6" s="13" t="inlineStr">
@@ -2876,7 +2848,7 @@
       </c>
       <c r="T6" s="13" t="inlineStr">
         <is>
-          <t>Schaalt met m². Goedkoopste met voorraad+snelle NL-levering. Drempel gratis verzending €150 excl. btw.</t>
+          <t>28 mm i.p.v. 47 mm: veel hogere belasting (150 kPa) → hardere vloer. Schaalt met m².</t>
         </is>
       </c>
       <c r="U6" s="28" t="inlineStr">
@@ -2906,26 +2878,26 @@
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>MAGNUM PE-RT buis 12×1,5 mm KOMO – rol 300 m</t>
+          <t>MAGNUM PE-RT buis 16×2 mm KOMO – rol 240 m</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>W12300</t>
+          <t>W16240</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>5-laags PE-RT ø12 mm, KOMO/EVOH.</t>
+          <t>5-laags PE-RT ø16 mm, KOMO/EVOH, tot 80 °C.</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Verwarmingscircuits.</t>
-        </is>
-      </c>
-      <c r="I7" s="14">
-        <f>MAX(1,CEILING(Parameters!$B$10/300,1))</f>
+          <t>Verwarmingscircuits (nat systeem).</t>
+        </is>
+      </c>
+      <c r="I7" s="30">
+        <f>Parameters!$B$13</f>
         <v/>
       </c>
       <c r="J7" s="13" t="inlineStr">
@@ -2934,14 +2906,14 @@
         </is>
       </c>
       <c r="K7" s="15" t="n">
-        <v>142.93</v>
+        <v>158.99</v>
       </c>
       <c r="L7" s="15" t="n">
-        <v>142.93</v>
+        <v>158.99</v>
       </c>
       <c r="M7" s="13" t="inlineStr">
         <is>
-          <t>behouden</t>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="N7" s="15">
@@ -2950,17 +2922,17 @@
       </c>
       <c r="O7" s="13" t="inlineStr">
         <is>
-          <t>NL · morgen in huis (vóór 14:30)</t>
+          <t>NL · 1 werkdag</t>
         </is>
       </c>
       <c r="P7" s="13" t="inlineStr">
         <is>
-          <t>123InstallatieMaterialen</t>
+          <t>Elektramat</t>
         </is>
       </c>
       <c r="Q7" s="13" t="inlineStr">
         <is>
-          <t>https://123installatiematerialen.nl/magnum-tube-vloerverwarmingsbuis-pe-rt-12-x-15-300-meter/</t>
+          <t>https://www.elektramat.nl/magnum-universele-vloerverwarmingsbuis-5-laags-pe-rt-16x2-mm-komo-rol-240-meter-w16240/</t>
         </is>
       </c>
       <c r="R7" s="13" t="inlineStr">
@@ -2969,11 +2941,11 @@
         </is>
       </c>
       <c r="S7" s="15" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="T7" s="13" t="inlineStr">
         <is>
-          <t>All-in: +€6,95 verzending (order &lt;€200 bij 123IM). Nog steeds goedkoper dan Elektramat €181,86.</t>
+          <t>16 mm standaard voor nat/zandcement. Bij 30 m² ≈ 240 m (8 m/m²). Bundel met noppen bij Elektramat.</t>
         </is>
       </c>
       <c r="U7" s="28" t="inlineStr">
@@ -3003,12 +2975,12 @@
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>MAGNUM Euroconus 12×1,5 mm × ¾″ (set van 2)</t>
+          <t>MAGNUM Euroconus 16×2 mm × ¾″ (set van 2)</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>W90012</t>
+          <t>W90016</t>
         </is>
       </c>
       <c r="G8" s="13" t="inlineStr">
@@ -3018,10 +2990,10 @@
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>1 set per groep.</t>
-        </is>
-      </c>
-      <c r="I8" s="14">
+          <t>1 set per groep op verdeler.</t>
+        </is>
+      </c>
+      <c r="I8" s="30">
         <f>Parameters!$B$5</f>
         <v/>
       </c>
@@ -3038,7 +3010,7 @@
       </c>
       <c r="M8" s="13" t="inlineStr">
         <is>
-          <t>behouden</t>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="N8" s="15">
@@ -3057,7 +3029,7 @@
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
-          <t>https://www.elektramat.nl/magnum-adaptor-euroconus-aansluitkoppeling-12x1-5mm-x-3-4-2-stuks-w90012/</t>
+          <t>https://www.elektramat.nl/magnum-adaptor-euroconus-aansluitkoppeling-16x2mm-x-3-4-2-stuks-w90016/</t>
         </is>
       </c>
       <c r="R8" s="13" t="inlineStr">
@@ -3066,11 +3038,11 @@
         </is>
       </c>
       <c r="S8" s="15" t="n">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="T8" s="13" t="inlineStr">
         <is>
-          <t>Schaalt met aantal groepen.</t>
+          <t>Schaalt met aantal groepen. Systeemecht Magnum 16 mm.</t>
         </is>
       </c>
       <c r="U8" s="28" t="inlineStr">
@@ -3100,38 +3072,38 @@
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>MAGNUM 90° bochtondersteuning ø10–12 mm (set van 2)</t>
+          <t>Henco geleidingsbocht ø12–18 mm</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>W90125</t>
+          <t>UFH-BEND1218</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>Ondersteunt bocht bij opgang.</t>
+          <t>Kunststof opgangbocht onder verdeler.</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Opgang verdeler→vloer.</t>
-        </is>
-      </c>
-      <c r="I9" s="14">
-        <f>Parameters!$B$5</f>
+          <t>Opgang verdeler→vloer (aanvoer+retour).</t>
+        </is>
+      </c>
+      <c r="I9" s="30">
+        <f>Parameters!$B$16</f>
         <v/>
       </c>
       <c r="J9" s="13" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>st</t>
         </is>
       </c>
       <c r="K9" s="15" t="n">
-        <v>1.18</v>
+        <v>1.45</v>
       </c>
       <c r="L9" s="15" t="n">
-        <v>1.18</v>
+        <v>1.45</v>
       </c>
       <c r="M9" s="13" t="inlineStr">
         <is>
@@ -3144,17 +3116,17 @@
       </c>
       <c r="O9" s="13" t="inlineStr">
         <is>
-          <t>NL · morgen in huis (vóór 14:30)</t>
+          <t>NL · 1 werkdag</t>
         </is>
       </c>
       <c r="P9" s="13" t="inlineStr">
         <is>
-          <t>123InstallatieMaterialen</t>
+          <t>Elektramat</t>
         </is>
       </c>
       <c r="Q9" s="13" t="inlineStr">
         <is>
-          <t>https://123installatiematerialen.nl/90-bochtondersteuning-buismaat-o-10-12mm-2-stuks/</t>
+          <t>https://www.elektramat.nl/henco-geleidingsbocht-voor-buis-o12-18mm-ufh-bend1218/</t>
         </is>
       </c>
       <c r="R9" s="13" t="inlineStr">
@@ -3163,11 +3135,11 @@
         </is>
       </c>
       <c r="S9" s="15" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="T9" s="13" t="inlineStr">
         <is>
-          <t>Schaalt met aantal groepen.</t>
+          <t>2 stuks per groep. Zelfde Elektramat-order als buis/noppen.</t>
         </is>
       </c>
       <c r="U9" s="28" t="inlineStr">
@@ -3192,47 +3164,47 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Lijm</t>
+          <t>Rand</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>MAGNUM Contactlijm 500 ml</t>
+          <t>NMC Climasol randisolatie 150×8 mm – rol 25 m</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>W61027</t>
+          <t>CLIMASOL</t>
         </is>
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Spuitlijm voor Magnum verlegsystemen.</t>
+          <t>Zelfklevend, met flap.</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>Matten vastzetten.</t>
-        </is>
-      </c>
-      <c r="I10" s="14">
-        <f>MAX(1,CEILING(Parameters!$B$4*0.2,1))</f>
+          <t>Rondom muren; voorkomt scheuren in dekvloer.</t>
+        </is>
+      </c>
+      <c r="I10" s="30">
+        <f>Parameters!$B$15</f>
         <v/>
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>bus</t>
+          <t>rol</t>
         </is>
       </c>
       <c r="K10" s="15" t="n">
-        <v>9.050000000000001</v>
+        <v>23.99</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>9.050000000000001</v>
+        <v>15.62</v>
       </c>
       <c r="M10" s="13" t="inlineStr">
         <is>
-          <t>behouden</t>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="N10" s="15">
@@ -3241,17 +3213,17 @@
       </c>
       <c r="O10" s="13" t="inlineStr">
         <is>
-          <t>NL · 1 werkdag</t>
+          <t>NL · vaak volgende werkdag</t>
         </is>
       </c>
       <c r="P10" s="13" t="inlineStr">
         <is>
-          <t>Elektramat</t>
+          <t>Installand</t>
         </is>
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
-          <t>https://www.elektramat.nl/magnum-contactlijm-voor-verlijmen-magnum-verlegsystemen-w61027/</t>
+          <t>https://www.installand.nl/gena-climasol-randisolatie-zelfklevend-150-x-8-mm-rol-25-m</t>
         </is>
       </c>
       <c r="R10" s="13" t="inlineStr">
@@ -3260,11 +3232,11 @@
         </is>
       </c>
       <c r="S10" s="15" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="T10" s="13" t="inlineStr">
         <is>
-          <t>~0,2 bus/m².</t>
+          <t>Kwaliteitsupgrade; essentieel bij zandcement.</t>
         </is>
       </c>
       <c r="U10" s="28" t="inlineStr">
@@ -3289,43 +3261,43 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Rand</t>
+          <t>Wapening</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>NMC Climasol randisolatie 150×8 mm – rol 25 m</t>
+          <t>Krimpnet verzinkt ø3 mm maas 100×100 – 120×210 cm</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>CLIMASOL</t>
+          <t>KN-3100</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>Zelfklevend, met flap.</t>
+          <t>≈2,52 m²/mat; wapening/krimpbeheersing in dekvloer.</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Rondom muren; voorkomt scheuren.</t>
-        </is>
-      </c>
-      <c r="I11" s="14">
-        <f>MAX(2,CEILING(Parameters!$B$4/10,1))</f>
+          <t>In/op zandcement boven buizen tegen scheuren.</t>
+        </is>
+      </c>
+      <c r="I11" s="30">
+        <f>Parameters!$B$12</f>
         <v/>
       </c>
       <c r="J11" s="13" t="inlineStr">
         <is>
-          <t>rol</t>
+          <t>mat</t>
         </is>
       </c>
       <c r="K11" s="15" t="n">
-        <v>23.99</v>
+        <v>9.789999999999999</v>
       </c>
       <c r="L11" s="15" t="n">
-        <v>15.62</v>
+        <v>5.66</v>
       </c>
       <c r="M11" s="13" t="inlineStr">
         <is>
@@ -3338,17 +3310,17 @@
       </c>
       <c r="O11" s="13" t="inlineStr">
         <is>
-          <t>NL · vaak volgende werkdag (vóór 16:30/17:00)</t>
+          <t>NL · ≤ 1 week</t>
         </is>
       </c>
       <c r="P11" s="13" t="inlineStr">
         <is>
-          <t>Installand</t>
+          <t>Overkamp Meddo</t>
         </is>
       </c>
       <c r="Q11" s="13" t="inlineStr">
         <is>
-          <t>https://www.installand.nl/gena-climasol-randisolatie-zelfklevend-150-x-8-mm-rol-25-m</t>
+          <t>https://overkampmeddo.nl/a/bouwstaalmat-3-100-mm-2100-1200-mm-verzinkt-krimpnet</t>
         </is>
       </c>
       <c r="R11" s="13" t="inlineStr">
@@ -3361,7 +3333,7 @@
       </c>
       <c r="T11" s="13" t="inlineStr">
         <is>
-          <t>Kwaliteitsupgrade; schaalt grof met m².</t>
+          <t>Kwaliteit: 100×100 i.p.v. grovere maas. Overlap ≥1 maas.</t>
         </is>
       </c>
       <c r="U11" s="28" t="inlineStr">
@@ -3386,47 +3358,47 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Primer</t>
+          <t>Dekvloer</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>Kreisel Gruntolit-W 301 voorstrijk 5 L</t>
+          <t>Zandcement dekvloer ≥50 mm boven buis (vloerzetter, indicatief)</t>
         </is>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>301</t>
+          <t>ZC-50</t>
         </is>
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>Voorstrijk bij Kreisel egaline.</t>
+          <t>Traditionele cementdekvloer; Magnum eist min. 50 mm boven buis.</t>
         </is>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>Onder egaline.</t>
-        </is>
-      </c>
-      <c r="I12" s="14">
-        <f>MAX(1,CEILING(Parameters!$B$4*2/30,1))</f>
+          <t>Harde, massieve loopvloer — geen golven.</t>
+        </is>
+      </c>
+      <c r="I12" s="30">
+        <f>Parameters!$B$18</f>
         <v/>
       </c>
       <c r="J12" s="13" t="inlineStr">
         <is>
-          <t>bus 5L</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="K12" s="15" t="n">
-        <v>9.289999999999999</v>
+        <v>35</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>9.289999999999999</v>
+        <v>25</v>
       </c>
       <c r="M12" s="13" t="inlineStr">
         <is>
-          <t>behouden</t>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="N12" s="15">
@@ -3435,17 +3407,17 @@
       </c>
       <c r="O12" s="13" t="inlineStr">
         <is>
-          <t>NL · 1–2 werkdagen (gebundeld met egaline)</t>
+          <t>NL · lokaal (vloerzetter; planning 1–2 wkn typisch)</t>
         </is>
       </c>
       <c r="P12" s="13" t="inlineStr">
         <is>
-          <t>EgalineXXL</t>
+          <t>Lokale vloerzetter NL</t>
         </is>
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
-          <t>https://egalinexxl.nl/</t>
+          <t>https://www.magnumheating.nl/product/noppenplaat/</t>
         </is>
       </c>
       <c r="R12" s="13" t="inlineStr">
@@ -3454,16 +3426,16 @@
         </is>
       </c>
       <c r="S12" s="15" t="n">
-        <v>600</v>
+        <v>0</v>
       </c>
       <c r="T12" s="13" t="inlineStr">
         <is>
-          <t>Zelfde shop als egaline (gebundeld voor verzending).</t>
+          <t>INDICATIEF €25–55/m² incl. arbeid. Vraag 2 offertes. Kern van “kwalitatief beste” t.o.v. SlimFit/egaline.</t>
         </is>
       </c>
       <c r="U12" s="28" t="inlineStr">
         <is>
-          <t>ZEKER — NL webshop</t>
+          <t>ZEKER — lokaal NL (geen webshop-SKU)</t>
         </is>
       </c>
     </row>
@@ -3483,47 +3455,46 @@
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Egaline</t>
+          <t>Verdeler</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>Kreisel 418 vezelversterkte egaline 25 kg</t>
+          <t>VTE Composiet 4-groeps mengverdeler + Grundfos UPM3 pomp</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>418</t>
+          <t>KU100104GU</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>1–50 mm, vezels, vloerverwarming.</t>
+          <t>Composiet, flowmeters, M30, koelbaar.</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>Inbedden SlimFit + buizen.</t>
-        </is>
-      </c>
-      <c r="I13" s="14">
-        <f>CEILING(Parameters!$B$4*1.5*Parameters!$B$7/25,1)</f>
-        <v/>
+          <t>Hart van het systeem.</t>
+        </is>
+      </c>
+      <c r="I13" s="30" t="n">
+        <v>1</v>
       </c>
       <c r="J13" s="13" t="inlineStr">
         <is>
-          <t>zak</t>
+          <t>st</t>
         </is>
       </c>
       <c r="K13" s="15" t="n">
-        <v>14.87</v>
+        <v>387.18</v>
       </c>
       <c r="L13" s="15" t="n">
-        <v>14.87</v>
+        <v>305.95</v>
       </c>
       <c r="M13" s="13" t="inlineStr">
         <is>
-          <t>behouden</t>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="N13" s="15">
@@ -3532,17 +3503,17 @@
       </c>
       <c r="O13" s="13" t="inlineStr">
         <is>
-          <t>NL · volgende werkdag / pallet in overleg</t>
+          <t>NL · op voorraad, volgende werkdag mogelijk</t>
         </is>
       </c>
       <c r="P13" s="13" t="inlineStr">
         <is>
-          <t>EgalineXXL</t>
+          <t>123Installatieshop</t>
         </is>
       </c>
       <c r="Q13" s="13" t="inlineStr">
         <is>
-          <t>https://egalinexxl.nl/products/kreisel-418-vezelversterkte-egalisatie-25kg-1-50mm</t>
+          <t>https://www.123installatieshop.nl/vte-composiet-verdeler-4-groepen-met-pomp-ku100104gu</t>
         </is>
       </c>
       <c r="R13" s="13" t="inlineStr">
@@ -3551,16 +3522,16 @@
         </is>
       </c>
       <c r="S13" s="15" t="n">
-        <v>600</v>
+        <v>150</v>
       </c>
       <c r="T13" s="13" t="inlineStr">
         <is>
-          <t>All-in: +pallet ~€60,50 als order &lt;€600 excl. Goedkoper dan extra zakken kopen voor gratis verzending.</t>
+          <t>PRIJS = 4-groeps. Bij andere groepen: andere SKU!</t>
         </is>
       </c>
       <c r="U13" s="28" t="inlineStr">
         <is>
-          <t>ZEKER — NL webshop (pallet)</t>
+          <t>ZEKER — NL webshop</t>
         </is>
       </c>
     </row>
@@ -3580,46 +3551,47 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>Verdeler</t>
+          <t>Leiding</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>VTE Composiet 4-groeps mengverdeler + Grundfos UPM3 pomp</t>
+          <t>Aanvoer + retourleiding (meerlagenbuis 16×2)</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
-          <t>KU100104GU</t>
+          <t>ML162</t>
         </is>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>Composiet, flowmeters, M30, koelbaar.</t>
+          <t>Primair cv/wp → verdeler.</t>
         </is>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>Hart van het systeem.</t>
-        </is>
-      </c>
-      <c r="I14" s="17" t="n">
-        <v>1</v>
+          <t>cv/wp → verdeler.</t>
+        </is>
+      </c>
+      <c r="I14" s="30">
+        <f>MAX(8,ROUND(Parameters!$B$4/3,0))</f>
+        <v/>
       </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>m</t>
         </is>
       </c>
       <c r="K14" s="15" t="n">
-        <v>387.18</v>
+        <v>6.5</v>
       </c>
       <c r="L14" s="15" t="n">
-        <v>305.95</v>
+        <v>6.5</v>
       </c>
       <c r="M14" s="13" t="inlineStr">
         <is>
-          <t>upgrade</t>
+          <t>behouden</t>
         </is>
       </c>
       <c r="N14" s="15">
@@ -3628,17 +3600,17 @@
       </c>
       <c r="O14" s="13" t="inlineStr">
         <is>
-          <t>NL · op voorraad, volgende werkdag mogelijk</t>
+          <t>NL · ≤ 1 week</t>
         </is>
       </c>
       <c r="P14" s="13" t="inlineStr">
         <is>
-          <t>123Installatieshop</t>
+          <t>123Installatieshop / bouwmarkt NL</t>
         </is>
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>https://www.123installatieshop.nl/vte-composiet-verdeler-4-groepen-met-pomp-ku100104gu</t>
+          <t>https://www.123installatieshop.nl/</t>
         </is>
       </c>
       <c r="R14" s="13" t="inlineStr">
@@ -3647,16 +3619,16 @@
         </is>
       </c>
       <c r="S14" s="15" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="T14" s="13" t="inlineStr">
         <is>
-          <t>PRIJS = 4-groeps. Bij andere groepen: andere SKU/prijs kiezen!</t>
+          <t>Situatie-afhankelijk.</t>
         </is>
       </c>
       <c r="U14" s="28" t="inlineStr">
         <is>
-          <t>ZEKER — NL webshop</t>
+          <t>ZEKER — NL</t>
         </is>
       </c>
     </row>
@@ -3676,43 +3648,42 @@
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Leiding</t>
+          <t>Afsluiters</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Aanvoer + retourleiding (meerlagenbuis 16×2)</t>
+          <t>Kogelkranen / koppelingen set</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
-          <t>ML162</t>
+          <t>KK-SET</t>
         </is>
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>Primair cv/wp → verdeler.</t>
+          <t>Afsluitbaar maken.</t>
         </is>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>cv/wp → verdeler.</t>
-        </is>
-      </c>
-      <c r="I15" s="14">
-        <f>MAX(8,ROUND(Parameters!$B$4/3,0))</f>
-        <v/>
+          <t>Service/afsluitbaar.</t>
+        </is>
+      </c>
+      <c r="I15" s="30" t="n">
+        <v>1</v>
       </c>
       <c r="J15" s="13" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>set</t>
         </is>
       </c>
       <c r="K15" s="15" t="n">
-        <v>6.5</v>
+        <v>34.95</v>
       </c>
       <c r="L15" s="15" t="n">
-        <v>6.5</v>
+        <v>34.95</v>
       </c>
       <c r="M15" s="13" t="inlineStr">
         <is>
@@ -3725,12 +3696,12 @@
       </c>
       <c r="O15" s="13" t="inlineStr">
         <is>
-          <t>NL · ≤ 1 week (standaard meerlagenbuis)</t>
+          <t>NL · ≤ 1 week</t>
         </is>
       </c>
       <c r="P15" s="13" t="inlineStr">
         <is>
-          <t>123Installatieshop / bouwmarkt NL</t>
+          <t>123Installatieshop</t>
         </is>
       </c>
       <c r="Q15" s="13" t="inlineStr">
@@ -3744,16 +3715,16 @@
         </is>
       </c>
       <c r="S15" s="15" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="T15" s="13" t="inlineStr">
         <is>
-          <t>Situatie-afhankelijk; schaalt licht met woninggrootte. Lokale bouwmarkt of NL-installatieshop; geen import.</t>
+          <t>Vast per installatie.</t>
         </is>
       </c>
       <c r="U15" s="28" t="inlineStr">
         <is>
-          <t>ZEKER — NL (generiek artikel)</t>
+          <t>ZEKER — NL webshop</t>
         </is>
       </c>
     </row>
@@ -3773,84 +3744,83 @@
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>Afsluiters</t>
+          <t>Actuator</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Kogelkranen / koppelingen set</t>
+          <t>Möhlenhoff Alpha 5 thermische motor 230V NC M30×1,5 (+ adapter)</t>
         </is>
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>KK-SET</t>
+          <t>A20405-00N80-1S</t>
         </is>
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>Afsluitbaar maken.</t>
+          <t>NC 230V, VA80 adapter, 1 W.</t>
         </is>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>Service/afsluitbaar.</t>
-        </is>
-      </c>
-      <c r="I16" s="17" t="n">
-        <v>1</v>
+          <t>1 per groep.</t>
+        </is>
+      </c>
+      <c r="I16" s="30">
+        <f>Parameters!$B$5</f>
+        <v/>
       </c>
       <c r="J16" s="13" t="inlineStr">
         <is>
-          <t>set</t>
-        </is>
-      </c>
-      <c r="K16" s="15" t="n">
-        <v>34.95</v>
-      </c>
-      <c r="L16" s="15" t="n">
-        <v>34.95</v>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="K16" s="15">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),20.12,9.99)</f>
+        <v/>
+      </c>
+      <c r="L16" s="15">
+        <f>K16</f>
+        <v/>
       </c>
       <c r="M16" s="13" t="inlineStr">
         <is>
-          <t>behouden</t>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="N16" s="15">
         <f>I16*K16</f>
         <v/>
       </c>
-      <c r="O16" s="13" t="inlineStr">
-        <is>
-          <t>NL · ≤ 1 week</t>
-        </is>
-      </c>
-      <c r="P16" s="13" t="inlineStr">
-        <is>
-          <t>123Installatieshop</t>
-        </is>
-      </c>
-      <c r="Q16" s="13" t="inlineStr">
-        <is>
-          <t>https://www.123installatieshop.nl/</t>
-        </is>
-      </c>
-      <c r="R16" s="13" t="inlineStr">
-        <is>
-          <t>NL</t>
-        </is>
-      </c>
-      <c r="S16" s="15" t="n">
-        <v>50</v>
+      <c r="O16" s="13">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"NL · 3–4 werkdagen (VerwarmingOnline)","DE→NL · 2–5 wd DE + NL-transit (eibhandel DHL)")</f>
+        <v/>
+      </c>
+      <c r="P16" s="13">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"VerwarmingOnline","eibhandel.de")</f>
+        <v/>
+      </c>
+      <c r="Q16" s="13">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"https://verwarmingonline.nl/productgroepen/mohlenhoff-thermische-servomotor-alpha-5-nc-m30x15mm-230v-a-20405-00n/","https://eibhandel.de/Alpha-Antrieb-230V-NC-incl-Adapter-VA80")</f>
+        <v/>
+      </c>
+      <c r="R16" s="13">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"NL","DE→NL")</f>
+        <v/>
+      </c>
+      <c r="S16" s="15">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),385,1000)</f>
+        <v/>
       </c>
       <c r="T16" s="13" t="inlineStr">
         <is>
-          <t>Vast per installatie.</t>
-        </is>
-      </c>
-      <c r="U16" s="28" t="inlineStr">
-        <is>
-          <t>ZEKER — NL webshop</t>
-        </is>
+          <t>Schakel via Parameters!B8. DE→NL: verzending ≈€15,41.</t>
+        </is>
+      </c>
+      <c r="U16" s="28">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"ZEKER — NL webshop","DE→NL bevestigd (DHL zone 1)")</f>
+        <v/>
       </c>
     </row>
     <row r="17">
@@ -3869,45 +3839,42 @@
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Actuator</t>
+          <t>Elektra</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>Möhlenhoff Alpha 5 thermische motor 230V NC M30×1,5 (+ adapter)</t>
+          <t>Elektrakabel 230V / signaalkabel (installatiekwaliteit)</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>A20405-00N80-1S</t>
+          <t>ELEKTRA</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>NC 230V, VA80 adapter, 1 W.</t>
+          <t>Voeding pomp/regeling/actuators.</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
-          <t>1 per groep.</t>
-        </is>
-      </c>
-      <c r="I17" s="14">
-        <f>Parameters!$B$5</f>
-        <v/>
+          <t>Elektra.</t>
+        </is>
+      </c>
+      <c r="I17" s="30" t="n">
+        <v>1</v>
       </c>
       <c r="J17" s="13" t="inlineStr">
         <is>
-          <t>st</t>
-        </is>
-      </c>
-      <c r="K17" s="15">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),20.12,9.99)</f>
-        <v/>
-      </c>
-      <c r="L17" s="15">
-        <f>K17</f>
-        <v/>
+          <t>kleinmateriaal</t>
+        </is>
+      </c>
+      <c r="K17" s="15" t="n">
+        <v>25</v>
+      </c>
+      <c r="L17" s="15" t="n">
+        <v>20</v>
       </c>
       <c r="M17" s="13" t="inlineStr">
         <is>
@@ -3918,34 +3885,38 @@
         <f>I17*K17</f>
         <v/>
       </c>
-      <c r="O17" s="13">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"NL · 3–4 werkdagen (VerwarmingOnline)","DE→NL · 2–5 wd DE + NL-transit (eibhandel DHL)")</f>
-        <v/>
-      </c>
-      <c r="P17" s="13">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"VerwarmingOnline","eibhandel.de")</f>
-        <v/>
-      </c>
-      <c r="Q17" s="13">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"https://verwarmingonline.nl/productgroepen/mohlenhoff-thermische-servomotor-alpha-5-nc-m30x15mm-230v-a-20405-00n/","https://eibhandel.de/Alpha-Antrieb-230V-NC-incl-Adapter-VA80")</f>
-        <v/>
-      </c>
-      <c r="R17" s="29">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"NL","DE→NL")</f>
-        <v/>
-      </c>
-      <c r="S17" s="15">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),385,1000)</f>
-        <v/>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>NL · 1 werkdag / afhalen</t>
+        </is>
+      </c>
+      <c r="P17" s="13" t="inlineStr">
+        <is>
+          <t>Elektramat</t>
+        </is>
+      </c>
+      <c r="Q17" s="13" t="inlineStr">
+        <is>
+          <t>https://www.elektramat.nl/draad-en-kabel/installatiekabel/</t>
+        </is>
+      </c>
+      <c r="R17" s="29" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="S17" s="15" t="n">
+        <v>0</v>
       </c>
       <c r="T17" s="13" t="inlineStr">
         <is>
-          <t>Schakel via Parameters!B8. DE→NL: verzending ≈€15,41 + levertijd 2–5 wd DE. NL zeker: €20,12/st, verzending €0 als order ≥€385 anders ~€6,95.</t>
-        </is>
-      </c>
-      <c r="U17">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"ZEKER — NL webshop","DE→NL bevestigd (DHL zone 1)")</f>
-        <v/>
+          <t>Vast; bij groter project licht ophogen. Bundel met Magnum-order.</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>ZEKER — NL</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -3959,51 +3930,51 @@
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>altijd</t>
+          <t>h64</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Elektra</t>
+          <t>Regeling</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>Elektrakabel 230V / signaalkabel (installatiekwaliteit)</t>
+          <t>MAGNUM H64-CC + master WiFi-thermostaat</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>ELEKTRA</t>
+          <t>W81000</t>
         </is>
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>Voeding pomp/regeling/actuators.</t>
+          <t>Control Center + master.</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>Elektra.</t>
-        </is>
-      </c>
-      <c r="I18" s="17" t="n">
+          <t>Alleen bij keuze H64.</t>
+        </is>
+      </c>
+      <c r="I18" s="30" t="n">
         <v>1</v>
       </c>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>kleinmateriaal</t>
+          <t>set</t>
         </is>
       </c>
       <c r="K18" s="15" t="n">
-        <v>25</v>
+        <v>194.92</v>
       </c>
       <c r="L18" s="15" t="n">
-        <v>20</v>
+        <v>194.92</v>
       </c>
       <c r="M18" s="13" t="inlineStr">
         <is>
-          <t>upgrade</t>
+          <t>behouden</t>
         </is>
       </c>
       <c r="N18" s="15">
@@ -4012,17 +3983,17 @@
       </c>
       <c r="O18" s="13" t="inlineStr">
         <is>
-          <t>NL · 1 werkdag / direct afhalen</t>
+          <t>NL · 1 werkdag</t>
         </is>
       </c>
       <c r="P18" s="13" t="inlineStr">
         <is>
-          <t>Elektramat / bouwmarkt NL</t>
+          <t>Warp Systems</t>
         </is>
       </c>
       <c r="Q18" s="13" t="inlineStr">
         <is>
-          <t>https://www.elektramat.nl/draad-en-kabel/installatiekabel/</t>
+          <t>https://shop.warp-systems.com/h64-control-center-master-wifi-thermostaat-wit-of-zwart-magh64cc-mt-c</t>
         </is>
       </c>
       <c r="R18" s="13" t="inlineStr">
@@ -4035,12 +4006,12 @@
       </c>
       <c r="T18" s="13" t="inlineStr">
         <is>
-          <t>Vast; bij groter project licht ophogen.</t>
+          <t>NL-fabrikant.</t>
         </is>
       </c>
       <c r="U18" s="28" t="inlineStr">
         <is>
-          <t>ZEKER — NL</t>
+          <t>ZEKER — NL fabrikant</t>
         </is>
       </c>
     </row>
@@ -4065,37 +4036,38 @@
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>MAGNUM H64-CC + master WiFi-thermostaat</t>
+          <t>MAGNUM H64-ST slave thermostaat</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>W81000</t>
+          <t>W81010</t>
         </is>
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>Control Center + master.</t>
+          <t>Slave per extra ruimte.</t>
         </is>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
-          <t>Alleen bij keuze H64.</t>
-        </is>
-      </c>
-      <c r="I19" s="17" t="n">
-        <v>1</v>
+          <t>Ruimte 2…N bij H64.</t>
+        </is>
+      </c>
+      <c r="I19" s="30">
+        <f>MAX(0,Parameters!$B$6-1)</f>
+        <v/>
       </c>
       <c r="J19" s="13" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>st</t>
         </is>
       </c>
       <c r="K19" s="15" t="n">
-        <v>194.92</v>
+        <v>44.58</v>
       </c>
       <c r="L19" s="15" t="n">
-        <v>194.92</v>
+        <v>44.58</v>
       </c>
       <c r="M19" s="13" t="inlineStr">
         <is>
@@ -4108,7 +4080,7 @@
       </c>
       <c r="O19" s="13" t="inlineStr">
         <is>
-          <t>NL · 1 werkdag (voor 12:00 zelfde dag verzonden)</t>
+          <t>NL · 1 werkdag</t>
         </is>
       </c>
       <c r="P19" s="13" t="inlineStr">
@@ -4118,7 +4090,7 @@
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>https://shop.warp-systems.com/h64-control-center-master-wifi-thermostaat-wit-of-zwart-magh64cc-mt-c</t>
+          <t>https://shop.warp-systems.com/catalogsearch/result/?q=slave+H64</t>
         </is>
       </c>
       <c r="R19" s="13" t="inlineStr">
@@ -4131,7 +4103,7 @@
       </c>
       <c r="T19" s="13" t="inlineStr">
         <is>
-          <t>NL-fabrikant, snelle levering.</t>
+          <t>Schaalt met ruimten−1.</t>
         </is>
       </c>
       <c r="U19" s="28" t="inlineStr">
@@ -4151,7 +4123,7 @@
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>h64</t>
+          <t>tado_draadloos</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
@@ -4161,38 +4133,38 @@
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>MAGNUM H64-ST slave thermostaat</t>
+          <t>tado° Draadloze Slimme Thermostaat X Starterskit</t>
         </is>
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
-          <t>W81010</t>
+          <t>TADO-WX</t>
         </is>
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t>Slave per extra ruimte.</t>
+          <t>Wireless X + Bridge.</t>
         </is>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>Ruimte 2…N bij H64.</t>
-        </is>
-      </c>
-      <c r="I20" s="14">
-        <f>MAX(0,Parameters!$B$6-1)</f>
+          <t>1 kit per ruimte (draadloos).</t>
+        </is>
+      </c>
+      <c r="I20" s="30">
+        <f>Parameters!$B$6</f>
         <v/>
       </c>
       <c r="J20" s="13" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>set</t>
         </is>
       </c>
       <c r="K20" s="15" t="n">
-        <v>44.58</v>
+        <v>129</v>
       </c>
       <c r="L20" s="15" t="n">
-        <v>44.58</v>
+        <v>129</v>
       </c>
       <c r="M20" s="13" t="inlineStr">
         <is>
@@ -4205,17 +4177,17 @@
       </c>
       <c r="O20" s="13" t="inlineStr">
         <is>
-          <t>NL · 1 werkdag</t>
+          <t>NL/EU · 2–4 werkdagen</t>
         </is>
       </c>
       <c r="P20" s="13" t="inlineStr">
         <is>
-          <t>Warp Systems</t>
+          <t>tado° Shop</t>
         </is>
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
-          <t>https://shop.warp-systems.com/catalogsearch/result/?q=slave+H64</t>
+          <t>https://shop.tado.com/nl-bx/products/wireless-smart-thermostat-x-starter-kit</t>
         </is>
       </c>
       <c r="R20" s="13" t="inlineStr">
@@ -4224,16 +4196,16 @@
         </is>
       </c>
       <c r="S20" s="15" t="n">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="T20" s="13" t="inlineStr">
         <is>
-          <t>Schaalt met ruimten−1.</t>
+          <t>Schaalt met ruimten.</t>
         </is>
       </c>
       <c r="U20" s="28" t="inlineStr">
         <is>
-          <t>ZEKER — NL fabrikant</t>
+          <t>ZEKER — tado° NL-shop</t>
         </is>
       </c>
     </row>
@@ -4248,7 +4220,7 @@
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>tado_draadloos</t>
+          <t>tado_bedraad</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
@@ -4258,27 +4230,26 @@
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>tado° Draadloze Slimme Thermostaat X Starterskit</t>
+          <t>tado° Slimme Thermostaat X Starterskit bedraad + Bridge X</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>TADO-WX</t>
+          <t>TADO-WX-W</t>
         </is>
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t>Wireless X + Bridge.</t>
+          <t>Wired starter + Bridge.</t>
         </is>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>1 kit per ruimte (draadloos).</t>
-        </is>
-      </c>
-      <c r="I21" s="14">
-        <f>Parameters!$B$6</f>
-        <v/>
+          <t>Kamer 1 + netwerk.</t>
+        </is>
+      </c>
+      <c r="I21" s="30" t="n">
+        <v>1</v>
       </c>
       <c r="J21" s="13" t="inlineStr">
         <is>
@@ -4286,14 +4257,14 @@
         </is>
       </c>
       <c r="K21" s="15" t="n">
-        <v>129</v>
+        <v>129.99</v>
       </c>
       <c r="L21" s="15" t="n">
-        <v>129</v>
+        <v>129.99</v>
       </c>
       <c r="M21" s="13" t="inlineStr">
         <is>
-          <t>behouden</t>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="N21" s="15">
@@ -4302,7 +4273,7 @@
       </c>
       <c r="O21" s="13" t="inlineStr">
         <is>
-          <t>NL/EU · 2–4 werkdagen (tado° levert NL)</t>
+          <t>NL/EU · 2–4 werkdagen</t>
         </is>
       </c>
       <c r="P21" s="13" t="inlineStr">
@@ -4312,7 +4283,7 @@
       </c>
       <c r="Q21" s="13" t="inlineStr">
         <is>
-          <t>https://shop.tado.com/nl-bx/products/wireless-smart-thermostat-x-starter-kit</t>
+          <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-starter-kit-1</t>
         </is>
       </c>
       <c r="R21" s="13" t="inlineStr">
@@ -4325,7 +4296,7 @@
       </c>
       <c r="T21" s="13" t="inlineStr">
         <is>
-          <t>Schaalt met ruimten. Officiële shop goedkoopst.</t>
+          <t>Aanbevolen pad (bedraad).</t>
         </is>
       </c>
       <c r="U21" s="28" t="inlineStr">
@@ -4355,37 +4326,38 @@
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>tado° Slimme Thermostaat X Starterskit bedraad + Bridge X</t>
+          <t>tado° Slimme Thermostaat X bedraad (uitbreiding)</t>
         </is>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
-          <t>TADO-WX-W</t>
+          <t>TADO-WX-E</t>
         </is>
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>Wired starter + Bridge.</t>
+          <t>Extra bedrade thermostaat.</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>Kamer 1 + netwerk.</t>
-        </is>
-      </c>
-      <c r="I22" s="17" t="n">
-        <v>1</v>
+          <t>Kamer 2…N.</t>
+        </is>
+      </c>
+      <c r="I22" s="30">
+        <f>MAX(0,Parameters!$B$6-1)</f>
+        <v/>
       </c>
       <c r="J22" s="13" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>st</t>
         </is>
       </c>
       <c r="K22" s="15" t="n">
-        <v>129.99</v>
+        <v>100</v>
       </c>
       <c r="L22" s="15" t="n">
-        <v>129.99</v>
+        <v>100</v>
       </c>
       <c r="M22" s="13" t="inlineStr">
         <is>
@@ -4408,7 +4380,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-starter-kit-1</t>
+          <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-wired</t>
         </is>
       </c>
       <c r="R22" s="13" t="inlineStr">
@@ -4421,7 +4393,7 @@
       </c>
       <c r="T22" s="13" t="inlineStr">
         <is>
-          <t>Aanbevolen pad (bedraad).</t>
+          <t>Schaalt met ruimten−1.</t>
         </is>
       </c>
       <c r="U22" s="28" t="inlineStr">
@@ -4441,7 +4413,7 @@
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>tado_bedraad</t>
+          <t>tado_optie</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
@@ -4451,27 +4423,26 @@
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>tado° Slimme Thermostaat X bedraad (uitbreiding)</t>
+          <t>tado° Bridge X (extra indien nodig)</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>TADO-WX-E</t>
+          <t>TADO-BR</t>
         </is>
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t>Extra bedrade thermostaat.</t>
+          <t>Alleen bij bereikproblemen.</t>
         </is>
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
-          <t>Kamer 2…N.</t>
-        </is>
-      </c>
-      <c r="I23" s="14">
-        <f>MAX(0,Parameters!$B$6-1)</f>
-        <v/>
+          <t>Optioneel.</t>
+        </is>
+      </c>
+      <c r="I23" s="30" t="n">
+        <v>0</v>
       </c>
       <c r="J23" s="13" t="inlineStr">
         <is>
@@ -4479,14 +4450,14 @@
         </is>
       </c>
       <c r="K23" s="15" t="n">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="L23" s="15" t="n">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="M23" s="13" t="inlineStr">
         <is>
-          <t>upgrade</t>
+          <t>behouden</t>
         </is>
       </c>
       <c r="N23" s="15">
@@ -4505,7 +4476,7 @@
       </c>
       <c r="Q23" s="13" t="inlineStr">
         <is>
-          <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-wired</t>
+          <t>https://shop.tado.com/nl-bx/</t>
         </is>
       </c>
       <c r="R23" s="13" t="inlineStr">
@@ -4518,7 +4489,7 @@
       </c>
       <c r="T23" s="13" t="inlineStr">
         <is>
-          <t>Schaalt met ruimten−1.</t>
+          <t>Standaard 0.</t>
         </is>
       </c>
       <c r="U23" s="28" t="inlineStr">
@@ -4528,113 +4499,30 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
-        <is>
-          <t>Vloerverwarming</t>
-        </is>
-      </c>
-      <c r="B24" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="C24" s="13" t="inlineStr">
-        <is>
-          <t>tado_optie</t>
-        </is>
-      </c>
-      <c r="D24" s="13" t="inlineStr">
-        <is>
-          <t>Regeling</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="inlineStr">
-        <is>
-          <t>tado° Bridge X (extra indien nodig)</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>TADO-BR</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>Alleen bij bereikproblemen.</t>
-        </is>
-      </c>
-      <c r="H24" s="13" t="inlineStr">
-        <is>
-          <t>Optioneel.</t>
-        </is>
-      </c>
-      <c r="I24" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" s="13" t="inlineStr">
-        <is>
-          <t>st</t>
-        </is>
-      </c>
-      <c r="K24" s="15" t="n">
-        <v>68</v>
-      </c>
-      <c r="L24" s="15" t="n">
-        <v>68</v>
-      </c>
-      <c r="M24" s="13" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="N24" s="15">
-        <f>I24*K24</f>
-        <v/>
-      </c>
-      <c r="O24" s="13" t="inlineStr">
-        <is>
-          <t>NL/EU · 2–4 werkdagen</t>
-        </is>
-      </c>
-      <c r="P24" s="13" t="inlineStr">
-        <is>
-          <t>tado° Shop</t>
-        </is>
-      </c>
-      <c r="Q24" s="13" t="inlineStr">
-        <is>
-          <t>https://shop.tado.com/nl-bx/</t>
-        </is>
-      </c>
-      <c r="R24" s="13" t="inlineStr">
-        <is>
-          <t>NL</t>
-        </is>
-      </c>
-      <c r="S24" s="15" t="n">
-        <v>150</v>
-      </c>
-      <c r="T24" s="13" t="inlineStr">
-        <is>
-          <t>Standaard 0; handmatig verhogen indien nodig.</t>
-        </is>
-      </c>
-      <c r="U24" s="28" t="inlineStr">
-        <is>
-          <t>ZEKER — tado° NL-shop</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Groen = hoeveelheid-formule (schaalt). Totaal = Hoeveelheid × Prijs/st. Verzendkosten: sheet Verzending.</t>
-        </is>
-      </c>
+      <c r="A24" s="12" t="n"/>
+      <c r="B24" s="13" t="n"/>
+      <c r="C24" s="13" t="n"/>
+      <c r="D24" s="13" t="n"/>
+      <c r="E24" s="13" t="n"/>
+      <c r="F24" s="13" t="n"/>
+      <c r="G24" s="13" t="n"/>
+      <c r="H24" s="13" t="n"/>
+      <c r="I24" s="17" t="n"/>
+      <c r="J24" s="13" t="n"/>
+      <c r="K24" s="15" t="n"/>
+      <c r="L24" s="15" t="n"/>
+      <c r="M24" s="13" t="n"/>
+      <c r="N24" s="15" t="n"/>
+      <c r="O24" s="13" t="n"/>
+      <c r="P24" s="13" t="n"/>
+      <c r="Q24" s="13" t="n"/>
+      <c r="R24" s="13" t="n"/>
+      <c r="S24" s="15" t="n"/>
+      <c r="T24" s="13" t="n"/>
+      <c r="U24" s="28" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:T24"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:T1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4645,7 +4533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4660,21 +4548,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>All-in check — prijs + verzending (nog steeds goedkoopste?)</t>
+          <t>All-in check — kwalitatief beste BOM</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Uitgangspunt: 30 m² · 4 groepen · 3 ruimten. Alleen NL-leverbare opties (of DE→NL met expliciete verzending/levertijd).</t>
+          <t>30 m² · 4 groepen · 3 ruimten · dekvloer ≥50 mm. Hardheid &gt; laagste opbouw.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="21" t="inlineStr">
         <is>
-          <t>Verdict: JA — alle gekozen shops blijven all-in het goedkoopst. Geen shopwissel nodig.</t>
+          <t>Verdict: BOM omgezet SlimFit/egaline → noppen 28 mm + PE-RT 16 + zandcement.</t>
         </is>
       </c>
     </row>
@@ -4691,12 +4579,12 @@
       </c>
       <c r="C5" s="22" t="inlineStr">
         <is>
-          <t>Gekozen (all-in)</t>
+          <t>Gekozen</t>
         </is>
       </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>Alternatief all-in</t>
+          <t>Alternatief</t>
         </is>
       </c>
       <c r="E5" s="22" t="inlineStr">
@@ -4706,7 +4594,7 @@
       </c>
       <c r="F5" s="22" t="inlineStr">
         <is>
-          <t>NL-leverbaar?</t>
+          <t>NL?</t>
         </is>
       </c>
       <c r="G5" s="22" t="inlineStr">
@@ -4721,27 +4609,27 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>SlimFit matten 8×</t>
+          <t>Noppen 28 mm 3×</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Elektramat €695,52 (ship €0; order ≫ €150 excl)</t>
+          <t>Elektramat 3×€136,58</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>123IM €711,92 · VV-direct €712</t>
+          <t>17 mm goedkoper, minder isolatie</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>−€16…€17</t>
+          <t>kwaliteit</t>
         </is>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>Ja NL 1 wd</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="G6" s="23" t="inlineStr">
@@ -4756,27 +4644,27 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>PE-RT 300 m</t>
+          <t>PE-RT 240 m</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>123IM €142,93 + €6,95 ship ≈ €149,88 (order &lt;€200)</t>
+          <t>Elektramat €158,99</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Elektramat €181,86 (ship €0 in combi)</t>
+          <t>losse rollen ≥</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>−€32</t>
+          <t>beste</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Ja NL morgen</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="G7" s="23" t="inlineStr">
@@ -4791,32 +4679,32 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Kreisel 418 33× + primer</t>
+          <t>Zandcement</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>EgalineXXL €509,29 + pallet €60,50 = €569,79</t>
+          <t>€35/m² indicatief</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>RBMB duurder/stuk · extra kopen tot €600 excl ≈ €610+</t>
+          <t>€25–55 lokaal</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>−€40…</t>
+          <t>offerte</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>Ja NL pallet</t>
+          <t>Ja lokaal</t>
         </is>
       </c>
       <c r="G8" s="23" t="inlineStr">
         <is>
-          <t>BEHOUDEN</t>
+          <t>OFFERTE</t>
         </is>
       </c>
     </row>
@@ -4826,27 +4714,27 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>VTE Composiet 4-gr.</t>
+          <t>VTE + Grundfos</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>123Installatieshop €387,18 (ship €0 ≥€150)</t>
+          <t>€387,18</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>VV-shop €405 · CVTotaal €423 · Jan Isolatieman €469</t>
+          <t>duurdere shops</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>−€18…€82</t>
+          <t>beste</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Ja NL ≤1 wk</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="G9" s="23" t="inlineStr">
@@ -4861,27 +4749,27 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Möhlenhoff Alpha 5 ×4</t>
+          <t>Möhlenhoff ×4</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>eibhandel.de €39,96 + €15,41 = €55,37</t>
+          <t>eibhandel ~€55 all-in</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Amazon~€52,64* · Home Perfect €69,94 · VerwarmingOnline €87,43</t>
+          <t>NL duurder</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>beste bevestigd</t>
+          <t>beste</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>Ja DE→NL DHL</t>
+          <t>DE→NL</t>
         </is>
       </c>
       <c r="G10" s="23" t="inlineStr">
@@ -4891,235 +4779,109 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>NMC Climasol 3×</t>
-        </is>
-      </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>Installand €71,97 (ship €0 ≥€60)</t>
-        </is>
-      </c>
-      <c r="D11" s="13" t="inlineStr">
-        <is>
-          <t>Generiek Distriheat goedkoper maar mindere kwaliteit</t>
-        </is>
-      </c>
-      <c r="E11" s="13" t="inlineStr">
-        <is>
-          <t>kwaliteit</t>
-        </is>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t>Ja NL</t>
-        </is>
-      </c>
-      <c r="G11" s="23" t="inlineStr">
-        <is>
-          <t>BEHOUDEN</t>
-        </is>
-      </c>
+      <c r="A11" s="13" t="n"/>
+      <c r="B11" s="13" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="13" t="n"/>
+      <c r="E11" s="13" t="n"/>
+      <c r="F11" s="13" t="n"/>
+      <c r="G11" s="23" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>H64-CC + slaves</t>
-        </is>
-      </c>
-      <c r="C12" s="13" t="inlineStr">
-        <is>
-          <t>Warp Systems €194,92 + 2×€44,58 (NL)</t>
-        </is>
-      </c>
-      <c r="D12" s="13" t="inlineStr">
-        <is>
-          <t>123IM H64-CC was €213,74</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
-          <t>−€19 CC</t>
-        </is>
-      </c>
-      <c r="F12" s="13" t="inlineStr">
-        <is>
-          <t>Ja NL 1 wd</t>
-        </is>
-      </c>
-      <c r="G12" s="23" t="inlineStr">
-        <is>
-          <t>BEHOUDEN</t>
-        </is>
-      </c>
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Live totalen</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
+      <c r="E12" s="13" t="n"/>
+      <c r="F12" s="13" t="n"/>
+      <c r="G12" s="23" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>Tado bedraad 3 ruimten</t>
-        </is>
-      </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>tado° Shop €329,99 (ship €0 ≥€150)</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>bol/retail vaak €189–€194 per starter alleen</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
-          <t>goedkoopst</t>
-        </is>
-      </c>
-      <c r="F13" s="13" t="inlineStr">
-        <is>
-          <t>Ja NL/EU</t>
-        </is>
-      </c>
-      <c r="G13" s="23" t="inlineStr">
-        <is>
-          <t>BEHOUDEN</t>
-        </is>
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Basis artikelen</t>
+        </is>
+      </c>
+      <c r="B13" s="13">
+        <f>Overzicht!B10</f>
+        <v/>
+      </c>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
+      <c r="E13" s="13" t="n"/>
+      <c r="F13" s="13" t="n"/>
+      <c r="G13" s="23" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Basis verzending</t>
+        </is>
+      </c>
+      <c r="B14">
+        <f>Overzicht!C10</f>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Consolidatie-check (minder shops = minder verzending?)</t>
-        </is>
+          <t>Basis all-in</t>
+        </is>
+      </c>
+      <c r="B15">
+        <f>Overzicht!D10</f>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>• PE-RT meenemen bij Elektramat (zelfde order als SlimFit): all-in €181,86 i.p.v. ~€149,88 → NIET doen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>• Extra egaline kopen tot gratis drempel (€600 excl): duurder dan pallet betalen → NIET doen.</t>
-        </is>
+          <t>All-in + Tado bedraad</t>
+        </is>
+      </c>
+      <c r="B16">
+        <f>Overzicht!D11</f>
+        <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>• Actuators bij VerwarmingOnline (pure NL): +€32 vs eibhandel → alleen als je DE wilt vermijden.</t>
+          <t>Zandcement-regel is INDICATIEF. Echt totaal = webshop-BOM + vloerzetter-offerte.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>• Home Perfect (€10,01/st) lijkt scherp maar +€29,90 ship + 7–10 wd → all-in slechter én trager.</t>
+          <t>Infrezen: vaak hardst als bestaande dekvloer geschikt is — apart laten beoordelen.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>Buitenland / NL-zekerheid</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Enige buitenlandse shop: eibhandel.de (actuators). Levert naar NL (DHL zone 1), verzending €15,41 incl, levertijd 2–5 wd DE (+NL-transit, meestal ≤1 week).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Alles overige: Nederlandse webshops met snelle levering.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>* Amazon.nl-prijs is indicatief (listings wisselen); eibhandel is stabiel bevestigd all-in.</t>
-        </is>
-      </c>
+      <c r="A21" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr">
-        <is>
-          <t>Live totalen (formules, schalen met m²)</t>
-        </is>
-      </c>
+      <c r="A26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>Basis artikelen</t>
-        </is>
-      </c>
-      <c r="B27" s="6">
-        <f>Overzicht!B10</f>
-        <v/>
-      </c>
+      <c r="B27" s="6" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Basis verzending</t>
-        </is>
-      </c>
-      <c r="B28" s="6">
-        <f>Overzicht!C10</f>
-        <v/>
-      </c>
+      <c r="B28" s="6" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>Basis all-in</t>
-        </is>
-      </c>
-      <c r="B29" s="6">
-        <f>Overzicht!D10</f>
-        <v/>
-      </c>
+      <c r="B29" s="6" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>All-in + Tado bedraad</t>
-        </is>
-      </c>
-      <c r="B30" s="6">
-        <f>Overzicht!D11</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>NL-update: schakelaar Parameters!B8. Default DE→NL blijft goedkoopst all-in; kies NL zeker indien je geen import wilt.</t>
-        </is>
-      </c>
+      <c r="B30" s="6" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5146,7 +4908,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Verzendkosten — berekend all-in (NL-leverbaar)</t>
+          <t>Verzendkosten — all-in (kwalitatief beste BOM)</t>
         </is>
       </c>
     </row>
@@ -5211,7 +4973,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A5,Boodschappenlijst!$C$6:$C$24,"altijd")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A5,Boodschappenlijst!$C$6:$C$23,"altijd")</f>
         <v/>
       </c>
       <c r="D5" s="5" t="n">
@@ -5232,14 +4994,14 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Drempel €150 excl. btw; onder: €4,09 excl ≈ €4,95 incl</t>
+          <t>Noppen+buis+euro+bocht. Noppen=lengtevracht; check pallet/afhaal bij Elektramat.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>123InstallatieMaterialen</t>
+          <t>Overkamp Meddo</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5248,14 +5010,14 @@
         </is>
       </c>
       <c r="C6" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A6,Boodschappenlijst!$C$6:$C$24,"altijd")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A6,Boodschappenlijst!$C$6:$C$23,"altijd")</f>
         <v/>
       </c>
       <c r="D6" s="5" t="n">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="E6" s="5">
-        <f>IF(C6&lt;=0,0,IF(C6&gt;=200,0,6.95))</f>
+        <f>IF(C6&lt;=0,0,IF(C6&gt;=50,0,6.95))</f>
         <v/>
       </c>
       <c r="F6" s="5">
@@ -5264,12 +5026,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>morgen</t>
+          <t>≤1 week</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Buis+bochten vaak &lt;€200 → €6,95 verzending; all-in nog steeds goedkoper dan Elektramat-buis</t>
+          <t>Krimpnetten</t>
         </is>
       </c>
     </row>
@@ -5285,7 +5047,7 @@
         </is>
       </c>
       <c r="C7" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A7,Boodschappenlijst!$C$6:$C$24,"altijd")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A7,Boodschappenlijst!$C$6:$C$23,"altijd")+SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,"123Installatieshop / bouwmarkt NL",Boodschappenlijst!$C$6:$C$23,"altijd")</f>
         <v/>
       </c>
       <c r="D7" s="5" t="n">
@@ -5306,14 +5068,14 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Verdeler alleen al &gt;€150 → gratis verzending</t>
+          <t>Verdeler+afsluiters (+ evt. ML-buis)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>EgalineXXL</t>
+          <t>Lokale vloerzetter NL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5322,15 +5084,14 @@
         </is>
       </c>
       <c r="C8" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A8,Boodschappenlijst!$C$6:$C$24,"altijd")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A8,Boodschappenlijst!$C$6:$C$23,"altijd")</f>
         <v/>
       </c>
       <c r="D8" s="5" t="n">
-        <v>600</v>
-      </c>
-      <c r="E8" s="5">
-        <f>IF(C8&lt;=0,0,IF(C8/1.21&gt;=600,0,60.5))</f>
-        <v/>
+        <v>0</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>0</v>
       </c>
       <c r="F8" s="5">
         <f>C8+E8</f>
@@ -5338,12 +5099,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>1–2 wd / pallet</t>
+          <t>lokaal</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Primer+egaline; drempel €600 excl. btw → deel door 1,21; pallet €60,50 incl</t>
+          <t>Zandcement: prijs is all-in indicatie</t>
         </is>
       </c>
     </row>
@@ -5357,7 +5118,7 @@
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>Boodschappenlijst!N17</f>
+        <f>Boodschappenlijst!N16</f>
         <v/>
       </c>
       <c r="D9" s="5">
@@ -5378,7 +5139,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Volgt Parameters!B8. DE: DHL zone 1 NL €15,41. NL: VerwarmingOnline drempel €385.</t>
+          <t>Actuators; volgt Parameters!B8</t>
         </is>
       </c>
     </row>
@@ -5394,7 +5155,7 @@
         </is>
       </c>
       <c r="C10" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A10,Boodschappenlijst!$C$6:$C$24,"h64")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A10,Boodschappenlijst!$C$6:$C$23,"h64")</f>
         <v/>
       </c>
       <c r="D10" s="5" t="n">
@@ -5414,7 +5175,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Alleen bij H64-pad</t>
+          <t>Alleen bij H64</t>
         </is>
       </c>
     </row>
@@ -5430,7 +5191,7 @@
         </is>
       </c>
       <c r="C11" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A11,Boodschappenlijst!$C$6:$C$24,"tado_bedraad")+SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A11,Boodschappenlijst!$C$6:$C$24,"tado_draadloos")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A11,Boodschappenlijst!$C$6:$C$23,"tado_bedraad")+SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A11,Boodschappenlijst!$C$6:$C$23,"tado_draadloos")</f>
         <v/>
       </c>
       <c r="D11" s="5" t="n">
@@ -5451,7 +5212,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Alleen bij Tado-pad</t>
+          <t>Alleen bij Tado</t>
         </is>
       </c>
     </row>
@@ -5467,7 +5228,7 @@
         </is>
       </c>
       <c r="C12" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A12,Boodschappenlijst!$C$6:$C$24,"altijd")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A12,Boodschappenlijst!$C$6:$C$23,"altijd")</f>
         <v/>
       </c>
       <c r="D12" s="5" t="n">
@@ -5488,7 +5249,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Gratis vanaf €60; 3 rollen Climasol ≈ €72 → meestal gratis</t>
+          <t>Climasol</t>
         </is>
       </c>
     </row>
@@ -5685,22 +5446,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Zakken</t>
+          <t>Noppen sets</t>
         </is>
       </c>
       <c r="B26">
-        <f>Parameters!B12</f>
+        <f>Parameters!B11</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Artikelkosten</t>
+          <t>Artikelkosten noppen</t>
         </is>
       </c>
       <c r="B27" s="5">
-        <f>B26*14.87</f>
+        <f>B26*136.58</f>
         <v/>
       </c>
     </row>
@@ -5718,24 +5479,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Verzending pallet</t>
+          <t>Verzending Elektramat (formule)</t>
         </is>
       </c>
       <c r="B29" s="5">
-        <f>IF(B28&gt;=600,0,60.5)</f>
+        <f>E5</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>All-in egaline</t>
-        </is>
-      </c>
-      <c r="B30" s="5">
-        <f>B27+B29</f>
-        <v/>
-      </c>
+          <t>Let op lengtevracht noppenplaten — check Elektramat bij bestelling</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5799,27 +5557,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Alleen upgrades die kwalitatief beter zijn (≤ 1 week leverbaar)</t>
+          <t>KWALITATIEF BESTE — harde vloer zonder golven (aug 2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Goedkoper alleen als kwaliteit gelijk blijft. Duurder alleen als kwaliteit aantoonbaar beter is.</t>
+          <t>Keuze: nat Magnum 16 mm + noppenplaat 28 mm + zandcement ≥50 mm. SlimFit/egaline bewust verlaten.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>KOPJE: Vloerverwarming — wat is geüpgraded?</t>
+          <t>KOPJE: Vloerverwarming — systeemkeuze</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5594,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Was (goedkoop)</t>
+          <t>Was</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -5848,14 +5606,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>UPGRADES (kwaliteit ↑)</t>
+          <t>SYSTEEM (kern)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>NMC Climasol randisolatie 150×8 mm – rol 25 m</t>
+          <t>MAGNUM noppenplaat 28 mm (150 kPa)</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -5865,19 +5623,19 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>€ 15.62 → € 23.99</t>
+          <t>SlimFit 12 matten</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>NMC is A-merk: vormvaster, betere flap/scheurstroken, betrouwbaarder bij egaline. +€8/rol is de moeite waard.</t>
+          <t>Stijvere basis + buis in noppen; daarna massieve zandcement.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>VTE Composiet 4-groeps mengverdeler + Grundfos UPM3 pomp</t>
+          <t>MAGNUM PE-RT 16×2</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5887,19 +5645,19 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>€ 305.95 → € 387.18</t>
+          <t>PE-RT 12×1,5 SlimFit</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Beter dan VTE SLIM: flowmeters (inregelen), geen corrosie, koelbaar, dubbelwandig. Gelijkwaardig/beter dan Magnum Basic (€406) op features, iets goedkoper.</t>
+          <t>Standaard natte-systeem diameter.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Möhlenhoff Alpha 5 thermische motor 230V NC M30×1,5 (+ adapter)</t>
+          <t>Zandcement ≥50 mm boven buis</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5909,19 +5667,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>€ 14.00 → € 20.12</t>
+          <t>Kreisel 418 egaline ~18 mm</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Möhlenhoff is kwalitatief duidelijk beter dan budget-Lovak (levensduur, lekkagebescherming, certificering). Marginaal duurder dan Magnum, merkbaar betrouwbaarder.</t>
+          <t>Dít maakt de vloer hard. Magnum eist min. 5 cm.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Elektrakabel 230V / signaalkabel (installatiekwaliteit)</t>
+          <t>Krimpnet 100×100</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -5931,369 +5689,83 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>€ 20.00 → € 25.00</t>
+          <t>(niet in SlimFit-BOM)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Gebruik nette installatiekabel + deugdelijke lasdozen; besparen op elektra is valse economie.</t>
+          <t>Scheurbeheersing in cementdekvloer.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>tado° Slimme Thermostaat X Starterskit bedraad + Bridge X</t>
+          <t>NMC Climasol / VTE Composiet / Möhlenhoff / Tado bedraad</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>UPGRADE</t>
+          <t>behouden</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>€ 129.99 → € 129.99</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Bedraad is kwalitatief beter dan 3× draadloos: stabielere voeding/communicatie, minder batterijen, betrouwbaarder bij VV.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>tado° Slimme Thermostaat X bedraad (uitbreiding)</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>UPGRADE</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>€ 100.00 → € 100.00</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>Onderdeel van bedrade (betere) Tado-setup.</t>
+          <t>Al kwaliteitskeuzes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Bewust niet gekozen</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BEHOUDEN (goedkoop genoeg / systeemecht / al optimaal)</t>
+          <t>• SlimFit + egaline: laagste opbouw, meer kans op “golven”.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>MAGNUM SlimFit 12 bevestigingsmat 3,75 m²</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>€ 86.94</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Geen beter alternatief: SlimFit is systeemecht; generieke matten passen niet betrouwbaar op Magnum 12 mm-buis.</t>
+          <t>• Noppenplaat 47 mm akoestisch: lagere max. belasting → zachter.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MAGNUM PE-RT buis 12×1,5 mm KOMO – rol 300 m</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>€ 142.93</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Blijf bij Magnum PE-RT: ontworpen voor SlimFit. Generieke 12 mm is niet automatisch beter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>MAGNUM Euroconus 12×1,5 mm × ¾″ (set van 2)</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>€ 4.69</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Systeemecht; past gegarandeerd op Magnum-buis + Euroconus-verdeler.</t>
+          <t>• Droogbouw/Heatboard: niet dezelfde massieve cementvloer-hardheid.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>MAGNUM 90° bochtondersteuning ø10–12 mm (set van 2)</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>€ 1.18</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Voldoende kwaliteit; duurdere merken bieden hier geen merkbare meerwaarde.</t>
+          <t>Absoluut hardst (als bestaande dekvloer geschikt is)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>MAGNUM Contactlijm 500 ml</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>€ 9.05</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Speciaal voor Magnum-verlegsystemen; generieke spuitlijm is niet beter.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Kreisel Gruntolit-W 301 voorstrijk 5 L</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>€ 9.29</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Houd primer bij dezelfde fabrikant als egaline (systeemcompatibiliteit).</t>
+          <t>INFREZEN in bestaande zandcement/anhydriet — laat beoordelen door freesbedrijf.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Kreisel 418 vezelversterkte egaline 25 kg</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>€ 14.87</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>Kreisel 418 is hier beter dan Uzin NC 170: tot 50 mm in 1 laag + vezels tegen thermische spanning. NC 170 is premium dun (0–15 mm) maar minder geschikt voor dikke SlimFit-dekking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Aanvoer + retourleiding (meerlagenbuis 16×2)</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>€ 6.50</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Kwaliteit zit in merk-meerlagenbuis; lengte is situatiespecifiek.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Kogelkranen / koppelingen set</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>€ 34.95</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Functioneel voldoende; premium messing-sets zijn niet merkbaar beter voor dit gebruik.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>MAGNUM H64-CC + master WiFi-thermostaat</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>€ 213.74</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Binnen H64-lijn is dit het juiste product; geen beter Magnum-alternatief.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>MAGNUM H64-ST slave thermostaat</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>€ 52.92</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Passend bij H64-CC; geen kwaliteitswinst bij andere slave.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>tado° Draadloze Slimme Thermostaat X Starterskit</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>€ 129.00</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>Prima, maar bedraad is kwalitatief stabieler (zie nr 17–18).</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>Niet gedaan (bewust)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>• Geen Uzin NC 170 i.p.v. Kreisel 418: NC 170 is premium dun-egaline; Kreisel 418 (vezels, tot 50 mm) past beter op SlimFit.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>• Geen generieke 12 mm-buis i.p.v. Magnum: systeemcompatibiliteit SlimFit &gt; kleine prijswinst.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>Prijszoek top-5 (aug 2026)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>Möhlenhoff → eibhandel.de €9,99 (+NL verzending). H64-CC → Warp €194,92. Overige top-5: geen betere shop binnen ≤1 week.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>m² is nu stuurvariabele op Parameters — hoeveelheden schalen automatisch.</t>
+          <t>Opbouw (indicatief): noppen 28 + buis 16 + ≥50 mm cement ≈ 70–90 mm. Check deurdorpels.</t>
         </is>
       </c>
     </row>
@@ -6308,20 +5780,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Prijszoek – 5 duurste items (alleen goedkoper + ≤1 week leverbaar)</t>
+          <t>Prijszoek – duurste items kwalitatief-beste BOM (aug 2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Gezocht NL + DE webshops, 22 aug 2026. Alleen gewijzigd als aantoonbaar goedkoper én binnen levertijd.</t>
+          <t>Focus: noppen/buis/verdeler/dekvloer.</t>
         </is>
       </c>
     </row>
@@ -6333,17 +5805,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Item (regeltotaal)</t>
+          <t>Item</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Was</t>
+          <t>Gekozen</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Beste gevonden</t>
+          <t>Alternatief</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -6353,241 +5825,164 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Besparing</t>
+          <t>Δ</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="A5" t="n">
+        <v>1</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MAGNUM SlimFit 12 matten (8×)</t>
+          <t>Noppenplaat 28 mm 3×10 m²</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Elektramat €86,94/st (€695,52)</t>
+          <t>Elektramat €136,58/set</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Bouwmaat €86,50 (geen voorraad/bezorging); VihamiJ €86,36 excl=duurder + 3–4 wkn; overige ≥€88,99</t>
+          <t>17 mm ongeïsoleerd €102,55 (alleen als al geïsoleerd)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BEHOUDEN Elektramat</t>
+          <t>BEHOUDEN 28 mm</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>kwaliteit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>PE-RT 16×2 240 m</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Elektramat €158,99</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2×120 m ≈ gelijk</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>€0</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Kreisel 418 egaline (33×)</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>EgalineXXL €14,87/st (€490,71)</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>RBMB ≥€16,55/st (bulkpas pas vanaf 41); geen goedkopere met snelle levering</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>BEHOUDEN EgalineXXL</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Zandcement 30 m²</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Indicatie €35/m² = €1.050</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Lokaal €25–55/m²</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>OFFERTE</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>variabel</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>VTE Composiet 4-gr.</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>123shop €387,18</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>andere shops hoger</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>€0</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>VTE Composiet 4-groeps + Grundfos</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>123Installatieshop €387,18</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>CVTotaal €423; VV-shop €404,95; Bouwbestel €440; Jan de Isolatieman €469</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>BEHOUDEN 123Installatieshop</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>€0</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>MAGNUM PE-RT 12×1,5 300 m</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>123InstallatieMaterialen €142,93</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Klusspullen €141,95 maar voorraad 0 / levertijd 1–2 wkn → afgewezen; Elektramat €181,86; VV-shop €164,70</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>BEHOUDEN 123IM</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>€0</t>
-        </is>
-      </c>
-    </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>5a</t>
-        </is>
+      <c r="A9" t="n">
+        <v>5</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Möhlenhoff Alpha 5 ×4 (altijd)</t>
+          <t>Möhlenhoff ×4</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>VerwarmingOnline €20,12 → €80,48</t>
+          <t>eibhandel + ship ~€55</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>eibhandel.de €9,99 + NL-verzending ~€15,41 = ~€55,37; Amazon.nl ~€13,16/st met Prime</t>
+          <t>VerwarmingOnline duurder</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>GEWIJZIGD → eibhandel</t>
+          <t>BEHOUDEN</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>~€25</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>5b</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>MAGNUM H64-CC + master (optie)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>123IM €213,74</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Warp Systems €194,92 (1 wd)</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>GEWIJZIGD → Warp</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>~€19</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Niet meegenomen</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>• PioTek DE (~€9,90): verzendt niet meer naar NL.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>• Bouwmaat SlimFit €86,50: tijdelijk niet beschikbaar / geen bezorging.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>• Klusspullen PE-RT €141,95: goedkoper op papier, maar 0 voorraad / 1–2 weken.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>• Tado: officiële tado° Shop blijft goedkoopst (bol/retail vaak duurder).</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>All-in met verzending: zie sheet Verzending (egaline pallet + eibhandel DE→NL).</t>
+          <t>beste</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>• SlimFit-pad bewust verlaten. Infrezen: apart offerte freesbedrijf.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fit SlimFit BOM to concrete subfloor and 30 mm max height
Revert wet 16 mm/sand-cement (too tall). Restore Magnum SlimFit 12
with fiber egaline at 22 mm (max 30 mm) on concrete, with height checks
and quality notes for a hard finish within the build-up limit.

Co-authored-by: bmverhagen <bmverhagen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Materiaalbenodigdheden_Vloerverwarming.xlsx
+++ b/Materiaalbenodigdheden_Vloerverwarming.xlsx
@@ -94,7 +94,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -131,11 +131,6 @@
         <fgColor rgb="00FDEBD0"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -163,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -194,7 +189,6 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -572,7 +566,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Vloerverwarming — KWALITATIEF BESTE (nat 16 mm). Speel met m² op Parameters</t>
+          <t>Vloerverwarming — SlimFit 12 op BETON (max 30 mm). Speel met m² op Parameters</t>
         </is>
       </c>
     </row>
@@ -729,42 +723,42 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>1. Parameters → gele cel Oppervlakte (m²) + dekvloer-mm (≥50).</t>
+          <t>1. Parameters: m², groepen, ruimten, opbouwhoogte (17–22 mm Magnum; max 30).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2. Pas Groepen/Ruimten aan (verdeler-SKU is 4-groeps!).</t>
+          <t>2. Ondergrond = beton (vast). Nat 16 mm past NIET in 3 cm.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>3. Boodschappenlijst = Magnum noppen 28 mm + PE-RT 16 + zandcement (niet SlimFit).</t>
+          <t>3. Boodschappenlijst = SlimFit + PE-RT 12 + Kreisel vezel-egaline.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>4. Zandcement: lokale offerte; Excel toont indicatie €35/m².</t>
+          <t>4. Check Verzending + hoogte-check Parameters!B21.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Nog beter als er al een stevige dekvloer is: INFREZEN i.p.v. opbouw — vraag een freesbedrijf. Anders is dit nat systeem het hardst.</t>
+          <t>Hardheid: beton helpt sterk. Vul egaline tot 22 mm (desnoods tot 28–30 mm). Tegels als afwerking = stevigst.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NL-leverzekerheid: sheet NL-leverbaarheid. Actuators: Parameters!B8.</t>
+          <t>Infrezen in beton: alleen als constructie/dikte het toelaat (vaak niet in constructief beton) — laat beoordelen. Anders: deze SlimFit-BOM.</t>
         </is>
       </c>
     </row>
@@ -1417,8 +1411,31 @@
       </c>
     </row>
     <row r="22">
-      <c r="D22" s="5" t="n"/>
-      <c r="E22" s="5" t="n"/>
+      <c r="A22">
+        <f>Boodschappenlijst!E24</f>
+        <v/>
+      </c>
+      <c r="B22">
+        <f>Boodschappenlijst!I24</f>
+        <v/>
+      </c>
+      <c r="C22">
+        <f>Boodschappenlijst!P24</f>
+        <v/>
+      </c>
+      <c r="D22" s="5">
+        <f>Boodschappenlijst!K24</f>
+        <v/>
+      </c>
+      <c r="E22" s="5">
+        <f>Boodschappenlijst!N24</f>
+        <v/>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1445,7 +1462,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>NL-leverbaarheid — kwalitatief beste BOM</t>
+          <t>NL-leverbaarheid — SlimFit op beton ≤30 mm</t>
         </is>
       </c>
     </row>
@@ -1967,6 +1984,32 @@
         <v/>
       </c>
     </row>
+    <row r="25">
+      <c r="A25">
+        <f>Boodschappenlijst!E24</f>
+        <v/>
+      </c>
+      <c r="B25">
+        <f>Boodschappenlijst!R24</f>
+        <v/>
+      </c>
+      <c r="C25">
+        <f>Boodschappenlijst!P24</f>
+        <v/>
+      </c>
+      <c r="D25">
+        <f>Boodschappenlijst!O24</f>
+        <v/>
+      </c>
+      <c r="E25">
+        <f>IF(OR(Boodschappenlijst!R24="NL",Boodschappenlijst!R24=""),"n.v.t. (NL)",IF(ISNUMBER(SEARCH("DE",Boodschappenlijst!R24&amp;"")),"JA — zie Verzending","check"))</f>
+        <v/>
+      </c>
+      <c r="F25">
+        <f>Boodschappenlijst!U24</f>
+        <v/>
+      </c>
+    </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
@@ -1977,28 +2020,28 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• Bijna alles NL-webshops (Elektramat, 123shop, Installand, Overkamp, Warp, tado°).</t>
+          <t>• SlimFit-BOM: NL-webshops + optioneel eibhandel DE→NL voor actuators.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>• Zandcement = lokale vloerzetter (indicatief in lijst).</t>
+          <t>• Hoogte: Parameters B7≤B10 (30 mm). Nat systeem verwijderd.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>• 1 regel mogelijk buitenland: Möhlenhoff via eibhandel.de (Parameters!B8).</t>
+          <t>• Ondergrond beton: primer verplicht (Kreisel in lijst).</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>• Noppenplaten: lengtevracht — plan bezorging/afhaal met Elektramat.</t>
+          <t>• Actuators: Parameters!B8 DE→NL of NL zeker.</t>
         </is>
       </c>
     </row>
@@ -2025,14 +2068,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>STUURVARIABELEN — pas gele cellen aan; rest schaalt automatisch</t>
+          <t>STUURVARIABELEN — beton + max. 30 mm opbouw; gele cellen aanpassen</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>PROJECT</t>
+          <t>PROJECT / RANDVOORWAARDEN</t>
         </is>
       </c>
     </row>
@@ -2052,7 +2095,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>← KEY: verander dit getal</t>
+          <t>← KEY</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2115,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Bepaalt verdeler/actuators/koppelingen (max ~100 m buis/groep)</t>
+          <t>max ~100 m buis/groep</t>
         </is>
       </c>
     </row>
@@ -2092,18 +2135,18 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bepaalt Tado/H64 thermostaten</t>
+          <t>Tado/H64</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Dekvloer boven buis</t>
+          <t>Totale opbouw VV+egaline</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>50</v>
+        <v>22</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -2112,7 +2155,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Magnum min. 50 mm zandcement boven buis (harde, niet-golvende vloer)</t>
+          <t>Magnum SlimFit 12: 17–22 mm. Jouw max = 30 mm. Hoger (tot 28–30) = meer dekking = harder.</t>
         </is>
       </c>
     </row>
@@ -2134,192 +2177,224 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Of: "NL zeker (VerwarmingOnline)" — duurder, 100% NL-webshop</t>
+          <t>Of: "NL zeker (VerwarmingOnline)"</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>AFGELEIDE WAARDEN (auto)</t>
+          <t>Ondergrond</t>
+        </is>
+      </c>
+      <c r="B9" s="25" t="inlineStr">
+        <is>
+          <t>Beton</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>vast</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Goed: stijve basis → minder kans op golven dan hout</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Buislengte (indicatie)</t>
-        </is>
-      </c>
-      <c r="B10">
-        <f>ROUND(B4*8,0)</f>
-        <v/>
+          <t>Max. beschikbare hoogte</t>
+        </is>
+      </c>
+      <c r="B10" s="25" t="n">
+        <v>30</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>mm</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>vuistregel 8 m/m² ≈ hart-op-hart 12,5 cm (kwaliteit nat 16 mm)</t>
+          <t>Harde limiet; nat 16 mm + zandcement past NIET</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Noppenplaat sets 10 m²</t>
+          <t>SlimFit pakken</t>
         </is>
       </c>
       <c r="B11">
-        <f>CEILING(B4/10,1)</f>
+        <f>CEILING(B4/3.75,1)</f>
         <v/>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>set à 10 m²</t>
+          <t>pak à 3,75 m²</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Krimpnetten 2,52 m²</t>
+          <t>AFGELEIDE WAARDEN (auto)</t>
         </is>
       </c>
       <c r="B12">
-        <f>CEILING(B4/2.52,1)</f>
+        <f>CEILING(B4*1.5*B7/25,1)</f>
         <v/>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>mat 120×210</t>
+          <t>zak à 25 kg</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PE-RT rollen 240 m</t>
+          <t>Buislengte (indicatie)</t>
         </is>
       </c>
       <c r="B13">
-        <f>MAX(1,CEILING(B10/240,1))</f>
+        <f>ROUND(B4*10,0)</f>
         <v/>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>rol</t>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>≈10 m/m² SlimFit 12 (h.o.h. 12,5 cm)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Euroconus sets</t>
+          <t>SlimFit pakken</t>
         </is>
       </c>
       <c r="B14">
-        <f>B5</f>
+        <f>CEILING(B4/3.75,1)</f>
         <v/>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>set (2 st)</t>
+          <t>pak à 3,75 m²</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Randisolatie rollen</t>
+          <t>Egaline zakken</t>
         </is>
       </c>
       <c r="B15">
-        <f>MAX(2,CEILING(B4/10,1))</f>
+        <f>CEILING(B4*1.5*B7/25,1)</f>
         <v/>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>rol à 25 m</t>
+          <t>zak à 25 kg</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>1,5 kg/m²/mm × totale opbouwhoogte B7</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Geleidingsbochten</t>
+          <t>PE-RT rollen 300 m</t>
         </is>
       </c>
       <c r="B16">
-        <f>B5*2</f>
+        <f>MAX(1,CEILING(B13/300,1))</f>
         <v/>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>st (aanvoer+retour/groep)</t>
+          <t>rol</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Tado/H64 slaves</t>
+          <t>Contactlijm bussen</t>
         </is>
       </c>
       <c r="B17">
-        <f>MAX(0,B6-1)</f>
+        <f>MAX(1,CEILING(B4*0.2,1))</f>
         <v/>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>bus</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Zandcement m²</t>
+          <t>Randisolatie rollen</t>
         </is>
       </c>
       <c r="B18">
-        <f>B4</f>
+        <f>MAX(2,CEILING(B4/10,1))</f>
         <v/>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>Indicatie vloerzetter; vraag lokale offerte</t>
+          <t>rol à 25 m</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>VERZENDREGELS (NL, all-in — gecorrigeerd)</t>
+          <t>Primer bussen 5 L</t>
+        </is>
+      </c>
+      <c r="B19">
+        <f>MAX(1,CEILING(B4*2/30,1))</f>
+        <v/>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>bus</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Beton: altijd primer</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="19" t="inlineStr">
         <is>
-          <t>Shop</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="inlineStr">
-        <is>
-          <t>Gratis vanaf</t>
-        </is>
+          <t>Tado/H64 slaves</t>
+        </is>
+      </c>
+      <c r="B20" s="19">
+        <f>MAX(0,B6-1)</f>
+        <v/>
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>Kosten onder drempel</t>
+          <t>st</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
@@ -2331,22 +2406,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Elektramat</t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>€150 excl. btw</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>€4,09 excl ≈ €4,95 incl</t>
-        </is>
-      </c>
+          <t>Hoogte-check</t>
+        </is>
+      </c>
+      <c r="B21" s="5">
+        <f>IF(B7&lt;=B10,"OK ≤ max","TE HOOG t.o.v. max")</f>
+        <v/>
+      </c>
+      <c r="C21" s="5" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NL · 1 wd · PostNL</t>
+          <t>B7 mag niet boven B10</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2445,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>123Installatieshop</t>
+          <t>VERZENDREGELS (NL, all-in)</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
@@ -2397,73 +2467,73 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>EgalineXXL / RBMB</t>
+          <t>Shop</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>€600 excl. btw</t>
+          <t>Gratis vanaf</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>pallet ≈ €60,50 incl</t>
+          <t>Kosten onder drempel</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>NL · 1–2 wd / palletplanning</t>
+          <t>Levertijd / land</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>eibhandel.de</t>
+          <t>Elektramat</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>€1000</t>
+          <t>€150 excl. btw</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>€12,95 excl ≈ €15,41 incl</t>
+          <t>≈ €4,95 incl</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>DE→NL DHL zone 1 · 2–5 wd DE (+NL)</t>
+          <t>NL · 1 wd</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Warp Systems</t>
+          <t>123InstallatieMaterialen</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>n.v.t. / laag</t>
+          <t>€200</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>€0 (typisch)</t>
+          <t>€6,95</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>NL · 1 wd (voor 12:00)</t>
+          <t>NL · morgen</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>tado° Shop</t>
+          <t>123Installatieshop</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
@@ -2473,92 +2543,144 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>€4,99</t>
+          <t>€6,95</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>NL/EU · 2–4 wd</t>
+          <t>NL · ≤1 week</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Installand</t>
+          <t>EgalineXXL / RBMB</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>€60</t>
+          <t>€600 excl. btw</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>var. / afhalen gratis</t>
+          <t>pallet ≈ €60,50</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NL · vaak volgende wd</t>
+          <t>NL · pallet</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>VerwarmingOnline</t>
+          <t>eibhandel.de</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>€385</t>
+          <t>€1000</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>~€6,95</t>
+          <t>≈ €15,41 incl</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NL · 3–4 wd</t>
+          <t>DE→NL DHL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Home Perfect (.nl/.de)</t>
+          <t>Warp Systems</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>€1000 pakket</t>
+          <t>n.v.t.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>€29,90–€69 NL-pakket</t>
+          <t>€0</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>DE-basis · 7–10 wd → te duur/traag all-in</t>
+          <t>NL · 1 wd</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>tado° Shop</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>€150</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>€4,99</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>NL/EU 2–4 wd</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="20" t="inlineStr">
         <is>
-          <t>Conclusie all-in (aug 2026): huidige shops blijven goedkoopst; zie sheet All-in-check. Geen shopwissel nodig.</t>
+          <t>Installand</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>€60</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>~€6,95</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>NL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Buitenland alleen eibhandel.de (actuators): NL-levering bevestigd, verzending + levertijd meegenomen.</t>
+          <t>VerwarmingOnline</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>€385</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>~€6,95</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>NL 3–4 wd</t>
         </is>
       </c>
     </row>
@@ -2606,7 +2728,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U24"/>
+  <dimension ref="A1:U26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2635,21 +2757,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Boodschappenlijst — KWALITATIEF BESTE (nat 16 mm + noppen + zandcement). Hoeveelheden schalen met Parameters!B4</t>
+          <t>Boodschappenlijst — SlimFit 12 op BETON, max 30 mm. Hoeveelheden schalen met Parameters!B4</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Doel: harde vloer zonder golven. SlimFit/egaline vervangen. Gele stuurcellen op Parameters. Verzending op sheet Verzending.</t>
+          <t>Nat 16 mm/zandcement past niet (te hoog). Beton = stijve basis → SlimFit + vezel-egaline tot 22–30 mm is hier de kwalitatief beste haalbare optie.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>KOPJE: Vloerverwarming — kwalitatief beste</t>
+          <t>KOPJE: Vloerverwarming</t>
         </is>
       </c>
     </row>
@@ -2776,47 +2898,47 @@
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>Noppenplaat</t>
+          <t>Bevestiging</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>MAGNUM noppenplaat geïsoleerd 28 mm (11 mm EPS) – set 10 m²</t>
+          <t>MAGNUM SlimFit 12 bevestigingsmat 3,75 m²</t>
         </is>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>W90117</t>
+          <t>W61012</t>
         </is>
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t>PS-noppen + 11 mm EPS, max. belasting 150 kPa, Rd 0,31. Voor 16/17 mm buis.</t>
+          <t>Kunststof klikmatten 5×75×100 cm = 3,75 m², opbouw ~14 mm.</t>
         </is>
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t>Buizen vastklikken + lichte isolatie; stijve basis i.p.v. SlimFit.</t>
-        </is>
-      </c>
-      <c r="I6" s="30">
-        <f>Parameters!$B$11</f>
+          <t>Basislaag voor buizen.</t>
+        </is>
+      </c>
+      <c r="I6" s="14">
+        <f>CEILING(Parameters!$B$4/3.75,1)</f>
         <v/>
       </c>
       <c r="J6" s="13" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>pak</t>
         </is>
       </c>
       <c r="K6" s="15" t="n">
-        <v>136.58</v>
+        <v>86.94</v>
       </c>
       <c r="L6" s="15" t="n">
-        <v>102.55</v>
+        <v>86.94</v>
       </c>
       <c r="M6" s="13" t="inlineStr">
         <is>
-          <t>upgrade</t>
+          <t>behouden</t>
         </is>
       </c>
       <c r="N6" s="15">
@@ -2825,7 +2947,7 @@
       </c>
       <c r="O6" s="13" t="inlineStr">
         <is>
-          <t>NL · 1 werkdag (lengtevracht)</t>
+          <t>NL · 1 werkdag (op voorraad)</t>
         </is>
       </c>
       <c r="P6" s="13" t="inlineStr">
@@ -2835,7 +2957,7 @@
       </c>
       <c r="Q6" s="13" t="inlineStr">
         <is>
-          <t>https://www.elektramat.nl/magnum-noppenplaat-geisoleerd-28mm-11mm-eps-10x1000x1000mm-set-van-10m2-w90117/</t>
+          <t>https://www.elektramat.nl/magnum-slimfit-12-bevestigingsmat-vloerverwarming-3-75-m2-5-stuks-van-75x100cm-w61012/</t>
         </is>
       </c>
       <c r="R6" s="13" t="inlineStr">
@@ -2848,7 +2970,7 @@
       </c>
       <c r="T6" s="13" t="inlineStr">
         <is>
-          <t>28 mm i.p.v. 47 mm: veel hogere belasting (150 kPa) → hardere vloer. Schaalt met m².</t>
+          <t>Schaalt met m². Op beton + vezel-egaline tot ≤30 mm = hardst haalbaar binnen hoogte.</t>
         </is>
       </c>
       <c r="U6" s="28" t="inlineStr">
@@ -2878,26 +3000,26 @@
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>MAGNUM PE-RT buis 16×2 mm KOMO – rol 240 m</t>
+          <t>MAGNUM PE-RT buis 12×1,5 mm KOMO – rol 300 m</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>W16240</t>
+          <t>W12300</t>
         </is>
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>5-laags PE-RT ø16 mm, KOMO/EVOH, tot 80 °C.</t>
+          <t>5-laags PE-RT ø12 mm, KOMO/EVOH.</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t>Verwarmingscircuits (nat systeem).</t>
-        </is>
-      </c>
-      <c r="I7" s="30">
-        <f>Parameters!$B$13</f>
+          <t>Verwarmingscircuits.</t>
+        </is>
+      </c>
+      <c r="I7" s="14">
+        <f>MAX(1,CEILING(Parameters!$B$13/300,1))</f>
         <v/>
       </c>
       <c r="J7" s="13" t="inlineStr">
@@ -2906,14 +3028,14 @@
         </is>
       </c>
       <c r="K7" s="15" t="n">
-        <v>158.99</v>
+        <v>142.93</v>
       </c>
       <c r="L7" s="15" t="n">
-        <v>158.99</v>
+        <v>142.93</v>
       </c>
       <c r="M7" s="13" t="inlineStr">
         <is>
-          <t>upgrade</t>
+          <t>behouden</t>
         </is>
       </c>
       <c r="N7" s="15">
@@ -2922,17 +3044,17 @@
       </c>
       <c r="O7" s="13" t="inlineStr">
         <is>
-          <t>NL · 1 werkdag</t>
+          <t>NL · morgen in huis (vóór 14:30)</t>
         </is>
       </c>
       <c r="P7" s="13" t="inlineStr">
         <is>
-          <t>Elektramat</t>
+          <t>123InstallatieMaterialen</t>
         </is>
       </c>
       <c r="Q7" s="13" t="inlineStr">
         <is>
-          <t>https://www.elektramat.nl/magnum-universele-vloerverwarmingsbuis-5-laags-pe-rt-16x2-mm-komo-rol-240-meter-w16240/</t>
+          <t>https://123installatiematerialen.nl/magnum-tube-vloerverwarmingsbuis-pe-rt-12-x-15-300-meter/</t>
         </is>
       </c>
       <c r="R7" s="13" t="inlineStr">
@@ -2941,11 +3063,11 @@
         </is>
       </c>
       <c r="S7" s="15" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="T7" s="13" t="inlineStr">
         <is>
-          <t>16 mm standaard voor nat/zandcement. Bij 30 m² ≈ 240 m (8 m/m²). Bundel met noppen bij Elektramat.</t>
+          <t>All-in: +€6,95 verzending (order &lt;€200 bij 123IM). Nog steeds goedkoper dan Elektramat €181,86.</t>
         </is>
       </c>
       <c r="U7" s="28" t="inlineStr">
@@ -2975,12 +3097,12 @@
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>MAGNUM Euroconus 16×2 mm × ¾″ (set van 2)</t>
+          <t>MAGNUM Euroconus 12×1,5 mm × ¾″ (set van 2)</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>W90016</t>
+          <t>W90012</t>
         </is>
       </c>
       <c r="G8" s="13" t="inlineStr">
@@ -2990,10 +3112,10 @@
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t>1 set per groep op verdeler.</t>
-        </is>
-      </c>
-      <c r="I8" s="30">
+          <t>1 set per groep.</t>
+        </is>
+      </c>
+      <c r="I8" s="14">
         <f>Parameters!$B$5</f>
         <v/>
       </c>
@@ -3010,7 +3132,7 @@
       </c>
       <c r="M8" s="13" t="inlineStr">
         <is>
-          <t>upgrade</t>
+          <t>behouden</t>
         </is>
       </c>
       <c r="N8" s="15">
@@ -3029,7 +3151,7 @@
       </c>
       <c r="Q8" s="13" t="inlineStr">
         <is>
-          <t>https://www.elektramat.nl/magnum-adaptor-euroconus-aansluitkoppeling-16x2mm-x-3-4-2-stuks-w90016/</t>
+          <t>https://www.elektramat.nl/magnum-adaptor-euroconus-aansluitkoppeling-12x1-5mm-x-3-4-2-stuks-w90012/</t>
         </is>
       </c>
       <c r="R8" s="13" t="inlineStr">
@@ -3038,11 +3160,11 @@
         </is>
       </c>
       <c r="S8" s="15" t="n">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="T8" s="13" t="inlineStr">
         <is>
-          <t>Schaalt met aantal groepen. Systeemecht Magnum 16 mm.</t>
+          <t>Schaalt met aantal groepen.</t>
         </is>
       </c>
       <c r="U8" s="28" t="inlineStr">
@@ -3072,38 +3194,38 @@
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>Henco geleidingsbocht ø12–18 mm</t>
+          <t>MAGNUM 90° bochtondersteuning ø10–12 mm (set van 2)</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>UFH-BEND1218</t>
+          <t>W90125</t>
         </is>
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>Kunststof opgangbocht onder verdeler.</t>
+          <t>Ondersteunt bocht bij opgang.</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t>Opgang verdeler→vloer (aanvoer+retour).</t>
-        </is>
-      </c>
-      <c r="I9" s="30">
-        <f>Parameters!$B$16</f>
+          <t>Opgang verdeler→vloer.</t>
+        </is>
+      </c>
+      <c r="I9" s="14">
+        <f>Parameters!$B$5</f>
         <v/>
       </c>
       <c r="J9" s="13" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>set</t>
         </is>
       </c>
       <c r="K9" s="15" t="n">
-        <v>1.45</v>
+        <v>1.18</v>
       </c>
       <c r="L9" s="15" t="n">
-        <v>1.45</v>
+        <v>1.18</v>
       </c>
       <c r="M9" s="13" t="inlineStr">
         <is>
@@ -3116,17 +3238,17 @@
       </c>
       <c r="O9" s="13" t="inlineStr">
         <is>
-          <t>NL · 1 werkdag</t>
+          <t>NL · morgen in huis (vóór 14:30)</t>
         </is>
       </c>
       <c r="P9" s="13" t="inlineStr">
         <is>
-          <t>Elektramat</t>
+          <t>123InstallatieMaterialen</t>
         </is>
       </c>
       <c r="Q9" s="13" t="inlineStr">
         <is>
-          <t>https://www.elektramat.nl/henco-geleidingsbocht-voor-buis-o12-18mm-ufh-bend1218/</t>
+          <t>https://123installatiematerialen.nl/90-bochtondersteuning-buismaat-o-10-12mm-2-stuks/</t>
         </is>
       </c>
       <c r="R9" s="13" t="inlineStr">
@@ -3135,11 +3257,11 @@
         </is>
       </c>
       <c r="S9" s="15" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="T9" s="13" t="inlineStr">
         <is>
-          <t>2 stuks per groep. Zelfde Elektramat-order als buis/noppen.</t>
+          <t>Schaalt met aantal groepen.</t>
         </is>
       </c>
       <c r="U9" s="28" t="inlineStr">
@@ -3164,47 +3286,47 @@
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>Rand</t>
+          <t>Lijm</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>NMC Climasol randisolatie 150×8 mm – rol 25 m</t>
+          <t>MAGNUM Contactlijm 500 ml</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>CLIMASOL</t>
+          <t>W61027</t>
         </is>
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t>Zelfklevend, met flap.</t>
+          <t>Spuitlijm voor Magnum verlegsystemen.</t>
         </is>
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t>Rondom muren; voorkomt scheuren in dekvloer.</t>
-        </is>
-      </c>
-      <c r="I10" s="30">
-        <f>Parameters!$B$15</f>
+          <t>Matten vastzetten.</t>
+        </is>
+      </c>
+      <c r="I10" s="14">
+        <f>MAX(1,CEILING(Parameters!$B$4*0.2,1))</f>
         <v/>
       </c>
       <c r="J10" s="13" t="inlineStr">
         <is>
-          <t>rol</t>
+          <t>bus</t>
         </is>
       </c>
       <c r="K10" s="15" t="n">
-        <v>23.99</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="L10" s="15" t="n">
-        <v>15.62</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="M10" s="13" t="inlineStr">
         <is>
-          <t>upgrade</t>
+          <t>behouden</t>
         </is>
       </c>
       <c r="N10" s="15">
@@ -3213,17 +3335,17 @@
       </c>
       <c r="O10" s="13" t="inlineStr">
         <is>
-          <t>NL · vaak volgende werkdag</t>
+          <t>NL · 1 werkdag</t>
         </is>
       </c>
       <c r="P10" s="13" t="inlineStr">
         <is>
-          <t>Installand</t>
+          <t>Elektramat</t>
         </is>
       </c>
       <c r="Q10" s="13" t="inlineStr">
         <is>
-          <t>https://www.installand.nl/gena-climasol-randisolatie-zelfklevend-150-x-8-mm-rol-25-m</t>
+          <t>https://www.elektramat.nl/magnum-contactlijm-voor-verlijmen-magnum-verlegsystemen-w61027/</t>
         </is>
       </c>
       <c r="R10" s="13" t="inlineStr">
@@ -3232,11 +3354,11 @@
         </is>
       </c>
       <c r="S10" s="15" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="T10" s="13" t="inlineStr">
         <is>
-          <t>Kwaliteitsupgrade; essentieel bij zandcement.</t>
+          <t>~0,2 bus/m².</t>
         </is>
       </c>
       <c r="U10" s="28" t="inlineStr">
@@ -3261,43 +3383,43 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Wapening</t>
+          <t>Rand</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Krimpnet verzinkt ø3 mm maas 100×100 – 120×210 cm</t>
+          <t>NMC Climasol randisolatie 150×8 mm – rol 25 m</t>
         </is>
       </c>
       <c r="F11" s="13" t="inlineStr">
         <is>
-          <t>KN-3100</t>
+          <t>CLIMASOL</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>≈2,52 m²/mat; wapening/krimpbeheersing in dekvloer.</t>
+          <t>Zelfklevend, met flap.</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>In/op zandcement boven buizen tegen scheuren.</t>
-        </is>
-      </c>
-      <c r="I11" s="30">
-        <f>Parameters!$B$12</f>
+          <t>Rondom muren; voorkomt scheuren.</t>
+        </is>
+      </c>
+      <c r="I11" s="14">
+        <f>MAX(2,CEILING(Parameters!$B$4/10,1))</f>
         <v/>
       </c>
       <c r="J11" s="13" t="inlineStr">
         <is>
-          <t>mat</t>
+          <t>rol</t>
         </is>
       </c>
       <c r="K11" s="15" t="n">
-        <v>9.789999999999999</v>
+        <v>23.99</v>
       </c>
       <c r="L11" s="15" t="n">
-        <v>5.66</v>
+        <v>15.62</v>
       </c>
       <c r="M11" s="13" t="inlineStr">
         <is>
@@ -3310,17 +3432,17 @@
       </c>
       <c r="O11" s="13" t="inlineStr">
         <is>
-          <t>NL · ≤ 1 week</t>
+          <t>NL · vaak volgende werkdag (vóór 16:30/17:00)</t>
         </is>
       </c>
       <c r="P11" s="13" t="inlineStr">
         <is>
-          <t>Overkamp Meddo</t>
+          <t>Installand</t>
         </is>
       </c>
       <c r="Q11" s="13" t="inlineStr">
         <is>
-          <t>https://overkampmeddo.nl/a/bouwstaalmat-3-100-mm-2100-1200-mm-verzinkt-krimpnet</t>
+          <t>https://www.installand.nl/gena-climasol-randisolatie-zelfklevend-150-x-8-mm-rol-25-m</t>
         </is>
       </c>
       <c r="R11" s="13" t="inlineStr">
@@ -3333,7 +3455,7 @@
       </c>
       <c r="T11" s="13" t="inlineStr">
         <is>
-          <t>Kwaliteit: 100×100 i.p.v. grovere maas. Overlap ≥1 maas.</t>
+          <t>Kwaliteitsupgrade; schaalt grof met m².</t>
         </is>
       </c>
       <c r="U11" s="28" t="inlineStr">
@@ -3358,47 +3480,47 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Dekvloer</t>
+          <t>Primer</t>
         </is>
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>Zandcement dekvloer ≥50 mm boven buis (vloerzetter, indicatief)</t>
+          <t>Kreisel Gruntolit-W 301 voorstrijk 5 L</t>
         </is>
       </c>
       <c r="F12" s="13" t="inlineStr">
         <is>
-          <t>ZC-50</t>
+          <t>301</t>
         </is>
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t>Traditionele cementdekvloer; Magnum eist min. 50 mm boven buis.</t>
+          <t>Voorstrijk op BETON vóór egaline (Kreisel-systeem).</t>
         </is>
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>Harde, massieve loopvloer — geen golven.</t>
-        </is>
-      </c>
-      <c r="I12" s="30">
-        <f>Parameters!$B$18</f>
+          <t>Onder egaline.</t>
+        </is>
+      </c>
+      <c r="I12" s="14">
+        <f>MAX(1,CEILING(Parameters!$B$4*2/30,1))</f>
         <v/>
       </c>
       <c r="J12" s="13" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>bus 5L</t>
         </is>
       </c>
       <c r="K12" s="15" t="n">
-        <v>35</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="L12" s="15" t="n">
-        <v>25</v>
+        <v>9.289999999999999</v>
       </c>
       <c r="M12" s="13" t="inlineStr">
         <is>
-          <t>upgrade</t>
+          <t>behouden</t>
         </is>
       </c>
       <c r="N12" s="15">
@@ -3407,17 +3529,17 @@
       </c>
       <c r="O12" s="13" t="inlineStr">
         <is>
-          <t>NL · lokaal (vloerzetter; planning 1–2 wkn typisch)</t>
+          <t>NL · 1–2 werkdagen (gebundeld met egaline)</t>
         </is>
       </c>
       <c r="P12" s="13" t="inlineStr">
         <is>
-          <t>Lokale vloerzetter NL</t>
+          <t>EgalineXXL</t>
         </is>
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
-          <t>https://www.magnumheating.nl/product/noppenplaat/</t>
+          <t>https://egalinexxl.nl/</t>
         </is>
       </c>
       <c r="R12" s="13" t="inlineStr">
@@ -3426,16 +3548,16 @@
         </is>
       </c>
       <c r="S12" s="15" t="n">
-        <v>0</v>
+        <v>600</v>
       </c>
       <c r="T12" s="13" t="inlineStr">
         <is>
-          <t>INDICATIEF €25–55/m² incl. arbeid. Vraag 2 offertes. Kern van “kwalitatief beste” t.o.v. SlimFit/egaline.</t>
+          <t>Zelfde shop als egaline (gebundeld voor verzending).</t>
         </is>
       </c>
       <c r="U12" s="28" t="inlineStr">
         <is>
-          <t>ZEKER — lokaal NL (geen webshop-SKU)</t>
+          <t>ZEKER — NL webshop</t>
         </is>
       </c>
     </row>
@@ -3455,46 +3577,47 @@
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
-          <t>Verdeler</t>
+          <t>Egaline</t>
         </is>
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>VTE Composiet 4-groeps mengverdeler + Grundfos UPM3 pomp</t>
+          <t>Kreisel 418 vezelversterkte egaline 25 kg</t>
         </is>
       </c>
       <c r="F13" s="13" t="inlineStr">
         <is>
-          <t>KU100104GU</t>
+          <t>418</t>
         </is>
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Composiet, flowmeters, M30, koelbaar.</t>
+          <t>1–50 mm, vezels, vloerverwarming. Totale opbouw SlimFit+egaline = Parameters!B7 mm.</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t>Hart van het systeem.</t>
-        </is>
-      </c>
-      <c r="I13" s="30" t="n">
-        <v>1</v>
+          <t>Inbedden SlimFit + buizen.</t>
+        </is>
+      </c>
+      <c r="I13" s="14">
+        <f>CEILING(Parameters!$B$4*1.5*Parameters!$B$7/25,1)</f>
+        <v/>
       </c>
       <c r="J13" s="13" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>zak</t>
         </is>
       </c>
       <c r="K13" s="15" t="n">
-        <v>387.18</v>
+        <v>14.87</v>
       </c>
       <c r="L13" s="15" t="n">
-        <v>305.95</v>
+        <v>14.87</v>
       </c>
       <c r="M13" s="13" t="inlineStr">
         <is>
-          <t>upgrade</t>
+          <t>behouden</t>
         </is>
       </c>
       <c r="N13" s="15">
@@ -3503,17 +3626,17 @@
       </c>
       <c r="O13" s="13" t="inlineStr">
         <is>
-          <t>NL · op voorraad, volgende werkdag mogelijk</t>
+          <t>NL · volgende werkdag / pallet in overleg</t>
         </is>
       </c>
       <c r="P13" s="13" t="inlineStr">
         <is>
-          <t>123Installatieshop</t>
+          <t>EgalineXXL</t>
         </is>
       </c>
       <c r="Q13" s="13" t="inlineStr">
         <is>
-          <t>https://www.123installatieshop.nl/vte-composiet-verdeler-4-groepen-met-pomp-ku100104gu</t>
+          <t>https://egalinexxl.nl/products/kreisel-418-vezelversterkte-egalisatie-25kg-1-50mm</t>
         </is>
       </c>
       <c r="R13" s="13" t="inlineStr">
@@ -3522,16 +3645,16 @@
         </is>
       </c>
       <c r="S13" s="15" t="n">
-        <v>150</v>
+        <v>600</v>
       </c>
       <c r="T13" s="13" t="inlineStr">
         <is>
-          <t>PRIJS = 4-groeps. Bij andere groepen: andere SKU!</t>
+          <t>All-in: +pallet ~€60,50 als &lt;€600 excl. Stort tot Parameters!B7 (22 mm aanbevolen; max 30). Vezels tegen spanning.</t>
         </is>
       </c>
       <c r="U13" s="28" t="inlineStr">
         <is>
-          <t>ZEKER — NL webshop</t>
+          <t>ZEKER — NL webshop (pallet)</t>
         </is>
       </c>
     </row>
@@ -3551,47 +3674,46 @@
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
-          <t>Leiding</t>
+          <t>Verdeler</t>
         </is>
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>Aanvoer + retourleiding (meerlagenbuis 16×2)</t>
+          <t>VTE Composiet 4-groeps mengverdeler + Grundfos UPM3 pomp</t>
         </is>
       </c>
       <c r="F14" s="13" t="inlineStr">
         <is>
-          <t>ML162</t>
+          <t>KU100104GU</t>
         </is>
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>Primair cv/wp → verdeler.</t>
+          <t>Composiet, flowmeters, M30, koelbaar.</t>
         </is>
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t>cv/wp → verdeler.</t>
-        </is>
-      </c>
-      <c r="I14" s="30">
-        <f>MAX(8,ROUND(Parameters!$B$4/3,0))</f>
-        <v/>
+          <t>Hart van het systeem.</t>
+        </is>
+      </c>
+      <c r="I14" s="17" t="n">
+        <v>1</v>
       </c>
       <c r="J14" s="13" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>st</t>
         </is>
       </c>
       <c r="K14" s="15" t="n">
-        <v>6.5</v>
+        <v>387.18</v>
       </c>
       <c r="L14" s="15" t="n">
-        <v>6.5</v>
+        <v>305.95</v>
       </c>
       <c r="M14" s="13" t="inlineStr">
         <is>
-          <t>behouden</t>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="N14" s="15">
@@ -3600,17 +3722,17 @@
       </c>
       <c r="O14" s="13" t="inlineStr">
         <is>
-          <t>NL · ≤ 1 week</t>
+          <t>NL · op voorraad, volgende werkdag mogelijk</t>
         </is>
       </c>
       <c r="P14" s="13" t="inlineStr">
         <is>
-          <t>123Installatieshop / bouwmarkt NL</t>
+          <t>123Installatieshop</t>
         </is>
       </c>
       <c r="Q14" s="13" t="inlineStr">
         <is>
-          <t>https://www.123installatieshop.nl/</t>
+          <t>https://www.123installatieshop.nl/vte-composiet-verdeler-4-groepen-met-pomp-ku100104gu</t>
         </is>
       </c>
       <c r="R14" s="13" t="inlineStr">
@@ -3619,16 +3741,16 @@
         </is>
       </c>
       <c r="S14" s="15" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="T14" s="13" t="inlineStr">
         <is>
-          <t>Situatie-afhankelijk.</t>
+          <t>PRIJS = 4-groeps. Bij andere groepen: andere SKU/prijs kiezen!</t>
         </is>
       </c>
       <c r="U14" s="28" t="inlineStr">
         <is>
-          <t>ZEKER — NL</t>
+          <t>ZEKER — NL webshop</t>
         </is>
       </c>
     </row>
@@ -3648,42 +3770,43 @@
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
-          <t>Afsluiters</t>
+          <t>Leiding</t>
         </is>
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Kogelkranen / koppelingen set</t>
+          <t>Aanvoer + retourleiding (meerlagenbuis 16×2)</t>
         </is>
       </c>
       <c r="F15" s="13" t="inlineStr">
         <is>
-          <t>KK-SET</t>
+          <t>ML162</t>
         </is>
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t>Afsluitbaar maken.</t>
+          <t>Primair cv/wp → verdeler.</t>
         </is>
       </c>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t>Service/afsluitbaar.</t>
-        </is>
-      </c>
-      <c r="I15" s="30" t="n">
-        <v>1</v>
+          <t>cv/wp → verdeler.</t>
+        </is>
+      </c>
+      <c r="I15" s="14">
+        <f>MAX(8,ROUND(Parameters!$B$4/3,0))</f>
+        <v/>
       </c>
       <c r="J15" s="13" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>m</t>
         </is>
       </c>
       <c r="K15" s="15" t="n">
-        <v>34.95</v>
+        <v>6.5</v>
       </c>
       <c r="L15" s="15" t="n">
-        <v>34.95</v>
+        <v>6.5</v>
       </c>
       <c r="M15" s="13" t="inlineStr">
         <is>
@@ -3696,12 +3819,12 @@
       </c>
       <c r="O15" s="13" t="inlineStr">
         <is>
-          <t>NL · ≤ 1 week</t>
+          <t>NL · ≤ 1 week (standaard meerlagenbuis)</t>
         </is>
       </c>
       <c r="P15" s="13" t="inlineStr">
         <is>
-          <t>123Installatieshop</t>
+          <t>123Installatieshop / bouwmarkt NL</t>
         </is>
       </c>
       <c r="Q15" s="13" t="inlineStr">
@@ -3715,16 +3838,16 @@
         </is>
       </c>
       <c r="S15" s="15" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="T15" s="13" t="inlineStr">
         <is>
-          <t>Vast per installatie.</t>
+          <t>Situatie-afhankelijk; schaalt licht met woninggrootte. Lokale bouwmarkt of NL-installatieshop; geen import.</t>
         </is>
       </c>
       <c r="U15" s="28" t="inlineStr">
         <is>
-          <t>ZEKER — NL webshop</t>
+          <t>ZEKER — NL (generiek artikel)</t>
         </is>
       </c>
     </row>
@@ -3744,83 +3867,84 @@
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>Actuator</t>
+          <t>Afsluiters</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Möhlenhoff Alpha 5 thermische motor 230V NC M30×1,5 (+ adapter)</t>
+          <t>Kogelkranen / koppelingen set</t>
         </is>
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>A20405-00N80-1S</t>
+          <t>KK-SET</t>
         </is>
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>NC 230V, VA80 adapter, 1 W.</t>
+          <t>Afsluitbaar maken.</t>
         </is>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>1 per groep.</t>
-        </is>
-      </c>
-      <c r="I16" s="30">
-        <f>Parameters!$B$5</f>
-        <v/>
+          <t>Service/afsluitbaar.</t>
+        </is>
+      </c>
+      <c r="I16" s="17" t="n">
+        <v>1</v>
       </c>
       <c r="J16" s="13" t="inlineStr">
         <is>
-          <t>st</t>
-        </is>
-      </c>
-      <c r="K16" s="15">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),20.12,9.99)</f>
-        <v/>
-      </c>
-      <c r="L16" s="15">
-        <f>K16</f>
-        <v/>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="K16" s="15" t="n">
+        <v>34.95</v>
+      </c>
+      <c r="L16" s="15" t="n">
+        <v>34.95</v>
       </c>
       <c r="M16" s="13" t="inlineStr">
         <is>
-          <t>upgrade</t>
+          <t>behouden</t>
         </is>
       </c>
       <c r="N16" s="15">
         <f>I16*K16</f>
         <v/>
       </c>
-      <c r="O16" s="13">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"NL · 3–4 werkdagen (VerwarmingOnline)","DE→NL · 2–5 wd DE + NL-transit (eibhandel DHL)")</f>
-        <v/>
-      </c>
-      <c r="P16" s="13">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"VerwarmingOnline","eibhandel.de")</f>
-        <v/>
-      </c>
-      <c r="Q16" s="13">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"https://verwarmingonline.nl/productgroepen/mohlenhoff-thermische-servomotor-alpha-5-nc-m30x15mm-230v-a-20405-00n/","https://eibhandel.de/Alpha-Antrieb-230V-NC-incl-Adapter-VA80")</f>
-        <v/>
-      </c>
-      <c r="R16" s="13">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"NL","DE→NL")</f>
-        <v/>
-      </c>
-      <c r="S16" s="15">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),385,1000)</f>
-        <v/>
+      <c r="O16" s="13" t="inlineStr">
+        <is>
+          <t>NL · ≤ 1 week</t>
+        </is>
+      </c>
+      <c r="P16" s="13" t="inlineStr">
+        <is>
+          <t>123Installatieshop</t>
+        </is>
+      </c>
+      <c r="Q16" s="13" t="inlineStr">
+        <is>
+          <t>https://www.123installatieshop.nl/</t>
+        </is>
+      </c>
+      <c r="R16" s="13" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="S16" s="15" t="n">
+        <v>50</v>
       </c>
       <c r="T16" s="13" t="inlineStr">
         <is>
-          <t>Schakel via Parameters!B8. DE→NL: verzending ≈€15,41.</t>
-        </is>
-      </c>
-      <c r="U16" s="28">
-        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"ZEKER — NL webshop","DE→NL bevestigd (DHL zone 1)")</f>
-        <v/>
+          <t>Vast per installatie.</t>
+        </is>
+      </c>
+      <c r="U16" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — NL webshop</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -3839,42 +3963,45 @@
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Elektra</t>
+          <t>Actuator</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>Elektrakabel 230V / signaalkabel (installatiekwaliteit)</t>
+          <t>Möhlenhoff Alpha 5 thermische motor 230V NC M30×1,5 (+ adapter)</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>ELEKTRA</t>
+          <t>A20405-00N80-1S</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>Voeding pomp/regeling/actuators.</t>
+          <t>NC 230V, VA80 adapter, 1 W.</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
-          <t>Elektra.</t>
-        </is>
-      </c>
-      <c r="I17" s="30" t="n">
-        <v>1</v>
+          <t>1 per groep.</t>
+        </is>
+      </c>
+      <c r="I17" s="14">
+        <f>Parameters!$B$5</f>
+        <v/>
       </c>
       <c r="J17" s="13" t="inlineStr">
         <is>
-          <t>kleinmateriaal</t>
-        </is>
-      </c>
-      <c r="K17" s="15" t="n">
-        <v>25</v>
-      </c>
-      <c r="L17" s="15" t="n">
-        <v>20</v>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="K17" s="15">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),20.12,9.99)</f>
+        <v/>
+      </c>
+      <c r="L17" s="15">
+        <f>K17</f>
+        <v/>
       </c>
       <c r="M17" s="13" t="inlineStr">
         <is>
@@ -3885,38 +4012,34 @@
         <f>I17*K17</f>
         <v/>
       </c>
-      <c r="O17" s="13" t="inlineStr">
-        <is>
-          <t>NL · 1 werkdag / afhalen</t>
-        </is>
-      </c>
-      <c r="P17" s="13" t="inlineStr">
-        <is>
-          <t>Elektramat</t>
-        </is>
-      </c>
-      <c r="Q17" s="13" t="inlineStr">
-        <is>
-          <t>https://www.elektramat.nl/draad-en-kabel/installatiekabel/</t>
-        </is>
-      </c>
-      <c r="R17" s="29" t="inlineStr">
-        <is>
-          <t>NL</t>
-        </is>
-      </c>
-      <c r="S17" s="15" t="n">
-        <v>0</v>
+      <c r="O17" s="13">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"NL · 3–4 werkdagen (VerwarmingOnline)","DE→NL · 2–5 wd DE + NL-transit (eibhandel DHL)")</f>
+        <v/>
+      </c>
+      <c r="P17" s="13">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"VerwarmingOnline","eibhandel.de")</f>
+        <v/>
+      </c>
+      <c r="Q17" s="13">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"https://verwarmingonline.nl/productgroepen/mohlenhoff-thermische-servomotor-alpha-5-nc-m30x15mm-230v-a-20405-00n/","https://eibhandel.de/Alpha-Antrieb-230V-NC-incl-Adapter-VA80")</f>
+        <v/>
+      </c>
+      <c r="R17" s="29">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"NL","DE→NL")</f>
+        <v/>
+      </c>
+      <c r="S17" s="15">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),385,1000)</f>
+        <v/>
       </c>
       <c r="T17" s="13" t="inlineStr">
         <is>
-          <t>Vast; bij groter project licht ophogen. Bundel met Magnum-order.</t>
-        </is>
-      </c>
-      <c r="U17" t="inlineStr">
-        <is>
-          <t>ZEKER — NL</t>
-        </is>
+          <t>Schakel via Parameters!B8. DE→NL: verzending ≈€15,41 + levertijd 2–5 wd DE. NL zeker: €20,12/st, verzending €0 als order ≥€385 anders ~€6,95.</t>
+        </is>
+      </c>
+      <c r="U17">
+        <f>IF(ISNUMBER(SEARCH("NL zeker",Parameters!$B$8)),"ZEKER — NL webshop","DE→NL bevestigd (DHL zone 1)")</f>
+        <v/>
       </c>
     </row>
     <row r="18">
@@ -3930,51 +4053,51 @@
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>h64</t>
+          <t>altijd</t>
         </is>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
-          <t>Regeling</t>
+          <t>Elektra</t>
         </is>
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>MAGNUM H64-CC + master WiFi-thermostaat</t>
+          <t>Elektrakabel 230V / signaalkabel (installatiekwaliteit)</t>
         </is>
       </c>
       <c r="F18" s="13" t="inlineStr">
         <is>
-          <t>W81000</t>
+          <t>ELEKTRA</t>
         </is>
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t>Control Center + master.</t>
+          <t>Voeding pomp/regeling/actuators.</t>
         </is>
       </c>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t>Alleen bij keuze H64.</t>
-        </is>
-      </c>
-      <c r="I18" s="30" t="n">
+          <t>Elektra.</t>
+        </is>
+      </c>
+      <c r="I18" s="17" t="n">
         <v>1</v>
       </c>
       <c r="J18" s="13" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>kleinmateriaal</t>
         </is>
       </c>
       <c r="K18" s="15" t="n">
-        <v>194.92</v>
+        <v>25</v>
       </c>
       <c r="L18" s="15" t="n">
-        <v>194.92</v>
+        <v>20</v>
       </c>
       <c r="M18" s="13" t="inlineStr">
         <is>
-          <t>behouden</t>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="N18" s="15">
@@ -3983,17 +4106,17 @@
       </c>
       <c r="O18" s="13" t="inlineStr">
         <is>
-          <t>NL · 1 werkdag</t>
+          <t>NL · 1 werkdag / direct afhalen</t>
         </is>
       </c>
       <c r="P18" s="13" t="inlineStr">
         <is>
-          <t>Warp Systems</t>
+          <t>Elektramat / bouwmarkt NL</t>
         </is>
       </c>
       <c r="Q18" s="13" t="inlineStr">
         <is>
-          <t>https://shop.warp-systems.com/h64-control-center-master-wifi-thermostaat-wit-of-zwart-magh64cc-mt-c</t>
+          <t>https://www.elektramat.nl/draad-en-kabel/installatiekabel/</t>
         </is>
       </c>
       <c r="R18" s="13" t="inlineStr">
@@ -4006,12 +4129,12 @@
       </c>
       <c r="T18" s="13" t="inlineStr">
         <is>
-          <t>NL-fabrikant.</t>
+          <t>Vast; bij groter project licht ophogen.</t>
         </is>
       </c>
       <c r="U18" s="28" t="inlineStr">
         <is>
-          <t>ZEKER — NL fabrikant</t>
+          <t>ZEKER — NL</t>
         </is>
       </c>
     </row>
@@ -4036,38 +4159,37 @@
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>MAGNUM H64-ST slave thermostaat</t>
+          <t>MAGNUM H64-CC + master WiFi-thermostaat</t>
         </is>
       </c>
       <c r="F19" s="13" t="inlineStr">
         <is>
-          <t>W81010</t>
+          <t>W81000</t>
         </is>
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>Slave per extra ruimte.</t>
+          <t>Control Center + master.</t>
         </is>
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
-          <t>Ruimte 2…N bij H64.</t>
-        </is>
-      </c>
-      <c r="I19" s="30">
-        <f>MAX(0,Parameters!$B$6-1)</f>
-        <v/>
+          <t>Alleen bij keuze H64.</t>
+        </is>
+      </c>
+      <c r="I19" s="17" t="n">
+        <v>1</v>
       </c>
       <c r="J19" s="13" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>set</t>
         </is>
       </c>
       <c r="K19" s="15" t="n">
-        <v>44.58</v>
+        <v>194.92</v>
       </c>
       <c r="L19" s="15" t="n">
-        <v>44.58</v>
+        <v>194.92</v>
       </c>
       <c r="M19" s="13" t="inlineStr">
         <is>
@@ -4080,7 +4202,7 @@
       </c>
       <c r="O19" s="13" t="inlineStr">
         <is>
-          <t>NL · 1 werkdag</t>
+          <t>NL · 1 werkdag (voor 12:00 zelfde dag verzonden)</t>
         </is>
       </c>
       <c r="P19" s="13" t="inlineStr">
@@ -4090,7 +4212,7 @@
       </c>
       <c r="Q19" s="13" t="inlineStr">
         <is>
-          <t>https://shop.warp-systems.com/catalogsearch/result/?q=slave+H64</t>
+          <t>https://shop.warp-systems.com/h64-control-center-master-wifi-thermostaat-wit-of-zwart-magh64cc-mt-c</t>
         </is>
       </c>
       <c r="R19" s="13" t="inlineStr">
@@ -4103,7 +4225,7 @@
       </c>
       <c r="T19" s="13" t="inlineStr">
         <is>
-          <t>Schaalt met ruimten−1.</t>
+          <t>NL-fabrikant, snelle levering.</t>
         </is>
       </c>
       <c r="U19" s="28" t="inlineStr">
@@ -4123,7 +4245,7 @@
       </c>
       <c r="C20" s="13" t="inlineStr">
         <is>
-          <t>tado_draadloos</t>
+          <t>h64</t>
         </is>
       </c>
       <c r="D20" s="13" t="inlineStr">
@@ -4133,38 +4255,38 @@
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>tado° Draadloze Slimme Thermostaat X Starterskit</t>
+          <t>MAGNUM H64-ST slave thermostaat</t>
         </is>
       </c>
       <c r="F20" s="13" t="inlineStr">
         <is>
-          <t>TADO-WX</t>
+          <t>W81010</t>
         </is>
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t>Wireless X + Bridge.</t>
+          <t>Slave per extra ruimte.</t>
         </is>
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>1 kit per ruimte (draadloos).</t>
-        </is>
-      </c>
-      <c r="I20" s="30">
-        <f>Parameters!$B$6</f>
+          <t>Ruimte 2…N bij H64.</t>
+        </is>
+      </c>
+      <c r="I20" s="14">
+        <f>MAX(0,Parameters!$B$6-1)</f>
         <v/>
       </c>
       <c r="J20" s="13" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>st</t>
         </is>
       </c>
       <c r="K20" s="15" t="n">
-        <v>129</v>
+        <v>44.58</v>
       </c>
       <c r="L20" s="15" t="n">
-        <v>129</v>
+        <v>44.58</v>
       </c>
       <c r="M20" s="13" t="inlineStr">
         <is>
@@ -4177,17 +4299,17 @@
       </c>
       <c r="O20" s="13" t="inlineStr">
         <is>
-          <t>NL/EU · 2–4 werkdagen</t>
+          <t>NL · 1 werkdag</t>
         </is>
       </c>
       <c r="P20" s="13" t="inlineStr">
         <is>
-          <t>tado° Shop</t>
+          <t>Warp Systems</t>
         </is>
       </c>
       <c r="Q20" s="13" t="inlineStr">
         <is>
-          <t>https://shop.tado.com/nl-bx/products/wireless-smart-thermostat-x-starter-kit</t>
+          <t>https://shop.warp-systems.com/catalogsearch/result/?q=slave+H64</t>
         </is>
       </c>
       <c r="R20" s="13" t="inlineStr">
@@ -4196,16 +4318,16 @@
         </is>
       </c>
       <c r="S20" s="15" t="n">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="T20" s="13" t="inlineStr">
         <is>
-          <t>Schaalt met ruimten.</t>
+          <t>Schaalt met ruimten−1.</t>
         </is>
       </c>
       <c r="U20" s="28" t="inlineStr">
         <is>
-          <t>ZEKER — tado° NL-shop</t>
+          <t>ZEKER — NL fabrikant</t>
         </is>
       </c>
     </row>
@@ -4220,7 +4342,7 @@
       </c>
       <c r="C21" s="13" t="inlineStr">
         <is>
-          <t>tado_bedraad</t>
+          <t>tado_draadloos</t>
         </is>
       </c>
       <c r="D21" s="13" t="inlineStr">
@@ -4230,26 +4352,27 @@
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>tado° Slimme Thermostaat X Starterskit bedraad + Bridge X</t>
+          <t>tado° Draadloze Slimme Thermostaat X Starterskit</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
         <is>
-          <t>TADO-WX-W</t>
+          <t>TADO-WX</t>
         </is>
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t>Wired starter + Bridge.</t>
+          <t>Wireless X + Bridge.</t>
         </is>
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>Kamer 1 + netwerk.</t>
-        </is>
-      </c>
-      <c r="I21" s="30" t="n">
-        <v>1</v>
+          <t>1 kit per ruimte (draadloos).</t>
+        </is>
+      </c>
+      <c r="I21" s="14">
+        <f>Parameters!$B$6</f>
+        <v/>
       </c>
       <c r="J21" s="13" t="inlineStr">
         <is>
@@ -4257,14 +4380,14 @@
         </is>
       </c>
       <c r="K21" s="15" t="n">
-        <v>129.99</v>
+        <v>129</v>
       </c>
       <c r="L21" s="15" t="n">
-        <v>129.99</v>
+        <v>129</v>
       </c>
       <c r="M21" s="13" t="inlineStr">
         <is>
-          <t>upgrade</t>
+          <t>behouden</t>
         </is>
       </c>
       <c r="N21" s="15">
@@ -4273,7 +4396,7 @@
       </c>
       <c r="O21" s="13" t="inlineStr">
         <is>
-          <t>NL/EU · 2–4 werkdagen</t>
+          <t>NL/EU · 2–4 werkdagen (tado° levert NL)</t>
         </is>
       </c>
       <c r="P21" s="13" t="inlineStr">
@@ -4283,7 +4406,7 @@
       </c>
       <c r="Q21" s="13" t="inlineStr">
         <is>
-          <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-starter-kit-1</t>
+          <t>https://shop.tado.com/nl-bx/products/wireless-smart-thermostat-x-starter-kit</t>
         </is>
       </c>
       <c r="R21" s="13" t="inlineStr">
@@ -4296,7 +4419,7 @@
       </c>
       <c r="T21" s="13" t="inlineStr">
         <is>
-          <t>Aanbevolen pad (bedraad).</t>
+          <t>Schaalt met ruimten. Officiële shop goedkoopst.</t>
         </is>
       </c>
       <c r="U21" s="28" t="inlineStr">
@@ -4326,38 +4449,37 @@
       </c>
       <c r="E22" s="13" t="inlineStr">
         <is>
-          <t>tado° Slimme Thermostaat X bedraad (uitbreiding)</t>
+          <t>tado° Slimme Thermostaat X Starterskit bedraad + Bridge X</t>
         </is>
       </c>
       <c r="F22" s="13" t="inlineStr">
         <is>
-          <t>TADO-WX-E</t>
+          <t>TADO-WX-W</t>
         </is>
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>Extra bedrade thermostaat.</t>
+          <t>Wired starter + Bridge.</t>
         </is>
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t>Kamer 2…N.</t>
-        </is>
-      </c>
-      <c r="I22" s="30">
-        <f>MAX(0,Parameters!$B$6-1)</f>
-        <v/>
+          <t>Kamer 1 + netwerk.</t>
+        </is>
+      </c>
+      <c r="I22" s="17" t="n">
+        <v>1</v>
       </c>
       <c r="J22" s="13" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>set</t>
         </is>
       </c>
       <c r="K22" s="15" t="n">
-        <v>100</v>
+        <v>129.99</v>
       </c>
       <c r="L22" s="15" t="n">
-        <v>100</v>
+        <v>129.99</v>
       </c>
       <c r="M22" s="13" t="inlineStr">
         <is>
@@ -4380,7 +4502,7 @@
       </c>
       <c r="Q22" s="13" t="inlineStr">
         <is>
-          <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-wired</t>
+          <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-starter-kit-1</t>
         </is>
       </c>
       <c r="R22" s="13" t="inlineStr">
@@ -4393,7 +4515,7 @@
       </c>
       <c r="T22" s="13" t="inlineStr">
         <is>
-          <t>Schaalt met ruimten−1.</t>
+          <t>Aanbevolen pad (bedraad).</t>
         </is>
       </c>
       <c r="U22" s="28" t="inlineStr">
@@ -4413,7 +4535,7 @@
       </c>
       <c r="C23" s="13" t="inlineStr">
         <is>
-          <t>tado_optie</t>
+          <t>tado_bedraad</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
@@ -4423,26 +4545,27 @@
       </c>
       <c r="E23" s="13" t="inlineStr">
         <is>
-          <t>tado° Bridge X (extra indien nodig)</t>
+          <t>tado° Slimme Thermostaat X bedraad (uitbreiding)</t>
         </is>
       </c>
       <c r="F23" s="13" t="inlineStr">
         <is>
-          <t>TADO-BR</t>
+          <t>TADO-WX-E</t>
         </is>
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t>Alleen bij bereikproblemen.</t>
+          <t>Extra bedrade thermostaat.</t>
         </is>
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
-          <t>Optioneel.</t>
-        </is>
-      </c>
-      <c r="I23" s="30" t="n">
-        <v>0</v>
+          <t>Kamer 2…N.</t>
+        </is>
+      </c>
+      <c r="I23" s="14">
+        <f>MAX(0,Parameters!$B$6-1)</f>
+        <v/>
       </c>
       <c r="J23" s="13" t="inlineStr">
         <is>
@@ -4450,14 +4573,14 @@
         </is>
       </c>
       <c r="K23" s="15" t="n">
-        <v>68</v>
+        <v>100</v>
       </c>
       <c r="L23" s="15" t="n">
-        <v>68</v>
+        <v>100</v>
       </c>
       <c r="M23" s="13" t="inlineStr">
         <is>
-          <t>behouden</t>
+          <t>upgrade</t>
         </is>
       </c>
       <c r="N23" s="15">
@@ -4476,7 +4599,7 @@
       </c>
       <c r="Q23" s="13" t="inlineStr">
         <is>
-          <t>https://shop.tado.com/nl-bx/</t>
+          <t>https://shop.tado.com/nl-bx/products/smart-thermostat-x-wired</t>
         </is>
       </c>
       <c r="R23" s="13" t="inlineStr">
@@ -4489,7 +4612,7 @@
       </c>
       <c r="T23" s="13" t="inlineStr">
         <is>
-          <t>Standaard 0.</t>
+          <t>Schaalt met ruimten−1.</t>
         </is>
       </c>
       <c r="U23" s="28" t="inlineStr">
@@ -4499,27 +4622,107 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n"/>
-      <c r="B24" s="13" t="n"/>
-      <c r="C24" s="13" t="n"/>
-      <c r="D24" s="13" t="n"/>
-      <c r="E24" s="13" t="n"/>
-      <c r="F24" s="13" t="n"/>
-      <c r="G24" s="13" t="n"/>
-      <c r="H24" s="13" t="n"/>
-      <c r="I24" s="17" t="n"/>
-      <c r="J24" s="13" t="n"/>
-      <c r="K24" s="15" t="n"/>
-      <c r="L24" s="15" t="n"/>
-      <c r="M24" s="13" t="n"/>
-      <c r="N24" s="15" t="n"/>
-      <c r="O24" s="13" t="n"/>
-      <c r="P24" s="13" t="n"/>
-      <c r="Q24" s="13" t="n"/>
-      <c r="R24" s="13" t="n"/>
-      <c r="S24" s="15" t="n"/>
-      <c r="T24" s="13" t="n"/>
-      <c r="U24" s="28" t="n"/>
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Vloerverwarming</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="n">
+        <v>19</v>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>tado_optie</t>
+        </is>
+      </c>
+      <c r="D24" s="13" t="inlineStr">
+        <is>
+          <t>Regeling</t>
+        </is>
+      </c>
+      <c r="E24" s="13" t="inlineStr">
+        <is>
+          <t>tado° Bridge X (extra indien nodig)</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>TADO-BR</t>
+        </is>
+      </c>
+      <c r="G24" s="13" t="inlineStr">
+        <is>
+          <t>Alleen bij bereikproblemen.</t>
+        </is>
+      </c>
+      <c r="H24" s="13" t="inlineStr">
+        <is>
+          <t>Optioneel.</t>
+        </is>
+      </c>
+      <c r="I24" s="17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="13" t="inlineStr">
+        <is>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="K24" s="15" t="n">
+        <v>68</v>
+      </c>
+      <c r="L24" s="15" t="n">
+        <v>68</v>
+      </c>
+      <c r="M24" s="13" t="inlineStr">
+        <is>
+          <t>behouden</t>
+        </is>
+      </c>
+      <c r="N24" s="15">
+        <f>I24*K24</f>
+        <v/>
+      </c>
+      <c r="O24" s="13" t="inlineStr">
+        <is>
+          <t>NL/EU · 2–4 werkdagen</t>
+        </is>
+      </c>
+      <c r="P24" s="13" t="inlineStr">
+        <is>
+          <t>tado° Shop</t>
+        </is>
+      </c>
+      <c r="Q24" s="13" t="inlineStr">
+        <is>
+          <t>https://shop.tado.com/nl-bx/</t>
+        </is>
+      </c>
+      <c r="R24" s="13" t="inlineStr">
+        <is>
+          <t>NL</t>
+        </is>
+      </c>
+      <c r="S24" s="15" t="n">
+        <v>150</v>
+      </c>
+      <c r="T24" s="13" t="inlineStr">
+        <is>
+          <t>Standaard 0; handmatig verhogen indien nodig.</t>
+        </is>
+      </c>
+      <c r="U24" s="28" t="inlineStr">
+        <is>
+          <t>ZEKER — tado° NL-shop</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Groen = hoeveelheid-formule (schaalt). Totaal = Hoeveelheid × Prijs/st. Verzendkosten: sheet Verzending.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A5:T24"/>
@@ -4533,7 +4736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -4548,21 +4751,21 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>All-in check — kwalitatief beste BOM</t>
+          <t>All-in check — SlimFit op beton ≤30 mm</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>30 m² · 4 groepen · 3 ruimten · dekvloer ≥50 mm. Hardheid &gt; laagste opbouw.</t>
+          <t>Terug naar SlimFit-BOM: zandcement paste niet in 3 cm. Beton + 22 mm egaline = kwalitatief best haalbaar.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="21" t="inlineStr">
         <is>
-          <t>Verdict: BOM omgezet SlimFit/egaline → noppen 28 mm + PE-RT 16 + zandcement.</t>
+          <t>Verdict: SlimFit-pad behouden t.o.v. nat systeem i.v.m. hoogte. Shops all-in ongewijzigd t.o.v. eerdere SlimFit-revisie.</t>
         </is>
       </c>
     </row>
@@ -4579,12 +4782,12 @@
       </c>
       <c r="C5" s="22" t="inlineStr">
         <is>
-          <t>Gekozen</t>
+          <t>Gekozen (all-in)</t>
         </is>
       </c>
       <c r="D5" s="22" t="inlineStr">
         <is>
-          <t>Alternatief</t>
+          <t>Alternatief all-in</t>
         </is>
       </c>
       <c r="E5" s="22" t="inlineStr">
@@ -4594,7 +4797,7 @@
       </c>
       <c r="F5" s="22" t="inlineStr">
         <is>
-          <t>NL?</t>
+          <t>NL-leverbaar?</t>
         </is>
       </c>
       <c r="G5" s="22" t="inlineStr">
@@ -4609,27 +4812,27 @@
       </c>
       <c r="B6" s="13" t="inlineStr">
         <is>
-          <t>Noppen 28 mm 3×</t>
+          <t>SlimFit matten 8×</t>
         </is>
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>Elektramat 3×€136,58</t>
+          <t>Elektramat €695,52 (ship €0; order ≫ €150 excl)</t>
         </is>
       </c>
       <c r="D6" s="13" t="inlineStr">
         <is>
-          <t>17 mm goedkoper, minder isolatie</t>
+          <t>123IM €711,92 · VV-direct €712</t>
         </is>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>kwaliteit</t>
+          <t>−€16…€17</t>
         </is>
       </c>
       <c r="F6" s="13" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Ja NL 1 wd</t>
         </is>
       </c>
       <c r="G6" s="23" t="inlineStr">
@@ -4644,27 +4847,27 @@
       </c>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>PE-RT 240 m</t>
+          <t>PE-RT 300 m</t>
         </is>
       </c>
       <c r="C7" s="13" t="inlineStr">
         <is>
-          <t>Elektramat €158,99</t>
+          <t>123IM €142,93 + €6,95 ship ≈ €149,88 (order &lt;€200)</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>losse rollen ≥</t>
+          <t>Elektramat €181,86 (ship €0 in combi)</t>
         </is>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>beste</t>
+          <t>−€32</t>
         </is>
       </c>
       <c r="F7" s="13" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Ja NL morgen</t>
         </is>
       </c>
       <c r="G7" s="23" t="inlineStr">
@@ -4679,32 +4882,32 @@
       </c>
       <c r="B8" s="13" t="inlineStr">
         <is>
-          <t>Zandcement</t>
+          <t>Kreisel 418 33× + primer</t>
         </is>
       </c>
       <c r="C8" s="13" t="inlineStr">
         <is>
-          <t>€35/m² indicatief</t>
+          <t>EgalineXXL €509,29 + pallet €60,50 = €569,79</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
         <is>
-          <t>€25–55 lokaal</t>
+          <t>RBMB duurder/stuk · extra kopen tot €600 excl ≈ €610+</t>
         </is>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>offerte</t>
+          <t>−€40…</t>
         </is>
       </c>
       <c r="F8" s="13" t="inlineStr">
         <is>
-          <t>Ja lokaal</t>
+          <t>Ja NL pallet</t>
         </is>
       </c>
       <c r="G8" s="23" t="inlineStr">
         <is>
-          <t>OFFERTE</t>
+          <t>BEHOUDEN</t>
         </is>
       </c>
     </row>
@@ -4714,27 +4917,27 @@
       </c>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>VTE + Grundfos</t>
+          <t>VTE Composiet 4-gr.</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>€387,18</t>
+          <t>123Installatieshop €387,18 (ship €0 ≥€150)</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
         <is>
-          <t>duurdere shops</t>
+          <t>VV-shop €405 · CVTotaal €423 · Jan Isolatieman €469</t>
         </is>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>beste</t>
+          <t>−€18…€82</t>
         </is>
       </c>
       <c r="F9" s="13" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Ja NL ≤1 wk</t>
         </is>
       </c>
       <c r="G9" s="23" t="inlineStr">
@@ -4749,27 +4952,27 @@
       </c>
       <c r="B10" s="13" t="inlineStr">
         <is>
-          <t>Möhlenhoff ×4</t>
+          <t>Möhlenhoff Alpha 5 ×4</t>
         </is>
       </c>
       <c r="C10" s="13" t="inlineStr">
         <is>
-          <t>eibhandel ~€55 all-in</t>
+          <t>eibhandel.de €39,96 + €15,41 = €55,37</t>
         </is>
       </c>
       <c r="D10" s="13" t="inlineStr">
         <is>
-          <t>NL duurder</t>
+          <t>Amazon~€52,64* · Home Perfect €69,94 · VerwarmingOnline €87,43</t>
         </is>
       </c>
       <c r="E10" s="13" t="inlineStr">
         <is>
-          <t>beste</t>
+          <t>beste bevestigd</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
         <is>
-          <t>DE→NL</t>
+          <t>Ja DE→NL DHL</t>
         </is>
       </c>
       <c r="G10" s="23" t="inlineStr">
@@ -4779,107 +4982,230 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="n"/>
-      <c r="B11" s="13" t="n"/>
-      <c r="C11" s="13" t="n"/>
-      <c r="D11" s="13" t="n"/>
-      <c r="E11" s="13" t="n"/>
-      <c r="F11" s="13" t="n"/>
-      <c r="G11" s="23" t="n"/>
+      <c r="A11" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>NMC Climasol 3×</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Installand €71,97 (ship €0 ≥€60)</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>Generiek Distriheat goedkoper maar mindere kwaliteit</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>kwaliteit</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="inlineStr">
+        <is>
+          <t>Ja NL</t>
+        </is>
+      </c>
+      <c r="G11" s="23" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Live totalen</t>
-        </is>
-      </c>
-      <c r="B12" s="13" t="n"/>
-      <c r="C12" s="13" t="n"/>
-      <c r="D12" s="13" t="n"/>
-      <c r="E12" s="13" t="n"/>
-      <c r="F12" s="13" t="n"/>
-      <c r="G12" s="23" t="n"/>
+      <c r="A12" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
+        <is>
+          <t>H64-CC + slaves</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Warp Systems €194,92 + 2×€44,58 (NL)</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>123IM H64-CC was €213,74</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>−€19 CC</t>
+        </is>
+      </c>
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Ja NL 1 wd</t>
+        </is>
+      </c>
+      <c r="G12" s="23" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>Basis artikelen</t>
-        </is>
-      </c>
-      <c r="B13" s="13">
-        <f>Overzicht!B10</f>
-        <v/>
-      </c>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="13" t="n"/>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="13" t="n"/>
-      <c r="G13" s="23" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Basis verzending</t>
-        </is>
-      </c>
-      <c r="B14">
-        <f>Overzicht!C10</f>
-        <v/>
+      <c r="A13" s="13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Tado bedraad 3 ruimten</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>tado° Shop €329,99 (ship €0 ≥€150)</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>bol/retail vaak €189–€194 per starter alleen</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>goedkoopst</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Ja NL/EU</t>
+        </is>
+      </c>
+      <c r="G13" s="23" t="inlineStr">
+        <is>
+          <t>BEHOUDEN</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Basis all-in</t>
-        </is>
-      </c>
-      <c r="B15">
-        <f>Overzicht!D10</f>
-        <v/>
+          <t>Consolidatie-check (minder shops = minder verzending?)</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>All-in + Tado bedraad</t>
-        </is>
-      </c>
-      <c r="B16">
-        <f>Overzicht!D11</f>
-        <v/>
+          <t>• PE-RT meenemen bij Elektramat (zelfde order als SlimFit): all-in €181,86 i.p.v. ~€149,88 → NIET doen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>• Extra egaline kopen tot gratis drempel (€600 excl): duurder dan pallet betalen → NIET doen.</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Zandcement-regel is INDICATIEF. Echt totaal = webshop-BOM + vloerzetter-offerte.</t>
+          <t>• Actuators bij VerwarmingOnline (pure NL): +€32 vs eibhandel → alleen als je DE wilt vermijden.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Infrezen: vaak hardst als bestaande dekvloer geschikt is — apart laten beoordelen.</t>
+          <t>• Home Perfect (€10,01/st) lijkt scherp maar +€29,90 ship + 7–10 wd → all-in slechter én trager.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n"/>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Buitenland / NL-zekerheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Enige buitenlandse shop: eibhandel.de (actuators). Levert naar NL (DHL zone 1), verzending €15,41 incl, levertijd 2–5 wd DE (+NL-transit, meestal ≤1 week).</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Alles overige: Nederlandse webshops met snelle levering.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>* Amazon.nl-prijs is indicatief (listings wisselen); eibhandel is stabiel bevestigd all-in.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n"/>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Live totalen (formules, schalen met m²)</t>
+        </is>
+      </c>
     </row>
     <row r="27">
-      <c r="B27" s="6" t="n"/>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Basis artikelen</t>
+        </is>
+      </c>
+      <c r="B27" s="6">
+        <f>Overzicht!B10</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
-      <c r="B28" s="6" t="n"/>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Basis verzending</t>
+        </is>
+      </c>
+      <c r="B28" s="6">
+        <f>Overzicht!C10</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
-      <c r="B29" s="6" t="n"/>
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Basis all-in</t>
+        </is>
+      </c>
+      <c r="B29" s="6">
+        <f>Overzicht!D10</f>
+        <v/>
+      </c>
     </row>
     <row r="30">
-      <c r="B30" s="6" t="n"/>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>All-in + Tado bedraad</t>
+        </is>
+      </c>
+      <c r="B30" s="6">
+        <f>Overzicht!D11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>NL-update: schakelaar Parameters!B8. Default DE→NL blijft goedkoopst all-in; kies NL zeker indien je geen import wilt.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4892,7 +5218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H30"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4908,7 +5234,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Verzendkosten — all-in (kwalitatief beste BOM)</t>
+          <t>Verzendkosten — berekend all-in (NL-leverbaar)</t>
         </is>
       </c>
     </row>
@@ -4919,6 +5245,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -4973,7 +5300,7 @@
         </is>
       </c>
       <c r="C5" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A5,Boodschappenlijst!$C$6:$C$23,"altijd")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A5,Boodschappenlijst!$C$6:$C$24,"altijd")</f>
         <v/>
       </c>
       <c r="D5" s="5" t="n">
@@ -4994,14 +5321,14 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Noppen+buis+euro+bocht. Noppen=lengtevracht; check pallet/afhaal bij Elektramat.</t>
+          <t>Drempel €150 excl. btw; onder: €4,09 excl ≈ €4,95 incl</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Overkamp Meddo</t>
+          <t>123InstallatieMaterialen</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -5010,14 +5337,14 @@
         </is>
       </c>
       <c r="C6" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A6,Boodschappenlijst!$C$6:$C$23,"altijd")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A6,Boodschappenlijst!$C$6:$C$24,"altijd")</f>
         <v/>
       </c>
       <c r="D6" s="5" t="n">
-        <v>50</v>
+        <v>200</v>
       </c>
       <c r="E6" s="5">
-        <f>IF(C6&lt;=0,0,IF(C6&gt;=50,0,6.95))</f>
+        <f>IF(C6&lt;=0,0,IF(C6&gt;=200,0,6.95))</f>
         <v/>
       </c>
       <c r="F6" s="5">
@@ -5026,12 +5353,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>≤1 week</t>
+          <t>morgen</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Krimpnetten</t>
+          <t>Buis+bochten vaak &lt;€200 → €6,95 verzending; all-in nog steeds goedkoper dan Elektramat-buis</t>
         </is>
       </c>
     </row>
@@ -5047,7 +5374,7 @@
         </is>
       </c>
       <c r="C7" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A7,Boodschappenlijst!$C$6:$C$23,"altijd")+SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,"123Installatieshop / bouwmarkt NL",Boodschappenlijst!$C$6:$C$23,"altijd")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A7,Boodschappenlijst!$C$6:$C$24,"altijd")</f>
         <v/>
       </c>
       <c r="D7" s="5" t="n">
@@ -5068,14 +5395,14 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Verdeler+afsluiters (+ evt. ML-buis)</t>
+          <t>Verdeler alleen al &gt;€150 → gratis verzending</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Lokale vloerzetter NL</t>
+          <t>EgalineXXL</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5084,14 +5411,15 @@
         </is>
       </c>
       <c r="C8" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A8,Boodschappenlijst!$C$6:$C$23,"altijd")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A8,Boodschappenlijst!$C$6:$C$24,"altijd")</f>
         <v/>
       </c>
       <c r="D8" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>0</v>
+        <v>600</v>
+      </c>
+      <c r="E8" s="5">
+        <f>IF(C8&lt;=0,0,IF(C8/1.21&gt;=600,0,60.5))</f>
+        <v/>
       </c>
       <c r="F8" s="5">
         <f>C8+E8</f>
@@ -5099,12 +5427,12 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>lokaal</t>
+          <t>1–2 wd / pallet</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Zandcement: prijs is all-in indicatie</t>
+          <t>Primer+egaline; drempel €600 excl. btw → deel door 1,21; pallet €60,50 incl</t>
         </is>
       </c>
     </row>
@@ -5118,7 +5446,7 @@
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>Boodschappenlijst!N16</f>
+        <f>Boodschappenlijst!N17</f>
         <v/>
       </c>
       <c r="D9" s="5">
@@ -5139,7 +5467,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Actuators; volgt Parameters!B8</t>
+          <t>Volgt Parameters!B8. DE: DHL zone 1 NL €15,41. NL: VerwarmingOnline drempel €385.</t>
         </is>
       </c>
     </row>
@@ -5155,7 +5483,7 @@
         </is>
       </c>
       <c r="C10" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A10,Boodschappenlijst!$C$6:$C$23,"h64")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A10,Boodschappenlijst!$C$6:$C$24,"h64")</f>
         <v/>
       </c>
       <c r="D10" s="5" t="n">
@@ -5175,7 +5503,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Alleen bij H64</t>
+          <t>Alleen bij H64-pad</t>
         </is>
       </c>
     </row>
@@ -5191,7 +5519,7 @@
         </is>
       </c>
       <c r="C11" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A11,Boodschappenlijst!$C$6:$C$23,"tado_bedraad")+SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A11,Boodschappenlijst!$C$6:$C$23,"tado_draadloos")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A11,Boodschappenlijst!$C$6:$C$24,"tado_bedraad")+SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A11,Boodschappenlijst!$C$6:$C$24,"tado_draadloos")</f>
         <v/>
       </c>
       <c r="D11" s="5" t="n">
@@ -5212,7 +5540,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Alleen bij Tado</t>
+          <t>Alleen bij Tado-pad</t>
         </is>
       </c>
     </row>
@@ -5228,7 +5556,7 @@
         </is>
       </c>
       <c r="C12" s="5">
-        <f>SUMIFS(Boodschappenlijst!$N$6:$N$23,Boodschappenlijst!$P$6:$P$23,A12,Boodschappenlijst!$C$6:$C$23,"altijd")</f>
+        <f>SUMIFS(Boodschappenlijst!$N$6:$N$24,Boodschappenlijst!$P$6:$P$24,A12,Boodschappenlijst!$C$6:$C$24,"altijd")</f>
         <v/>
       </c>
       <c r="D12" s="5" t="n">
@@ -5249,10 +5577,11 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Climasol</t>
-        </is>
-      </c>
-    </row>
+          <t>Gratis vanaf €60; 3 rollen Climasol ≈ €72 → meestal gratis</t>
+        </is>
+      </c>
+    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
@@ -5286,6 +5615,7 @@
         <v/>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
@@ -5446,22 +5776,22 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Noppen sets</t>
+          <t>Zakken</t>
         </is>
       </c>
       <c r="B26">
-        <f>Parameters!B11</f>
+        <f>Parameters!B15</f>
         <v/>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Artikelkosten noppen</t>
+          <t>Artikelkosten</t>
         </is>
       </c>
       <c r="B27" s="5">
-        <f>B26*136.58</f>
+        <f>B26*14.87</f>
         <v/>
       </c>
     </row>
@@ -5479,22 +5809,29 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Verzending Elektramat (formule)</t>
+          <t>Verzending pallet</t>
         </is>
       </c>
       <c r="B29" s="5">
-        <f>E5</f>
+        <f>IF(B28&gt;=600,0,60.5)</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Let op lengtevracht noppenplaten — check Elektramat bij bestelling</t>
-        </is>
-      </c>
-      <c r="B30" s="5" t="n"/>
-    </row>
+          <t>All-in egaline</t>
+        </is>
+      </c>
+      <c r="B30" s="5">
+        <f>B27+B29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5557,218 +5894,132 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>KWALITATIEF BESTE — harde vloer zonder golven (aug 2026)</t>
+          <t>KWALITEIT binnen 30 mm op BETON (aug 2026)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Keuze: nat Magnum 16 mm + noppenplaat 28 mm + zandcement ≥50 mm. SlimFit/egaline bewust verlaten.</t>
-        </is>
-      </c>
-    </row>
+          <t>Randvoorwaarden: beton + max. 3 cm totale VV-opbouw → nat 16 mm/zandcement onmogelijk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>KOPJE: Vloerverwarming — systeemkeuze</t>
+          <t>Beste haalbare keuze</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Keuze</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Was</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Waarom</t>
+          <t>MAGNUM SlimFit 12 + PE-RT 12×1,5 + Kreisel 418 vezel-egaline tot 22 mm (tot 30 mm max)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SYSTEEM (kern)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>MAGNUM noppenplaat 28 mm (150 kPa)</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>UPGRADE</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>SlimFit 12 matten</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Stijvere basis + buis in noppen; daarna massieve zandcement.</t>
-        </is>
-      </c>
-    </row>
+          <t>Waarom: Magnum-spec 17–22 mm past ruim in 30 mm. Beton = stijve ondergrond → veel minder “golven” dan op hout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MAGNUM PE-RT 16×2</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>UPGRADE</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>PE-RT 12×1,5 SlimFit</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Standaard natte-systeem diameter.</t>
+          <t>Bewust afgewezen</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Zandcement ≥50 mm boven buis</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>UPGRADE</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Kreisel 418 egaline ~18 mm</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Dít maakt de vloer hard. Magnum eist min. 5 cm.</t>
+          <t>• Nat 16 mm + zandcement ≥50 mm: te hoog (~70–90 mm).</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Krimpnet 100×100</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>UPGRADE</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>(niet in SlimFit-BOM)</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Scheurbeheersing in cementdekvloer.</t>
+          <t>• Noppenplaat 28 mm: al ~28 mm zonder dekvloer → past niet + dekvloer.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>NMC Climasol / VTE Composiet / Möhlenhoff / Tado bedraad</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>behouden</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Al kwaliteitskeuzes.</t>
-        </is>
-      </c>
-    </row>
+          <t>• Heatboard droog: mogelijk, maar egaline-sandwich op beton is hier massiever/harder voor dezelfde hoogte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Bewust niet gekozen</t>
+          <t>Tips hardheid</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>• SlimFit + egaline: laagste opbouw, meer kans op “golven”.</t>
+          <t>1) Primer op beton. 2) Matten goed verlijmen. 3) Egaline tot min. 22 mm, liever dichter bij 28–30 mm als hoogte toelaat.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>• Noppenplaat 47 mm akoestisch: lagere max. belasting → zachter.</t>
+          <t>4) Afwerking: tegels &gt; PVC/laminaat voor het hardste gevoel (tegeldikte komt BOVENOP de 30 mm VV-opbouw).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>• Droogbouw/Heatboard: niet dezelfde massieve cementvloer-hardheid.</t>
-        </is>
-      </c>
-    </row>
+          <t>5) Geen zachte ondervloer tussen beton en SlimFit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Absoluut hardst (als bestaande dekvloer geschikt is)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>INFREZEN in bestaande zandcement/anhydriet — laat beoordelen door freesbedrijf.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Opbouw (indicatief): noppen 28 + buis 16 + ≥50 mm cement ≈ 70–90 mm. Check deurdorpels.</t>
-        </is>
-      </c>
-    </row>
+          <t>Behouden upgrades: NMC Climasol, VTE Composiet+Grundfos, Möhlenhoff Alpha 5, Tado bedraad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
+    <row r="20"/>
+    <row r="21"/>
+    <row r="22"/>
+    <row r="23"/>
+    <row r="24"/>
+    <row r="25"/>
+    <row r="26"/>
+    <row r="27"/>
+    <row r="28"/>
+    <row r="29"/>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5780,20 +6031,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Prijszoek – duurste items kwalitatief-beste BOM (aug 2026)</t>
+          <t>Prijszoek – SlimFit-BOM (beton, max 30 mm)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Focus: noppen/buis/verdeler/dekvloer.</t>
+          <t>Gezocht NL + DE webshops, 22 aug 2026. Alleen gewijzigd als aantoonbaar goedkoper én binnen levertijd.</t>
         </is>
       </c>
     </row>
@@ -5805,17 +6056,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Item</t>
+          <t>Item (regeltotaal)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Gekozen</t>
+          <t>Was</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Alternatief</t>
+          <t>Beste gevonden</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -5825,62 +6076,66 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Δ</t>
+          <t>Besparing</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>1</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Noppenplaat 28 mm 3×10 m²</t>
+          <t>MAGNUM SlimFit 12 matten (8×)</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Elektramat €136,58/set</t>
+          <t>Elektramat €86,94/st (€695,52)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>17 mm ongeïsoleerd €102,55 (alleen als al geïsoleerd)</t>
+          <t>Bouwmaat €86,50 (geen voorraad/bezorging); VihamiJ €86,36 excl=duurder + 3–4 wkn; overige ≥€88,99</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>BEHOUDEN 28 mm</t>
+          <t>BEHOUDEN Elektramat</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>kwaliteit</t>
+          <t>€0</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>2</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PE-RT 16×2 240 m</t>
+          <t>Kreisel 418 egaline (33×)</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Elektramat €158,99</t>
+          <t>EgalineXXL €14,87/st (€490,71)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2×120 m ≈ gelijk</t>
+          <t>RBMB ≥€16,55/st (bulkpas pas vanaf 41); geen goedkopere met snelle levering</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>BEHOUDEN</t>
+          <t>BEHOUDEN EgalineXXL</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -5890,57 +6145,61 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>3</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Zandcement 30 m²</t>
+          <t>VTE Composiet 4-groeps + Grundfos</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Indicatie €35/m² = €1.050</t>
+          <t>123Installatieshop €387,18</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Lokaal €25–55/m²</t>
+          <t>CVTotaal €423; VV-shop €404,95; Bouwbestel €440; Jan de Isolatieman €469</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>OFFERTE</t>
+          <t>BEHOUDEN 123Installatieshop</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>variabel</t>
+          <t>€0</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>4</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>VTE Composiet 4-gr.</t>
+          <t>MAGNUM PE-RT 12×1,5 300 m</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>123shop €387,18</t>
+          <t>123InstallatieMaterialen €142,93</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>andere shops hoger</t>
+          <t>Klusspullen €141,95 maar voorraad 0 / levertijd 1–2 wkn → afgewezen; Elektramat €181,86; VV-shop €164,70</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>BEHOUDEN</t>
+          <t>BEHOUDEN 123IM</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -5950,39 +6209,108 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>5</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5a</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Möhlenhoff ×4</t>
+          <t>Möhlenhoff Alpha 5 ×4 (altijd)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>eibhandel + ship ~€55</t>
+          <t>VerwarmingOnline €20,12 → €80,48</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>VerwarmingOnline duurder</t>
+          <t>eibhandel.de €9,99 + NL-verzending ~€15,41 = ~€55,37; Amazon.nl ~€13,16/st met Prime</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BEHOUDEN</t>
+          <t>GEWIJZIGD → eibhandel</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>beste</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>• SlimFit-pad bewust verlaten. Infrezen: apart offerte freesbedrijf.</t>
+          <t>~€25</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>5b</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>MAGNUM H64-CC + master (optie)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>123IM €213,74</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Warp Systems €194,92 (1 wd)</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>GEWIJZIGD → Warp</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>~€19</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Niet meegenomen</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>• PioTek DE (~€9,90): verzendt niet meer naar NL.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>• Bouwmaat SlimFit €86,50: tijdelijk niet beschikbaar / geen bezorging.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>• Klusspullen PE-RT €141,95: goedkoper op papier, maar 0 voorraad / 1–2 weken.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>• Tado: officiële tado° Shop blijft goedkoopst (bol/retail vaak duurder).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>All-in met verzending: zie sheet Verzending (egaline pallet + eibhandel DE→NL).</t>
         </is>
       </c>
     </row>

</xml_diff>